<commit_message>
Fixed error at EV calculation
</commit_message>
<xml_diff>
--- a/AAPL.xlsx
+++ b/AAPL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/KINGSTON/MyStockData/Finance-StockLists/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E15C707B-16D4-BA43-B121-A09F2792B191}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B229DD2F-3C74-9541-9B5C-BEC699157B91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14400" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14400" firstSheet="7" activeTab="17" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -119,7 +119,7 @@
       </extLst>
     </bk>
   </futureMetadata>
-  <futureMetadata name="XLRICHVALUE" count="5">
+  <futureMetadata name="XLRICHVALUE" count="2">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
@@ -130,28 +130,7 @@
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="3"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="4"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
           <xlrd:rvb i="5"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="8"/>
         </ext>
       </extLst>
     </bk>
@@ -161,21 +140,12 @@
       <rc t="1" v="0"/>
     </bk>
   </cellMetadata>
-  <valueMetadata count="5">
+  <valueMetadata count="2">
     <bk>
       <rc t="2" v="0"/>
     </bk>
     <bk>
       <rc t="2" v="1"/>
-    </bk>
-    <bk>
-      <rc t="2" v="2"/>
-    </bk>
-    <bk>
-      <rc t="2" v="3"/>
-    </bk>
-    <bk>
-      <rc t="2" v="4"/>
     </bk>
   </valueMetadata>
 </metadata>
@@ -2342,10 +2312,42 @@
     <xf numFmtId="39" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="10" fontId="0" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="39" fontId="10" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="7" fillId="9" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="18" fillId="17" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="18" fillId="17" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2357,36 +2359,6 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="18" fillId="17" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="18" fillId="17" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2396,8 +2368,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="7" fillId="9" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -15516,7 +15486,7 @@
 </file>
 
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="9">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="6">
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1mou2&amp;q=XNAS%3aAAPL&amp;form=skydnc</v>
     <v>Learn more on Bing</v>
@@ -15536,8 +15506,10 @@
     <v>345.34</v>
     <v>243.42</v>
     <v>1.0718000000000001</v>
-    <v>4.3049999999999997</v>
-    <v>1.2816000000000001E-2</v>
+    <v>5.15</v>
+    <v>1.5330999999999999E-2</v>
+    <v>-0.21</v>
+    <v>-6.1569999999999995E-4</v>
     <v>USD</v>
     <v>Apple Inc. designs, manufactures and markets smartphones, personal computers, tablets, wearables and accessories, and sells a variety of related services. Its product categories include iPhone, Mac, iPad, Wearables, Home and Accessories. Its services include advertising, AppleCare, cloud services, digital content, and payment services. The Company operates various platforms, including the App Store, that allow customers to discover and download applications and digital content, such as books, music, video, games and podcasts. It also offers digital content through subscription-based services, including Apple Arcade, Apple Fitness+, Apple Music, Apple News+, and Apple TV+. Its wearables include smartwatches, wireless headphones, and spatial computers. Its products include iPhone 16 Pro, iPhone 16, iPhone 15, iPhone 14, iPhone SE, MacBook Air, MacBook Pro, iMac, Mac mini, Mac Studio, Mac Pro, iPad Pro, iPad Air, AirPods, AirPods Pro, AirPods Max, Apple TV, Apple Vision Pro and others.</v>
     <v>166000</v>
@@ -15545,49 +15517,35 @@
     <v>XNAS</v>
     <v>XNAS</v>
     <v>One Apple Park Way, CUPERTINO, CA, 95014 US</v>
-    <v>340.48</v>
+    <v>341.67</v>
     <v>Computers, Phones &amp; Household Electronics</v>
     <v>Stock</v>
-    <v>46290.815623495313</v>
+    <v>46290.841611724216</v>
     <v>0</v>
     <v>334.53</v>
-    <v>4965304890500</v>
+    <v>4977636972600</v>
     <v>APPLE INC.</v>
     <v>APPLE INC.</v>
     <v>335.92</v>
-    <v>39.148600000000002</v>
+    <v>39.245899999999999</v>
     <v>335.92</v>
-    <v>340.22500000000002</v>
+    <v>341.07</v>
+    <v>340.86</v>
     <v>14594180000</v>
     <v>AAPL</v>
     <v>APPLE INC. (XNAS:AAPL)</v>
-    <v>18921928</v>
+    <v>29401485</v>
     <v>41709089</v>
     <v>1977</v>
   </rv>
   <rv s="2">
     <v>1</v>
   </rv>
-  <rv s="3">
-    <v>12</v>
-    <v>Price (Extended hours)</v>
-    <v>0</v>
-  </rv>
-  <rv s="3">
-    <v>12</v>
-    <v>Change (extended hours)</v>
-    <v>0</v>
-  </rv>
-  <rv s="3">
-    <v>12</v>
-    <v>Change % (extended hours)</v>
-    <v>0</v>
-  </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a33knm&amp;q=10+Y+TSY+YLD+NDX&amp;form=skydnc</v>
     <v>Learn more on Bing</v>
   </rv>
-  <rv s="4">
+  <rv s="3">
     <v>5</v>
     <v>10 Y TSY YLD NDX</v>
     <v>6</v>
@@ -15606,7 +15564,7 @@
     <v>US</v>
     <v>51.81</v>
     <v>Index</v>
-    <v>6</v>
+    <v>3</v>
     <v>50.87</v>
     <v>10 Y TSY YLD NDX</v>
     <v>51.21</v>
@@ -15616,13 +15574,13 @@
     <v>10 Y TSY YLD NDX</v>
   </rv>
   <rv s="2">
-    <v>7</v>
+    <v>4</v>
   </rv>
 </rvData>
 </file>
 
 <file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
-<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="5">
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="4">
   <s t="_hyperlink">
     <k n="Address" t="s"/>
     <k n="Text" t="s"/>
@@ -15644,6 +15602,8 @@
     <k n="Beta"/>
     <k n="Change"/>
     <k n="Change (%)"/>
+    <k n="Change (Extended hours)"/>
+    <k n="Change % (Extended hours)"/>
     <k n="Currency" t="s"/>
     <k n="Description" t="s"/>
     <k n="Employees"/>
@@ -15664,6 +15624,7 @@
     <k n="P/E"/>
     <k n="Previous close"/>
     <k n="Price"/>
+    <k n="Price (Extended hours)"/>
     <k n="Shares outstanding"/>
     <k n="Ticker symbol" t="s"/>
     <k n="UniqueName" t="s"/>
@@ -15673,11 +15634,6 @@
   </s>
   <s t="_linkedentity">
     <k n="%cvi" t="r"/>
-  </s>
-  <s t="_error">
-    <k n="errorType" t="i"/>
-    <k n="field" t="s"/>
-    <k n="subType" t="i"/>
   </s>
   <s t="_linkedentitycore">
     <k n="_Display" t="spb"/>
@@ -15713,7 +15669,7 @@
 <file path=xl/richData/rdsupportingpropertybag.xml><?xml version="1.0" encoding="utf-8"?>
 <supportingPropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2">
   <spbArrays count="2">
-    <a count="42">
+    <a count="45">
       <v t="s">%EntityServiceId</v>
       <v t="s">_Format</v>
       <v t="s">%IsRefreshable</v>
@@ -15724,13 +15680,16 @@
       <v t="s">Name</v>
       <v t="s">_SubLabel</v>
       <v t="s">Price</v>
+      <v t="s">Price (Extended hours)</v>
       <v t="s">Exchange</v>
       <v t="s">Official name</v>
       <v t="s">Last trade time</v>
       <v t="s">Ticker symbol</v>
       <v t="s">Exchange abbreviation</v>
       <v t="s">Change</v>
+      <v t="s">Change (Extended hours)</v>
       <v t="s">Change (%)</v>
+      <v t="s">Change % (Extended hours)</v>
       <v t="s">Currency</v>
       <v t="s">Previous close</v>
       <v t="s">Open</v>
@@ -15824,13 +15783,19 @@
       <v>8</v>
       <v>9</v>
       <v>4</v>
+      <v>1</v>
+      <v>1</v>
+      <v>5</v>
     </spb>
     <spb s="4">
-      <v>Real-Time Nasdaq Last Sale</v>
+      <v>at close</v>
       <v>from previous close</v>
       <v>from previous close</v>
       <v>Source: Nasdaq Last Sale</v>
       <v>GMT</v>
+      <v>Real-Time Nasdaq Last Sale</v>
+      <v>from close</v>
+      <v>from close</v>
     </spb>
     <spb s="0">
       <v>1</v>
@@ -15902,6 +15867,9 @@
     <k n="Year incorporated" t="i"/>
     <k n="`%EntityServiceId" t="i"/>
     <k n="Shares outstanding" t="i"/>
+    <k n="Price (Extended hours)" t="i"/>
+    <k n="Change (Extended hours)" t="i"/>
+    <k n="Change % (Extended hours)" t="i"/>
   </s>
   <s>
     <k n="Price" t="s"/>
@@ -15909,6 +15877,9 @@
     <k n="Change (%)" t="s"/>
     <k n="ExchangeID" t="s"/>
     <k n="Last trade time" t="s"/>
+    <k n="Price (Extended hours)" t="s"/>
+    <k n="Change (Extended hours)" t="s"/>
+    <k n="Change % (Extended hours)" t="s"/>
   </s>
   <s>
     <k n="UniqueName" t="spb"/>
@@ -16393,18 +16364,18 @@
   <sheetData>
     <row r="1" spans="2:9" ht="11" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="2" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="239" t="s">
+      <c r="B2" s="237" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="240"/>
-      <c r="E2" s="239" t="s">
+      <c r="C2" s="238"/>
+      <c r="E2" s="237" t="s">
         <v>281</v>
       </c>
-      <c r="F2" s="240"/>
-      <c r="H2" s="239" t="s">
+      <c r="F2" s="238"/>
+      <c r="H2" s="237" t="s">
         <v>319</v>
       </c>
-      <c r="I2" s="240"/>
+      <c r="I2" s="238"/>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B3" s="179" t="s">
@@ -16419,7 +16390,7 @@
       </c>
       <c r="F3" s="181">
         <f ca="1">Statement!AC143</f>
-        <v>4985316.9250000007</v>
+        <v>4997698.71</v>
       </c>
       <c r="H3" s="179" t="str">
         <f>'AVG target price'!B5</f>
@@ -16427,7 +16398,7 @@
       </c>
       <c r="I3" s="205">
         <f ca="1">'AVG target price'!C5</f>
-        <v>114.58092461460862</v>
+        <v>114.57736714629849</v>
       </c>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.2">
@@ -16443,7 +16414,7 @@
       </c>
       <c r="F4" s="182">
         <f ca="1">Statement!AC144</f>
-        <v>4923143.9250000007</v>
+        <v>4935525.71</v>
       </c>
       <c r="H4" s="179" t="str">
         <f>'AVG target price'!B6</f>
@@ -16451,7 +16422,7 @@
       </c>
       <c r="I4" s="205">
         <f ca="1">'AVG target price'!C6</f>
-        <v>231.99401211300611</v>
+        <v>229.68744916265044</v>
       </c>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.2">
@@ -16460,7 +16431,7 @@
       </c>
       <c r="C5" s="202" cm="1">
         <f t="array" aca="1" ref="C5" ca="1">_FV(C3,"Price",TRUE)</f>
-        <v>340.22500000000002</v>
+        <v>341.07</v>
       </c>
       <c r="E5" s="179" t="s">
         <v>237</v>
@@ -16482,16 +16453,16 @@
       <c r="B6" s="179" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="202" t="e" cm="1" vm="2">
-        <f t="array" ref="C6">_FV(C3,"Price (Extended hours)",TRUE)</f>
-        <v>#VALUE!</v>
+      <c r="C6" s="202" cm="1">
+        <f t="array" aca="1" ref="C6" ca="1">_FV(C3,"Price (Extended hours)",TRUE)</f>
+        <v>340.86</v>
       </c>
       <c r="E6" s="179" t="s">
         <v>231</v>
       </c>
       <c r="F6" s="184">
         <f ca="1">Statement!AC140</f>
-        <v>39.016628440366979</v>
+        <v>39.113532110091747</v>
       </c>
       <c r="H6" s="179" t="str">
         <f>'AVG target price'!B8</f>
@@ -16499,7 +16470,7 @@
       </c>
       <c r="I6" s="205">
         <f ca="1">'AVG target price'!C8</f>
-        <v>153.58097582972349</v>
+        <v>151.27529713145577</v>
       </c>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.2">
@@ -16508,14 +16479,14 @@
       </c>
       <c r="C7" s="6" cm="1">
         <f t="array" aca="1" ref="C7" ca="1">_FV(C3,"Change")</f>
-        <v>4.3049999999999997</v>
+        <v>5.15</v>
       </c>
       <c r="E7" s="180" t="s">
         <v>198</v>
       </c>
       <c r="F7" s="185">
         <f ca="1">Statement!AC141</f>
-        <v>10.770892219856348</v>
+        <v>10.797643351977086</v>
       </c>
       <c r="H7" s="178" t="str">
         <f>'AVG target price'!B9</f>
@@ -16523,23 +16494,23 @@
       </c>
       <c r="I7" s="206">
         <f ca="1">'AVG target price'!C9</f>
-        <v>175.35263739282055</v>
+        <v>174.1986876135872</v>
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B8" s="179" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="6" t="e" cm="1" vm="3">
-        <f t="array" ref="C8">_FV(C3,"Change (extended hours)",TRUE)</f>
-        <v>#VALUE!</v>
+      <c r="C8" s="6" cm="1">
+        <f t="array" aca="1" ref="C8" ca="1">_FV(C3,"Change (extended hours)",TRUE)</f>
+        <v>-0.21</v>
       </c>
       <c r="E8" s="179" t="s">
         <v>259</v>
       </c>
       <c r="F8" s="186">
         <f ca="1">Statement!AC151</f>
-        <v>2.4667839948811273E-2</v>
+        <v>2.4606725442238592E-2</v>
       </c>
       <c r="H8" s="178" t="str">
         <f>'AVG target price'!B11</f>
@@ -16547,7 +16518,7 @@
       </c>
       <c r="I8" s="207">
         <f ca="1">'AVG target price'!C11</f>
-        <v>-0.48459802368191479</v>
+        <v>-0.4892582531046788</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
@@ -16556,30 +16527,30 @@
       </c>
       <c r="C9" s="73" cm="1">
         <f t="array" aca="1" ref="C9" ca="1">_FV(C3,"Change (%)",TRUE)</f>
-        <v>1.2816000000000001E-2</v>
+        <v>1.5330999999999999E-2</v>
       </c>
       <c r="E9" s="179" t="s">
         <v>282</v>
       </c>
       <c r="F9" s="186">
         <f ca="1">Statement!AC152</f>
-        <v>2.5630097729443746E-2</v>
+        <v>2.5566599231829239E-2</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B10" s="179" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="73" t="e" cm="1" vm="4">
-        <f t="array" ref="C10">_FV(C3,"Change % (extended hours)",TRUE)</f>
-        <v>#VALUE!</v>
+      <c r="C10" s="73" cm="1">
+        <f t="array" aca="1" ref="C10" ca="1">_FV(C3,"Change % (extended hours)",TRUE)</f>
+        <v>-6.1569999999999995E-4</v>
       </c>
       <c r="E10" s="179" t="s">
         <v>287</v>
       </c>
       <c r="F10" s="186">
         <f ca="1">Statement!AC154</f>
-        <v>1.6493635457288401E-2</v>
+        <v>1.6452772520174592E-2</v>
       </c>
       <c r="H10" s="178" t="s">
         <v>394</v>
@@ -16602,7 +16573,7 @@
       </c>
       <c r="F11" s="187">
         <f ca="1">Statement!AC153</f>
-        <v>3.0861929605408185E-3</v>
+        <v>3.0785469258509984E-3</v>
       </c>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.2">
@@ -16659,7 +16630,7 @@
       </c>
       <c r="F15" s="186">
         <f ca="1">Statement!AC166</f>
-        <v>1.2471223181061851E-2</v>
+        <v>1.2440325759453395E-2</v>
       </c>
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.2">
@@ -16672,10 +16643,10 @@
       </c>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B17" s="241" t="s">
+      <c r="B17" s="239" t="s">
         <v>88</v>
       </c>
-      <c r="C17" s="241"/>
+      <c r="C17" s="239"/>
       <c r="E17" s="178" t="s">
         <v>290</v>
       </c>
@@ -16748,14 +16719,14 @@
       </c>
     </row>
     <row r="25" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B25" s="241" t="s">
+      <c r="B25" s="239" t="s">
         <v>104</v>
       </c>
-      <c r="C25" s="241"/>
-      <c r="E25" s="239" t="s">
+      <c r="C25" s="239"/>
+      <c r="E25" s="237" t="s">
         <v>332</v>
       </c>
-      <c r="F25" s="240"/>
+      <c r="F25" s="238"/>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B26" s="178" t="s">
@@ -16764,7 +16735,7 @@
       <c r="C26" s="164">
         <v>0.21</v>
       </c>
-      <c r="E26" s="179" t="e" vm="5">
+      <c r="E26" s="179" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
       <c r="F26" s="213" cm="1">
@@ -16804,15 +16775,15 @@
       </c>
     </row>
     <row r="33" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B33" s="235" t="s">
+      <c r="B33" s="236" t="s">
         <v>327</v>
       </c>
-      <c r="C33" s="235"/>
-      <c r="D33" s="235"/>
-      <c r="E33" s="235"/>
-      <c r="F33" s="235"/>
-      <c r="G33" s="235"/>
-      <c r="H33" s="235"/>
+      <c r="C33" s="236"/>
+      <c r="D33" s="236"/>
+      <c r="E33" s="236"/>
+      <c r="F33" s="236"/>
+      <c r="G33" s="236"/>
+      <c r="H33" s="236"/>
     </row>
     <row r="35" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B35" s="16" t="s">
@@ -16831,24 +16802,24 @@
       </c>
     </row>
     <row r="39" spans="2:8" ht="6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B39" s="235"/>
-      <c r="C39" s="235"/>
-      <c r="D39" s="235"/>
-      <c r="E39" s="235"/>
-      <c r="F39" s="235"/>
-      <c r="G39" s="235"/>
-      <c r="H39" s="235"/>
+      <c r="B39" s="236"/>
+      <c r="C39" s="236"/>
+      <c r="D39" s="236"/>
+      <c r="E39" s="236"/>
+      <c r="F39" s="236"/>
+      <c r="G39" s="236"/>
+      <c r="H39" s="236"/>
     </row>
     <row r="42" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B42" s="235" t="s">
+      <c r="B42" s="236" t="s">
         <v>330</v>
       </c>
-      <c r="C42" s="235"/>
-      <c r="D42" s="235"/>
-      <c r="E42" s="235"/>
-      <c r="F42" s="235"/>
-      <c r="G42" s="235"/>
-      <c r="H42" s="235"/>
+      <c r="C42" s="236"/>
+      <c r="D42" s="236"/>
+      <c r="E42" s="236"/>
+      <c r="F42" s="236"/>
+      <c r="G42" s="236"/>
+      <c r="H42" s="236"/>
     </row>
     <row r="44" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B44" s="41" t="s">
@@ -16863,24 +16834,24 @@
       </c>
     </row>
     <row r="49" spans="2:8" ht="5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B49" s="235"/>
-      <c r="C49" s="235"/>
-      <c r="D49" s="235"/>
-      <c r="E49" s="235"/>
-      <c r="F49" s="235"/>
-      <c r="G49" s="235"/>
-      <c r="H49" s="235"/>
+      <c r="B49" s="236"/>
+      <c r="C49" s="236"/>
+      <c r="D49" s="236"/>
+      <c r="E49" s="236"/>
+      <c r="F49" s="236"/>
+      <c r="G49" s="236"/>
+      <c r="H49" s="236"/>
     </row>
     <row r="52" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B52" s="235" t="s">
+      <c r="B52" s="236" t="s">
         <v>106</v>
       </c>
-      <c r="C52" s="235"/>
-      <c r="D52" s="235"/>
-      <c r="E52" s="235"/>
-      <c r="F52" s="235"/>
-      <c r="G52" s="235"/>
-      <c r="H52" s="235"/>
+      <c r="C52" s="236"/>
+      <c r="D52" s="236"/>
+      <c r="E52" s="236"/>
+      <c r="F52" s="236"/>
+      <c r="G52" s="236"/>
+      <c r="H52" s="236"/>
     </row>
     <row r="54" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B54" s="41" t="s">
@@ -16895,28 +16866,28 @@
       </c>
     </row>
     <row r="59" spans="2:8" ht="5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B59" s="235"/>
-      <c r="C59" s="235"/>
-      <c r="D59" s="235"/>
-      <c r="E59" s="235"/>
-      <c r="F59" s="235"/>
-      <c r="G59" s="235"/>
-      <c r="H59" s="235"/>
+      <c r="B59" s="236"/>
+      <c r="C59" s="236"/>
+      <c r="D59" s="236"/>
+      <c r="E59" s="236"/>
+      <c r="F59" s="236"/>
+      <c r="G59" s="236"/>
+      <c r="H59" s="236"/>
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="E25:F25"/>
     <mergeCell ref="B52:H52"/>
     <mergeCell ref="B59:H59"/>
     <mergeCell ref="B33:H33"/>
     <mergeCell ref="B39:H39"/>
     <mergeCell ref="B42:H42"/>
     <mergeCell ref="B49:H49"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="E2:F2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="E25:F25"/>
   </mergeCells>
   <conditionalFormatting sqref="C7:C10">
     <cfRule type="cellIs" dxfId="2" priority="4" operator="lessThan">
@@ -16986,36 +16957,36 @@
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
-      <c r="C2" s="235" t="s">
+      <c r="C2" s="236" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="235"/>
-      <c r="E2" s="235"/>
-      <c r="F2" s="235"/>
-      <c r="G2" s="236"/>
-      <c r="H2" s="237" t="s">
+      <c r="D2" s="236"/>
+      <c r="E2" s="236"/>
+      <c r="F2" s="236"/>
+      <c r="G2" s="248"/>
+      <c r="H2" s="249" t="s">
         <v>111</v>
       </c>
-      <c r="I2" s="235"/>
-      <c r="J2" s="235"/>
-      <c r="K2" s="235"/>
-      <c r="L2" s="235"/>
+      <c r="I2" s="236"/>
+      <c r="J2" s="236"/>
+      <c r="K2" s="236"/>
+      <c r="L2" s="236"/>
       <c r="O2" s="5"/>
-      <c r="S2" s="235" t="s">
+      <c r="S2" s="236" t="s">
         <v>110</v>
       </c>
-      <c r="T2" s="235"/>
-      <c r="U2" s="235"/>
-      <c r="V2" s="235"/>
-      <c r="W2" s="235"/>
-      <c r="X2" s="235"/>
-      <c r="Y2" s="235"/>
-      <c r="Z2" s="235"/>
-      <c r="AA2" s="235" t="s">
+      <c r="T2" s="236"/>
+      <c r="U2" s="236"/>
+      <c r="V2" s="236"/>
+      <c r="W2" s="236"/>
+      <c r="X2" s="236"/>
+      <c r="Y2" s="236"/>
+      <c r="Z2" s="236"/>
+      <c r="AA2" s="236" t="s">
         <v>111</v>
       </c>
-      <c r="AB2" s="235"/>
-      <c r="AC2" s="235"/>
+      <c r="AB2" s="236"/>
+      <c r="AC2" s="236"/>
       <c r="AE2" s="85" t="s">
         <v>112</v>
       </c>
@@ -17026,32 +16997,32 @@
     <row r="4" spans="1:31" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="86"/>
       <c r="B4" s="60"/>
-      <c r="C4" s="234" t="s">
+      <c r="C4" s="245" t="s">
         <v>113</v>
       </c>
-      <c r="D4" s="234"/>
-      <c r="E4" s="234"/>
-      <c r="F4" s="234"/>
-      <c r="G4" s="234"/>
-      <c r="H4" s="234"/>
-      <c r="I4" s="234"/>
-      <c r="J4" s="234"/>
-      <c r="K4" s="234"/>
-      <c r="L4" s="234"/>
+      <c r="D4" s="245"/>
+      <c r="E4" s="245"/>
+      <c r="F4" s="245"/>
+      <c r="G4" s="245"/>
+      <c r="H4" s="245"/>
+      <c r="I4" s="245"/>
+      <c r="J4" s="245"/>
+      <c r="K4" s="245"/>
+      <c r="L4" s="245"/>
       <c r="O4" s="5"/>
-      <c r="S4" s="247" t="s">
+      <c r="S4" s="246" t="s">
         <v>113</v>
       </c>
-      <c r="T4" s="248"/>
-      <c r="U4" s="248"/>
-      <c r="V4" s="248"/>
-      <c r="W4" s="248"/>
-      <c r="X4" s="248"/>
-      <c r="Y4" s="248"/>
-      <c r="Z4" s="248"/>
-      <c r="AA4" s="248"/>
-      <c r="AB4" s="248"/>
-      <c r="AC4" s="248"/>
+      <c r="T4" s="247"/>
+      <c r="U4" s="247"/>
+      <c r="V4" s="247"/>
+      <c r="W4" s="247"/>
+      <c r="X4" s="247"/>
+      <c r="Y4" s="247"/>
+      <c r="Z4" s="247"/>
+      <c r="AA4" s="247"/>
+      <c r="AB4" s="247"/>
+      <c r="AC4" s="247"/>
       <c r="AE4" s="87"/>
     </row>
     <row r="5" spans="1:31" x14ac:dyDescent="0.2">
@@ -17739,33 +17710,33 @@
       <c r="Q12" s="91"/>
     </row>
     <row r="13" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="C13" s="234" t="s">
+      <c r="C13" s="245" t="s">
         <v>119</v>
       </c>
-      <c r="D13" s="234"/>
-      <c r="E13" s="234"/>
-      <c r="F13" s="234"/>
-      <c r="G13" s="234"/>
-      <c r="H13" s="234"/>
-      <c r="I13" s="234"/>
-      <c r="J13" s="234"/>
-      <c r="K13" s="234"/>
-      <c r="L13" s="234"/>
+      <c r="D13" s="245"/>
+      <c r="E13" s="245"/>
+      <c r="F13" s="245"/>
+      <c r="G13" s="245"/>
+      <c r="H13" s="245"/>
+      <c r="I13" s="245"/>
+      <c r="J13" s="245"/>
+      <c r="K13" s="245"/>
+      <c r="L13" s="245"/>
       <c r="O13" s="5"/>
       <c r="Q13" s="91"/>
-      <c r="S13" s="247" t="s">
+      <c r="S13" s="246" t="s">
         <v>119</v>
       </c>
-      <c r="T13" s="248"/>
-      <c r="U13" s="248"/>
-      <c r="V13" s="248"/>
-      <c r="W13" s="248"/>
-      <c r="X13" s="248"/>
-      <c r="Y13" s="248"/>
-      <c r="Z13" s="248"/>
-      <c r="AA13" s="248"/>
-      <c r="AB13" s="248"/>
-      <c r="AC13" s="248"/>
+      <c r="T13" s="247"/>
+      <c r="U13" s="247"/>
+      <c r="V13" s="247"/>
+      <c r="W13" s="247"/>
+      <c r="X13" s="247"/>
+      <c r="Y13" s="247"/>
+      <c r="Z13" s="247"/>
+      <c r="AA13" s="247"/>
+      <c r="AB13" s="247"/>
+      <c r="AC13" s="247"/>
     </row>
     <row r="14" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B14" s="16" t="s">
@@ -18386,35 +18357,35 @@
     </row>
     <row r="2" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
-      <c r="C2" s="235" t="s">
+      <c r="C2" s="236" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="235"/>
-      <c r="E2" s="235"/>
-      <c r="F2" s="235"/>
-      <c r="G2" s="236"/>
-      <c r="H2" s="237" t="s">
+      <c r="D2" s="236"/>
+      <c r="E2" s="236"/>
+      <c r="F2" s="236"/>
+      <c r="G2" s="248"/>
+      <c r="H2" s="249" t="s">
         <v>111</v>
       </c>
-      <c r="I2" s="235"/>
-      <c r="J2" s="235"/>
-      <c r="K2" s="235"/>
-      <c r="L2" s="235"/>
-      <c r="P2" s="235" t="s">
+      <c r="I2" s="236"/>
+      <c r="J2" s="236"/>
+      <c r="K2" s="236"/>
+      <c r="L2" s="236"/>
+      <c r="P2" s="236" t="s">
         <v>110</v>
       </c>
-      <c r="Q2" s="235"/>
-      <c r="R2" s="235"/>
-      <c r="S2" s="235"/>
-      <c r="T2" s="235"/>
-      <c r="U2" s="235"/>
-      <c r="V2" s="235"/>
-      <c r="W2" s="235"/>
-      <c r="X2" s="235" t="s">
+      <c r="Q2" s="236"/>
+      <c r="R2" s="236"/>
+      <c r="S2" s="236"/>
+      <c r="T2" s="236"/>
+      <c r="U2" s="236"/>
+      <c r="V2" s="236"/>
+      <c r="W2" s="236"/>
+      <c r="X2" s="236" t="s">
         <v>111</v>
       </c>
-      <c r="Y2" s="235"/>
-      <c r="Z2" s="235"/>
+      <c r="Y2" s="236"/>
+      <c r="Z2" s="236"/>
       <c r="AB2" s="85" t="s">
         <v>112</v>
       </c>
@@ -18423,31 +18394,31 @@
     <row r="4" spans="1:28" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="86"/>
       <c r="B4" s="60"/>
-      <c r="C4" s="234" t="s">
+      <c r="C4" s="245" t="s">
         <v>113</v>
       </c>
-      <c r="D4" s="234"/>
-      <c r="E4" s="234"/>
-      <c r="F4" s="234"/>
-      <c r="G4" s="234"/>
-      <c r="H4" s="234"/>
-      <c r="I4" s="234"/>
-      <c r="J4" s="234"/>
-      <c r="K4" s="234"/>
-      <c r="L4" s="234"/>
-      <c r="P4" s="248" t="s">
+      <c r="D4" s="245"/>
+      <c r="E4" s="245"/>
+      <c r="F4" s="245"/>
+      <c r="G4" s="245"/>
+      <c r="H4" s="245"/>
+      <c r="I4" s="245"/>
+      <c r="J4" s="245"/>
+      <c r="K4" s="245"/>
+      <c r="L4" s="245"/>
+      <c r="P4" s="247" t="s">
         <v>113</v>
       </c>
-      <c r="Q4" s="248"/>
-      <c r="R4" s="248"/>
-      <c r="S4" s="248"/>
-      <c r="T4" s="248"/>
-      <c r="U4" s="248"/>
-      <c r="V4" s="248"/>
-      <c r="W4" s="248"/>
-      <c r="X4" s="248"/>
-      <c r="Y4" s="248"/>
-      <c r="Z4" s="248"/>
+      <c r="Q4" s="247"/>
+      <c r="R4" s="247"/>
+      <c r="S4" s="247"/>
+      <c r="T4" s="247"/>
+      <c r="U4" s="247"/>
+      <c r="V4" s="247"/>
+      <c r="W4" s="247"/>
+      <c r="X4" s="247"/>
+      <c r="Y4" s="247"/>
+      <c r="Z4" s="247"/>
       <c r="AB4" s="87"/>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.2">
@@ -18642,32 +18613,32 @@
       <c r="N8" s="91"/>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="C9" s="234" t="s">
+      <c r="C9" s="245" t="s">
         <v>122</v>
       </c>
-      <c r="D9" s="234"/>
-      <c r="E9" s="234"/>
-      <c r="F9" s="234"/>
-      <c r="G9" s="234"/>
-      <c r="H9" s="234"/>
-      <c r="I9" s="234"/>
-      <c r="J9" s="234"/>
-      <c r="K9" s="234"/>
-      <c r="L9" s="234"/>
+      <c r="D9" s="245"/>
+      <c r="E9" s="245"/>
+      <c r="F9" s="245"/>
+      <c r="G9" s="245"/>
+      <c r="H9" s="245"/>
+      <c r="I9" s="245"/>
+      <c r="J9" s="245"/>
+      <c r="K9" s="245"/>
+      <c r="L9" s="245"/>
       <c r="N9" s="91"/>
-      <c r="P9" s="248" t="s">
+      <c r="P9" s="247" t="s">
         <v>123</v>
       </c>
-      <c r="Q9" s="248"/>
-      <c r="R9" s="248"/>
-      <c r="S9" s="248"/>
-      <c r="T9" s="248"/>
-      <c r="U9" s="248"/>
-      <c r="V9" s="248"/>
-      <c r="W9" s="248"/>
-      <c r="X9" s="248"/>
-      <c r="Y9" s="248"/>
-      <c r="Z9" s="248"/>
+      <c r="Q9" s="247"/>
+      <c r="R9" s="247"/>
+      <c r="S9" s="247"/>
+      <c r="T9" s="247"/>
+      <c r="U9" s="247"/>
+      <c r="V9" s="247"/>
+      <c r="W9" s="247"/>
+      <c r="X9" s="247"/>
+      <c r="Y9" s="247"/>
+      <c r="Z9" s="247"/>
       <c r="AB9" s="87">
         <f>AB4</f>
         <v>0</v>
@@ -19143,31 +19114,31 @@
       </c>
     </row>
     <row r="17" spans="2:26" x14ac:dyDescent="0.2">
-      <c r="C17" s="234" t="s">
+      <c r="C17" s="245" t="s">
         <v>125</v>
       </c>
-      <c r="D17" s="234"/>
-      <c r="E17" s="234"/>
-      <c r="F17" s="234"/>
-      <c r="G17" s="234"/>
-      <c r="H17" s="234"/>
-      <c r="I17" s="234"/>
-      <c r="J17" s="234"/>
-      <c r="K17" s="234"/>
-      <c r="L17" s="234"/>
-      <c r="P17" s="248" t="s">
+      <c r="D17" s="245"/>
+      <c r="E17" s="245"/>
+      <c r="F17" s="245"/>
+      <c r="G17" s="245"/>
+      <c r="H17" s="245"/>
+      <c r="I17" s="245"/>
+      <c r="J17" s="245"/>
+      <c r="K17" s="245"/>
+      <c r="L17" s="245"/>
+      <c r="P17" s="247" t="s">
         <v>125</v>
       </c>
-      <c r="Q17" s="248"/>
-      <c r="R17" s="248"/>
-      <c r="S17" s="248"/>
-      <c r="T17" s="248"/>
-      <c r="U17" s="248"/>
-      <c r="V17" s="248"/>
-      <c r="W17" s="248"/>
-      <c r="X17" s="248"/>
-      <c r="Y17" s="248"/>
-      <c r="Z17" s="248"/>
+      <c r="Q17" s="247"/>
+      <c r="R17" s="247"/>
+      <c r="S17" s="247"/>
+      <c r="T17" s="247"/>
+      <c r="U17" s="247"/>
+      <c r="V17" s="247"/>
+      <c r="W17" s="247"/>
+      <c r="X17" s="247"/>
+      <c r="Y17" s="247"/>
+      <c r="Z17" s="247"/>
     </row>
     <row r="18" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B18" s="16" t="s">
@@ -19645,60 +19616,60 @@
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A3" s="4"/>
-      <c r="C3" s="235" t="s">
+      <c r="C3" s="236" t="s">
         <v>110</v>
       </c>
-      <c r="D3" s="235"/>
-      <c r="E3" s="235"/>
-      <c r="F3" s="235"/>
-      <c r="G3" s="236"/>
-      <c r="H3" s="237" t="s">
+      <c r="D3" s="236"/>
+      <c r="E3" s="236"/>
+      <c r="F3" s="236"/>
+      <c r="G3" s="248"/>
+      <c r="H3" s="249" t="s">
         <v>111</v>
       </c>
-      <c r="I3" s="235"/>
-      <c r="J3" s="235"/>
-      <c r="K3" s="235"/>
-      <c r="L3" s="235"/>
-      <c r="P3" s="238"/>
-      <c r="Q3" s="238"/>
-      <c r="R3" s="238"/>
-      <c r="S3" s="238"/>
-      <c r="T3" s="238"/>
-      <c r="U3" s="238"/>
-      <c r="V3" s="238"/>
-      <c r="W3" s="238"/>
-      <c r="X3" s="238"/>
-      <c r="Y3" s="238"/>
-      <c r="Z3" s="238"/>
+      <c r="I3" s="236"/>
+      <c r="J3" s="236"/>
+      <c r="K3" s="236"/>
+      <c r="L3" s="236"/>
+      <c r="P3" s="250"/>
+      <c r="Q3" s="250"/>
+      <c r="R3" s="250"/>
+      <c r="S3" s="250"/>
+      <c r="T3" s="250"/>
+      <c r="U3" s="250"/>
+      <c r="V3" s="250"/>
+      <c r="W3" s="250"/>
+      <c r="X3" s="250"/>
+      <c r="Y3" s="250"/>
+      <c r="Z3" s="250"/>
       <c r="AB3" s="109"/>
     </row>
     <row r="4" spans="1:28" ht="10" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="5" spans="1:28" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="86"/>
       <c r="B5" s="60"/>
-      <c r="C5" s="234" t="s">
+      <c r="C5" s="245" t="s">
         <v>113</v>
       </c>
-      <c r="D5" s="234"/>
-      <c r="E5" s="234"/>
-      <c r="F5" s="234"/>
-      <c r="G5" s="234"/>
-      <c r="H5" s="234"/>
-      <c r="I5" s="234"/>
-      <c r="J5" s="234"/>
-      <c r="K5" s="234"/>
-      <c r="L5" s="234"/>
-      <c r="P5" s="238"/>
-      <c r="Q5" s="238"/>
-      <c r="R5" s="238"/>
-      <c r="S5" s="238"/>
-      <c r="T5" s="238"/>
-      <c r="U5" s="238"/>
-      <c r="V5" s="238"/>
-      <c r="W5" s="238"/>
-      <c r="X5" s="238"/>
-      <c r="Y5" s="238"/>
-      <c r="Z5" s="238"/>
+      <c r="D5" s="245"/>
+      <c r="E5" s="245"/>
+      <c r="F5" s="245"/>
+      <c r="G5" s="245"/>
+      <c r="H5" s="245"/>
+      <c r="I5" s="245"/>
+      <c r="J5" s="245"/>
+      <c r="K5" s="245"/>
+      <c r="L5" s="245"/>
+      <c r="P5" s="250"/>
+      <c r="Q5" s="250"/>
+      <c r="R5" s="250"/>
+      <c r="S5" s="250"/>
+      <c r="T5" s="250"/>
+      <c r="U5" s="250"/>
+      <c r="V5" s="250"/>
+      <c r="W5" s="250"/>
+      <c r="X5" s="250"/>
+      <c r="Y5" s="250"/>
+      <c r="Z5" s="250"/>
       <c r="AB5" s="110"/>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.2">
@@ -19884,30 +19855,30 @@
       <c r="N10" s="91"/>
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="C11" s="234" t="s">
+      <c r="C11" s="245" t="s">
         <v>129</v>
       </c>
-      <c r="D11" s="234"/>
-      <c r="E11" s="234"/>
-      <c r="F11" s="234"/>
-      <c r="G11" s="234"/>
-      <c r="H11" s="234"/>
-      <c r="I11" s="234"/>
-      <c r="J11" s="234"/>
-      <c r="K11" s="234"/>
-      <c r="L11" s="234"/>
+      <c r="D11" s="245"/>
+      <c r="E11" s="245"/>
+      <c r="F11" s="245"/>
+      <c r="G11" s="245"/>
+      <c r="H11" s="245"/>
+      <c r="I11" s="245"/>
+      <c r="J11" s="245"/>
+      <c r="K11" s="245"/>
+      <c r="L11" s="245"/>
       <c r="N11" s="91"/>
-      <c r="P11" s="238"/>
-      <c r="Q11" s="238"/>
-      <c r="R11" s="238"/>
-      <c r="S11" s="238"/>
-      <c r="T11" s="238"/>
-      <c r="U11" s="238"/>
-      <c r="V11" s="238"/>
-      <c r="W11" s="238"/>
-      <c r="X11" s="238"/>
-      <c r="Y11" s="238"/>
-      <c r="Z11" s="238"/>
+      <c r="P11" s="250"/>
+      <c r="Q11" s="250"/>
+      <c r="R11" s="250"/>
+      <c r="S11" s="250"/>
+      <c r="T11" s="250"/>
+      <c r="U11" s="250"/>
+      <c r="V11" s="250"/>
+      <c r="W11" s="250"/>
+      <c r="X11" s="250"/>
+      <c r="Y11" s="250"/>
+      <c r="Z11" s="250"/>
       <c r="AB11" s="110"/>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.2">
@@ -20149,18 +20120,18 @@
       <c r="D16" s="24"/>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="C18" s="234" t="s">
+      <c r="C18" s="245" t="s">
         <v>134</v>
       </c>
-      <c r="D18" s="234"/>
-      <c r="E18" s="234"/>
-      <c r="F18" s="234"/>
-      <c r="G18" s="234"/>
-      <c r="H18" s="234"/>
-      <c r="I18" s="234"/>
-      <c r="J18" s="234"/>
-      <c r="K18" s="234"/>
-      <c r="L18" s="234"/>
+      <c r="D18" s="245"/>
+      <c r="E18" s="245"/>
+      <c r="F18" s="245"/>
+      <c r="G18" s="245"/>
+      <c r="H18" s="245"/>
+      <c r="I18" s="245"/>
+      <c r="J18" s="245"/>
+      <c r="K18" s="245"/>
+      <c r="L18" s="245"/>
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B19" s="16" t="s">
@@ -20373,23 +20344,23 @@
       </c>
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B25" s="238"/>
-      <c r="C25" s="238"/>
+      <c r="B25" s="250"/>
+      <c r="C25" s="250"/>
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B26" s="109"/>
-      <c r="C26" s="234" t="s">
+      <c r="C26" s="245" t="s">
         <v>140</v>
       </c>
-      <c r="D26" s="234"/>
-      <c r="E26" s="234"/>
-      <c r="F26" s="234"/>
-      <c r="G26" s="234"/>
-      <c r="H26" s="234"/>
-      <c r="I26" s="234"/>
-      <c r="J26" s="234"/>
-      <c r="K26" s="234"/>
-      <c r="L26" s="234"/>
+      <c r="D26" s="245"/>
+      <c r="E26" s="245"/>
+      <c r="F26" s="245"/>
+      <c r="G26" s="245"/>
+      <c r="H26" s="245"/>
+      <c r="I26" s="245"/>
+      <c r="J26" s="245"/>
+      <c r="K26" s="245"/>
+      <c r="L26" s="245"/>
     </row>
     <row r="27" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B27" s="16" t="s">
@@ -20581,18 +20552,18 @@
     </row>
     <row r="33" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B33" s="109"/>
-      <c r="C33" s="234" t="s">
+      <c r="C33" s="245" t="s">
         <v>144</v>
       </c>
-      <c r="D33" s="234"/>
-      <c r="E33" s="234"/>
-      <c r="F33" s="234"/>
-      <c r="G33" s="234"/>
-      <c r="H33" s="234"/>
-      <c r="I33" s="234"/>
-      <c r="J33" s="234"/>
-      <c r="K33" s="234"/>
-      <c r="L33" s="234"/>
+      <c r="D33" s="245"/>
+      <c r="E33" s="245"/>
+      <c r="F33" s="245"/>
+      <c r="G33" s="245"/>
+      <c r="H33" s="245"/>
+      <c r="I33" s="245"/>
+      <c r="J33" s="245"/>
+      <c r="K33" s="245"/>
+      <c r="L33" s="245"/>
     </row>
     <row r="34" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B34" s="16" t="s">
@@ -20776,18 +20747,18 @@
       <c r="C39" s="125"/>
     </row>
     <row r="40" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="C40" s="234" t="s">
+      <c r="C40" s="245" t="s">
         <v>147</v>
       </c>
-      <c r="D40" s="234"/>
-      <c r="E40" s="234"/>
-      <c r="F40" s="234"/>
-      <c r="G40" s="234"/>
-      <c r="H40" s="234"/>
-      <c r="I40" s="234"/>
-      <c r="J40" s="234"/>
-      <c r="K40" s="234"/>
-      <c r="L40" s="234"/>
+      <c r="D40" s="245"/>
+      <c r="E40" s="245"/>
+      <c r="F40" s="245"/>
+      <c r="G40" s="245"/>
+      <c r="H40" s="245"/>
+      <c r="I40" s="245"/>
+      <c r="J40" s="245"/>
+      <c r="K40" s="245"/>
+      <c r="L40" s="245"/>
     </row>
     <row r="41" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B41" s="16" t="s">
@@ -21051,12 +21022,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="C3:G3"/>
-    <mergeCell ref="H3:L3"/>
-    <mergeCell ref="P3:W3"/>
-    <mergeCell ref="X3:Z3"/>
-    <mergeCell ref="C5:L5"/>
-    <mergeCell ref="P5:Z5"/>
     <mergeCell ref="C40:L40"/>
     <mergeCell ref="C11:L11"/>
     <mergeCell ref="P11:Z11"/>
@@ -21064,6 +21029,12 @@
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="C26:L26"/>
     <mergeCell ref="C33:L33"/>
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="H3:L3"/>
+    <mergeCell ref="P3:W3"/>
+    <mergeCell ref="X3:Z3"/>
+    <mergeCell ref="C5:L5"/>
+    <mergeCell ref="P5:Z5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -21101,60 +21072,60 @@
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
-      <c r="C2" s="235" t="s">
+      <c r="C2" s="236" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="235"/>
-      <c r="E2" s="235"/>
-      <c r="F2" s="235"/>
-      <c r="G2" s="236"/>
-      <c r="H2" s="237" t="s">
+      <c r="D2" s="236"/>
+      <c r="E2" s="236"/>
+      <c r="F2" s="236"/>
+      <c r="G2" s="248"/>
+      <c r="H2" s="249" t="s">
         <v>111</v>
       </c>
-      <c r="I2" s="235"/>
-      <c r="J2" s="235"/>
-      <c r="K2" s="235"/>
-      <c r="L2" s="235"/>
-      <c r="S2" s="238"/>
-      <c r="T2" s="238"/>
-      <c r="U2" s="238"/>
-      <c r="V2" s="238"/>
-      <c r="W2" s="238"/>
-      <c r="X2" s="238"/>
-      <c r="Y2" s="238"/>
-      <c r="Z2" s="238"/>
-      <c r="AA2" s="238"/>
-      <c r="AB2" s="238"/>
-      <c r="AC2" s="238"/>
+      <c r="I2" s="236"/>
+      <c r="J2" s="236"/>
+      <c r="K2" s="236"/>
+      <c r="L2" s="236"/>
+      <c r="S2" s="250"/>
+      <c r="T2" s="250"/>
+      <c r="U2" s="250"/>
+      <c r="V2" s="250"/>
+      <c r="W2" s="250"/>
+      <c r="X2" s="250"/>
+      <c r="Y2" s="250"/>
+      <c r="Z2" s="250"/>
+      <c r="AA2" s="250"/>
+      <c r="AB2" s="250"/>
+      <c r="AC2" s="250"/>
       <c r="AE2" s="109"/>
     </row>
     <row r="3" spans="1:31" ht="10" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:31" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="86"/>
       <c r="B4" s="60"/>
-      <c r="C4" s="234" t="s">
+      <c r="C4" s="245" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="234"/>
-      <c r="E4" s="234"/>
-      <c r="F4" s="234"/>
-      <c r="G4" s="234"/>
-      <c r="H4" s="234"/>
-      <c r="I4" s="234"/>
-      <c r="J4" s="234"/>
-      <c r="K4" s="234"/>
-      <c r="L4" s="234"/>
-      <c r="S4" s="238"/>
-      <c r="T4" s="238"/>
-      <c r="U4" s="238"/>
-      <c r="V4" s="238"/>
-      <c r="W4" s="238"/>
-      <c r="X4" s="238"/>
-      <c r="Y4" s="238"/>
-      <c r="Z4" s="238"/>
-      <c r="AA4" s="238"/>
-      <c r="AB4" s="238"/>
-      <c r="AC4" s="238"/>
+      <c r="D4" s="245"/>
+      <c r="E4" s="245"/>
+      <c r="F4" s="245"/>
+      <c r="G4" s="245"/>
+      <c r="H4" s="245"/>
+      <c r="I4" s="245"/>
+      <c r="J4" s="245"/>
+      <c r="K4" s="245"/>
+      <c r="L4" s="245"/>
+      <c r="S4" s="250"/>
+      <c r="T4" s="250"/>
+      <c r="U4" s="250"/>
+      <c r="V4" s="250"/>
+      <c r="W4" s="250"/>
+      <c r="X4" s="250"/>
+      <c r="Y4" s="250"/>
+      <c r="Z4" s="250"/>
+      <c r="AA4" s="250"/>
+      <c r="AB4" s="250"/>
+      <c r="AC4" s="250"/>
       <c r="AE4" s="110"/>
     </row>
     <row r="5" spans="1:31" x14ac:dyDescent="0.2">
@@ -21517,18 +21488,18 @@
       <c r="AE10" s="64"/>
     </row>
     <row r="13" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="C13" s="234" t="s">
+      <c r="C13" s="245" t="s">
         <v>155</v>
       </c>
-      <c r="D13" s="234"/>
-      <c r="E13" s="234"/>
-      <c r="F13" s="234"/>
-      <c r="G13" s="234"/>
-      <c r="H13" s="234"/>
-      <c r="I13" s="234"/>
-      <c r="J13" s="234"/>
-      <c r="K13" s="234"/>
-      <c r="L13" s="234"/>
+      <c r="D13" s="245"/>
+      <c r="E13" s="245"/>
+      <c r="F13" s="245"/>
+      <c r="G13" s="245"/>
+      <c r="H13" s="245"/>
+      <c r="I13" s="245"/>
+      <c r="J13" s="245"/>
+      <c r="K13" s="245"/>
+      <c r="L13" s="245"/>
     </row>
     <row r="14" spans="1:31" x14ac:dyDescent="0.2">
       <c r="C14" s="12">
@@ -21621,18 +21592,18 @@
       </c>
     </row>
     <row r="18" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="C18" s="234" t="s">
+      <c r="C18" s="245" t="s">
         <v>156</v>
       </c>
-      <c r="D18" s="234"/>
-      <c r="E18" s="234"/>
-      <c r="F18" s="234"/>
-      <c r="G18" s="234"/>
-      <c r="H18" s="234"/>
-      <c r="I18" s="234"/>
-      <c r="J18" s="234"/>
-      <c r="K18" s="234"/>
-      <c r="L18" s="234"/>
+      <c r="D18" s="245"/>
+      <c r="E18" s="245"/>
+      <c r="F18" s="245"/>
+      <c r="G18" s="245"/>
+      <c r="H18" s="245"/>
+      <c r="I18" s="245"/>
+      <c r="J18" s="245"/>
+      <c r="K18" s="245"/>
+      <c r="L18" s="245"/>
     </row>
     <row r="19" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B19" s="16" t="s">
@@ -21824,18 +21795,18 @@
       </c>
     </row>
     <row r="25" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="C25" s="234" t="s">
+      <c r="C25" s="245" t="s">
         <v>256</v>
       </c>
-      <c r="D25" s="234"/>
-      <c r="E25" s="234"/>
-      <c r="F25" s="234"/>
-      <c r="G25" s="234"/>
-      <c r="H25" s="234"/>
-      <c r="I25" s="234"/>
-      <c r="J25" s="234"/>
-      <c r="K25" s="234"/>
-      <c r="L25" s="234"/>
+      <c r="D25" s="245"/>
+      <c r="E25" s="245"/>
+      <c r="F25" s="245"/>
+      <c r="G25" s="245"/>
+      <c r="H25" s="245"/>
+      <c r="I25" s="245"/>
+      <c r="J25" s="245"/>
+      <c r="K25" s="245"/>
+      <c r="L25" s="245"/>
     </row>
     <row r="26" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B26" s="16" t="s">
@@ -21973,18 +21944,18 @@
       </c>
     </row>
     <row r="31" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="C31" s="234" t="s">
+      <c r="C31" s="245" t="s">
         <v>75</v>
       </c>
-      <c r="D31" s="234"/>
-      <c r="E31" s="234"/>
-      <c r="F31" s="234"/>
-      <c r="G31" s="234"/>
-      <c r="H31" s="234"/>
-      <c r="I31" s="234"/>
-      <c r="J31" s="234"/>
-      <c r="K31" s="234"/>
-      <c r="L31" s="234"/>
+      <c r="D31" s="245"/>
+      <c r="E31" s="245"/>
+      <c r="F31" s="245"/>
+      <c r="G31" s="245"/>
+      <c r="H31" s="245"/>
+      <c r="I31" s="245"/>
+      <c r="J31" s="245"/>
+      <c r="K31" s="245"/>
+      <c r="L31" s="245"/>
     </row>
     <row r="32" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B32" s="16" t="s">
@@ -22123,16 +22094,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="C31:L31"/>
+    <mergeCell ref="C25:L25"/>
+    <mergeCell ref="C2:G2"/>
+    <mergeCell ref="H2:L2"/>
+    <mergeCell ref="S2:Z2"/>
     <mergeCell ref="AA2:AC2"/>
     <mergeCell ref="C4:L4"/>
     <mergeCell ref="S4:AC4"/>
     <mergeCell ref="C13:L13"/>
     <mergeCell ref="C18:L18"/>
-    <mergeCell ref="C31:L31"/>
-    <mergeCell ref="C25:L25"/>
-    <mergeCell ref="C2:G2"/>
-    <mergeCell ref="H2:L2"/>
-    <mergeCell ref="S2:Z2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -22195,10 +22166,10 @@
     </row>
     <row r="3" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="235" t="s">
+      <c r="B4" s="236" t="s">
         <v>163</v>
       </c>
-      <c r="C4" s="235"/>
+      <c r="C4" s="236"/>
     </row>
     <row r="5" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
@@ -22215,7 +22186,7 @@
       </c>
       <c r="C6" s="133">
         <f ca="1">Overview!C5</f>
-        <v>340.22500000000002</v>
+        <v>341.07</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22224,7 +22195,7 @@
       </c>
       <c r="C7" s="134">
         <f ca="1">C5*C6</f>
-        <v>4985316.9250000007</v>
+        <v>4997698.71</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22283,10 +22254,10 @@
     </row>
     <row r="14" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="15" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="235" t="s">
+      <c r="B15" s="236" t="s">
         <v>170</v>
       </c>
-      <c r="C15" s="235"/>
+      <c r="C15" s="236"/>
     </row>
     <row r="16" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="1" t="s">
@@ -22294,7 +22265,7 @@
       </c>
       <c r="C16" s="46">
         <f ca="1">C8/(C8+C7)</f>
-        <v>1.6637010097475105E-2</v>
+        <v>1.6596476026074169E-2</v>
       </c>
     </row>
     <row r="17" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22303,7 +22274,7 @@
       </c>
       <c r="C17" s="46">
         <f ca="1">C7/(C8+C7)</f>
-        <v>0.98336298990252491</v>
+        <v>0.98340352397392583</v>
       </c>
     </row>
     <row r="18" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22330,7 +22301,7 @@
       </c>
       <c r="C20" s="46">
         <f ca="1">(C17*C19)+(C16*C18)</f>
-        <v>9.8833796565630266E-2</v>
+        <v>9.8836274859289808E-2</v>
       </c>
     </row>
   </sheetData>
@@ -22375,60 +22346,60 @@
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A3" s="4"/>
-      <c r="C3" s="235" t="s">
+      <c r="C3" s="236" t="s">
         <v>110</v>
       </c>
-      <c r="D3" s="235"/>
-      <c r="E3" s="235"/>
-      <c r="F3" s="235"/>
-      <c r="G3" s="236"/>
-      <c r="H3" s="237" t="s">
+      <c r="D3" s="236"/>
+      <c r="E3" s="236"/>
+      <c r="F3" s="236"/>
+      <c r="G3" s="248"/>
+      <c r="H3" s="249" t="s">
         <v>111</v>
       </c>
-      <c r="I3" s="235"/>
-      <c r="J3" s="235"/>
-      <c r="K3" s="235"/>
-      <c r="L3" s="235"/>
-      <c r="P3" s="238"/>
-      <c r="Q3" s="238"/>
-      <c r="R3" s="238"/>
-      <c r="S3" s="238"/>
-      <c r="T3" s="238"/>
-      <c r="U3" s="238"/>
-      <c r="V3" s="238"/>
-      <c r="W3" s="238"/>
-      <c r="X3" s="238"/>
-      <c r="Y3" s="238"/>
-      <c r="Z3" s="238"/>
+      <c r="I3" s="236"/>
+      <c r="J3" s="236"/>
+      <c r="K3" s="236"/>
+      <c r="L3" s="236"/>
+      <c r="P3" s="250"/>
+      <c r="Q3" s="250"/>
+      <c r="R3" s="250"/>
+      <c r="S3" s="250"/>
+      <c r="T3" s="250"/>
+      <c r="U3" s="250"/>
+      <c r="V3" s="250"/>
+      <c r="W3" s="250"/>
+      <c r="X3" s="250"/>
+      <c r="Y3" s="250"/>
+      <c r="Z3" s="250"/>
       <c r="AB3" s="109"/>
     </row>
     <row r="4" spans="1:28" ht="10" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="5" spans="1:28" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="86"/>
       <c r="B5" s="60"/>
-      <c r="C5" s="234" t="s">
+      <c r="C5" s="245" t="s">
         <v>177</v>
       </c>
-      <c r="D5" s="234"/>
-      <c r="E5" s="234"/>
-      <c r="F5" s="234"/>
-      <c r="G5" s="234"/>
-      <c r="H5" s="234"/>
-      <c r="I5" s="234"/>
-      <c r="J5" s="234"/>
-      <c r="K5" s="234"/>
-      <c r="L5" s="234"/>
-      <c r="P5" s="238"/>
-      <c r="Q5" s="238"/>
-      <c r="R5" s="238"/>
-      <c r="S5" s="238"/>
-      <c r="T5" s="238"/>
-      <c r="U5" s="238"/>
-      <c r="V5" s="238"/>
-      <c r="W5" s="238"/>
-      <c r="X5" s="238"/>
-      <c r="Y5" s="238"/>
-      <c r="Z5" s="238"/>
+      <c r="D5" s="245"/>
+      <c r="E5" s="245"/>
+      <c r="F5" s="245"/>
+      <c r="G5" s="245"/>
+      <c r="H5" s="245"/>
+      <c r="I5" s="245"/>
+      <c r="J5" s="245"/>
+      <c r="K5" s="245"/>
+      <c r="L5" s="245"/>
+      <c r="P5" s="250"/>
+      <c r="Q5" s="250"/>
+      <c r="R5" s="250"/>
+      <c r="S5" s="250"/>
+      <c r="T5" s="250"/>
+      <c r="U5" s="250"/>
+      <c r="V5" s="250"/>
+      <c r="W5" s="250"/>
+      <c r="X5" s="250"/>
+      <c r="Y5" s="250"/>
+      <c r="Z5" s="250"/>
       <c r="AB5" s="110"/>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.2">
@@ -22581,7 +22552,7 @@
       </c>
       <c r="L8" s="126">
         <f ca="1">L7*(1+C14)/(C15-C14)</f>
-        <v>1838737.1276046229</v>
+        <v>1838679.3251453738</v>
       </c>
       <c r="N8" s="91"/>
       <c r="O8" s="16"/>
@@ -22635,23 +22606,23 @@
       <c r="G10" s="138"/>
       <c r="H10" s="126">
         <f ca="1">H7/(1+$C$15)^H9</f>
-        <v>100432.85543948702</v>
+        <v>100432.62892520591</v>
       </c>
       <c r="I10" s="126">
         <f t="shared" ref="I10:L10" ca="1" si="0">I7/(1+$C$15)^I9</f>
-        <v>97108.00119072423</v>
+        <v>97107.56316027735</v>
       </c>
       <c r="J10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>93374.960808008371</v>
+        <v>93374.329021298967</v>
       </c>
       <c r="K10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>89373.103671124671</v>
+        <v>89372.297392511886</v>
       </c>
       <c r="L10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>88709.855886179692</v>
+        <v>88708.855518396362</v>
       </c>
       <c r="N10" s="91"/>
     </row>
@@ -22670,14 +22641,14 @@
       <c r="K11" s="137"/>
       <c r="L11" s="126">
         <f ca="1">L8/(1+C15)^L9</f>
-        <v>1147782.511382336</v>
+        <v>1147733.4867770211</v>
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="B13" s="235" t="s">
+      <c r="B13" s="236" t="s">
         <v>181</v>
       </c>
-      <c r="C13" s="235"/>
+      <c r="C13" s="236"/>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B14" s="1" t="s">
@@ -22693,14 +22664,14 @@
       </c>
       <c r="C15" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.8833796565630266E-2</v>
+        <v>9.8836274859289808E-2</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B18" s="235" t="s">
+      <c r="B18" s="236" t="s">
         <v>183</v>
       </c>
-      <c r="C18" s="235"/>
+      <c r="C18" s="236"/>
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B19" s="1" t="s">
@@ -22708,7 +22679,7 @@
       </c>
       <c r="C19" s="64">
         <f ca="1">SUM(H10:L10)</f>
-        <v>468998.77699552395</v>
+        <v>468995.67401769047</v>
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.2">
@@ -22717,7 +22688,7 @@
       </c>
       <c r="C20" s="64">
         <f ca="1">L11</f>
-        <v>1147782.511382336</v>
+        <v>1147733.4867770211</v>
       </c>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.2">
@@ -22726,7 +22697,7 @@
       </c>
       <c r="C21" s="94">
         <f ca="1">C19+C20</f>
-        <v>1616781.2883778601</v>
+        <v>1616729.1607947117</v>
       </c>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.2">
@@ -22753,7 +22724,7 @@
       </c>
       <c r="C24" s="94">
         <f ca="1">C21+C22-C23</f>
-        <v>1678954.2883778601</v>
+        <v>1678902.1607947117</v>
       </c>
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.2">
@@ -22766,12 +22737,12 @@
       </c>
     </row>
     <row r="26" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B26" s="252" t="s">
+      <c r="B26" s="234" t="s">
         <v>189</v>
       </c>
-      <c r="C26" s="253">
+      <c r="C26" s="235">
         <f ca="1">C24/C25</f>
-        <v>114.58092461460862</v>
+        <v>114.57736714629849</v>
       </c>
     </row>
   </sheetData>
@@ -22814,37 +22785,37 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
-      <c r="C2" s="235" t="s">
+      <c r="C2" s="236" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="235"/>
-      <c r="E2" s="235"/>
-      <c r="F2" s="235"/>
-      <c r="G2" s="236"/>
-      <c r="H2" s="237" t="s">
+      <c r="D2" s="236"/>
+      <c r="E2" s="236"/>
+      <c r="F2" s="236"/>
+      <c r="G2" s="248"/>
+      <c r="H2" s="249" t="s">
         <v>111</v>
       </c>
-      <c r="I2" s="235"/>
-      <c r="J2" s="235"/>
-      <c r="K2" s="235"/>
-      <c r="L2" s="235"/>
+      <c r="I2" s="236"/>
+      <c r="J2" s="236"/>
+      <c r="K2" s="236"/>
+      <c r="L2" s="236"/>
     </row>
     <row r="3" spans="1:14" ht="10" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:14" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="86"/>
       <c r="B4" s="60"/>
-      <c r="C4" s="234" t="s">
+      <c r="C4" s="245" t="s">
         <v>191</v>
       </c>
-      <c r="D4" s="234"/>
-      <c r="E4" s="234"/>
-      <c r="F4" s="234"/>
-      <c r="G4" s="234"/>
-      <c r="H4" s="234"/>
-      <c r="I4" s="234"/>
-      <c r="J4" s="234"/>
-      <c r="K4" s="234"/>
-      <c r="L4" s="234"/>
+      <c r="D4" s="245"/>
+      <c r="E4" s="245"/>
+      <c r="F4" s="245"/>
+      <c r="G4" s="245"/>
+      <c r="H4" s="245"/>
+      <c r="I4" s="245"/>
+      <c r="J4" s="245"/>
+      <c r="K4" s="245"/>
+      <c r="L4" s="245"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B5" s="16" t="s">
@@ -23040,23 +23011,23 @@
       <c r="G9" s="138"/>
       <c r="H9" s="92">
         <f ca="1">DCF!H10</f>
-        <v>100432.85543948702</v>
+        <v>100432.62892520591</v>
       </c>
       <c r="I9" s="92">
         <f ca="1">DCF!I10</f>
-        <v>97108.00119072423</v>
+        <v>97107.56316027735</v>
       </c>
       <c r="J9" s="92">
         <f ca="1">DCF!J10</f>
-        <v>93374.960808008371</v>
+        <v>93374.329021298967</v>
       </c>
       <c r="K9" s="92">
         <f ca="1">DCF!K10</f>
-        <v>89373.103671124671</v>
+        <v>89372.297392511886</v>
       </c>
       <c r="L9" s="92">
         <f ca="1">DCF!L10</f>
-        <v>88709.855886179692</v>
+        <v>88708.855518396362</v>
       </c>
       <c r="N9" s="91"/>
     </row>
@@ -23064,18 +23035,18 @@
       <c r="N10" s="91"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="C11" s="234" t="s">
+      <c r="C11" s="245" t="s">
         <v>119</v>
       </c>
-      <c r="D11" s="234"/>
-      <c r="E11" s="234"/>
-      <c r="F11" s="234"/>
-      <c r="G11" s="234"/>
-      <c r="H11" s="234"/>
-      <c r="I11" s="234"/>
-      <c r="J11" s="234"/>
-      <c r="K11" s="234"/>
-      <c r="L11" s="234"/>
+      <c r="D11" s="245"/>
+      <c r="E11" s="245"/>
+      <c r="F11" s="245"/>
+      <c r="G11" s="245"/>
+      <c r="H11" s="245"/>
+      <c r="I11" s="245"/>
+      <c r="J11" s="245"/>
+      <c r="K11" s="245"/>
+      <c r="L11" s="245"/>
       <c r="N11" s="91"/>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.2">
@@ -23269,18 +23240,18 @@
       <c r="N16" s="91"/>
     </row>
     <row r="17" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="C17" s="234" t="s">
+      <c r="C17" s="245" t="s">
         <v>193</v>
       </c>
-      <c r="D17" s="234"/>
-      <c r="E17" s="234"/>
-      <c r="F17" s="234"/>
-      <c r="G17" s="234"/>
-      <c r="H17" s="234"/>
-      <c r="I17" s="234"/>
-      <c r="J17" s="234"/>
-      <c r="K17" s="234"/>
-      <c r="L17" s="234"/>
+      <c r="D17" s="245"/>
+      <c r="E17" s="245"/>
+      <c r="F17" s="245"/>
+      <c r="G17" s="245"/>
+      <c r="H17" s="245"/>
+      <c r="I17" s="245"/>
+      <c r="J17" s="245"/>
+      <c r="K17" s="245"/>
+      <c r="L17" s="245"/>
       <c r="N17" s="91"/>
     </row>
     <row r="18" spans="2:14" x14ac:dyDescent="0.2">
@@ -23414,18 +23385,18 @@
       <c r="N21" s="91"/>
     </row>
     <row r="22" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="C22" s="234" t="s">
+      <c r="C22" s="245" t="s">
         <v>196</v>
       </c>
-      <c r="D22" s="234"/>
-      <c r="E22" s="234"/>
-      <c r="F22" s="234"/>
-      <c r="G22" s="234"/>
-      <c r="H22" s="234"/>
-      <c r="I22" s="234"/>
-      <c r="J22" s="234"/>
-      <c r="K22" s="234"/>
-      <c r="L22" s="234"/>
+      <c r="D22" s="245"/>
+      <c r="E22" s="245"/>
+      <c r="F22" s="245"/>
+      <c r="G22" s="245"/>
+      <c r="H22" s="245"/>
+      <c r="I22" s="245"/>
+      <c r="J22" s="245"/>
+      <c r="K22" s="245"/>
+      <c r="L22" s="245"/>
       <c r="N22" s="91"/>
     </row>
     <row r="23" spans="2:14" x14ac:dyDescent="0.2">
@@ -23509,18 +23480,18 @@
       <c r="N26" s="91"/>
     </row>
     <row r="27" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="C27" s="234" t="s">
+      <c r="C27" s="245" t="s">
         <v>197</v>
       </c>
-      <c r="D27" s="234"/>
-      <c r="E27" s="234"/>
-      <c r="F27" s="234"/>
-      <c r="G27" s="234"/>
-      <c r="H27" s="234"/>
-      <c r="I27" s="234"/>
-      <c r="J27" s="234"/>
-      <c r="K27" s="234"/>
-      <c r="L27" s="234"/>
+      <c r="D27" s="245"/>
+      <c r="E27" s="245"/>
+      <c r="F27" s="245"/>
+      <c r="G27" s="245"/>
+      <c r="H27" s="245"/>
+      <c r="I27" s="245"/>
+      <c r="J27" s="245"/>
+      <c r="K27" s="245"/>
+      <c r="L27" s="245"/>
       <c r="N27" s="91"/>
     </row>
     <row r="28" spans="2:14" x14ac:dyDescent="0.2">
@@ -23790,10 +23761,10 @@
       <c r="N37" s="91"/>
     </row>
     <row r="38" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B38" s="235" t="s">
+      <c r="B38" s="236" t="s">
         <v>202</v>
       </c>
-      <c r="C38" s="235"/>
+      <c r="C38" s="236"/>
       <c r="N38" s="91"/>
     </row>
     <row r="39" spans="2:14" x14ac:dyDescent="0.2">
@@ -23811,7 +23782,7 @@
       </c>
       <c r="C40" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.8833796565630266E-2</v>
+        <v>9.8836274859289808E-2</v>
       </c>
     </row>
     <row r="41" spans="2:14" x14ac:dyDescent="0.2">
@@ -23836,8 +23807,8 @@
         <v>410</v>
       </c>
       <c r="C43" s="24">
-        <f ca="1">C42/(1+C40)^5-G31+G32</f>
-        <v>2956946.3383825342</v>
+        <f ca="1">C42/(1+C40)^5</f>
+        <v>2923150.3740810226</v>
       </c>
     </row>
     <row r="44" spans="2:14" x14ac:dyDescent="0.2">
@@ -23846,7 +23817,7 @@
       </c>
       <c r="C44" s="108">
         <f ca="1">SUM(H9:K9)+C43</f>
-        <v>3337235.2594918786</v>
+        <v>3303437.1925803167</v>
       </c>
     </row>
     <row r="45" spans="2:14" x14ac:dyDescent="0.2">
@@ -23873,7 +23844,7 @@
       </c>
       <c r="C47" s="94">
         <f ca="1">C44+C45-C46</f>
-        <v>3399408.2594918786</v>
+        <v>3365610.1925803167</v>
       </c>
     </row>
     <row r="48" spans="2:14" x14ac:dyDescent="0.2">
@@ -23886,19 +23857,19 @@
       </c>
     </row>
     <row r="49" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B49" s="252" t="s">
+      <c r="B49" s="234" t="s">
         <v>206</v>
       </c>
-      <c r="C49" s="253">
+      <c r="C49" s="235">
         <f ca="1">C47/C48</f>
-        <v>231.99401211300611</v>
+        <v>229.68744916265044</v>
       </c>
     </row>
     <row r="51" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B51" s="235" t="s">
+      <c r="B51" s="236" t="s">
         <v>207</v>
       </c>
-      <c r="C51" s="235"/>
+      <c r="C51" s="236"/>
     </row>
     <row r="52" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B52" s="1" t="s">
@@ -23945,19 +23916,19 @@
       </c>
     </row>
     <row r="57" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B57" s="252" t="s">
+      <c r="B57" s="234" t="s">
         <v>206</v>
       </c>
-      <c r="C57" s="253">
+      <c r="C57" s="235">
         <f ca="1">C56/(1+C53)^5</f>
         <v>201.25463701394406</v>
       </c>
     </row>
     <row r="59" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B59" s="235" t="s">
+      <c r="B59" s="236" t="s">
         <v>316</v>
       </c>
-      <c r="C59" s="235"/>
+      <c r="C59" s="236"/>
     </row>
     <row r="60" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B60" s="1" t="s">
@@ -23974,7 +23945,7 @@
       </c>
       <c r="C61" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.8833796565630266E-2</v>
+        <v>9.8836274859289808E-2</v>
       </c>
     </row>
     <row r="62" spans="2:3" x14ac:dyDescent="0.2">
@@ -23999,8 +23970,8 @@
         <v>410</v>
       </c>
       <c r="C64" s="24">
-        <f ca="1">C63/(1+C61)^5-G31+G32</f>
-        <v>1807960.117723594</v>
+        <f ca="1">C63/(1+C61)^5</f>
+        <v>1774177.1103679272</v>
       </c>
     </row>
     <row r="65" spans="2:3" x14ac:dyDescent="0.2">
@@ -24009,7 +23980,7 @@
       </c>
       <c r="C65" s="108">
         <f ca="1">SUM(H9:K9)+C64</f>
-        <v>2188249.0388329383</v>
+        <v>2154463.9288672213</v>
       </c>
     </row>
     <row r="66" spans="2:3" x14ac:dyDescent="0.2">
@@ -24036,7 +24007,7 @@
       </c>
       <c r="C68" s="94">
         <f ca="1">C65+C66-C67</f>
-        <v>2250422.0388329383</v>
+        <v>2216636.9288672213</v>
       </c>
     </row>
     <row r="69" spans="2:3" x14ac:dyDescent="0.2">
@@ -24049,12 +24020,12 @@
       </c>
     </row>
     <row r="70" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B70" s="252" t="s">
+      <c r="B70" s="234" t="s">
         <v>206</v>
       </c>
-      <c r="C70" s="253">
+      <c r="C70" s="235">
         <f ca="1">C68/C69</f>
-        <v>153.58097582972349</v>
+        <v>151.27529713145577</v>
       </c>
     </row>
   </sheetData>
@@ -24106,10 +24077,10 @@
       <c r="N3" s="91"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B4" s="235" t="s">
+      <c r="B4" s="236" t="s">
         <v>211</v>
       </c>
-      <c r="C4" s="235"/>
+      <c r="C4" s="236"/>
       <c r="N4" s="91"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
@@ -24118,7 +24089,7 @@
       </c>
       <c r="C5" s="133">
         <f ca="1">DCF!C26</f>
-        <v>114.58092461460862</v>
+        <v>114.57736714629849</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -24127,7 +24098,7 @@
       </c>
       <c r="C6" s="133">
         <f ca="1">Multiples!C49</f>
-        <v>231.99401211300611</v>
+        <v>229.68744916265044</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
@@ -24145,16 +24116,16 @@
       </c>
       <c r="C8" s="133">
         <f ca="1">Multiples!C70</f>
-        <v>153.58097582972349</v>
+        <v>151.27529713145577</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B9" s="252" t="s">
+      <c r="B9" s="234" t="s">
         <v>215</v>
       </c>
-      <c r="C9" s="253">
+      <c r="C9" s="235">
         <f ca="1">AVERAGE(C5:C8)</f>
-        <v>175.35263739282055</v>
+        <v>174.1986876135872</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
@@ -24163,7 +24134,7 @@
       </c>
       <c r="C10" s="133">
         <f ca="1">Overview!C5</f>
-        <v>340.22500000000002</v>
+        <v>341.07</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
@@ -24172,7 +24143,7 @@
       </c>
       <c r="C11" s="149">
         <f ca="1">(C9-C10)/C10</f>
-        <v>-0.48459802368191479</v>
+        <v>-0.4892582531046788</v>
       </c>
     </row>
   </sheetData>
@@ -24228,37 +24199,37 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
-      <c r="C2" s="235" t="s">
+      <c r="C2" s="236" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="235"/>
-      <c r="E2" s="235"/>
-      <c r="F2" s="235"/>
-      <c r="G2" s="236"/>
-      <c r="H2" s="237" t="s">
+      <c r="D2" s="236"/>
+      <c r="E2" s="236"/>
+      <c r="F2" s="236"/>
+      <c r="G2" s="248"/>
+      <c r="H2" s="249" t="s">
         <v>111</v>
       </c>
-      <c r="I2" s="235"/>
-      <c r="J2" s="235"/>
-      <c r="K2" s="235"/>
-      <c r="L2" s="235"/>
+      <c r="I2" s="236"/>
+      <c r="J2" s="236"/>
+      <c r="K2" s="236"/>
+      <c r="L2" s="236"/>
     </row>
     <row r="3" spans="1:14" ht="10" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:14" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="86"/>
       <c r="B4" s="60"/>
-      <c r="C4" s="234" t="s">
+      <c r="C4" s="245" t="s">
         <v>191</v>
       </c>
-      <c r="D4" s="234"/>
-      <c r="E4" s="234"/>
-      <c r="F4" s="234"/>
-      <c r="G4" s="234"/>
-      <c r="H4" s="234"/>
-      <c r="I4" s="234"/>
-      <c r="J4" s="234"/>
-      <c r="K4" s="234"/>
-      <c r="L4" s="234"/>
+      <c r="D4" s="245"/>
+      <c r="E4" s="245"/>
+      <c r="F4" s="245"/>
+      <c r="G4" s="245"/>
+      <c r="H4" s="245"/>
+      <c r="I4" s="245"/>
+      <c r="J4" s="245"/>
+      <c r="K4" s="245"/>
+      <c r="L4" s="245"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B5" s="16" t="s">
@@ -24371,18 +24342,18 @@
       <c r="N8" s="91"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="C9" s="234" t="s">
+      <c r="C9" s="245" t="s">
         <v>119</v>
       </c>
-      <c r="D9" s="234"/>
-      <c r="E9" s="234"/>
-      <c r="F9" s="234"/>
-      <c r="G9" s="234"/>
-      <c r="H9" s="234"/>
-      <c r="I9" s="234"/>
-      <c r="J9" s="234"/>
-      <c r="K9" s="234"/>
-      <c r="L9" s="234"/>
+      <c r="D9" s="245"/>
+      <c r="E9" s="245"/>
+      <c r="F9" s="245"/>
+      <c r="G9" s="245"/>
+      <c r="H9" s="245"/>
+      <c r="I9" s="245"/>
+      <c r="J9" s="245"/>
+      <c r="K9" s="245"/>
+      <c r="L9" s="245"/>
       <c r="N9" s="91"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
@@ -24503,18 +24474,18 @@
       <c r="N13" s="91"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="C14" s="234" t="s">
+      <c r="C14" s="245" t="s">
         <v>397</v>
       </c>
-      <c r="D14" s="234"/>
-      <c r="E14" s="234"/>
-      <c r="F14" s="234"/>
-      <c r="G14" s="234"/>
-      <c r="H14" s="234"/>
-      <c r="I14" s="234"/>
-      <c r="J14" s="234"/>
-      <c r="K14" s="234"/>
-      <c r="L14" s="234"/>
+      <c r="D14" s="245"/>
+      <c r="E14" s="245"/>
+      <c r="F14" s="245"/>
+      <c r="G14" s="245"/>
+      <c r="H14" s="245"/>
+      <c r="I14" s="245"/>
+      <c r="J14" s="245"/>
+      <c r="K14" s="245"/>
+      <c r="L14" s="245"/>
       <c r="N14" s="91"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.2">
@@ -24604,10 +24575,10 @@
       <c r="N19" s="91"/>
     </row>
     <row r="20" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B20" s="235" t="s">
+      <c r="B20" s="236" t="s">
         <v>399</v>
       </c>
-      <c r="C20" s="235"/>
+      <c r="C20" s="236"/>
       <c r="N20" s="91"/>
     </row>
     <row r="21" spans="2:14" x14ac:dyDescent="0.2">
@@ -24654,10 +24625,10 @@
       </c>
     </row>
     <row r="26" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B26" s="252" t="s">
+      <c r="B26" s="234" t="s">
         <v>206</v>
       </c>
-      <c r="C26" s="253">
+      <c r="C26" s="235">
         <f ca="1">C23/(C24-C25)</f>
         <v>13.284742833527446</v>
       </c>
@@ -24708,60 +24679,60 @@
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A3" s="4"/>
-      <c r="C3" s="235" t="s">
+      <c r="C3" s="236" t="s">
         <v>110</v>
       </c>
-      <c r="D3" s="235"/>
-      <c r="E3" s="235"/>
-      <c r="F3" s="235"/>
-      <c r="G3" s="236"/>
-      <c r="H3" s="237" t="s">
+      <c r="D3" s="236"/>
+      <c r="E3" s="236"/>
+      <c r="F3" s="236"/>
+      <c r="G3" s="248"/>
+      <c r="H3" s="249" t="s">
         <v>111</v>
       </c>
-      <c r="I3" s="235"/>
-      <c r="J3" s="235"/>
-      <c r="K3" s="235"/>
-      <c r="L3" s="235"/>
-      <c r="P3" s="238"/>
-      <c r="Q3" s="238"/>
-      <c r="R3" s="238"/>
-      <c r="S3" s="238"/>
-      <c r="T3" s="238"/>
-      <c r="U3" s="238"/>
-      <c r="V3" s="238"/>
-      <c r="W3" s="238"/>
-      <c r="X3" s="238"/>
-      <c r="Y3" s="238"/>
-      <c r="Z3" s="238"/>
+      <c r="I3" s="236"/>
+      <c r="J3" s="236"/>
+      <c r="K3" s="236"/>
+      <c r="L3" s="236"/>
+      <c r="P3" s="250"/>
+      <c r="Q3" s="250"/>
+      <c r="R3" s="250"/>
+      <c r="S3" s="250"/>
+      <c r="T3" s="250"/>
+      <c r="U3" s="250"/>
+      <c r="V3" s="250"/>
+      <c r="W3" s="250"/>
+      <c r="X3" s="250"/>
+      <c r="Y3" s="250"/>
+      <c r="Z3" s="250"/>
       <c r="AB3" s="109"/>
     </row>
     <row r="4" spans="1:28" ht="10" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="5" spans="1:28" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="86"/>
       <c r="B5" s="60"/>
-      <c r="C5" s="234" t="s">
+      <c r="C5" s="245" t="s">
         <v>177</v>
       </c>
-      <c r="D5" s="234"/>
-      <c r="E5" s="234"/>
-      <c r="F5" s="234"/>
-      <c r="G5" s="234"/>
-      <c r="H5" s="234"/>
-      <c r="I5" s="234"/>
-      <c r="J5" s="234"/>
-      <c r="K5" s="234"/>
-      <c r="L5" s="234"/>
-      <c r="P5" s="238"/>
-      <c r="Q5" s="238"/>
-      <c r="R5" s="238"/>
-      <c r="S5" s="238"/>
-      <c r="T5" s="238"/>
-      <c r="U5" s="238"/>
-      <c r="V5" s="238"/>
-      <c r="W5" s="238"/>
-      <c r="X5" s="238"/>
-      <c r="Y5" s="238"/>
-      <c r="Z5" s="238"/>
+      <c r="D5" s="245"/>
+      <c r="E5" s="245"/>
+      <c r="F5" s="245"/>
+      <c r="G5" s="245"/>
+      <c r="H5" s="245"/>
+      <c r="I5" s="245"/>
+      <c r="J5" s="245"/>
+      <c r="K5" s="245"/>
+      <c r="L5" s="245"/>
+      <c r="P5" s="250"/>
+      <c r="Q5" s="250"/>
+      <c r="R5" s="250"/>
+      <c r="S5" s="250"/>
+      <c r="T5" s="250"/>
+      <c r="U5" s="250"/>
+      <c r="V5" s="250"/>
+      <c r="W5" s="250"/>
+      <c r="X5" s="250"/>
+      <c r="Y5" s="250"/>
+      <c r="Z5" s="250"/>
       <c r="AB5" s="110"/>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.2">
@@ -24896,7 +24867,7 @@
       <c r="K8" s="137"/>
       <c r="L8" s="126">
         <f ca="1">L7*(1+C20)/(C21-C20)</f>
-        <v>6331388.698795232</v>
+        <v>6331189.6655393308</v>
       </c>
       <c r="N8" s="91"/>
       <c r="O8" s="16"/>
@@ -24950,23 +24921,23 @@
       <c r="G10" s="138"/>
       <c r="H10" s="126">
         <f ca="1">H7/(1+$C$21)^H9</f>
-        <v>111084.50377973144</v>
+        <v>111084.25324193278</v>
       </c>
       <c r="I10" s="126">
         <f t="shared" ref="I10:L10" ca="1" si="1">I7/(1+$C$21)^I9</f>
-        <v>143046.72220639311</v>
+        <v>143046.07695760948</v>
       </c>
       <c r="J10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>184205.39353146552</v>
+        <v>184204.14717464327</v>
       </c>
       <c r="K10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>237206.60272889215</v>
+        <v>237204.46277176033</v>
       </c>
       <c r="L10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>305457.78980446124</v>
+        <v>305454.3452026294</v>
       </c>
       <c r="N10" s="91"/>
     </row>
@@ -24985,15 +24956,15 @@
       <c r="K11" s="137"/>
       <c r="L11" s="126">
         <f ca="1">L8/(1+C21)^L9</f>
-        <v>3952200.1879126369</v>
+        <v>3952031.3797521903</v>
       </c>
     </row>
     <row r="13" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="14" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="B14" s="249" t="s">
+      <c r="B14" s="251" t="s">
         <v>219</v>
       </c>
-      <c r="C14" s="250"/>
+      <c r="C14" s="252"/>
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B15" s="150" t="s">
@@ -25001,7 +24972,7 @@
       </c>
       <c r="C15" s="151">
         <f ca="1">Overview!C5</f>
-        <v>340.22500000000002</v>
+        <v>341.07</v>
       </c>
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.2">
@@ -25010,7 +24981,7 @@
       </c>
       <c r="C16" s="151">
         <f ca="1">C36</f>
-        <v>342.28958475836515</v>
+        <v>342.27748835828186</v>
       </c>
     </row>
     <row r="17" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -25020,20 +24991,20 @@
       <c r="C17" s="153">
         <v>0.41499999999999998</v>
       </c>
-      <c r="E17" s="251" t="s">
+      <c r="E17" s="253" t="s">
         <v>222</v>
       </c>
-      <c r="F17" s="251"/>
-      <c r="G17" s="251"/>
-      <c r="H17" s="251"/>
-      <c r="I17" s="251"/>
+      <c r="F17" s="253"/>
+      <c r="G17" s="253"/>
+      <c r="H17" s="253"/>
+      <c r="I17" s="253"/>
     </row>
     <row r="18" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B19" s="249" t="s">
+      <c r="B19" s="251" t="s">
         <v>181</v>
       </c>
-      <c r="C19" s="250"/>
+      <c r="C19" s="252"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B20" s="154" t="s">
@@ -25049,7 +25020,7 @@
       </c>
       <c r="C21" s="216">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.8833796565630266E-2</v>
+        <v>9.8836274859289808E-2</v>
       </c>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.2">
@@ -25067,7 +25038,7 @@
       </c>
       <c r="C23" s="156">
         <f ca="1">C15*C22</f>
-        <v>4965243.6500000004</v>
+        <v>4977575.58</v>
       </c>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.2">
@@ -25094,15 +25065,15 @@
       </c>
       <c r="C26" s="157">
         <f ca="1">C23+C25-C24</f>
-        <v>4903070.6500000004</v>
+        <v>4915402.58</v>
       </c>
     </row>
     <row r="27" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="28" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B28" s="249" t="s">
+      <c r="B28" s="251" t="s">
         <v>183</v>
       </c>
-      <c r="C28" s="250"/>
+      <c r="C28" s="252"/>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B29" s="154" t="s">
@@ -25110,7 +25081,7 @@
       </c>
       <c r="C29" s="156">
         <f ca="1">SUM(H10:L10)</f>
-        <v>981001.01205094345</v>
+        <v>980993.28534857533</v>
       </c>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
@@ -25119,7 +25090,7 @@
       </c>
       <c r="C30" s="156">
         <f ca="1">L11</f>
-        <v>3952200.1879126369</v>
+        <v>3952031.3797521903</v>
       </c>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.2">
@@ -25128,7 +25099,7 @@
       </c>
       <c r="C31" s="159">
         <f ca="1">C29+C30</f>
-        <v>4933201.1999635808</v>
+        <v>4933024.6651007654</v>
       </c>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.2">
@@ -25155,7 +25126,7 @@
       </c>
       <c r="C34" s="159">
         <f ca="1">C31+C32-C33</f>
-        <v>4995374.1999635808</v>
+        <v>4995197.6651007654</v>
       </c>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.2">
@@ -25173,21 +25144,21 @@
       </c>
       <c r="C36" s="162">
         <f ca="1">C34/C35</f>
-        <v>342.28958475836515</v>
+        <v>342.27748835828186</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="E17:I17"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B28:C28"/>
     <mergeCell ref="C3:G3"/>
     <mergeCell ref="H3:L3"/>
     <mergeCell ref="P3:W3"/>
     <mergeCell ref="X3:Z3"/>
     <mergeCell ref="C5:L5"/>
     <mergeCell ref="P5:Z5"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="E17:I17"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B28:C28"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -31692,7 +31663,7 @@
       </c>
       <c r="AC114" s="63">
         <f ca="1">Overview!C5</f>
-        <v>340.22500000000002</v>
+        <v>341.07</v>
       </c>
     </row>
     <row r="115" spans="1:31" x14ac:dyDescent="0.2">
@@ -31763,7 +31734,7 @@
       </c>
       <c r="AC115" s="65">
         <f ca="1">AC114/AC84</f>
-        <v>340.22500000000002</v>
+        <v>341.07</v>
       </c>
     </row>
     <row r="117" spans="1:31" x14ac:dyDescent="0.2">
@@ -32677,7 +32648,7 @@
       <c r="AA140" s="49"/>
       <c r="AC140" s="72">
         <f ca="1">AC115/Statement!AC25</f>
-        <v>39.016628440366979</v>
+        <v>39.113532110091747</v>
       </c>
     </row>
     <row r="141" spans="2:29" x14ac:dyDescent="0.2">
@@ -32714,7 +32685,7 @@
       <c r="AA141" s="49"/>
       <c r="AC141" s="72">
         <f ca="1">AC115/(Statement!AC5/Statement!AC21)</f>
-        <v>10.770892219856348</v>
+        <v>10.797643351977086</v>
       </c>
     </row>
     <row r="142" spans="2:29" x14ac:dyDescent="0.2">
@@ -32775,7 +32746,7 @@
       </c>
       <c r="AC142" s="72">
         <f ca="1">AC115/(Statement!AC48/Statement!AC74)</f>
-        <v>46.179721447172618</v>
+        <v>46.294415736607142</v>
       </c>
     </row>
     <row r="143" spans="2:29" x14ac:dyDescent="0.2">
@@ -32836,7 +32807,7 @@
       </c>
       <c r="AC143" s="141">
         <f ca="1">Statement!AC115*Statement!AC77</f>
-        <v>4985316.9250000007</v>
+        <v>4997698.71</v>
       </c>
     </row>
     <row r="144" spans="2:29" x14ac:dyDescent="0.2">
@@ -32897,7 +32868,7 @@
       </c>
       <c r="AC144" s="141">
         <f ca="1">AC143+AC106-AC105+AC47+AC44</f>
-        <v>4923143.9250000007</v>
+        <v>4935525.71</v>
       </c>
     </row>
     <row r="145" spans="2:29" x14ac:dyDescent="0.2">
@@ -32934,7 +32905,7 @@
       <c r="AA145" s="49"/>
       <c r="AC145" s="177">
         <f ca="1">AC144/AC5</f>
-        <v>10.546061194499844</v>
+        <v>10.572584705552211</v>
       </c>
     </row>
     <row r="146" spans="2:29" x14ac:dyDescent="0.2">
@@ -32971,7 +32942,7 @@
       <c r="AA146" s="49"/>
       <c r="AC146" s="177">
         <f ca="1">AC144/AC11</f>
-        <v>31.79113855184394</v>
+        <v>31.871093769170663</v>
       </c>
     </row>
     <row r="147" spans="2:29" x14ac:dyDescent="0.2">
@@ -33106,7 +33077,7 @@
       <c r="AA149" s="49"/>
       <c r="AC149" s="72">
         <f t="shared" ref="AC149:AC150" ca="1" si="137">AC143/AC147</f>
-        <v>40.538612301487277</v>
+        <v>40.639296047228342</v>
       </c>
     </row>
     <row r="150" spans="2:29" x14ac:dyDescent="0.2">
@@ -33143,7 +33114,7 @@
       <c r="AA150" s="49"/>
       <c r="AC150" s="72">
         <f t="shared" ca="1" si="137"/>
-        <v>38.530345023722319</v>
+        <v>38.627249452137846</v>
       </c>
     </row>
     <row r="151" spans="2:29" x14ac:dyDescent="0.2">
@@ -33180,7 +33151,7 @@
       <c r="AA151" s="49"/>
       <c r="AC151" s="74">
         <f t="shared" ref="AC151" ca="1" si="140">AC147/AC143</f>
-        <v>2.4667839948811273E-2</v>
+        <v>2.4606725442238592E-2</v>
       </c>
     </row>
     <row r="152" spans="2:29" x14ac:dyDescent="0.2">
@@ -33217,7 +33188,7 @@
       <c r="AA152" s="49"/>
       <c r="AC152" s="74">
         <f ca="1">AC25/AC115</f>
-        <v>2.5630097729443746E-2</v>
+        <v>2.5566599231829239E-2</v>
       </c>
     </row>
     <row r="153" spans="2:29" x14ac:dyDescent="0.2">
@@ -33254,7 +33225,7 @@
       <c r="AA153" s="49"/>
       <c r="AC153" s="149">
         <f ca="1">AC81/AC115</f>
-        <v>3.0861929605408185E-3</v>
+        <v>3.0785469258509984E-3</v>
       </c>
     </row>
     <row r="154" spans="2:29" x14ac:dyDescent="0.2">
@@ -33291,7 +33262,7 @@
       <c r="AA154" s="49"/>
       <c r="AC154" s="149">
         <f ca="1">-AC62/AC143</f>
-        <v>1.6493635457288401E-2</v>
+        <v>1.6452772520174592E-2</v>
       </c>
     </row>
     <row r="155" spans="2:29" x14ac:dyDescent="0.2">
@@ -33328,7 +33299,7 @@
       <c r="AA155" s="49"/>
       <c r="AC155" s="149">
         <f ca="1">-(AC62+AC63)/AC143</f>
-        <v>1.963084824341433E-2</v>
+        <v>1.9582212870131181E-2</v>
       </c>
     </row>
     <row r="156" spans="2:29" x14ac:dyDescent="0.2">
@@ -33831,7 +33802,7 @@
       <c r="AA166" s="49"/>
       <c r="AC166" s="149">
         <f ca="1">(AC105-AC106)/AC143</f>
-        <v>1.2471223181061851E-2</v>
+        <v>1.2440325759453395E-2</v>
       </c>
     </row>
     <row r="167" spans="1:31" x14ac:dyDescent="0.2">
@@ -35828,15 +35799,15 @@
       </c>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B4" s="235" t="s">
+      <c r="B4" s="236" t="s">
         <v>227</v>
       </c>
-      <c r="C4" s="235"/>
-      <c r="E4" s="235" t="s">
+      <c r="C4" s="236"/>
+      <c r="E4" s="236" t="s">
         <v>234</v>
       </c>
-      <c r="F4" s="235"/>
-      <c r="G4" s="235"/>
+      <c r="F4" s="236"/>
+      <c r="G4" s="236"/>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B5" s="20" t="s">
@@ -35844,7 +35815,7 @@
       </c>
       <c r="C5" s="166">
         <f ca="1">Overview!C5</f>
-        <v>340.22500000000002</v>
+        <v>341.07</v>
       </c>
       <c r="E5" s="12"/>
       <c r="F5" s="132" t="s">
@@ -35860,7 +35831,7 @@
       </c>
       <c r="C6" s="167">
         <f ca="1">Statement!AC143</f>
-        <v>4985316.9250000007</v>
+        <v>4997698.71</v>
       </c>
       <c r="E6" s="20" t="s">
         <v>19</v>
@@ -35880,7 +35851,7 @@
       </c>
       <c r="C7" s="167">
         <f ca="1">Statement!AC144</f>
-        <v>4923143.9250000007</v>
+        <v>4935525.71</v>
       </c>
       <c r="E7" s="20" t="s">
         <v>29</v>
@@ -35900,7 +35871,7 @@
       </c>
       <c r="C8" s="168">
         <f ca="1">Statement!AC140</f>
-        <v>39.016628440366979</v>
+        <v>39.113532110091747</v>
       </c>
       <c r="E8" s="20" t="s">
         <v>237</v>
@@ -35920,7 +35891,7 @@
       </c>
       <c r="C9" s="168">
         <f ca="1">Statement!AC141</f>
-        <v>10.770892219856348</v>
+        <v>10.797643351977086</v>
       </c>
       <c r="E9" s="20" t="s">
         <v>238</v>
@@ -35940,7 +35911,7 @@
       </c>
       <c r="C10" s="168">
         <f ca="1">Statement!AC142</f>
-        <v>46.179721447172618</v>
+        <v>46.294415736607142</v>
       </c>
       <c r="E10" s="20" t="s">
         <v>1</v>
@@ -35960,7 +35931,7 @@
       </c>
       <c r="C11" s="168">
         <f ca="1">Statement!AC145</f>
-        <v>10.546061194499844</v>
+        <v>10.572584705552211</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.2">
@@ -35969,18 +35940,18 @@
       </c>
       <c r="C12" s="168">
         <f ca="1">Statement!AC146</f>
-        <v>31.79113855184394</v>
+        <v>31.871093769170663</v>
       </c>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B15" s="235" t="s">
+      <c r="B15" s="236" t="s">
         <v>75</v>
       </c>
-      <c r="C15" s="235"/>
-      <c r="E15" s="235" t="s">
+      <c r="C15" s="236"/>
+      <c r="E15" s="236" t="s">
         <v>240</v>
       </c>
-      <c r="F15" s="235"/>
+      <c r="F15" s="236"/>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B16" s="20" t="s">
@@ -36031,14 +36002,14 @@
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B21" s="235" t="s">
+      <c r="B21" s="236" t="s">
         <v>239</v>
       </c>
-      <c r="C21" s="235"/>
-      <c r="E21" s="235" t="s">
+      <c r="C21" s="236"/>
+      <c r="E21" s="236" t="s">
         <v>243</v>
       </c>
-      <c r="F21" s="235"/>
+      <c r="F21" s="236"/>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B22" s="20" t="s">
@@ -36107,14 +36078,14 @@
       </c>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B29" s="235" t="s">
+      <c r="B29" s="236" t="s">
         <v>244</v>
       </c>
-      <c r="C29" s="235"/>
-      <c r="E29" s="235" t="s">
+      <c r="C29" s="236"/>
+      <c r="E29" s="236" t="s">
         <v>250</v>
       </c>
-      <c r="F29" s="235"/>
+      <c r="F29" s="236"/>
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B30" s="20" t="s">
@@ -36190,14 +36161,14 @@
       </c>
     </row>
     <row r="37" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B37" s="235" t="s">
+      <c r="B37" s="236" t="s">
         <v>262</v>
       </c>
-      <c r="C37" s="235"/>
-      <c r="E37" s="235" t="s">
+      <c r="C37" s="236"/>
+      <c r="E37" s="236" t="s">
         <v>265</v>
       </c>
-      <c r="F37" s="235"/>
+      <c r="F37" s="236"/>
     </row>
     <row r="38" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B38" s="20" t="s">
@@ -36205,7 +36176,7 @@
       </c>
       <c r="C38" s="169">
         <f ca="1">Statement!AC152</f>
-        <v>2.5630097729443746E-2</v>
+        <v>2.5566599231829239E-2</v>
       </c>
       <c r="E38" s="20" t="s">
         <v>264</v>
@@ -36221,7 +36192,7 @@
       </c>
       <c r="C39" s="209">
         <f ca="1">Statement!AC151</f>
-        <v>2.4667839948811273E-2</v>
+        <v>2.4606725442238592E-2</v>
       </c>
       <c r="E39" s="20" t="s">
         <v>266</v>
@@ -36237,7 +36208,7 @@
       </c>
       <c r="C40" s="169">
         <f ca="1">Statement!AC153</f>
-        <v>3.0861929605408185E-3</v>
+        <v>3.0785469258509984E-3</v>
       </c>
       <c r="E40" s="20" t="s">
         <v>267</v>
@@ -36253,7 +36224,7 @@
       </c>
       <c r="C41" s="169">
         <f ca="1">Statement!AC154</f>
-        <v>1.6493635457288401E-2</v>
+        <v>1.6452772520174592E-2</v>
       </c>
     </row>
     <row r="42" spans="2:6" x14ac:dyDescent="0.2">
@@ -36262,18 +36233,18 @@
       </c>
       <c r="C42" s="169">
         <f ca="1">Statement!AC155</f>
-        <v>1.963084824341433E-2</v>
+        <v>1.9582212870131181E-2</v>
       </c>
     </row>
     <row r="45" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B45" s="235" t="s">
+      <c r="B45" s="236" t="s">
         <v>273</v>
       </c>
-      <c r="C45" s="235"/>
-      <c r="E45" s="235" t="s">
+      <c r="C45" s="236"/>
+      <c r="E45" s="236" t="s">
         <v>279</v>
       </c>
-      <c r="F45" s="235"/>
+      <c r="F45" s="236"/>
     </row>
     <row r="46" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B46" s="20" t="s">
@@ -36306,18 +36277,18 @@
       </c>
       <c r="F48" s="169">
         <f ca="1">Statement!AC166</f>
-        <v>1.2471223181061851E-2</v>
+        <v>1.2440325759453395E-2</v>
       </c>
     </row>
     <row r="51" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B51" s="235" t="s">
+      <c r="B51" s="236" t="s">
         <v>276</v>
       </c>
-      <c r="C51" s="235"/>
-      <c r="E51" s="235" t="s">
+      <c r="C51" s="236"/>
+      <c r="E51" s="236" t="s">
         <v>297</v>
       </c>
-      <c r="F51" s="235"/>
+      <c r="F51" s="236"/>
     </row>
     <row r="52" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B52" s="20" t="s">
@@ -36485,7 +36456,7 @@
       </c>
       <c r="I6" s="166">
         <f ca="1">Statement!AC114</f>
-        <v>340.22500000000002</v>
+        <v>341.07</v>
       </c>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.2">
@@ -36514,7 +36485,7 @@
       </c>
       <c r="I7" s="167">
         <f ca="1">Statement!AC143</f>
-        <v>4985316.9250000007</v>
+        <v>4997698.71</v>
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
@@ -36543,7 +36514,7 @@
       </c>
       <c r="I8" s="167">
         <f ca="1">Statement!AC144</f>
-        <v>4923143.9250000007</v>
+        <v>4935525.71</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
@@ -36572,7 +36543,7 @@
       </c>
       <c r="I9" s="168">
         <f ca="1">Statement!AC140</f>
-        <v>39.016628440366979</v>
+        <v>39.113532110091747</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.2">
@@ -36601,7 +36572,7 @@
       </c>
       <c r="I10" s="168">
         <f ca="1">Statement!AC141</f>
-        <v>10.770892219856348</v>
+        <v>10.797643351977086</v>
       </c>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.2">
@@ -36630,7 +36601,7 @@
       </c>
       <c r="I11" s="168">
         <f ca="1">Statement!AC142</f>
-        <v>46.179721447172618</v>
+        <v>46.294415736607142</v>
       </c>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.2">
@@ -36659,7 +36630,7 @@
       </c>
       <c r="I12" s="168">
         <f ca="1">Statement!AC145</f>
-        <v>10.546061194499844</v>
+        <v>10.572584705552211</v>
       </c>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
@@ -36688,7 +36659,7 @@
       </c>
       <c r="I13" s="168">
         <f ca="1">Statement!AC146</f>
-        <v>31.79113855184394</v>
+        <v>31.871093769170663</v>
       </c>
     </row>
     <row r="15" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -37461,7 +37432,7 @@
       </c>
       <c r="I51" s="169">
         <f ca="1">Statement!AC152</f>
-        <v>2.5630097729443746E-2</v>
+        <v>2.5566599231829239E-2</v>
       </c>
     </row>
     <row r="52" spans="2:9" x14ac:dyDescent="0.2">
@@ -37490,7 +37461,7 @@
       </c>
       <c r="I52" s="169">
         <f ca="1">Statement!AC151</f>
-        <v>2.4667839948811273E-2</v>
+        <v>2.4606725442238592E-2</v>
       </c>
     </row>
     <row r="53" spans="2:9" x14ac:dyDescent="0.2">
@@ -37519,7 +37490,7 @@
       </c>
       <c r="I53" s="169">
         <f ca="1">Statement!AC153</f>
-        <v>3.0861929605408185E-3</v>
+        <v>3.0785469258509984E-3</v>
       </c>
     </row>
     <row r="54" spans="2:9" x14ac:dyDescent="0.2">
@@ -37548,7 +37519,7 @@
       </c>
       <c r="I54" s="169">
         <f ca="1">Statement!AC154</f>
-        <v>1.6493635457288401E-2</v>
+        <v>1.6452772520174592E-2</v>
       </c>
     </row>
     <row r="55" spans="2:9" x14ac:dyDescent="0.2">
@@ -37577,7 +37548,7 @@
       </c>
       <c r="I55" s="169">
         <f ca="1">Statement!AC155</f>
-        <v>1.963084824341433E-2</v>
+        <v>1.9582212870131181E-2</v>
       </c>
     </row>
     <row r="57" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -37813,7 +37784,7 @@
       </c>
       <c r="I68" s="190">
         <f ca="1">Statement!AC166</f>
-        <v>1.2471223181061851E-2</v>
+        <v>1.2440325759453395E-2</v>
       </c>
     </row>
     <row r="70" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -38505,14 +38476,14 @@
     <row r="1" spans="2:7" ht="12" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="3" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B3" s="8"/>
-      <c r="C3" s="244" t="s">
+      <c r="C3" s="240" t="s">
         <v>307</v>
       </c>
-      <c r="D3" s="245"/>
-      <c r="F3" s="246" t="s">
+      <c r="D3" s="241"/>
+      <c r="F3" s="242" t="s">
         <v>308</v>
       </c>
-      <c r="G3" s="245"/>
+      <c r="G3" s="241"/>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B4" s="8"/>
@@ -38579,19 +38550,19 @@
       <c r="B7" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C7" s="242">
+      <c r="C7" s="243">
         <f>Statement!AA88</f>
         <v>-1.5892574471146927E-2</v>
       </c>
-      <c r="D7" s="243"/>
-      <c r="F7" s="242">
+      <c r="D7" s="244"/>
+      <c r="F7" s="243">
         <f>IF(F6=0,
 IF(G6=0,0,IF(G6&gt;0,1,-1)),
 (G6-F6)/ABS(F6)
 )</f>
         <v>0.16356501765281381</v>
       </c>
-      <c r="G7" s="243"/>
+      <c r="G7" s="244"/>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B8" s="201" t="s">
@@ -38618,19 +38589,19 @@
       <c r="B9" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C9" s="242">
+      <c r="C9" s="243">
         <f>Statement!AA89</f>
         <v>-3.1133095757317875E-2</v>
       </c>
-      <c r="D9" s="243"/>
-      <c r="F9" s="242">
+      <c r="D9" s="244"/>
+      <c r="F9" s="243">
         <f>IF(F8=0,
 IF(G8=0,0,IF(G8&gt;0,1,-1)),
 (G8-F8)/ABS(F8)
 )</f>
         <v>8.6032831193608647E-2</v>
       </c>
-      <c r="G9" s="243"/>
+      <c r="G9" s="244"/>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B10" s="201" t="s">
@@ -38657,19 +38628,19 @@
       <c r="B11" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C11" s="242">
+      <c r="C11" s="243">
         <f>Statement!AA90</f>
         <v>-2.0079954728829339E-4</v>
       </c>
-      <c r="D11" s="243"/>
-      <c r="F11" s="242">
+      <c r="D11" s="244"/>
+      <c r="F11" s="243">
         <f>IF(F10=0,
 IF(G10=0,0,IF(G10&gt;0,1,-1)),
 (G10-F10)/ABS(F10)
 )</f>
         <v>0.25280204949906215</v>
       </c>
-      <c r="G11" s="243"/>
+      <c r="G11" s="244"/>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B12" s="201" t="s">
@@ -38696,19 +38667,19 @@
       <c r="B13" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C13" s="242">
+      <c r="C13" s="243">
         <f>Statement!AA93</f>
         <v>9.4729043183742583E-3</v>
       </c>
-      <c r="D13" s="243"/>
-      <c r="F13" s="242">
+      <c r="D13" s="244"/>
+      <c r="F13" s="243">
         <f>IF(F12=0,
 IF(G12=0,0,IF(G12&gt;0,1,-1)),
 (G12-F12)/ABS(F12)
 )</f>
         <v>0.22937612786800721</v>
       </c>
-      <c r="G13" s="243"/>
+      <c r="G13" s="244"/>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B14" s="201" t="s">
@@ -38735,19 +38706,19 @@
       <c r="B15" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C15" s="242">
+      <c r="C15" s="243">
         <f>Statement!AA94</f>
         <v>-5.2946913752264175E-3</v>
       </c>
-      <c r="D15" s="243"/>
-      <c r="F15" s="242">
+      <c r="D15" s="244"/>
+      <c r="F15" s="243">
         <f>IF(F14=0,
 IF(G14=0,0,IF(G14&gt;0,1,-1)),
 (G14-F14)/ABS(F14)
 )</f>
         <v>0.26569037656903766</v>
       </c>
-      <c r="G15" s="243"/>
+      <c r="G15" s="244"/>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B16" s="201" t="s">
@@ -38774,19 +38745,19 @@
       <c r="B17" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C17" s="242">
+      <c r="C17" s="243">
         <f>Statement!AA96</f>
         <v>7.1336804381635002E-3</v>
       </c>
-      <c r="D17" s="243"/>
-      <c r="F17" s="242">
+      <c r="D17" s="244"/>
+      <c r="F17" s="243">
         <f>IF(F16=0,
 IF(G16=0,0,IF(G16&gt;0,1,-1)),
 (G16-F16)/ABS(F16)
 )</f>
         <v>0.27118716394981651</v>
       </c>
-      <c r="G17" s="243"/>
+      <c r="G17" s="244"/>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B18" s="201" t="s">
@@ -38813,22 +38784,22 @@
       <c r="B19" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C19" s="242">
+      <c r="C19" s="243">
         <f>IF(C18=0,
 IF(D18=0,0,IF(D18&gt;0,1,-1)),
 (D18-C18)/ABS(C18)
 )</f>
         <v>-7.4697813391280731E-4</v>
       </c>
-      <c r="D19" s="243"/>
-      <c r="F19" s="242">
+      <c r="D19" s="244"/>
+      <c r="F19" s="243">
         <f>IF(F18=0,
 IF(G18=0,0,IF(G18&gt;0,1,-1)),
 (G18-F18)/ABS(F18)
 )</f>
         <v>-1.5587369547765587E-2</v>
       </c>
-      <c r="G19" s="243"/>
+      <c r="G19" s="244"/>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B20" s="201" t="s">
@@ -38855,22 +38826,22 @@
       <c r="B21" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C21" s="242">
+      <c r="C21" s="243">
         <f>IF(C20=0,
 IF(D20=0,0,IF(D20&gt;0,1,-1)),
 (D20-C20)/ABS(C20)
 )</f>
         <v>4.975124378109568E-3</v>
       </c>
-      <c r="D21" s="243"/>
-      <c r="F21" s="242">
+      <c r="D21" s="244"/>
+      <c r="F21" s="243">
         <f>IF(F20=0,
 IF(G20=0,0,IF(G20&gt;0,1,-1)),
 (G20-F20)/ABS(F20)
 )</f>
         <v>0.28662420382165599</v>
       </c>
-      <c r="G21" s="243"/>
+      <c r="G21" s="244"/>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23" s="8" t="s">
@@ -38918,22 +38889,22 @@
       <c r="B25" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C25" s="242">
+      <c r="C25" s="243">
         <f>IF(C24=0,
 IF(D24=0,0,IF(D24&gt;0,1,-1)),
 (D24-C24)/ABS(C24)
 )</f>
         <v>1.5257357017718937E-2</v>
       </c>
-      <c r="D25" s="243"/>
-      <c r="F25" s="242">
+      <c r="D25" s="244"/>
+      <c r="F25" s="243">
         <f>IF(F24=0,
 IF(G24=0,0,IF(G24&gt;0,1,-1)),
 (G24-F24)/ABS(F24)
 )</f>
         <v>0.11124326423612797</v>
       </c>
-      <c r="G25" s="243"/>
+      <c r="G25" s="244"/>
     </row>
     <row r="26" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B26" s="20" t="s">
@@ -38960,22 +38931,22 @@
       <c r="B27" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C27" s="242">
+      <c r="C27" s="243">
         <f>IF(C26=0,
 IF(D26=0,0,IF(D26&gt;0,1,-1)),
 (D26-C26)/ABS(C26)
 )</f>
         <v>4.7692033505613969E-2</v>
       </c>
-      <c r="D27" s="243"/>
-      <c r="F27" s="242">
+      <c r="D27" s="244"/>
+      <c r="F27" s="243">
         <f>IF(F26=0,
 IF(G26=0,0,IF(G26&gt;0,1,-1)),
 (G26-F26)/ABS(F26)
 )</f>
         <v>0.22399433663696178</v>
       </c>
-      <c r="G27" s="243"/>
+      <c r="G27" s="244"/>
     </row>
     <row r="28" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B28" s="20" t="s">
@@ -39002,22 +38973,22 @@
       <c r="B29" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C29" s="242">
+      <c r="C29" s="243">
         <f>IF(C28=0,
 IF(D28=0,0,IF(D28&gt;0,1,-1)),
 (D28-C28)/ABS(C28)
 )</f>
         <v>-8.2012001756354591E-2</v>
       </c>
-      <c r="D29" s="243"/>
-      <c r="F29" s="242">
+      <c r="D29" s="244"/>
+      <c r="F29" s="243">
         <f>IF(F28=0,
 IF(G28=0,0,IF(G28&gt;0,1,-1)),
 (G28-F28)/ABS(F28)
 )</f>
         <v>0.22428264688658989</v>
       </c>
-      <c r="G29" s="243"/>
+      <c r="G29" s="244"/>
     </row>
     <row r="30" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B30" s="20" t="s">
@@ -39044,22 +39015,22 @@
       <c r="B31" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C31" s="242">
+      <c r="C31" s="243">
         <f>IF(C30=0,
 IF(D30=0,0,IF(D30&gt;0,1,-1)),
 (D30-C30)/ABS(C30)
 )</f>
         <v>-0.21985477919295321</v>
       </c>
-      <c r="D31" s="243"/>
-      <c r="F31" s="242">
+      <c r="D31" s="244"/>
+      <c r="F31" s="243">
         <f>IF(F30=0,
 IF(G30=0,0,IF(G30&gt;0,1,-1)),
 (G30-F30)/ABS(F30)
 )</f>
         <v>0.1335178139052231</v>
       </c>
-      <c r="G31" s="243"/>
+      <c r="G31" s="244"/>
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B32" s="20" t="s">
@@ -39086,22 +39057,22 @@
       <c r="B33" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C33" s="242">
+      <c r="C33" s="243">
         <f>IF(C32=0,
 IF(D32=0,0,IF(D32&gt;0,1,-1)),
 (D32-C32)/ABS(C32)
 )</f>
         <v>-2.9218647406434668E-2</v>
       </c>
-      <c r="D33" s="243"/>
-      <c r="F33" s="242">
+      <c r="D33" s="244"/>
+      <c r="F33" s="243">
         <f>IF(F32=0,
 IF(G32=0,0,IF(G32&gt;0,1,-1)),
 (G32-F32)/ABS(F32)
 )</f>
         <v>0.15613189104652678</v>
       </c>
-      <c r="G33" s="243"/>
+      <c r="G33" s="244"/>
     </row>
     <row r="35" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B35" s="224" t="s">
@@ -39128,22 +39099,22 @@
       <c r="B36" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C36" s="242">
+      <c r="C36" s="243">
         <f>IF(C35=0,
 IF(D35=0,0,IF(D35&gt;0,1,-1)),
 (D35-C35)/ABS(C35)
 )</f>
         <v>-4.8110327402884512E-2</v>
       </c>
-      <c r="D36" s="243"/>
-      <c r="F36" s="242">
+      <c r="D36" s="244"/>
+      <c r="F36" s="243">
         <f>IF(F35=0,
 IF(G35=0,0,IF(G35&gt;0,1,-1)),
 (G35-F35)/ABS(F35)
 )</f>
         <v>0.21690368310080302</v>
       </c>
-      <c r="G36" s="243"/>
+      <c r="G36" s="244"/>
     </row>
     <row r="37" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B37" s="224" t="s">
@@ -39170,22 +39141,22 @@
       <c r="B38" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C38" s="242">
+      <c r="C38" s="243">
         <f>IF(C37=0,
 IF(D37=0,0,IF(D37&gt;0,1,-1)),
 (D37-C37)/ABS(C37)
 )</f>
         <v>0.23252768186688891</v>
       </c>
-      <c r="D38" s="243"/>
-      <c r="F38" s="242">
+      <c r="D38" s="244"/>
+      <c r="F38" s="243">
         <f>IF(F37=0,
 IF(G37=0,0,IF(G37&gt;0,1,-1)),
 (G37-F37)/ABS(F37)
 )</f>
         <v>0.28660203827989061</v>
       </c>
-      <c r="G38" s="243"/>
+      <c r="G38" s="244"/>
     </row>
     <row r="39" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B39" s="224" t="s">
@@ -39212,22 +39183,22 @@
       <c r="B40" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C40" s="242">
+      <c r="C40" s="243">
         <f>IF(C39=0,
 IF(D39=0,0,IF(D39&gt;0,1,-1)),
 (D39-C39)/ABS(C39)
 )</f>
         <v>-0.10457043679490888</v>
       </c>
-      <c r="D40" s="243"/>
-      <c r="F40" s="242">
+      <c r="D40" s="244"/>
+      <c r="F40" s="243">
         <f>IF(F39=0,
 IF(G39=0,0,IF(G39&gt;0,1,-1)),
 (G39-F39)/ABS(F39)
 )</f>
         <v>-5.9261510408752466E-2</v>
       </c>
-      <c r="G40" s="243"/>
+      <c r="G40" s="244"/>
     </row>
     <row r="41" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B41" s="224" t="s">
@@ -39254,22 +39225,22 @@
       <c r="B42" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C42" s="242">
+      <c r="C42" s="243">
         <f>IF(C41=0,
 IF(D41=0,0,IF(D41&gt;0,1,-1)),
 (D41-C41)/ABS(C41)
 )</f>
         <v>-2.2781926338438173E-3</v>
       </c>
-      <c r="D42" s="243"/>
-      <c r="F42" s="242">
+      <c r="D42" s="244"/>
+      <c r="F42" s="243">
         <f>IF(F41=0,
 IF(G41=0,0,IF(G41&gt;0,1,-1)),
 (G41-F41)/ABS(F41)
 )</f>
         <v>6.4694759589411135E-2</v>
       </c>
-      <c r="G42" s="243"/>
+      <c r="G42" s="244"/>
     </row>
     <row r="43" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B43" s="224" t="s">
@@ -39296,55 +39267,25 @@
       <c r="B44" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C44" s="242">
+      <c r="C44" s="243">
         <f>IF(C43=0,
 IF(D43=0,0,IF(D43&gt;0,1,-1)),
 (D43-C43)/ABS(C43)
 )</f>
         <v>-7.6510847107438013E-3</v>
       </c>
-      <c r="D44" s="243"/>
-      <c r="F44" s="242">
+      <c r="D44" s="244"/>
+      <c r="F44" s="243">
         <f>IF(F43=0,
 IF(G43=0,0,IF(G43&gt;0,1,-1)),
 (G43-F43)/ABS(F43)
 )</f>
         <v>0.12092039528862633</v>
       </c>
-      <c r="G44" s="243"/>
+      <c r="G44" s="244"/>
     </row>
   </sheetData>
   <mergeCells count="38">
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="F36:G36"/>
     <mergeCell ref="C44:D44"/>
     <mergeCell ref="F44:G44"/>
     <mergeCell ref="C38:D38"/>
@@ -39353,6 +39294,36 @@
     <mergeCell ref="F40:G40"/>
     <mergeCell ref="C42:D42"/>
     <mergeCell ref="F42:G42"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="F36:G36"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="F9:G9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>

</xml_diff>

<commit_message>
Added the EV/Sales value on the front page
</commit_message>
<xml_diff>
--- a/AAPL.xlsx
+++ b/AAPL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/KINGSTON/MyStockData/Finance-StockLists/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5B2F8EE-0F64-F947-90DB-A93C0C99C867}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02A09294-29B9-AF43-9492-6F52668346FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14400" firstSheet="8" activeTab="18" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14400" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -152,7 +152,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="800" uniqueCount="418">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="801" uniqueCount="419">
   <si>
     <t>Ticker</t>
   </si>
@@ -1406,6 +1406,9 @@
   </si>
   <si>
     <t>Applied EV/Sales ratio</t>
+  </si>
+  <si>
+    <t>Reverse DCF rate</t>
   </si>
 </sst>
 </file>
@@ -2329,18 +2332,6 @@
     <xf numFmtId="39" fontId="10" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="7" fillId="9" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2350,10 +2341,7 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="18" fillId="17" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="18" fillId="17" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2365,23 +2353,38 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="168" fontId="18" fillId="17" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="18" fillId="17" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -15520,11 +15523,11 @@
     <v>Powered by Refinitiv</v>
     <v>345.34</v>
     <v>243.42</v>
-    <v>1.0737000000000001</v>
-    <v>5.15</v>
-    <v>1.5330999999999999E-2</v>
-    <v>0.39</v>
-    <v>1.1429999999999999E-3</v>
+    <v>1.0696000000000001</v>
+    <v>-9</v>
+    <v>-2.6596000000000002E-2</v>
+    <v>0.68</v>
+    <v>2.0639999999999999E-3</v>
     <v>USD</v>
     <v>Apple Inc. designs, manufactures and markets smartphones, personal computers, tablets, wearables and accessories, and sells a variety of related services. Its product categories include iPhone, Mac, iPad, Wearables, Home and Accessories. Its services include advertising, AppleCare, cloud services, digital content, and payment services. The Company operates various platforms, including the App Store, that allow customers to discover and download applications and digital content, such as books, music, video, games and podcasts. It also offers digital content through subscription-based services, including Apple Arcade, Apple Fitness+, Apple Music, Apple News+, and Apple TV+. Its wearables include smartwatches, wireless headphones, and spatial computers. Its products include iPhone 16 Pro, iPhone 16, iPhone 15, iPhone 14, iPhone SE, MacBook Air, MacBook Pro, iMac, Mac mini, Mac Studio, Mac Pro, iPad Pro, iPad Air, AirPods, AirPods Pro, AirPods Max, Apple TV, Apple Vision Pro and others.</v>
     <v>166000</v>
@@ -15532,25 +15535,25 @@
     <v>XNAS</v>
     <v>XNAS</v>
     <v>One Apple Park Way, CUPERTINO, CA, 95014 US</v>
-    <v>341.67</v>
+    <v>337.08499999999998</v>
     <v>Computers, Phones &amp; Household Electronics</v>
     <v>Stock</v>
-    <v>46290.99998606406</v>
+    <v>46294.96824790469</v>
     <v>0</v>
-    <v>334.53</v>
-    <v>4977636972600</v>
+    <v>328.7</v>
+    <v>4807322892000</v>
     <v>APPLE INC.</v>
     <v>APPLE INC.</v>
-    <v>336.04</v>
-    <v>38.653300000000002</v>
-    <v>335.92</v>
-    <v>341.07</v>
-    <v>341.46</v>
+    <v>336.96499999999997</v>
+    <v>38.938699999999997</v>
+    <v>338.4</v>
+    <v>329.4</v>
+    <v>330.08</v>
     <v>14594180000</v>
     <v>AAPL</v>
     <v>APPLE INC. (XNAS:AAPL)</v>
-    <v>30002507</v>
-    <v>41709089</v>
+    <v>38455644</v>
+    <v>40708584</v>
     <v>1977</v>
   </rv>
   <rv s="2">
@@ -15572,19 +15575,19 @@
     <v>268435456</v>
     <v>1</v>
     <v>Powered by Refinitiv</v>
-    <v>52.3</v>
+    <v>52.93</v>
     <v>39.47</v>
-    <v>0.22</v>
-    <v>4.2620000000000002E-3</v>
+    <v>0.15</v>
+    <v>2.8630000000000001E-3</v>
     <v>US</v>
-    <v>52.3</v>
+    <v>52.93</v>
     <v>Index</v>
     <v>3</v>
-    <v>51.62</v>
+    <v>52.13</v>
     <v>10 Y TSY YLD NDX</v>
-    <v>51.86</v>
-    <v>51.62</v>
-    <v>51.84</v>
+    <v>52.13</v>
+    <v>52.4</v>
+    <v>52.55</v>
     <v>TNX</v>
     <v>10 Y TSY YLD NDX</v>
   </rv>
@@ -15806,9 +15809,9 @@
       <v>at close</v>
       <v>from previous close</v>
       <v>from previous close</v>
-      <v>Source: Nasdaq</v>
+      <v>Source: Nasdaq Last Sale</v>
       <v>GMT</v>
-      <v>Delayed 15 minutes</v>
+      <v>Real-Time Nasdaq Last Sale</v>
       <v>from close</v>
       <v>from close</v>
     </spb>
@@ -16379,18 +16382,18 @@
   <sheetData>
     <row r="1" spans="2:9" ht="11" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="2" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="240" t="s">
+      <c r="B2" s="236" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="241"/>
-      <c r="E2" s="240" t="s">
+      <c r="C2" s="237"/>
+      <c r="E2" s="236" t="s">
         <v>281</v>
       </c>
-      <c r="F2" s="241"/>
-      <c r="H2" s="240" t="s">
+      <c r="F2" s="237"/>
+      <c r="H2" s="236" t="s">
         <v>319</v>
       </c>
-      <c r="I2" s="241"/>
+      <c r="I2" s="237"/>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B3" s="179" t="s">
@@ -16405,7 +16408,7 @@
       </c>
       <c r="F3" s="181">
         <f ca="1">Statement!AC143</f>
-        <v>4997698.71</v>
+        <v>4826698.1999999993</v>
       </c>
       <c r="H3" s="179" t="str">
         <f>'AVG target price'!B5</f>
@@ -16413,7 +16416,7 @@
       </c>
       <c r="I3" s="205">
         <f ca="1">'AVG target price'!C5</f>
-        <v>114.14777193331305</v>
+        <v>113.46679690078477</v>
       </c>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.2">
@@ -16429,7 +16432,7 @@
       </c>
       <c r="F4" s="182">
         <f ca="1">Statement!AC144</f>
-        <v>4935525.71</v>
+        <v>4764525.1999999993</v>
       </c>
       <c r="H4" s="179" t="str">
         <f>'AVG target price'!B6</f>
@@ -16437,7 +16440,7 @@
       </c>
       <c r="I4" s="205">
         <f ca="1">'AVG target price'!C6</f>
-        <v>229.39757505520808</v>
+        <v>228.93447629680676</v>
       </c>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.2">
@@ -16446,7 +16449,7 @@
       </c>
       <c r="C5" s="202" cm="1">
         <f t="array" aca="1" ref="C5" ca="1">_FV(C3,"Price",TRUE)</f>
-        <v>341.07</v>
+        <v>329.4</v>
       </c>
       <c r="E5" s="179" t="s">
         <v>237</v>
@@ -16461,7 +16464,7 @@
       </c>
       <c r="I5" s="205">
         <f ca="1">'AVG target price'!C7</f>
-        <v>200.97536240722781</v>
+        <v>200.49606068515598</v>
       </c>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.2">
@@ -16470,14 +16473,14 @@
       </c>
       <c r="C6" s="202" cm="1">
         <f t="array" aca="1" ref="C6" ca="1">_FV(C3,"Price (Extended hours)",TRUE)</f>
-        <v>341.46</v>
+        <v>330.08</v>
       </c>
       <c r="E6" s="179" t="s">
         <v>231</v>
       </c>
       <c r="F6" s="184">
         <f ca="1">Statement!AC140</f>
-        <v>39.113532110091747</v>
+        <v>37.775229357798167</v>
       </c>
       <c r="H6" s="179" t="str">
         <f>'AVG target price'!B8</f>
@@ -16485,7 +16488,7 @@
       </c>
       <c r="I6" s="205">
         <f ca="1">'AVG target price'!C8</f>
-        <v>199.45815175947126</v>
+        <v>199.06047234671664</v>
       </c>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.2">
@@ -16494,22 +16497,22 @@
       </c>
       <c r="C7" s="6" cm="1">
         <f t="array" aca="1" ref="C7" ca="1">_FV(C3,"Change")</f>
-        <v>5.15</v>
+        <v>-9</v>
       </c>
       <c r="E7" s="180" t="s">
         <v>198</v>
       </c>
       <c r="F7" s="185">
         <f ca="1">Statement!AC141</f>
-        <v>10.797643351977086</v>
-      </c>
-      <c r="H7" s="178" t="str">
-        <f>'AVG target price'!B10</f>
-        <v>AVG price</v>
-      </c>
-      <c r="I7" s="206">
-        <f ca="1">'AVG target price'!C10</f>
-        <v>191.49113324644583</v>
+        <v>10.428192805410186</v>
+      </c>
+      <c r="H7" s="179" t="str">
+        <f>'AVG target price'!B9</f>
+        <v>EV/Sales price</v>
+      </c>
+      <c r="I7" s="205">
+        <f ca="1">'AVG target price'!C9</f>
+        <v>213.04849410806756</v>
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
@@ -16518,22 +16521,22 @@
       </c>
       <c r="C8" s="6" cm="1">
         <f t="array" aca="1" ref="C8" ca="1">_FV(C3,"Change (extended hours)",TRUE)</f>
-        <v>0.39</v>
+        <v>0.68</v>
       </c>
       <c r="E8" s="179" t="s">
         <v>259</v>
       </c>
       <c r="F8" s="186">
         <f ca="1">Statement!AC151</f>
-        <v>2.4606725442238592E-2</v>
+        <v>2.5478493766194044E-2</v>
       </c>
       <c r="H8" s="178" t="str">
-        <f>'AVG target price'!B12</f>
-        <v>Upside/Downside</v>
-      </c>
-      <c r="I8" s="207">
-        <f ca="1">'AVG target price'!C12</f>
-        <v>-0.43855767658707645</v>
+        <f>'AVG target price'!B10</f>
+        <v>AVG price</v>
+      </c>
+      <c r="I8" s="206">
+        <f ca="1">'AVG target price'!C10</f>
+        <v>191.00126006750634</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
@@ -16542,14 +16545,22 @@
       </c>
       <c r="C9" s="73" cm="1">
         <f t="array" aca="1" ref="C9" ca="1">_FV(C3,"Change (%)",TRUE)</f>
-        <v>1.5330999999999999E-2</v>
+        <v>-2.6596000000000002E-2</v>
       </c>
       <c r="E9" s="179" t="s">
         <v>282</v>
       </c>
       <c r="F9" s="186">
         <f ca="1">Statement!AC152</f>
-        <v>2.5566599231829239E-2</v>
+        <v>2.6472374013357617E-2</v>
+      </c>
+      <c r="H9" s="178" t="str">
+        <f>'AVG target price'!B12</f>
+        <v>Upside/Downside</v>
+      </c>
+      <c r="I9" s="207">
+        <f ca="1">'AVG target price'!C12</f>
+        <v>-0.42015403743926427</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.2">
@@ -16558,21 +16569,14 @@
       </c>
       <c r="C10" s="73" cm="1">
         <f t="array" aca="1" ref="C10" ca="1">_FV(C3,"Change % (extended hours)",TRUE)</f>
-        <v>1.1429999999999999E-3</v>
+        <v>2.0639999999999999E-3</v>
       </c>
       <c r="E10" s="179" t="s">
         <v>287</v>
       </c>
       <c r="F10" s="186">
         <f ca="1">Statement!AC154</f>
-        <v>1.6452772520174592E-2</v>
-      </c>
-      <c r="H10" s="178" t="s">
-        <v>394</v>
-      </c>
-      <c r="I10" s="206">
-        <f ca="1">DDM!C26</f>
-        <v>13.234110770804612</v>
+        <v>1.7035662184140706E-2</v>
       </c>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.2">
@@ -16588,7 +16592,14 @@
       </c>
       <c r="F11" s="187">
         <f ca="1">Statement!AC153</f>
-        <v>3.0785469258509984E-3</v>
+        <v>3.1876138433515485E-3</v>
+      </c>
+      <c r="H11" s="178" t="s">
+        <v>394</v>
+      </c>
+      <c r="I11" s="206">
+        <f ca="1">DDM!C26</f>
+        <v>13.147914032869787</v>
       </c>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.2">
@@ -16613,7 +16624,7 @@
       </c>
       <c r="C13" s="203" cm="1">
         <f t="array" aca="1" ref="C13" ca="1">_FV(C3,"Beta")</f>
-        <v>1.0737000000000001</v>
+        <v>1.0696000000000001</v>
       </c>
       <c r="E13" s="179" t="s">
         <v>101</v>
@@ -16622,6 +16633,13 @@
         <f>Statement!AC123</f>
         <v>1.1991257440476193</v>
       </c>
+      <c r="H13" s="178" t="s">
+        <v>418</v>
+      </c>
+      <c r="I13" s="207">
+        <f>'Reverse DCF'!C17</f>
+        <v>0.41499999999999998</v>
+      </c>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B14" s="180" t="s">
@@ -16629,7 +16647,7 @@
       </c>
       <c r="C14" s="204" cm="1">
         <f t="array" aca="1" ref="C14" ca="1">_FV(C3,"Volume average",TRUE)</f>
-        <v>41709089</v>
+        <v>40708584</v>
       </c>
       <c r="E14" s="180" t="s">
         <v>102</v>
@@ -16645,7 +16663,7 @@
       </c>
       <c r="F15" s="186">
         <f ca="1">Statement!AC166</f>
-        <v>1.2440325759453395E-2</v>
+        <v>1.2881062254938585E-2</v>
       </c>
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.2">
@@ -16658,10 +16676,10 @@
       </c>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B17" s="242" t="s">
+      <c r="B17" s="238" t="s">
         <v>88</v>
       </c>
-      <c r="C17" s="242"/>
+      <c r="C17" s="238"/>
       <c r="E17" s="178" t="s">
         <v>290</v>
       </c>
@@ -16684,7 +16702,6 @@
         <f>Statement!AC134</f>
         <v>-56.814895644278849</v>
       </c>
-      <c r="I18" s="50"/>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B19" s="178" t="s">
@@ -16700,6 +16717,7 @@
         <f>Statement!AC136</f>
         <v>-0.57824590773809526</v>
       </c>
+      <c r="I19" s="50"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B20" s="178" t="s">
@@ -16723,7 +16741,6 @@
       <c r="C21" s="69" t="s">
         <v>91</v>
       </c>
-      <c r="I21" s="50"/>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B22" s="178" t="s">
@@ -16732,16 +16749,17 @@
       <c r="C22" s="69" t="s">
         <v>392</v>
       </c>
+      <c r="I22" s="50"/>
     </row>
     <row r="25" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B25" s="242" t="s">
+      <c r="B25" s="238" t="s">
         <v>104</v>
       </c>
-      <c r="C25" s="242"/>
-      <c r="E25" s="240" t="s">
+      <c r="C25" s="238"/>
+      <c r="E25" s="236" t="s">
         <v>332</v>
       </c>
-      <c r="F25" s="241"/>
+      <c r="F25" s="237"/>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B26" s="178" t="s">
@@ -16755,7 +16773,7 @@
       </c>
       <c r="F26" s="213" cm="1">
         <f t="array" aca="1" ref="F26" ca="1">_FV(E26,"Price")</f>
-        <v>51.84</v>
+        <v>52.55</v>
       </c>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.2">
@@ -16770,7 +16788,7 @@
       </c>
       <c r="F27" s="214">
         <f ca="1">F26/1000</f>
-        <v>5.1840000000000004E-2</v>
+        <v>5.2549999999999999E-2</v>
       </c>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.2">
@@ -16790,15 +16808,15 @@
       </c>
     </row>
     <row r="33" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B33" s="237" t="s">
+      <c r="B33" s="132" t="s">
         <v>327</v>
       </c>
-      <c r="C33" s="237"/>
-      <c r="D33" s="237"/>
-      <c r="E33" s="237"/>
-      <c r="F33" s="237"/>
-      <c r="G33" s="237"/>
-      <c r="H33" s="237"/>
+      <c r="C33" s="132"/>
+      <c r="D33" s="132"/>
+      <c r="E33" s="132"/>
+      <c r="F33" s="132"/>
+      <c r="G33" s="132"/>
+      <c r="H33" s="132"/>
     </row>
     <row r="35" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B35" s="16" t="s">
@@ -16817,24 +16835,24 @@
       </c>
     </row>
     <row r="39" spans="2:8" ht="6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B39" s="237"/>
-      <c r="C39" s="237"/>
-      <c r="D39" s="237"/>
-      <c r="E39" s="237"/>
-      <c r="F39" s="237"/>
-      <c r="G39" s="237"/>
-      <c r="H39" s="237"/>
+      <c r="B39" s="132"/>
+      <c r="C39" s="132"/>
+      <c r="D39" s="132"/>
+      <c r="E39" s="132"/>
+      <c r="F39" s="132"/>
+      <c r="G39" s="132"/>
+      <c r="H39" s="132"/>
     </row>
     <row r="42" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B42" s="237" t="s">
+      <c r="B42" s="132" t="s">
         <v>330</v>
       </c>
-      <c r="C42" s="237"/>
-      <c r="D42" s="237"/>
-      <c r="E42" s="237"/>
-      <c r="F42" s="237"/>
-      <c r="G42" s="237"/>
-      <c r="H42" s="237"/>
+      <c r="C42" s="132"/>
+      <c r="D42" s="132"/>
+      <c r="E42" s="132"/>
+      <c r="F42" s="132"/>
+      <c r="G42" s="132"/>
+      <c r="H42" s="132"/>
     </row>
     <row r="44" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B44" s="41" t="s">
@@ -16849,24 +16867,24 @@
       </c>
     </row>
     <row r="49" spans="2:8" ht="5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B49" s="237"/>
-      <c r="C49" s="237"/>
-      <c r="D49" s="237"/>
-      <c r="E49" s="237"/>
-      <c r="F49" s="237"/>
-      <c r="G49" s="237"/>
-      <c r="H49" s="237"/>
+      <c r="B49" s="132"/>
+      <c r="C49" s="132"/>
+      <c r="D49" s="132"/>
+      <c r="E49" s="132"/>
+      <c r="F49" s="132"/>
+      <c r="G49" s="132"/>
+      <c r="H49" s="132"/>
     </row>
     <row r="52" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B52" s="237" t="s">
+      <c r="B52" s="132" t="s">
         <v>106</v>
       </c>
-      <c r="C52" s="237"/>
-      <c r="D52" s="237"/>
-      <c r="E52" s="237"/>
-      <c r="F52" s="237"/>
-      <c r="G52" s="237"/>
-      <c r="H52" s="237"/>
+      <c r="C52" s="132"/>
+      <c r="D52" s="132"/>
+      <c r="E52" s="132"/>
+      <c r="F52" s="132"/>
+      <c r="G52" s="132"/>
+      <c r="H52" s="132"/>
     </row>
     <row r="54" spans="2:8" x14ac:dyDescent="0.2">
       <c r="B54" s="41" t="s">
@@ -16881,22 +16899,16 @@
       </c>
     </row>
     <row r="59" spans="2:8" ht="5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B59" s="237"/>
-      <c r="C59" s="237"/>
-      <c r="D59" s="237"/>
-      <c r="E59" s="237"/>
-      <c r="F59" s="237"/>
-      <c r="G59" s="237"/>
-      <c r="H59" s="237"/>
+      <c r="B59" s="132"/>
+      <c r="C59" s="132"/>
+      <c r="D59" s="132"/>
+      <c r="E59" s="132"/>
+      <c r="F59" s="132"/>
+      <c r="G59" s="132"/>
+      <c r="H59" s="132"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="B52:H52"/>
-    <mergeCell ref="B59:H59"/>
-    <mergeCell ref="B33:H33"/>
-    <mergeCell ref="B39:H39"/>
-    <mergeCell ref="B42:H42"/>
-    <mergeCell ref="B49:H49"/>
+  <mergeCells count="6">
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B17:C17"/>
     <mergeCell ref="B25:C25"/>
@@ -16972,36 +16984,36 @@
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
-      <c r="C2" s="237" t="s">
+      <c r="C2" s="239" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="237"/>
-      <c r="E2" s="237"/>
-      <c r="F2" s="237"/>
-      <c r="G2" s="238"/>
-      <c r="H2" s="239" t="s">
+      <c r="D2" s="239"/>
+      <c r="E2" s="239"/>
+      <c r="F2" s="239"/>
+      <c r="G2" s="248"/>
+      <c r="H2" s="249" t="s">
         <v>111</v>
       </c>
-      <c r="I2" s="237"/>
-      <c r="J2" s="237"/>
-      <c r="K2" s="237"/>
-      <c r="L2" s="237"/>
+      <c r="I2" s="239"/>
+      <c r="J2" s="239"/>
+      <c r="K2" s="239"/>
+      <c r="L2" s="239"/>
       <c r="O2" s="5"/>
-      <c r="S2" s="237" t="s">
+      <c r="S2" s="239" t="s">
         <v>110</v>
       </c>
-      <c r="T2" s="237"/>
-      <c r="U2" s="237"/>
-      <c r="V2" s="237"/>
-      <c r="W2" s="237"/>
-      <c r="X2" s="237"/>
-      <c r="Y2" s="237"/>
-      <c r="Z2" s="237"/>
-      <c r="AA2" s="237" t="s">
+      <c r="T2" s="239"/>
+      <c r="U2" s="239"/>
+      <c r="V2" s="239"/>
+      <c r="W2" s="239"/>
+      <c r="X2" s="239"/>
+      <c r="Y2" s="239"/>
+      <c r="Z2" s="239"/>
+      <c r="AA2" s="239" t="s">
         <v>111</v>
       </c>
-      <c r="AB2" s="237"/>
-      <c r="AC2" s="237"/>
+      <c r="AB2" s="239"/>
+      <c r="AC2" s="239"/>
       <c r="AE2" s="85" t="s">
         <v>112</v>
       </c>
@@ -17012,32 +17024,32 @@
     <row r="4" spans="1:31" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="86"/>
       <c r="B4" s="60"/>
-      <c r="C4" s="236" t="s">
+      <c r="C4" s="245" t="s">
         <v>113</v>
       </c>
-      <c r="D4" s="236"/>
-      <c r="E4" s="236"/>
-      <c r="F4" s="236"/>
-      <c r="G4" s="236"/>
-      <c r="H4" s="236"/>
-      <c r="I4" s="236"/>
-      <c r="J4" s="236"/>
-      <c r="K4" s="236"/>
-      <c r="L4" s="236"/>
+      <c r="D4" s="245"/>
+      <c r="E4" s="245"/>
+      <c r="F4" s="245"/>
+      <c r="G4" s="245"/>
+      <c r="H4" s="245"/>
+      <c r="I4" s="245"/>
+      <c r="J4" s="245"/>
+      <c r="K4" s="245"/>
+      <c r="L4" s="245"/>
       <c r="O4" s="5"/>
-      <c r="S4" s="248" t="s">
+      <c r="S4" s="246" t="s">
         <v>113</v>
       </c>
-      <c r="T4" s="249"/>
-      <c r="U4" s="249"/>
-      <c r="V4" s="249"/>
-      <c r="W4" s="249"/>
-      <c r="X4" s="249"/>
-      <c r="Y4" s="249"/>
-      <c r="Z4" s="249"/>
-      <c r="AA4" s="249"/>
-      <c r="AB4" s="249"/>
-      <c r="AC4" s="249"/>
+      <c r="T4" s="247"/>
+      <c r="U4" s="247"/>
+      <c r="V4" s="247"/>
+      <c r="W4" s="247"/>
+      <c r="X4" s="247"/>
+      <c r="Y4" s="247"/>
+      <c r="Z4" s="247"/>
+      <c r="AA4" s="247"/>
+      <c r="AB4" s="247"/>
+      <c r="AC4" s="247"/>
       <c r="AE4" s="87"/>
     </row>
     <row r="5" spans="1:31" x14ac:dyDescent="0.2">
@@ -17725,33 +17737,33 @@
       <c r="Q12" s="91"/>
     </row>
     <row r="13" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="C13" s="236" t="s">
+      <c r="C13" s="245" t="s">
         <v>119</v>
       </c>
-      <c r="D13" s="236"/>
-      <c r="E13" s="236"/>
-      <c r="F13" s="236"/>
-      <c r="G13" s="236"/>
-      <c r="H13" s="236"/>
-      <c r="I13" s="236"/>
-      <c r="J13" s="236"/>
-      <c r="K13" s="236"/>
-      <c r="L13" s="236"/>
+      <c r="D13" s="245"/>
+      <c r="E13" s="245"/>
+      <c r="F13" s="245"/>
+      <c r="G13" s="245"/>
+      <c r="H13" s="245"/>
+      <c r="I13" s="245"/>
+      <c r="J13" s="245"/>
+      <c r="K13" s="245"/>
+      <c r="L13" s="245"/>
       <c r="O13" s="5"/>
       <c r="Q13" s="91"/>
-      <c r="S13" s="248" t="s">
+      <c r="S13" s="246" t="s">
         <v>119</v>
       </c>
-      <c r="T13" s="249"/>
-      <c r="U13" s="249"/>
-      <c r="V13" s="249"/>
-      <c r="W13" s="249"/>
-      <c r="X13" s="249"/>
-      <c r="Y13" s="249"/>
-      <c r="Z13" s="249"/>
-      <c r="AA13" s="249"/>
-      <c r="AB13" s="249"/>
-      <c r="AC13" s="249"/>
+      <c r="T13" s="247"/>
+      <c r="U13" s="247"/>
+      <c r="V13" s="247"/>
+      <c r="W13" s="247"/>
+      <c r="X13" s="247"/>
+      <c r="Y13" s="247"/>
+      <c r="Z13" s="247"/>
+      <c r="AA13" s="247"/>
+      <c r="AB13" s="247"/>
+      <c r="AC13" s="247"/>
     </row>
     <row r="14" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B14" s="16" t="s">
@@ -18372,35 +18384,35 @@
     </row>
     <row r="2" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
-      <c r="C2" s="237" t="s">
+      <c r="C2" s="239" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="237"/>
-      <c r="E2" s="237"/>
-      <c r="F2" s="237"/>
-      <c r="G2" s="238"/>
-      <c r="H2" s="239" t="s">
+      <c r="D2" s="239"/>
+      <c r="E2" s="239"/>
+      <c r="F2" s="239"/>
+      <c r="G2" s="248"/>
+      <c r="H2" s="249" t="s">
         <v>111</v>
       </c>
-      <c r="I2" s="237"/>
-      <c r="J2" s="237"/>
-      <c r="K2" s="237"/>
-      <c r="L2" s="237"/>
-      <c r="P2" s="237" t="s">
+      <c r="I2" s="239"/>
+      <c r="J2" s="239"/>
+      <c r="K2" s="239"/>
+      <c r="L2" s="239"/>
+      <c r="P2" s="239" t="s">
         <v>110</v>
       </c>
-      <c r="Q2" s="237"/>
-      <c r="R2" s="237"/>
-      <c r="S2" s="237"/>
-      <c r="T2" s="237"/>
-      <c r="U2" s="237"/>
-      <c r="V2" s="237"/>
-      <c r="W2" s="237"/>
-      <c r="X2" s="237" t="s">
+      <c r="Q2" s="239"/>
+      <c r="R2" s="239"/>
+      <c r="S2" s="239"/>
+      <c r="T2" s="239"/>
+      <c r="U2" s="239"/>
+      <c r="V2" s="239"/>
+      <c r="W2" s="239"/>
+      <c r="X2" s="239" t="s">
         <v>111</v>
       </c>
-      <c r="Y2" s="237"/>
-      <c r="Z2" s="237"/>
+      <c r="Y2" s="239"/>
+      <c r="Z2" s="239"/>
       <c r="AB2" s="85" t="s">
         <v>112</v>
       </c>
@@ -18409,31 +18421,31 @@
     <row r="4" spans="1:28" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="86"/>
       <c r="B4" s="60"/>
-      <c r="C4" s="236" t="s">
+      <c r="C4" s="245" t="s">
         <v>113</v>
       </c>
-      <c r="D4" s="236"/>
-      <c r="E4" s="236"/>
-      <c r="F4" s="236"/>
-      <c r="G4" s="236"/>
-      <c r="H4" s="236"/>
-      <c r="I4" s="236"/>
-      <c r="J4" s="236"/>
-      <c r="K4" s="236"/>
-      <c r="L4" s="236"/>
-      <c r="P4" s="249" t="s">
+      <c r="D4" s="245"/>
+      <c r="E4" s="245"/>
+      <c r="F4" s="245"/>
+      <c r="G4" s="245"/>
+      <c r="H4" s="245"/>
+      <c r="I4" s="245"/>
+      <c r="J4" s="245"/>
+      <c r="K4" s="245"/>
+      <c r="L4" s="245"/>
+      <c r="P4" s="247" t="s">
         <v>113</v>
       </c>
-      <c r="Q4" s="249"/>
-      <c r="R4" s="249"/>
-      <c r="S4" s="249"/>
-      <c r="T4" s="249"/>
-      <c r="U4" s="249"/>
-      <c r="V4" s="249"/>
-      <c r="W4" s="249"/>
-      <c r="X4" s="249"/>
-      <c r="Y4" s="249"/>
-      <c r="Z4" s="249"/>
+      <c r="Q4" s="247"/>
+      <c r="R4" s="247"/>
+      <c r="S4" s="247"/>
+      <c r="T4" s="247"/>
+      <c r="U4" s="247"/>
+      <c r="V4" s="247"/>
+      <c r="W4" s="247"/>
+      <c r="X4" s="247"/>
+      <c r="Y4" s="247"/>
+      <c r="Z4" s="247"/>
       <c r="AB4" s="87"/>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.2">
@@ -18628,32 +18640,32 @@
       <c r="N8" s="91"/>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="C9" s="236" t="s">
+      <c r="C9" s="245" t="s">
         <v>122</v>
       </c>
-      <c r="D9" s="236"/>
-      <c r="E9" s="236"/>
-      <c r="F9" s="236"/>
-      <c r="G9" s="236"/>
-      <c r="H9" s="236"/>
-      <c r="I9" s="236"/>
-      <c r="J9" s="236"/>
-      <c r="K9" s="236"/>
-      <c r="L9" s="236"/>
+      <c r="D9" s="245"/>
+      <c r="E9" s="245"/>
+      <c r="F9" s="245"/>
+      <c r="G9" s="245"/>
+      <c r="H9" s="245"/>
+      <c r="I9" s="245"/>
+      <c r="J9" s="245"/>
+      <c r="K9" s="245"/>
+      <c r="L9" s="245"/>
       <c r="N9" s="91"/>
-      <c r="P9" s="249" t="s">
+      <c r="P9" s="247" t="s">
         <v>123</v>
       </c>
-      <c r="Q9" s="249"/>
-      <c r="R9" s="249"/>
-      <c r="S9" s="249"/>
-      <c r="T9" s="249"/>
-      <c r="U9" s="249"/>
-      <c r="V9" s="249"/>
-      <c r="W9" s="249"/>
-      <c r="X9" s="249"/>
-      <c r="Y9" s="249"/>
-      <c r="Z9" s="249"/>
+      <c r="Q9" s="247"/>
+      <c r="R9" s="247"/>
+      <c r="S9" s="247"/>
+      <c r="T9" s="247"/>
+      <c r="U9" s="247"/>
+      <c r="V9" s="247"/>
+      <c r="W9" s="247"/>
+      <c r="X9" s="247"/>
+      <c r="Y9" s="247"/>
+      <c r="Z9" s="247"/>
       <c r="AB9" s="87">
         <f>AB4</f>
         <v>0</v>
@@ -19129,31 +19141,31 @@
       </c>
     </row>
     <row r="17" spans="2:26" x14ac:dyDescent="0.2">
-      <c r="C17" s="236" t="s">
+      <c r="C17" s="245" t="s">
         <v>125</v>
       </c>
-      <c r="D17" s="236"/>
-      <c r="E17" s="236"/>
-      <c r="F17" s="236"/>
-      <c r="G17" s="236"/>
-      <c r="H17" s="236"/>
-      <c r="I17" s="236"/>
-      <c r="J17" s="236"/>
-      <c r="K17" s="236"/>
-      <c r="L17" s="236"/>
-      <c r="P17" s="249" t="s">
+      <c r="D17" s="245"/>
+      <c r="E17" s="245"/>
+      <c r="F17" s="245"/>
+      <c r="G17" s="245"/>
+      <c r="H17" s="245"/>
+      <c r="I17" s="245"/>
+      <c r="J17" s="245"/>
+      <c r="K17" s="245"/>
+      <c r="L17" s="245"/>
+      <c r="P17" s="247" t="s">
         <v>125</v>
       </c>
-      <c r="Q17" s="249"/>
-      <c r="R17" s="249"/>
-      <c r="S17" s="249"/>
-      <c r="T17" s="249"/>
-      <c r="U17" s="249"/>
-      <c r="V17" s="249"/>
-      <c r="W17" s="249"/>
-      <c r="X17" s="249"/>
-      <c r="Y17" s="249"/>
-      <c r="Z17" s="249"/>
+      <c r="Q17" s="247"/>
+      <c r="R17" s="247"/>
+      <c r="S17" s="247"/>
+      <c r="T17" s="247"/>
+      <c r="U17" s="247"/>
+      <c r="V17" s="247"/>
+      <c r="W17" s="247"/>
+      <c r="X17" s="247"/>
+      <c r="Y17" s="247"/>
+      <c r="Z17" s="247"/>
     </row>
     <row r="18" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B18" s="16" t="s">
@@ -19631,20 +19643,20 @@
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A3" s="4"/>
-      <c r="C3" s="237" t="s">
+      <c r="C3" s="239" t="s">
         <v>110</v>
       </c>
-      <c r="D3" s="237"/>
-      <c r="E3" s="237"/>
-      <c r="F3" s="237"/>
-      <c r="G3" s="238"/>
-      <c r="H3" s="239" t="s">
+      <c r="D3" s="239"/>
+      <c r="E3" s="239"/>
+      <c r="F3" s="239"/>
+      <c r="G3" s="248"/>
+      <c r="H3" s="249" t="s">
         <v>111</v>
       </c>
-      <c r="I3" s="237"/>
-      <c r="J3" s="237"/>
-      <c r="K3" s="237"/>
-      <c r="L3" s="237"/>
+      <c r="I3" s="239"/>
+      <c r="J3" s="239"/>
+      <c r="K3" s="239"/>
+      <c r="L3" s="239"/>
       <c r="P3" s="250"/>
       <c r="Q3" s="250"/>
       <c r="R3" s="250"/>
@@ -19662,18 +19674,18 @@
     <row r="5" spans="1:28" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="86"/>
       <c r="B5" s="60"/>
-      <c r="C5" s="236" t="s">
+      <c r="C5" s="245" t="s">
         <v>113</v>
       </c>
-      <c r="D5" s="236"/>
-      <c r="E5" s="236"/>
-      <c r="F5" s="236"/>
-      <c r="G5" s="236"/>
-      <c r="H5" s="236"/>
-      <c r="I5" s="236"/>
-      <c r="J5" s="236"/>
-      <c r="K5" s="236"/>
-      <c r="L5" s="236"/>
+      <c r="D5" s="245"/>
+      <c r="E5" s="245"/>
+      <c r="F5" s="245"/>
+      <c r="G5" s="245"/>
+      <c r="H5" s="245"/>
+      <c r="I5" s="245"/>
+      <c r="J5" s="245"/>
+      <c r="K5" s="245"/>
+      <c r="L5" s="245"/>
       <c r="P5" s="250"/>
       <c r="Q5" s="250"/>
       <c r="R5" s="250"/>
@@ -19870,18 +19882,18 @@
       <c r="N10" s="91"/>
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="C11" s="236" t="s">
+      <c r="C11" s="245" t="s">
         <v>129</v>
       </c>
-      <c r="D11" s="236"/>
-      <c r="E11" s="236"/>
-      <c r="F11" s="236"/>
-      <c r="G11" s="236"/>
-      <c r="H11" s="236"/>
-      <c r="I11" s="236"/>
-      <c r="J11" s="236"/>
-      <c r="K11" s="236"/>
-      <c r="L11" s="236"/>
+      <c r="D11" s="245"/>
+      <c r="E11" s="245"/>
+      <c r="F11" s="245"/>
+      <c r="G11" s="245"/>
+      <c r="H11" s="245"/>
+      <c r="I11" s="245"/>
+      <c r="J11" s="245"/>
+      <c r="K11" s="245"/>
+      <c r="L11" s="245"/>
       <c r="N11" s="91"/>
       <c r="P11" s="250"/>
       <c r="Q11" s="250"/>
@@ -20135,18 +20147,18 @@
       <c r="D16" s="24"/>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="C18" s="236" t="s">
+      <c r="C18" s="245" t="s">
         <v>134</v>
       </c>
-      <c r="D18" s="236"/>
-      <c r="E18" s="236"/>
-      <c r="F18" s="236"/>
-      <c r="G18" s="236"/>
-      <c r="H18" s="236"/>
-      <c r="I18" s="236"/>
-      <c r="J18" s="236"/>
-      <c r="K18" s="236"/>
-      <c r="L18" s="236"/>
+      <c r="D18" s="245"/>
+      <c r="E18" s="245"/>
+      <c r="F18" s="245"/>
+      <c r="G18" s="245"/>
+      <c r="H18" s="245"/>
+      <c r="I18" s="245"/>
+      <c r="J18" s="245"/>
+      <c r="K18" s="245"/>
+      <c r="L18" s="245"/>
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B19" s="16" t="s">
@@ -20364,18 +20376,18 @@
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B26" s="109"/>
-      <c r="C26" s="236" t="s">
+      <c r="C26" s="245" t="s">
         <v>140</v>
       </c>
-      <c r="D26" s="236"/>
-      <c r="E26" s="236"/>
-      <c r="F26" s="236"/>
-      <c r="G26" s="236"/>
-      <c r="H26" s="236"/>
-      <c r="I26" s="236"/>
-      <c r="J26" s="236"/>
-      <c r="K26" s="236"/>
-      <c r="L26" s="236"/>
+      <c r="D26" s="245"/>
+      <c r="E26" s="245"/>
+      <c r="F26" s="245"/>
+      <c r="G26" s="245"/>
+      <c r="H26" s="245"/>
+      <c r="I26" s="245"/>
+      <c r="J26" s="245"/>
+      <c r="K26" s="245"/>
+      <c r="L26" s="245"/>
     </row>
     <row r="27" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B27" s="16" t="s">
@@ -20567,18 +20579,18 @@
     </row>
     <row r="33" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B33" s="109"/>
-      <c r="C33" s="236" t="s">
+      <c r="C33" s="245" t="s">
         <v>144</v>
       </c>
-      <c r="D33" s="236"/>
-      <c r="E33" s="236"/>
-      <c r="F33" s="236"/>
-      <c r="G33" s="236"/>
-      <c r="H33" s="236"/>
-      <c r="I33" s="236"/>
-      <c r="J33" s="236"/>
-      <c r="K33" s="236"/>
-      <c r="L33" s="236"/>
+      <c r="D33" s="245"/>
+      <c r="E33" s="245"/>
+      <c r="F33" s="245"/>
+      <c r="G33" s="245"/>
+      <c r="H33" s="245"/>
+      <c r="I33" s="245"/>
+      <c r="J33" s="245"/>
+      <c r="K33" s="245"/>
+      <c r="L33" s="245"/>
     </row>
     <row r="34" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B34" s="16" t="s">
@@ -20762,18 +20774,18 @@
       <c r="C39" s="125"/>
     </row>
     <row r="40" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="C40" s="236" t="s">
+      <c r="C40" s="245" t="s">
         <v>147</v>
       </c>
-      <c r="D40" s="236"/>
-      <c r="E40" s="236"/>
-      <c r="F40" s="236"/>
-      <c r="G40" s="236"/>
-      <c r="H40" s="236"/>
-      <c r="I40" s="236"/>
-      <c r="J40" s="236"/>
-      <c r="K40" s="236"/>
-      <c r="L40" s="236"/>
+      <c r="D40" s="245"/>
+      <c r="E40" s="245"/>
+      <c r="F40" s="245"/>
+      <c r="G40" s="245"/>
+      <c r="H40" s="245"/>
+      <c r="I40" s="245"/>
+      <c r="J40" s="245"/>
+      <c r="K40" s="245"/>
+      <c r="L40" s="245"/>
     </row>
     <row r="41" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B41" s="16" t="s">
@@ -21037,12 +21049,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="C3:G3"/>
-    <mergeCell ref="H3:L3"/>
-    <mergeCell ref="P3:W3"/>
-    <mergeCell ref="X3:Z3"/>
-    <mergeCell ref="C5:L5"/>
-    <mergeCell ref="P5:Z5"/>
     <mergeCell ref="C40:L40"/>
     <mergeCell ref="C11:L11"/>
     <mergeCell ref="P11:Z11"/>
@@ -21050,6 +21056,12 @@
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="C26:L26"/>
     <mergeCell ref="C33:L33"/>
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="H3:L3"/>
+    <mergeCell ref="P3:W3"/>
+    <mergeCell ref="X3:Z3"/>
+    <mergeCell ref="C5:L5"/>
+    <mergeCell ref="P5:Z5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -21087,20 +21099,20 @@
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
-      <c r="C2" s="237" t="s">
+      <c r="C2" s="239" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="237"/>
-      <c r="E2" s="237"/>
-      <c r="F2" s="237"/>
-      <c r="G2" s="238"/>
-      <c r="H2" s="239" t="s">
+      <c r="D2" s="239"/>
+      <c r="E2" s="239"/>
+      <c r="F2" s="239"/>
+      <c r="G2" s="248"/>
+      <c r="H2" s="249" t="s">
         <v>111</v>
       </c>
-      <c r="I2" s="237"/>
-      <c r="J2" s="237"/>
-      <c r="K2" s="237"/>
-      <c r="L2" s="237"/>
+      <c r="I2" s="239"/>
+      <c r="J2" s="239"/>
+      <c r="K2" s="239"/>
+      <c r="L2" s="239"/>
       <c r="S2" s="250"/>
       <c r="T2" s="250"/>
       <c r="U2" s="250"/>
@@ -21118,18 +21130,18 @@
     <row r="4" spans="1:31" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="86"/>
       <c r="B4" s="60"/>
-      <c r="C4" s="236" t="s">
+      <c r="C4" s="245" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="236"/>
-      <c r="E4" s="236"/>
-      <c r="F4" s="236"/>
-      <c r="G4" s="236"/>
-      <c r="H4" s="236"/>
-      <c r="I4" s="236"/>
-      <c r="J4" s="236"/>
-      <c r="K4" s="236"/>
-      <c r="L4" s="236"/>
+      <c r="D4" s="245"/>
+      <c r="E4" s="245"/>
+      <c r="F4" s="245"/>
+      <c r="G4" s="245"/>
+      <c r="H4" s="245"/>
+      <c r="I4" s="245"/>
+      <c r="J4" s="245"/>
+      <c r="K4" s="245"/>
+      <c r="L4" s="245"/>
       <c r="S4" s="250"/>
       <c r="T4" s="250"/>
       <c r="U4" s="250"/>
@@ -21503,18 +21515,18 @@
       <c r="AE10" s="64"/>
     </row>
     <row r="13" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="C13" s="236" t="s">
+      <c r="C13" s="245" t="s">
         <v>155</v>
       </c>
-      <c r="D13" s="236"/>
-      <c r="E13" s="236"/>
-      <c r="F13" s="236"/>
-      <c r="G13" s="236"/>
-      <c r="H13" s="236"/>
-      <c r="I13" s="236"/>
-      <c r="J13" s="236"/>
-      <c r="K13" s="236"/>
-      <c r="L13" s="236"/>
+      <c r="D13" s="245"/>
+      <c r="E13" s="245"/>
+      <c r="F13" s="245"/>
+      <c r="G13" s="245"/>
+      <c r="H13" s="245"/>
+      <c r="I13" s="245"/>
+      <c r="J13" s="245"/>
+      <c r="K13" s="245"/>
+      <c r="L13" s="245"/>
     </row>
     <row r="14" spans="1:31" x14ac:dyDescent="0.2">
       <c r="C14" s="12">
@@ -21607,18 +21619,18 @@
       </c>
     </row>
     <row r="18" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="C18" s="236" t="s">
+      <c r="C18" s="245" t="s">
         <v>156</v>
       </c>
-      <c r="D18" s="236"/>
-      <c r="E18" s="236"/>
-      <c r="F18" s="236"/>
-      <c r="G18" s="236"/>
-      <c r="H18" s="236"/>
-      <c r="I18" s="236"/>
-      <c r="J18" s="236"/>
-      <c r="K18" s="236"/>
-      <c r="L18" s="236"/>
+      <c r="D18" s="245"/>
+      <c r="E18" s="245"/>
+      <c r="F18" s="245"/>
+      <c r="G18" s="245"/>
+      <c r="H18" s="245"/>
+      <c r="I18" s="245"/>
+      <c r="J18" s="245"/>
+      <c r="K18" s="245"/>
+      <c r="L18" s="245"/>
     </row>
     <row r="19" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B19" s="16" t="s">
@@ -21810,18 +21822,18 @@
       </c>
     </row>
     <row r="25" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="C25" s="236" t="s">
+      <c r="C25" s="245" t="s">
         <v>256</v>
       </c>
-      <c r="D25" s="236"/>
-      <c r="E25" s="236"/>
-      <c r="F25" s="236"/>
-      <c r="G25" s="236"/>
-      <c r="H25" s="236"/>
-      <c r="I25" s="236"/>
-      <c r="J25" s="236"/>
-      <c r="K25" s="236"/>
-      <c r="L25" s="236"/>
+      <c r="D25" s="245"/>
+      <c r="E25" s="245"/>
+      <c r="F25" s="245"/>
+      <c r="G25" s="245"/>
+      <c r="H25" s="245"/>
+      <c r="I25" s="245"/>
+      <c r="J25" s="245"/>
+      <c r="K25" s="245"/>
+      <c r="L25" s="245"/>
     </row>
     <row r="26" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B26" s="16" t="s">
@@ -21959,18 +21971,18 @@
       </c>
     </row>
     <row r="31" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="C31" s="236" t="s">
+      <c r="C31" s="245" t="s">
         <v>75</v>
       </c>
-      <c r="D31" s="236"/>
-      <c r="E31" s="236"/>
-      <c r="F31" s="236"/>
-      <c r="G31" s="236"/>
-      <c r="H31" s="236"/>
-      <c r="I31" s="236"/>
-      <c r="J31" s="236"/>
-      <c r="K31" s="236"/>
-      <c r="L31" s="236"/>
+      <c r="D31" s="245"/>
+      <c r="E31" s="245"/>
+      <c r="F31" s="245"/>
+      <c r="G31" s="245"/>
+      <c r="H31" s="245"/>
+      <c r="I31" s="245"/>
+      <c r="J31" s="245"/>
+      <c r="K31" s="245"/>
+      <c r="L31" s="245"/>
     </row>
     <row r="32" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B32" s="16" t="s">
@@ -22109,16 +22121,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="C31:L31"/>
+    <mergeCell ref="C25:L25"/>
+    <mergeCell ref="C2:G2"/>
+    <mergeCell ref="H2:L2"/>
+    <mergeCell ref="S2:Z2"/>
     <mergeCell ref="AA2:AC2"/>
     <mergeCell ref="C4:L4"/>
     <mergeCell ref="S4:AC4"/>
     <mergeCell ref="C13:L13"/>
     <mergeCell ref="C18:L18"/>
-    <mergeCell ref="C31:L31"/>
-    <mergeCell ref="C25:L25"/>
-    <mergeCell ref="C2:G2"/>
-    <mergeCell ref="H2:L2"/>
-    <mergeCell ref="S2:Z2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -22181,10 +22193,10 @@
     </row>
     <row r="3" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="237" t="s">
+      <c r="B4" s="239" t="s">
         <v>163</v>
       </c>
-      <c r="C4" s="237"/>
+      <c r="C4" s="239"/>
     </row>
     <row r="5" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
@@ -22201,7 +22213,7 @@
       </c>
       <c r="C6" s="133">
         <f ca="1">Overview!C5</f>
-        <v>341.07</v>
+        <v>329.4</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22210,7 +22222,7 @@
       </c>
       <c r="C7" s="134">
         <f ca="1">C5*C6</f>
-        <v>4997698.71</v>
+        <v>4826698.1999999993</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22228,7 +22240,7 @@
       </c>
       <c r="C9" s="135">
         <f ca="1">Overview!F27</f>
-        <v>5.1840000000000004E-2</v>
+        <v>5.2549999999999999E-2</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22237,7 +22249,7 @@
       </c>
       <c r="C10" s="133">
         <f ca="1">Overview!C13</f>
-        <v>1.0737000000000001</v>
+        <v>1.0696000000000001</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22269,10 +22281,10 @@
     </row>
     <row r="14" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="15" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="237" t="s">
+      <c r="B15" s="239" t="s">
         <v>170</v>
       </c>
-      <c r="C15" s="237"/>
+      <c r="C15" s="239"/>
     </row>
     <row r="16" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="1" t="s">
@@ -22280,7 +22292,7 @@
       </c>
       <c r="C16" s="46">
         <f ca="1">C8/(C8+C7)</f>
-        <v>1.6596476026074169E-2</v>
+        <v>1.7174358632063885E-2</v>
       </c>
     </row>
     <row r="17" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22289,7 +22301,7 @@
       </c>
       <c r="C17" s="46">
         <f ca="1">C7/(C8+C7)</f>
-        <v>0.98340352397392583</v>
+        <v>0.98282564136793615</v>
       </c>
     </row>
     <row r="18" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22307,7 +22319,7 @@
       </c>
       <c r="C19" s="46">
         <f ca="1">C9+C10*C11</f>
-        <v>0.10015650000000001</v>
+        <v>0.10068199999999999</v>
       </c>
     </row>
     <row r="20" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22316,7 +22328,7 @@
       </c>
       <c r="C20" s="46">
         <f ca="1">(C17*C19)+(C16*C18)</f>
-        <v>9.9136704635863854E-2</v>
+        <v>9.9617670646853729E-2</v>
       </c>
     </row>
   </sheetData>
@@ -22361,20 +22373,20 @@
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A3" s="4"/>
-      <c r="C3" s="237" t="s">
+      <c r="C3" s="239" t="s">
         <v>110</v>
       </c>
-      <c r="D3" s="237"/>
-      <c r="E3" s="237"/>
-      <c r="F3" s="237"/>
-      <c r="G3" s="238"/>
-      <c r="H3" s="239" t="s">
+      <c r="D3" s="239"/>
+      <c r="E3" s="239"/>
+      <c r="F3" s="239"/>
+      <c r="G3" s="248"/>
+      <c r="H3" s="249" t="s">
         <v>111</v>
       </c>
-      <c r="I3" s="237"/>
-      <c r="J3" s="237"/>
-      <c r="K3" s="237"/>
-      <c r="L3" s="237"/>
+      <c r="I3" s="239"/>
+      <c r="J3" s="239"/>
+      <c r="K3" s="239"/>
+      <c r="L3" s="239"/>
       <c r="P3" s="250"/>
       <c r="Q3" s="250"/>
       <c r="R3" s="250"/>
@@ -22392,18 +22404,18 @@
     <row r="5" spans="1:28" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="86"/>
       <c r="B5" s="60"/>
-      <c r="C5" s="236" t="s">
+      <c r="C5" s="245" t="s">
         <v>177</v>
       </c>
-      <c r="D5" s="236"/>
-      <c r="E5" s="236"/>
-      <c r="F5" s="236"/>
-      <c r="G5" s="236"/>
-      <c r="H5" s="236"/>
-      <c r="I5" s="236"/>
-      <c r="J5" s="236"/>
-      <c r="K5" s="236"/>
-      <c r="L5" s="236"/>
+      <c r="D5" s="245"/>
+      <c r="E5" s="245"/>
+      <c r="F5" s="245"/>
+      <c r="G5" s="245"/>
+      <c r="H5" s="245"/>
+      <c r="I5" s="245"/>
+      <c r="J5" s="245"/>
+      <c r="K5" s="245"/>
+      <c r="L5" s="245"/>
       <c r="P5" s="250"/>
       <c r="Q5" s="250"/>
       <c r="R5" s="250"/>
@@ -22567,7 +22579,7 @@
       </c>
       <c r="L8" s="126">
         <f ca="1">L7*(1+C14)/(C15-C14)</f>
-        <v>1831699.0746865442</v>
+        <v>1820633.88036312</v>
       </c>
       <c r="N8" s="91"/>
       <c r="O8" s="16"/>
@@ -22621,23 +22633,23 @@
       <c r="G10" s="138"/>
       <c r="H10" s="126">
         <f ca="1">H7/(1+$C$15)^H9</f>
-        <v>100405.17742427663</v>
+        <v>100361.2608167524</v>
       </c>
       <c r="I10" s="126">
         <f t="shared" ref="I10:L10" ca="1" si="0">I7/(1+$C$15)^I9</f>
-        <v>97054.485110423731</v>
+        <v>96969.601607647288</v>
       </c>
       <c r="J10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>93297.78323292089</v>
+        <v>93175.413141498604</v>
       </c>
       <c r="K10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>89274.624035873872</v>
+        <v>89118.533795059731</v>
       </c>
       <c r="L10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>88587.686711715622</v>
+        <v>88394.117569124312</v>
       </c>
       <c r="N10" s="91"/>
     </row>
@@ -22656,14 +22668,14 @@
       <c r="K11" s="137"/>
       <c r="L11" s="126">
         <f ca="1">L8/(1+C15)^L9</f>
-        <v>1141814.5456236254</v>
+        <v>1132437.048057117</v>
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="B13" s="237" t="s">
+      <c r="B13" s="239" t="s">
         <v>181</v>
       </c>
-      <c r="C13" s="237"/>
+      <c r="C13" s="239"/>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B14" s="1" t="s">
@@ -22679,14 +22691,14 @@
       </c>
       <c r="C15" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.9136704635863854E-2</v>
+        <v>9.9617670646853729E-2</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B18" s="237" t="s">
+      <c r="B18" s="239" t="s">
         <v>183</v>
       </c>
-      <c r="C18" s="237"/>
+      <c r="C18" s="239"/>
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B19" s="1" t="s">
@@ -22694,7 +22706,7 @@
       </c>
       <c r="C19" s="64">
         <f ca="1">SUM(H10:L10)</f>
-        <v>468619.75651521073</v>
+        <v>468018.92693008232</v>
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.2">
@@ -22703,7 +22715,7 @@
       </c>
       <c r="C20" s="64">
         <f ca="1">L11</f>
-        <v>1141814.5456236254</v>
+        <v>1132437.048057117</v>
       </c>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.2">
@@ -22712,7 +22724,7 @@
       </c>
       <c r="C21" s="94">
         <f ca="1">C19+C20</f>
-        <v>1610434.3021388361</v>
+        <v>1600455.9749871993</v>
       </c>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.2">
@@ -22739,7 +22751,7 @@
       </c>
       <c r="C24" s="94">
         <f ca="1">C21+C22-C23</f>
-        <v>1672607.3021388361</v>
+        <v>1662628.9749871993</v>
       </c>
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.2">
@@ -22757,7 +22769,7 @@
       </c>
       <c r="C26" s="235">
         <f ca="1">C24/C25</f>
-        <v>114.14777193331305</v>
+        <v>113.46679690078477</v>
       </c>
     </row>
   </sheetData>
@@ -22800,37 +22812,37 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
-      <c r="C2" s="237" t="s">
+      <c r="C2" s="239" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="237"/>
-      <c r="E2" s="237"/>
-      <c r="F2" s="237"/>
-      <c r="G2" s="238"/>
-      <c r="H2" s="239" t="s">
+      <c r="D2" s="239"/>
+      <c r="E2" s="239"/>
+      <c r="F2" s="239"/>
+      <c r="G2" s="248"/>
+      <c r="H2" s="249" t="s">
         <v>111</v>
       </c>
-      <c r="I2" s="237"/>
-      <c r="J2" s="237"/>
-      <c r="K2" s="237"/>
-      <c r="L2" s="237"/>
+      <c r="I2" s="239"/>
+      <c r="J2" s="239"/>
+      <c r="K2" s="239"/>
+      <c r="L2" s="239"/>
     </row>
     <row r="3" spans="1:14" ht="10" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:14" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="86"/>
       <c r="B4" s="60"/>
-      <c r="C4" s="236" t="s">
+      <c r="C4" s="245" t="s">
         <v>191</v>
       </c>
-      <c r="D4" s="236"/>
-      <c r="E4" s="236"/>
-      <c r="F4" s="236"/>
-      <c r="G4" s="236"/>
-      <c r="H4" s="236"/>
-      <c r="I4" s="236"/>
-      <c r="J4" s="236"/>
-      <c r="K4" s="236"/>
-      <c r="L4" s="236"/>
+      <c r="D4" s="245"/>
+      <c r="E4" s="245"/>
+      <c r="F4" s="245"/>
+      <c r="G4" s="245"/>
+      <c r="H4" s="245"/>
+      <c r="I4" s="245"/>
+      <c r="J4" s="245"/>
+      <c r="K4" s="245"/>
+      <c r="L4" s="245"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B5" s="16" t="s">
@@ -23026,23 +23038,23 @@
       <c r="G9" s="138"/>
       <c r="H9" s="92">
         <f ca="1">DCF!H10</f>
-        <v>100405.17742427663</v>
+        <v>100361.2608167524</v>
       </c>
       <c r="I9" s="92">
         <f ca="1">DCF!I10</f>
-        <v>97054.485110423731</v>
+        <v>96969.601607647288</v>
       </c>
       <c r="J9" s="92">
         <f ca="1">DCF!J10</f>
-        <v>93297.78323292089</v>
+        <v>93175.413141498604</v>
       </c>
       <c r="K9" s="92">
         <f ca="1">DCF!K10</f>
-        <v>89274.624035873872</v>
+        <v>89118.533795059731</v>
       </c>
       <c r="L9" s="92">
         <f ca="1">DCF!L10</f>
-        <v>88587.686711715622</v>
+        <v>88394.117569124312</v>
       </c>
       <c r="N9" s="91"/>
     </row>
@@ -23050,18 +23062,18 @@
       <c r="N10" s="91"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="C11" s="236" t="s">
+      <c r="C11" s="245" t="s">
         <v>119</v>
       </c>
-      <c r="D11" s="236"/>
-      <c r="E11" s="236"/>
-      <c r="F11" s="236"/>
-      <c r="G11" s="236"/>
-      <c r="H11" s="236"/>
-      <c r="I11" s="236"/>
-      <c r="J11" s="236"/>
-      <c r="K11" s="236"/>
-      <c r="L11" s="236"/>
+      <c r="D11" s="245"/>
+      <c r="E11" s="245"/>
+      <c r="F11" s="245"/>
+      <c r="G11" s="245"/>
+      <c r="H11" s="245"/>
+      <c r="I11" s="245"/>
+      <c r="J11" s="245"/>
+      <c r="K11" s="245"/>
+      <c r="L11" s="245"/>
       <c r="N11" s="91"/>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.2">
@@ -23255,18 +23267,18 @@
       <c r="N16" s="91"/>
     </row>
     <row r="17" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="C17" s="236" t="s">
+      <c r="C17" s="245" t="s">
         <v>193</v>
       </c>
-      <c r="D17" s="236"/>
-      <c r="E17" s="236"/>
-      <c r="F17" s="236"/>
-      <c r="G17" s="236"/>
-      <c r="H17" s="236"/>
-      <c r="I17" s="236"/>
-      <c r="J17" s="236"/>
-      <c r="K17" s="236"/>
-      <c r="L17" s="236"/>
+      <c r="D17" s="245"/>
+      <c r="E17" s="245"/>
+      <c r="F17" s="245"/>
+      <c r="G17" s="245"/>
+      <c r="H17" s="245"/>
+      <c r="I17" s="245"/>
+      <c r="J17" s="245"/>
+      <c r="K17" s="245"/>
+      <c r="L17" s="245"/>
       <c r="N17" s="91"/>
     </row>
     <row r="18" spans="2:14" x14ac:dyDescent="0.2">
@@ -23400,18 +23412,18 @@
       <c r="N21" s="91"/>
     </row>
     <row r="22" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="C22" s="236" t="s">
+      <c r="C22" s="245" t="s">
         <v>196</v>
       </c>
-      <c r="D22" s="236"/>
-      <c r="E22" s="236"/>
-      <c r="F22" s="236"/>
-      <c r="G22" s="236"/>
-      <c r="H22" s="236"/>
-      <c r="I22" s="236"/>
-      <c r="J22" s="236"/>
-      <c r="K22" s="236"/>
-      <c r="L22" s="236"/>
+      <c r="D22" s="245"/>
+      <c r="E22" s="245"/>
+      <c r="F22" s="245"/>
+      <c r="G22" s="245"/>
+      <c r="H22" s="245"/>
+      <c r="I22" s="245"/>
+      <c r="J22" s="245"/>
+      <c r="K22" s="245"/>
+      <c r="L22" s="245"/>
       <c r="N22" s="91"/>
     </row>
     <row r="23" spans="2:14" x14ac:dyDescent="0.2">
@@ -23495,18 +23507,18 @@
       <c r="N26" s="91"/>
     </row>
     <row r="27" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="C27" s="236" t="s">
+      <c r="C27" s="245" t="s">
         <v>197</v>
       </c>
-      <c r="D27" s="236"/>
-      <c r="E27" s="236"/>
-      <c r="F27" s="236"/>
-      <c r="G27" s="236"/>
-      <c r="H27" s="236"/>
-      <c r="I27" s="236"/>
-      <c r="J27" s="236"/>
-      <c r="K27" s="236"/>
-      <c r="L27" s="236"/>
+      <c r="D27" s="245"/>
+      <c r="E27" s="245"/>
+      <c r="F27" s="245"/>
+      <c r="G27" s="245"/>
+      <c r="H27" s="245"/>
+      <c r="I27" s="245"/>
+      <c r="J27" s="245"/>
+      <c r="K27" s="245"/>
+      <c r="L27" s="245"/>
       <c r="N27" s="91"/>
     </row>
     <row r="28" spans="2:14" x14ac:dyDescent="0.2">
@@ -23807,10 +23819,10 @@
       <c r="N38" s="91"/>
     </row>
     <row r="39" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B39" s="237" t="s">
+      <c r="B39" s="239" t="s">
         <v>202</v>
       </c>
-      <c r="C39" s="237"/>
+      <c r="C39" s="239"/>
       <c r="N39" s="91"/>
     </row>
     <row r="40" spans="2:14" x14ac:dyDescent="0.2">
@@ -23828,7 +23840,7 @@
       </c>
       <c r="C41" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.9136704635863854E-2</v>
+        <v>9.9617670646853729E-2</v>
       </c>
     </row>
     <row r="42" spans="2:14" x14ac:dyDescent="0.2">
@@ -23854,7 +23866,7 @@
       </c>
       <c r="C44" s="24">
         <f ca="1">C43/(1+C41)^5</f>
-        <v>2919157.5974804689</v>
+        <v>2912779.0718161515</v>
       </c>
     </row>
     <row r="45" spans="2:14" x14ac:dyDescent="0.2">
@@ -23863,7 +23875,7 @@
       </c>
       <c r="C45" s="108">
         <f ca="1">SUM(H9:K9)+C44</f>
-        <v>3299189.6672839639</v>
+        <v>3292403.8811771097</v>
       </c>
     </row>
     <row r="46" spans="2:14" x14ac:dyDescent="0.2">
@@ -23890,7 +23902,7 @@
       </c>
       <c r="C48" s="94">
         <f ca="1">C45+C46-C47</f>
-        <v>3361362.6672839639</v>
+        <v>3354576.8811771097</v>
       </c>
     </row>
     <row r="49" spans="2:3" x14ac:dyDescent="0.2">
@@ -23908,14 +23920,14 @@
       </c>
       <c r="C50" s="235">
         <f ca="1">C48/C49</f>
-        <v>229.39757505520808</v>
+        <v>228.93447629680676</v>
       </c>
     </row>
     <row r="52" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B52" s="237" t="s">
+      <c r="B52" s="239" t="s">
         <v>207</v>
       </c>
-      <c r="C52" s="237"/>
+      <c r="C52" s="239"/>
     </row>
     <row r="53" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B53" s="1" t="s">
@@ -23932,7 +23944,7 @@
       </c>
       <c r="C54" s="135">
         <f ca="1">IF(Overview!C29&gt;0,Overview!C29,WACC!C19)</f>
-        <v>0.10015650000000001</v>
+        <v>0.10068199999999999</v>
       </c>
     </row>
     <row r="55" spans="2:3" x14ac:dyDescent="0.2">
@@ -23967,14 +23979,14 @@
       </c>
       <c r="C58" s="235">
         <f ca="1">C57/(1+C54)^5</f>
-        <v>200.97536240722781</v>
+        <v>200.49606068515598</v>
       </c>
     </row>
     <row r="60" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B60" s="237" t="s">
+      <c r="B60" s="239" t="s">
         <v>316</v>
       </c>
-      <c r="C60" s="237"/>
+      <c r="C60" s="239"/>
     </row>
     <row r="61" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B61" s="1" t="s">
@@ -23991,7 +24003,7 @@
       </c>
       <c r="C62" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.9136704635863854E-2</v>
+        <v>9.9617670646853729E-2</v>
       </c>
     </row>
     <row r="63" spans="2:3" x14ac:dyDescent="0.2">
@@ -24017,7 +24029,7 @@
       </c>
       <c r="C65" s="24">
         <f ca="1">C64/(1+C62)^5</f>
-        <v>2480455.2279280373</v>
+        <v>2475035.2919354807</v>
       </c>
     </row>
     <row r="66" spans="2:3" x14ac:dyDescent="0.2">
@@ -24026,7 +24038,7 @@
       </c>
       <c r="C66" s="108">
         <f ca="1">SUM(H9:K9)+C65</f>
-        <v>2860487.2977315322</v>
+        <v>2854660.1012964388</v>
       </c>
     </row>
     <row r="67" spans="2:3" x14ac:dyDescent="0.2">
@@ -24053,7 +24065,7 @@
       </c>
       <c r="C69" s="94">
         <f ca="1">C66+C67-C68</f>
-        <v>2922660.2977315322</v>
+        <v>2916833.1012964388</v>
       </c>
     </row>
     <row r="70" spans="2:3" x14ac:dyDescent="0.2">
@@ -24071,14 +24083,14 @@
       </c>
       <c r="C71" s="235">
         <f ca="1">C69/C70</f>
-        <v>199.45815175947126</v>
+        <v>199.06047234671664</v>
       </c>
     </row>
     <row r="73" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B73" s="237" t="s">
+      <c r="B73" s="239" t="s">
         <v>414</v>
       </c>
-      <c r="C73" s="237"/>
+      <c r="C73" s="239"/>
     </row>
     <row r="74" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B74" s="1" t="s">
@@ -24095,7 +24107,7 @@
       </c>
       <c r="C75" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.9136704635863854E-2</v>
+        <v>9.9617670646853729E-2</v>
       </c>
     </row>
     <row r="76" spans="2:3" x14ac:dyDescent="0.2">
@@ -24121,7 +24133,7 @@
       </c>
       <c r="C78" s="24">
         <f ca="1">C77/(1+C75)^5</f>
-        <v>2685870.5549899163</v>
+        <v>2680001.7748045558</v>
       </c>
     </row>
     <row r="79" spans="2:3" x14ac:dyDescent="0.2">
@@ -24130,7 +24142,7 @@
       </c>
       <c r="C79" s="108">
         <f ca="1">SUM(H9:K9)+C78</f>
-        <v>3065902.6247934112</v>
+        <v>3059626.584165514</v>
       </c>
     </row>
     <row r="80" spans="2:3" x14ac:dyDescent="0.2">
@@ -24157,7 +24169,7 @@
       </c>
       <c r="C82" s="94">
         <f ca="1">C79+C80-C81</f>
-        <v>3128075.6247934112</v>
+        <v>3121799.584165514</v>
       </c>
     </row>
     <row r="83" spans="2:3" x14ac:dyDescent="0.2">
@@ -24175,22 +24187,22 @@
       </c>
       <c r="C84" s="235">
         <f ca="1">C82/C83</f>
-        <v>213.47680507700889</v>
+        <v>213.04849410806756</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B73:C73"/>
-    <mergeCell ref="C27:L27"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="B60:C60"/>
     <mergeCell ref="C22:L22"/>
     <mergeCell ref="C2:G2"/>
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="C4:L4"/>
     <mergeCell ref="C11:L11"/>
     <mergeCell ref="C17:L17"/>
+    <mergeCell ref="B73:C73"/>
+    <mergeCell ref="C27:L27"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="B60:C60"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -24228,10 +24240,10 @@
       <c r="N3" s="91"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B4" s="237" t="s">
+      <c r="B4" s="239" t="s">
         <v>211</v>
       </c>
-      <c r="C4" s="237"/>
+      <c r="C4" s="239"/>
       <c r="N4" s="91"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
@@ -24240,7 +24252,7 @@
       </c>
       <c r="C5" s="133">
         <f ca="1">DCF!C26</f>
-        <v>114.14777193331305</v>
+        <v>113.46679690078477</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -24249,7 +24261,7 @@
       </c>
       <c r="C6" s="133">
         <f ca="1">Multiples!C50</f>
-        <v>229.39757505520808</v>
+        <v>228.93447629680676</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
@@ -24258,7 +24270,7 @@
       </c>
       <c r="C7" s="133">
         <f ca="1">Multiples!C58</f>
-        <v>200.97536240722781</v>
+        <v>200.49606068515598</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
@@ -24267,7 +24279,7 @@
       </c>
       <c r="C8" s="133">
         <f ca="1">Multiples!C71</f>
-        <v>199.45815175947126</v>
+        <v>199.06047234671664</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
@@ -24276,7 +24288,7 @@
       </c>
       <c r="C9" s="133">
         <f ca="1">Multiples!C84</f>
-        <v>213.47680507700889</v>
+        <v>213.04849410806756</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
@@ -24285,7 +24297,7 @@
       </c>
       <c r="C10" s="235">
         <f ca="1">AVERAGE(C5:C9)</f>
-        <v>191.49113324644583</v>
+        <v>191.00126006750634</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
@@ -24294,7 +24306,7 @@
       </c>
       <c r="C11" s="133">
         <f ca="1">Overview!C5</f>
-        <v>341.07</v>
+        <v>329.4</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.2">
@@ -24303,7 +24315,7 @@
       </c>
       <c r="C12" s="149">
         <f ca="1">(C10-C11)/C11</f>
-        <v>-0.43855767658707645</v>
+        <v>-0.42015403743926427</v>
       </c>
     </row>
   </sheetData>
@@ -24359,37 +24371,37 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
-      <c r="C2" s="237" t="s">
+      <c r="C2" s="239" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="237"/>
-      <c r="E2" s="237"/>
-      <c r="F2" s="237"/>
-      <c r="G2" s="238"/>
-      <c r="H2" s="239" t="s">
+      <c r="D2" s="239"/>
+      <c r="E2" s="239"/>
+      <c r="F2" s="239"/>
+      <c r="G2" s="248"/>
+      <c r="H2" s="249" t="s">
         <v>111</v>
       </c>
-      <c r="I2" s="237"/>
-      <c r="J2" s="237"/>
-      <c r="K2" s="237"/>
-      <c r="L2" s="237"/>
+      <c r="I2" s="239"/>
+      <c r="J2" s="239"/>
+      <c r="K2" s="239"/>
+      <c r="L2" s="239"/>
     </row>
     <row r="3" spans="1:14" ht="10" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:14" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="86"/>
       <c r="B4" s="60"/>
-      <c r="C4" s="236" t="s">
+      <c r="C4" s="245" t="s">
         <v>191</v>
       </c>
-      <c r="D4" s="236"/>
-      <c r="E4" s="236"/>
-      <c r="F4" s="236"/>
-      <c r="G4" s="236"/>
-      <c r="H4" s="236"/>
-      <c r="I4" s="236"/>
-      <c r="J4" s="236"/>
-      <c r="K4" s="236"/>
-      <c r="L4" s="236"/>
+      <c r="D4" s="245"/>
+      <c r="E4" s="245"/>
+      <c r="F4" s="245"/>
+      <c r="G4" s="245"/>
+      <c r="H4" s="245"/>
+      <c r="I4" s="245"/>
+      <c r="J4" s="245"/>
+      <c r="K4" s="245"/>
+      <c r="L4" s="245"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B5" s="16" t="s">
@@ -24502,18 +24514,18 @@
       <c r="N8" s="91"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="C9" s="236" t="s">
+      <c r="C9" s="245" t="s">
         <v>119</v>
       </c>
-      <c r="D9" s="236"/>
-      <c r="E9" s="236"/>
-      <c r="F9" s="236"/>
-      <c r="G9" s="236"/>
-      <c r="H9" s="236"/>
-      <c r="I9" s="236"/>
-      <c r="J9" s="236"/>
-      <c r="K9" s="236"/>
-      <c r="L9" s="236"/>
+      <c r="D9" s="245"/>
+      <c r="E9" s="245"/>
+      <c r="F9" s="245"/>
+      <c r="G9" s="245"/>
+      <c r="H9" s="245"/>
+      <c r="I9" s="245"/>
+      <c r="J9" s="245"/>
+      <c r="K9" s="245"/>
+      <c r="L9" s="245"/>
       <c r="N9" s="91"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
@@ -24634,18 +24646,18 @@
       <c r="N13" s="91"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="C14" s="236" t="s">
+      <c r="C14" s="245" t="s">
         <v>397</v>
       </c>
-      <c r="D14" s="236"/>
-      <c r="E14" s="236"/>
-      <c r="F14" s="236"/>
-      <c r="G14" s="236"/>
-      <c r="H14" s="236"/>
-      <c r="I14" s="236"/>
-      <c r="J14" s="236"/>
-      <c r="K14" s="236"/>
-      <c r="L14" s="236"/>
+      <c r="D14" s="245"/>
+      <c r="E14" s="245"/>
+      <c r="F14" s="245"/>
+      <c r="G14" s="245"/>
+      <c r="H14" s="245"/>
+      <c r="I14" s="245"/>
+      <c r="J14" s="245"/>
+      <c r="K14" s="245"/>
+      <c r="L14" s="245"/>
       <c r="N14" s="91"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.2">
@@ -24735,10 +24747,10 @@
       <c r="N19" s="91"/>
     </row>
     <row r="20" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B20" s="237" t="s">
+      <c r="B20" s="239" t="s">
         <v>399</v>
       </c>
-      <c r="C20" s="237"/>
+      <c r="C20" s="239"/>
       <c r="N20" s="91"/>
     </row>
     <row r="21" spans="2:14" x14ac:dyDescent="0.2">
@@ -24773,7 +24785,7 @@
       </c>
       <c r="C24" s="135">
         <f ca="1">IF(Overview!C29&gt;0,Overview!C29,WACC!C19)</f>
-        <v>0.10015650000000001</v>
+        <v>0.10068199999999999</v>
       </c>
     </row>
     <row r="25" spans="2:14" x14ac:dyDescent="0.2">
@@ -24790,7 +24802,7 @@
       </c>
       <c r="C26" s="235">
         <f ca="1">C23/(C24-C25)</f>
-        <v>13.234110770804612</v>
+        <v>13.147914032869787</v>
       </c>
     </row>
   </sheetData>
@@ -24839,20 +24851,20 @@
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A3" s="4"/>
-      <c r="C3" s="237" t="s">
+      <c r="C3" s="239" t="s">
         <v>110</v>
       </c>
-      <c r="D3" s="237"/>
-      <c r="E3" s="237"/>
-      <c r="F3" s="237"/>
-      <c r="G3" s="238"/>
-      <c r="H3" s="239" t="s">
+      <c r="D3" s="239"/>
+      <c r="E3" s="239"/>
+      <c r="F3" s="239"/>
+      <c r="G3" s="248"/>
+      <c r="H3" s="249" t="s">
         <v>111</v>
       </c>
-      <c r="I3" s="237"/>
-      <c r="J3" s="237"/>
-      <c r="K3" s="237"/>
-      <c r="L3" s="237"/>
+      <c r="I3" s="239"/>
+      <c r="J3" s="239"/>
+      <c r="K3" s="239"/>
+      <c r="L3" s="239"/>
       <c r="P3" s="250"/>
       <c r="Q3" s="250"/>
       <c r="R3" s="250"/>
@@ -24870,18 +24882,18 @@
     <row r="5" spans="1:28" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="86"/>
       <c r="B5" s="60"/>
-      <c r="C5" s="236" t="s">
+      <c r="C5" s="245" t="s">
         <v>177</v>
       </c>
-      <c r="D5" s="236"/>
-      <c r="E5" s="236"/>
-      <c r="F5" s="236"/>
-      <c r="G5" s="236"/>
-      <c r="H5" s="236"/>
-      <c r="I5" s="236"/>
-      <c r="J5" s="236"/>
-      <c r="K5" s="236"/>
-      <c r="L5" s="236"/>
+      <c r="D5" s="245"/>
+      <c r="E5" s="245"/>
+      <c r="F5" s="245"/>
+      <c r="G5" s="245"/>
+      <c r="H5" s="245"/>
+      <c r="I5" s="245"/>
+      <c r="J5" s="245"/>
+      <c r="K5" s="245"/>
+      <c r="L5" s="245"/>
       <c r="P5" s="250"/>
       <c r="Q5" s="250"/>
       <c r="R5" s="250"/>
@@ -25027,7 +25039,7 @@
       <c r="K8" s="137"/>
       <c r="L8" s="126">
         <f ca="1">L7*(1+C20)/(C21-C20)</f>
-        <v>6307154.3218209138</v>
+        <v>6269053.1461620694</v>
       </c>
       <c r="N8" s="91"/>
       <c r="O8" s="16"/>
@@ -25081,23 +25093,23 @@
       <c r="G10" s="138"/>
       <c r="H10" s="126">
         <f ca="1">H7/(1+$C$21)^H9</f>
-        <v>111053.89030596531</v>
+        <v>111005.31601687268</v>
       </c>
       <c r="I10" s="126">
         <f t="shared" ref="I10:L10" ca="1" si="1">I7/(1+$C$21)^I9</f>
-        <v>142967.88936277106</v>
+        <v>142842.85016216265</v>
       </c>
       <c r="J10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>184053.14152013644</v>
+        <v>183811.7360014421</v>
       </c>
       <c r="K10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>236945.22633312788</v>
+        <v>236530.94469556829</v>
       </c>
       <c r="L10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>305037.12035751826</v>
+        <v>304370.5968705886</v>
       </c>
       <c r="N10" s="91"/>
     </row>
@@ -25116,15 +25128,15 @@
       <c r="K11" s="137"/>
       <c r="L11" s="126">
         <f ca="1">L8/(1+C21)^L9</f>
-        <v>3931650.4799678572</v>
+        <v>3899360.6103479848</v>
       </c>
     </row>
     <row r="13" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="14" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="B14" s="252" t="s">
+      <c r="B14" s="251" t="s">
         <v>219</v>
       </c>
-      <c r="C14" s="253"/>
+      <c r="C14" s="252"/>
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B15" s="150" t="s">
@@ -25132,7 +25144,7 @@
       </c>
       <c r="C15" s="151">
         <f ca="1">Overview!C5</f>
-        <v>341.07</v>
+        <v>329.4</v>
       </c>
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.2">
@@ -25141,7 +25153,7 @@
       </c>
       <c r="C16" s="151">
         <f ca="1">C36</f>
-        <v>340.8168252602012</v>
+        <v>338.50178526069749</v>
       </c>
     </row>
     <row r="17" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -25151,20 +25163,20 @@
       <c r="C17" s="153">
         <v>0.41499999999999998</v>
       </c>
-      <c r="E17" s="251" t="s">
+      <c r="E17" s="253" t="s">
         <v>222</v>
       </c>
-      <c r="F17" s="251"/>
-      <c r="G17" s="251"/>
-      <c r="H17" s="251"/>
-      <c r="I17" s="251"/>
+      <c r="F17" s="253"/>
+      <c r="G17" s="253"/>
+      <c r="H17" s="253"/>
+      <c r="I17" s="253"/>
     </row>
     <row r="18" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B19" s="252" t="s">
+      <c r="B19" s="251" t="s">
         <v>181</v>
       </c>
-      <c r="C19" s="253"/>
+      <c r="C19" s="252"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B20" s="154" t="s">
@@ -25180,7 +25192,7 @@
       </c>
       <c r="C21" s="216">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.9136704635863854E-2</v>
+        <v>9.9617670646853729E-2</v>
       </c>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.2">
@@ -25198,7 +25210,7 @@
       </c>
       <c r="C23" s="156">
         <f ca="1">C15*C22</f>
-        <v>4977575.58</v>
+        <v>4807263.5999999996</v>
       </c>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.2">
@@ -25225,15 +25237,15 @@
       </c>
       <c r="C26" s="157">
         <f ca="1">C23+C25-C24</f>
-        <v>4915402.58</v>
+        <v>4745090.5999999996</v>
       </c>
     </row>
     <row r="27" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="28" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B28" s="252" t="s">
+      <c r="B28" s="251" t="s">
         <v>183</v>
       </c>
-      <c r="C28" s="253"/>
+      <c r="C28" s="252"/>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B29" s="154" t="s">
@@ -25241,7 +25253,7 @@
       </c>
       <c r="C29" s="156">
         <f ca="1">SUM(H10:L10)</f>
-        <v>980057.26787951891</v>
+        <v>978561.44374663429</v>
       </c>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
@@ -25250,7 +25262,7 @@
       </c>
       <c r="C30" s="156">
         <f ca="1">L11</f>
-        <v>3931650.4799678572</v>
+        <v>3899360.6103479848</v>
       </c>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.2">
@@ -25259,7 +25271,7 @@
       </c>
       <c r="C31" s="159">
         <f ca="1">C29+C30</f>
-        <v>4911707.7478473764</v>
+        <v>4877922.0540946191</v>
       </c>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.2">
@@ -25286,7 +25298,7 @@
       </c>
       <c r="C34" s="159">
         <f ca="1">C31+C32-C33</f>
-        <v>4973880.7478473764</v>
+        <v>4940095.0540946191</v>
       </c>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.2">
@@ -25304,21 +25316,21 @@
       </c>
       <c r="C36" s="162">
         <f ca="1">C34/C35</f>
-        <v>340.8168252602012</v>
+        <v>338.50178526069749</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="E17:I17"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="H3:L3"/>
     <mergeCell ref="P3:W3"/>
     <mergeCell ref="X3:Z3"/>
     <mergeCell ref="C5:L5"/>
     <mergeCell ref="P5:Z5"/>
     <mergeCell ref="B14:C14"/>
-    <mergeCell ref="E17:I17"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="C3:G3"/>
-    <mergeCell ref="H3:L3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -31823,7 +31835,7 @@
       </c>
       <c r="AC114" s="63">
         <f ca="1">Overview!C5</f>
-        <v>341.07</v>
+        <v>329.4</v>
       </c>
     </row>
     <row r="115" spans="1:31" x14ac:dyDescent="0.2">
@@ -31894,7 +31906,7 @@
       </c>
       <c r="AC115" s="65">
         <f ca="1">AC114/AC84</f>
-        <v>341.07</v>
+        <v>329.4</v>
       </c>
     </row>
     <row r="117" spans="1:31" x14ac:dyDescent="0.2">
@@ -32808,7 +32820,7 @@
       <c r="AA140" s="49"/>
       <c r="AC140" s="72">
         <f ca="1">AC115/Statement!AC25</f>
-        <v>39.113532110091747</v>
+        <v>37.775229357798167</v>
       </c>
     </row>
     <row r="141" spans="2:29" x14ac:dyDescent="0.2">
@@ -32845,7 +32857,7 @@
       <c r="AA141" s="49"/>
       <c r="AC141" s="72">
         <f ca="1">AC115/(Statement!AC5/Statement!AC21)</f>
-        <v>10.797643351977086</v>
+        <v>10.428192805410186</v>
       </c>
     </row>
     <row r="142" spans="2:29" x14ac:dyDescent="0.2">
@@ -32906,7 +32918,7 @@
       </c>
       <c r="AC142" s="72">
         <f ca="1">AC115/(Statement!AC48/Statement!AC74)</f>
-        <v>46.294415736607142</v>
+        <v>44.710412946428569</v>
       </c>
     </row>
     <row r="143" spans="2:29" x14ac:dyDescent="0.2">
@@ -32967,7 +32979,7 @@
       </c>
       <c r="AC143" s="141">
         <f ca="1">Statement!AC115*Statement!AC77</f>
-        <v>4997698.71</v>
+        <v>4826698.1999999993</v>
       </c>
     </row>
     <row r="144" spans="2:29" x14ac:dyDescent="0.2">
@@ -33028,7 +33040,7 @@
       </c>
       <c r="AC144" s="141">
         <f ca="1">AC143+AC106-AC105+AC47+AC44</f>
-        <v>4935525.71</v>
+        <v>4764525.1999999993</v>
       </c>
     </row>
     <row r="145" spans="2:29" x14ac:dyDescent="0.2">
@@ -33065,7 +33077,7 @@
       <c r="AA145" s="49"/>
       <c r="AC145" s="177">
         <f ca="1">AC144/AC5</f>
-        <v>10.572584705552211</v>
+        <v>10.206277754095234</v>
       </c>
     </row>
     <row r="146" spans="2:29" x14ac:dyDescent="0.2">
@@ -33102,7 +33114,7 @@
       <c r="AA146" s="49"/>
       <c r="AC146" s="177">
         <f ca="1">AC144/AC11</f>
-        <v>31.871093769170663</v>
+        <v>30.766860176031095</v>
       </c>
     </row>
     <row r="147" spans="2:29" x14ac:dyDescent="0.2">
@@ -33237,7 +33249,7 @@
       <c r="AA149" s="49"/>
       <c r="AC149" s="72">
         <f t="shared" ref="AC149:AC150" ca="1" si="137">AC143/AC147</f>
-        <v>40.639296047228342</v>
+        <v>39.248787984745107</v>
       </c>
     </row>
     <row r="150" spans="2:29" x14ac:dyDescent="0.2">
@@ -33274,7 +33286,7 @@
       <c r="AA150" s="49"/>
       <c r="AC150" s="72">
         <f t="shared" ca="1" si="137"/>
-        <v>38.627249452137846</v>
+        <v>37.288936221830959</v>
       </c>
     </row>
     <row r="151" spans="2:29" x14ac:dyDescent="0.2">
@@ -33311,7 +33323,7 @@
       <c r="AA151" s="49"/>
       <c r="AC151" s="74">
         <f t="shared" ref="AC151" ca="1" si="140">AC147/AC143</f>
-        <v>2.4606725442238592E-2</v>
+        <v>2.5478493766194044E-2</v>
       </c>
     </row>
     <row r="152" spans="2:29" x14ac:dyDescent="0.2">
@@ -33348,7 +33360,7 @@
       <c r="AA152" s="49"/>
       <c r="AC152" s="74">
         <f ca="1">AC25/AC115</f>
-        <v>2.5566599231829239E-2</v>
+        <v>2.6472374013357617E-2</v>
       </c>
     </row>
     <row r="153" spans="2:29" x14ac:dyDescent="0.2">
@@ -33385,7 +33397,7 @@
       <c r="AA153" s="49"/>
       <c r="AC153" s="149">
         <f ca="1">AC81/AC115</f>
-        <v>3.0785469258509984E-3</v>
+        <v>3.1876138433515485E-3</v>
       </c>
     </row>
     <row r="154" spans="2:29" x14ac:dyDescent="0.2">
@@ -33422,7 +33434,7 @@
       <c r="AA154" s="49"/>
       <c r="AC154" s="149">
         <f ca="1">-AC62/AC143</f>
-        <v>1.6452772520174592E-2</v>
+        <v>1.7035662184140706E-2</v>
       </c>
     </row>
     <row r="155" spans="2:29" x14ac:dyDescent="0.2">
@@ -33459,7 +33471,7 @@
       <c r="AA155" s="49"/>
       <c r="AC155" s="149">
         <f ca="1">-(AC62+AC63)/AC143</f>
-        <v>1.9582212870131181E-2</v>
+        <v>2.0275972506422716E-2</v>
       </c>
     </row>
     <row r="156" spans="2:29" x14ac:dyDescent="0.2">
@@ -33962,7 +33974,7 @@
       <c r="AA166" s="49"/>
       <c r="AC166" s="149">
         <f ca="1">(AC105-AC106)/AC143</f>
-        <v>1.2440325759453395E-2</v>
+        <v>1.2881062254938585E-2</v>
       </c>
     </row>
     <row r="167" spans="1:31" x14ac:dyDescent="0.2">
@@ -35959,15 +35971,15 @@
       </c>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B4" s="237" t="s">
+      <c r="B4" s="239" t="s">
         <v>227</v>
       </c>
-      <c r="C4" s="237"/>
-      <c r="E4" s="237" t="s">
+      <c r="C4" s="239"/>
+      <c r="E4" s="239" t="s">
         <v>234</v>
       </c>
-      <c r="F4" s="237"/>
-      <c r="G4" s="237"/>
+      <c r="F4" s="239"/>
+      <c r="G4" s="239"/>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B5" s="20" t="s">
@@ -35975,7 +35987,7 @@
       </c>
       <c r="C5" s="166">
         <f ca="1">Overview!C5</f>
-        <v>341.07</v>
+        <v>329.4</v>
       </c>
       <c r="E5" s="12"/>
       <c r="F5" s="132" t="s">
@@ -35991,7 +36003,7 @@
       </c>
       <c r="C6" s="167">
         <f ca="1">Statement!AC143</f>
-        <v>4997698.71</v>
+        <v>4826698.1999999993</v>
       </c>
       <c r="E6" s="20" t="s">
         <v>19</v>
@@ -36011,7 +36023,7 @@
       </c>
       <c r="C7" s="167">
         <f ca="1">Statement!AC144</f>
-        <v>4935525.71</v>
+        <v>4764525.1999999993</v>
       </c>
       <c r="E7" s="20" t="s">
         <v>29</v>
@@ -36031,7 +36043,7 @@
       </c>
       <c r="C8" s="168">
         <f ca="1">Statement!AC140</f>
-        <v>39.113532110091747</v>
+        <v>37.775229357798167</v>
       </c>
       <c r="E8" s="20" t="s">
         <v>237</v>
@@ -36051,7 +36063,7 @@
       </c>
       <c r="C9" s="168">
         <f ca="1">Statement!AC141</f>
-        <v>10.797643351977086</v>
+        <v>10.428192805410186</v>
       </c>
       <c r="E9" s="20" t="s">
         <v>238</v>
@@ -36071,7 +36083,7 @@
       </c>
       <c r="C10" s="168">
         <f ca="1">Statement!AC142</f>
-        <v>46.294415736607142</v>
+        <v>44.710412946428569</v>
       </c>
       <c r="E10" s="20" t="s">
         <v>1</v>
@@ -36091,7 +36103,7 @@
       </c>
       <c r="C11" s="168">
         <f ca="1">Statement!AC145</f>
-        <v>10.572584705552211</v>
+        <v>10.206277754095234</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.2">
@@ -36100,18 +36112,18 @@
       </c>
       <c r="C12" s="168">
         <f ca="1">Statement!AC146</f>
-        <v>31.871093769170663</v>
+        <v>30.766860176031095</v>
       </c>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B15" s="237" t="s">
+      <c r="B15" s="239" t="s">
         <v>75</v>
       </c>
-      <c r="C15" s="237"/>
-      <c r="E15" s="237" t="s">
+      <c r="C15" s="239"/>
+      <c r="E15" s="239" t="s">
         <v>240</v>
       </c>
-      <c r="F15" s="237"/>
+      <c r="F15" s="239"/>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B16" s="20" t="s">
@@ -36162,14 +36174,14 @@
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B21" s="237" t="s">
+      <c r="B21" s="239" t="s">
         <v>239</v>
       </c>
-      <c r="C21" s="237"/>
-      <c r="E21" s="237" t="s">
+      <c r="C21" s="239"/>
+      <c r="E21" s="239" t="s">
         <v>243</v>
       </c>
-      <c r="F21" s="237"/>
+      <c r="F21" s="239"/>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B22" s="20" t="s">
@@ -36238,14 +36250,14 @@
       </c>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B29" s="237" t="s">
+      <c r="B29" s="239" t="s">
         <v>244</v>
       </c>
-      <c r="C29" s="237"/>
-      <c r="E29" s="237" t="s">
+      <c r="C29" s="239"/>
+      <c r="E29" s="239" t="s">
         <v>250</v>
       </c>
-      <c r="F29" s="237"/>
+      <c r="F29" s="239"/>
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B30" s="20" t="s">
@@ -36321,14 +36333,14 @@
       </c>
     </row>
     <row r="37" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B37" s="237" t="s">
+      <c r="B37" s="239" t="s">
         <v>262</v>
       </c>
-      <c r="C37" s="237"/>
-      <c r="E37" s="237" t="s">
+      <c r="C37" s="239"/>
+      <c r="E37" s="239" t="s">
         <v>265</v>
       </c>
-      <c r="F37" s="237"/>
+      <c r="F37" s="239"/>
     </row>
     <row r="38" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B38" s="20" t="s">
@@ -36336,7 +36348,7 @@
       </c>
       <c r="C38" s="169">
         <f ca="1">Statement!AC152</f>
-        <v>2.5566599231829239E-2</v>
+        <v>2.6472374013357617E-2</v>
       </c>
       <c r="E38" s="20" t="s">
         <v>264</v>
@@ -36352,7 +36364,7 @@
       </c>
       <c r="C39" s="209">
         <f ca="1">Statement!AC151</f>
-        <v>2.4606725442238592E-2</v>
+        <v>2.5478493766194044E-2</v>
       </c>
       <c r="E39" s="20" t="s">
         <v>266</v>
@@ -36368,7 +36380,7 @@
       </c>
       <c r="C40" s="169">
         <f ca="1">Statement!AC153</f>
-        <v>3.0785469258509984E-3</v>
+        <v>3.1876138433515485E-3</v>
       </c>
       <c r="E40" s="20" t="s">
         <v>267</v>
@@ -36384,7 +36396,7 @@
       </c>
       <c r="C41" s="169">
         <f ca="1">Statement!AC154</f>
-        <v>1.6452772520174592E-2</v>
+        <v>1.7035662184140706E-2</v>
       </c>
     </row>
     <row r="42" spans="2:6" x14ac:dyDescent="0.2">
@@ -36393,18 +36405,18 @@
       </c>
       <c r="C42" s="169">
         <f ca="1">Statement!AC155</f>
-        <v>1.9582212870131181E-2</v>
+        <v>2.0275972506422716E-2</v>
       </c>
     </row>
     <row r="45" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B45" s="237" t="s">
+      <c r="B45" s="239" t="s">
         <v>273</v>
       </c>
-      <c r="C45" s="237"/>
-      <c r="E45" s="237" t="s">
+      <c r="C45" s="239"/>
+      <c r="E45" s="239" t="s">
         <v>279</v>
       </c>
-      <c r="F45" s="237"/>
+      <c r="F45" s="239"/>
     </row>
     <row r="46" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B46" s="20" t="s">
@@ -36437,18 +36449,18 @@
       </c>
       <c r="F48" s="169">
         <f ca="1">Statement!AC166</f>
-        <v>1.2440325759453395E-2</v>
+        <v>1.2881062254938585E-2</v>
       </c>
     </row>
     <row r="51" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B51" s="237" t="s">
+      <c r="B51" s="239" t="s">
         <v>276</v>
       </c>
-      <c r="C51" s="237"/>
-      <c r="E51" s="237" t="s">
+      <c r="C51" s="239"/>
+      <c r="E51" s="239" t="s">
         <v>297</v>
       </c>
-      <c r="F51" s="237"/>
+      <c r="F51" s="239"/>
     </row>
     <row r="52" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B52" s="20" t="s">
@@ -36616,7 +36628,7 @@
       </c>
       <c r="I6" s="166">
         <f ca="1">Statement!AC114</f>
-        <v>341.07</v>
+        <v>329.4</v>
       </c>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.2">
@@ -36645,7 +36657,7 @@
       </c>
       <c r="I7" s="167">
         <f ca="1">Statement!AC143</f>
-        <v>4997698.71</v>
+        <v>4826698.1999999993</v>
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
@@ -36674,7 +36686,7 @@
       </c>
       <c r="I8" s="167">
         <f ca="1">Statement!AC144</f>
-        <v>4935525.71</v>
+        <v>4764525.1999999993</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
@@ -36703,7 +36715,7 @@
       </c>
       <c r="I9" s="168">
         <f ca="1">Statement!AC140</f>
-        <v>39.113532110091747</v>
+        <v>37.775229357798167</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.2">
@@ -36732,7 +36744,7 @@
       </c>
       <c r="I10" s="168">
         <f ca="1">Statement!AC141</f>
-        <v>10.797643351977086</v>
+        <v>10.428192805410186</v>
       </c>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.2">
@@ -36761,7 +36773,7 @@
       </c>
       <c r="I11" s="168">
         <f ca="1">Statement!AC142</f>
-        <v>46.294415736607142</v>
+        <v>44.710412946428569</v>
       </c>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.2">
@@ -36790,7 +36802,7 @@
       </c>
       <c r="I12" s="168">
         <f ca="1">Statement!AC145</f>
-        <v>10.572584705552211</v>
+        <v>10.206277754095234</v>
       </c>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
@@ -36819,7 +36831,7 @@
       </c>
       <c r="I13" s="168">
         <f ca="1">Statement!AC146</f>
-        <v>31.871093769170663</v>
+        <v>30.766860176031095</v>
       </c>
     </row>
     <row r="15" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -37592,7 +37604,7 @@
       </c>
       <c r="I51" s="169">
         <f ca="1">Statement!AC152</f>
-        <v>2.5566599231829239E-2</v>
+        <v>2.6472374013357617E-2</v>
       </c>
     </row>
     <row r="52" spans="2:9" x14ac:dyDescent="0.2">
@@ -37621,7 +37633,7 @@
       </c>
       <c r="I52" s="169">
         <f ca="1">Statement!AC151</f>
-        <v>2.4606725442238592E-2</v>
+        <v>2.5478493766194044E-2</v>
       </c>
     </row>
     <row r="53" spans="2:9" x14ac:dyDescent="0.2">
@@ -37650,7 +37662,7 @@
       </c>
       <c r="I53" s="169">
         <f ca="1">Statement!AC153</f>
-        <v>3.0785469258509984E-3</v>
+        <v>3.1876138433515485E-3</v>
       </c>
     </row>
     <row r="54" spans="2:9" x14ac:dyDescent="0.2">
@@ -37679,7 +37691,7 @@
       </c>
       <c r="I54" s="169">
         <f ca="1">Statement!AC154</f>
-        <v>1.6452772520174592E-2</v>
+        <v>1.7035662184140706E-2</v>
       </c>
     </row>
     <row r="55" spans="2:9" x14ac:dyDescent="0.2">
@@ -37708,7 +37720,7 @@
       </c>
       <c r="I55" s="169">
         <f ca="1">Statement!AC155</f>
-        <v>1.9582212870131181E-2</v>
+        <v>2.0275972506422716E-2</v>
       </c>
     </row>
     <row r="57" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -37944,7 +37956,7 @@
       </c>
       <c r="I68" s="190">
         <f ca="1">Statement!AC166</f>
-        <v>1.2440325759453395E-2</v>
+        <v>1.2881062254938585E-2</v>
       </c>
     </row>
     <row r="70" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -38636,14 +38648,14 @@
     <row r="1" spans="2:7" ht="12" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="3" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B3" s="8"/>
-      <c r="C3" s="245" t="s">
+      <c r="C3" s="240" t="s">
         <v>307</v>
       </c>
-      <c r="D3" s="246"/>
-      <c r="F3" s="247" t="s">
+      <c r="D3" s="241"/>
+      <c r="F3" s="242" t="s">
         <v>308</v>
       </c>
-      <c r="G3" s="246"/>
+      <c r="G3" s="241"/>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B4" s="8"/>
@@ -39446,36 +39458,6 @@
     </row>
   </sheetData>
   <mergeCells count="38">
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="F36:G36"/>
     <mergeCell ref="C44:D44"/>
     <mergeCell ref="F44:G44"/>
     <mergeCell ref="C38:D38"/>
@@ -39484,6 +39466,36 @@
     <mergeCell ref="F40:G40"/>
     <mergeCell ref="C42:D42"/>
     <mergeCell ref="F42:G42"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="F36:G36"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="F9:G9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>

</xml_diff>

<commit_message>
Fixed a bug in the formula for FCFF in the TTM column
</commit_message>
<xml_diff>
--- a/AAPL.xlsx
+++ b/AAPL.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/KINGSTON/MyStockData/Finance-StockLists/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC17B24C-5CB2-5E41-BFE3-E728F8000197}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F62E2388-65B4-0E4B-B5A6-9C27A724E166}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14400" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14400" activeTab="2" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -2344,12 +2344,6 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="18" fillId="17" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="18" fillId="17" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2357,6 +2351,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="18" fillId="17" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="18" fillId="17" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2377,14 +2377,14 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -15523,11 +15523,11 @@
     <v>Powered by Refinitiv</v>
     <v>345.34</v>
     <v>243.42</v>
-    <v>1.069</v>
-    <v>-2.7</v>
-    <v>-8.1079999999999989E-3</v>
-    <v>0.16339999999999999</v>
-    <v>4.9470000000000004E-4</v>
+    <v>1.0795999999999999</v>
+    <v>-0.8</v>
+    <v>-2.3969999999999998E-3</v>
+    <v>7.4999999999999997E-3</v>
+    <v>2.2529999999999999E-5</v>
     <v>USD</v>
     <v>Apple Inc. designs, manufactures and markets smartphones, personal computers, tablets, wearables and accessories, and sells a variety of related services. Its product categories include iPhone, Mac, iPad, Wearables, Home and Accessories. Its services include advertising, AppleCare, cloud services, digital content, and payment services. The Company operates various platforms, including the App Store, that allow customers to discover and download applications and digital content, such as books, music, video, games and podcasts. It also offers digital content through subscription-based services, including Apple Arcade, Apple Fitness+, Apple Music, Apple News+, and Apple TV+. Its wearables include smartwatches, wireless headphones, and spatial computers. Its products include iPhone 16 Pro, iPhone 16, iPhone 15, iPhone 14, iPhone SE, MacBook Air, MacBook Pro, iMac, Mac mini, Mac Studio, Mac Pro, iPad Pro, iPad Air, AirPods, AirPods Pro, AirPods Max, Apple TV, Apple Vision Pro and others.</v>
     <v>166000</v>
@@ -15535,25 +15535,25 @@
     <v>XNAS</v>
     <v>XNAS</v>
     <v>One Apple Park Way, CUPERTINO, CA, 95014 US</v>
-    <v>332.48160000000001</v>
+    <v>336.21</v>
     <v>Computers, Phones &amp; Household Electronics</v>
     <v>Stock</v>
-    <v>46296.843086411718</v>
+    <v>46300.889066863281</v>
     <v>0</v>
-    <v>325.81</v>
-    <v>4820749537600</v>
+    <v>331.65</v>
+    <v>4858256580200</v>
     <v>APPLE INC.</v>
     <v>APPLE INC.</v>
-    <v>329.6</v>
-    <v>38.008899999999997</v>
-    <v>333.02</v>
-    <v>330.32</v>
-    <v>330.48340000000002</v>
+    <v>332.815</v>
+    <v>38.396700000000003</v>
+    <v>333.69</v>
+    <v>332.89</v>
+    <v>332.89749999999998</v>
     <v>14594180000</v>
     <v>AAPL</v>
     <v>APPLE INC. (XNAS:AAPL)</v>
-    <v>34959379</v>
-    <v>41825512</v>
+    <v>34335686</v>
+    <v>41951159</v>
     <v>1977</v>
   </rv>
   <rv s="2">
@@ -15575,19 +15575,19 @@
     <v>268435456</v>
     <v>1</v>
     <v>Powered by Refinitiv</v>
-    <v>53.06</v>
+    <v>53.42</v>
     <v>39.47</v>
-    <v>0.38</v>
-    <v>7.2309999999999996E-3</v>
+    <v>0.4</v>
+    <v>7.6380000000000007E-3</v>
     <v>US</v>
-    <v>53.06</v>
+    <v>52.98</v>
     <v>Index</v>
     <v>3</v>
-    <v>52.05</v>
+    <v>51.57</v>
     <v>10 Y TSY YLD NDX</v>
-    <v>52.43</v>
-    <v>52.55</v>
-    <v>52.93</v>
+    <v>52.16</v>
+    <v>52.37</v>
+    <v>52.77</v>
     <v>TNX</v>
     <v>10 Y TSY YLD NDX</v>
   </rv>
@@ -16408,7 +16408,7 @@
       </c>
       <c r="F3" s="181">
         <f ca="1">Statement!AC143</f>
-        <v>4840178.96</v>
+        <v>4877837.17</v>
       </c>
       <c r="H3" s="179" t="str">
         <f>'AVG target price'!B5</f>
@@ -16416,7 +16416,7 @@
       </c>
       <c r="I3" s="205">
         <f ca="1">'AVG target price'!C5</f>
-        <v>112.97660356325736</v>
+        <v>112.5324096820578</v>
       </c>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.2">
@@ -16432,7 +16432,7 @@
       </c>
       <c r="F4" s="182">
         <f ca="1">Statement!AC144</f>
-        <v>4778005.96</v>
+        <v>4815664.17</v>
       </c>
       <c r="H4" s="179" t="str">
         <f>'AVG target price'!B6</f>
@@ -16440,7 +16440,7 @@
       </c>
       <c r="I4" s="205">
         <f ca="1">'AVG target price'!C6</f>
-        <v>228.59835302710741</v>
+        <v>228.29174889122544</v>
       </c>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.2">
@@ -16449,7 +16449,7 @@
       </c>
       <c r="C5" s="202" cm="1">
         <f t="array" aca="1" ref="C5" ca="1">_FV(C3,"Price",TRUE)</f>
-        <v>330.32</v>
+        <v>332.89</v>
       </c>
       <c r="E5" s="179" t="s">
         <v>237</v>
@@ -16464,7 +16464,7 @@
       </c>
       <c r="I5" s="205">
         <f ca="1">'AVG target price'!C7</f>
-        <v>200.17486407506783</v>
+        <v>199.8869501569128</v>
       </c>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.2">
@@ -16473,14 +16473,14 @@
       </c>
       <c r="C6" s="202" cm="1">
         <f t="array" aca="1" ref="C6" ca="1">_FV(C3,"Price (Extended hours)",TRUE)</f>
-        <v>330.48340000000002</v>
+        <v>332.89749999999998</v>
       </c>
       <c r="E6" s="179" t="s">
         <v>231</v>
       </c>
       <c r="F6" s="184">
         <f ca="1">Statement!AC140</f>
-        <v>37.88073394495413</v>
+        <v>38.175458715596335</v>
       </c>
       <c r="H6" s="179" t="str">
         <f>'AVG target price'!B8</f>
@@ -16488,7 +16488,7 @@
       </c>
       <c r="I6" s="205">
         <f ca="1">'AVG target price'!C8</f>
-        <v>198.77182911427875</v>
+        <v>198.50853359075884</v>
       </c>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.2">
@@ -16497,14 +16497,14 @@
       </c>
       <c r="C7" s="6" cm="1">
         <f t="array" aca="1" ref="C7" ca="1">_FV(C3,"Change")</f>
-        <v>-2.7</v>
+        <v>-0.8</v>
       </c>
       <c r="E7" s="180" t="s">
         <v>198</v>
       </c>
       <c r="F7" s="185">
         <f ca="1">Statement!AC141</f>
-        <v>10.457318298370046</v>
+        <v>10.53867972979052</v>
       </c>
       <c r="H7" s="179" t="str">
         <f>'AVG target price'!B9</f>
@@ -16512,7 +16512,7 @@
       </c>
       <c r="I7" s="205">
         <f ca="1">'AVG target price'!C9</f>
-        <v>212.73761911200157</v>
+        <v>212.45404502745629</v>
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
@@ -16521,14 +16521,14 @@
       </c>
       <c r="C8" s="6" cm="1">
         <f t="array" aca="1" ref="C8" ca="1">_FV(C3,"Change (extended hours)",TRUE)</f>
-        <v>0.16339999999999999</v>
+        <v>7.4999999999999997E-3</v>
       </c>
       <c r="E8" s="179" t="s">
         <v>259</v>
       </c>
       <c r="F8" s="186">
         <f ca="1">Statement!AC151</f>
-        <v>2.5407531625648818E-2</v>
+        <v>2.521137867338856E-2</v>
       </c>
       <c r="H8" s="178" t="str">
         <f>'AVG target price'!B10</f>
@@ -16536,7 +16536,7 @@
       </c>
       <c r="I8" s="206">
         <f ca="1">'AVG target price'!C10</f>
-        <v>190.65185377834257</v>
+        <v>190.33473746968221</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
@@ -16545,14 +16545,14 @@
       </c>
       <c r="C9" s="73" cm="1">
         <f t="array" aca="1" ref="C9" ca="1">_FV(C3,"Change (%)",TRUE)</f>
-        <v>-8.1079999999999989E-3</v>
+        <v>-2.3969999999999998E-3</v>
       </c>
       <c r="E9" s="179" t="s">
         <v>282</v>
       </c>
       <c r="F9" s="186">
         <f ca="1">Statement!AC152</f>
-        <v>2.6398643739404211E-2</v>
+        <v>2.6194839136050946E-2</v>
       </c>
       <c r="H9" s="178" t="str">
         <f>'AVG target price'!B12</f>
@@ -16560,7 +16560,7 @@
       </c>
       <c r="I9" s="207">
         <f ca="1">'AVG target price'!C12</f>
-        <v>-0.42282679287254005</v>
+        <v>-0.4282353405939433</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.2">
@@ -16569,14 +16569,14 @@
       </c>
       <c r="C10" s="73" cm="1">
         <f t="array" aca="1" ref="C10" ca="1">_FV(C3,"Change % (extended hours)",TRUE)</f>
-        <v>4.9470000000000004E-4</v>
+        <v>2.2529999999999999E-5</v>
       </c>
       <c r="E10" s="179" t="s">
         <v>287</v>
       </c>
       <c r="F10" s="186">
         <f ca="1">Statement!AC154</f>
-        <v>1.6988214832453219E-2</v>
+        <v>1.68570612618461E-2</v>
       </c>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.2">
@@ -16592,14 +16592,14 @@
       </c>
       <c r="F11" s="187">
         <f ca="1">Statement!AC153</f>
-        <v>3.1787357713732142E-3</v>
+        <v>3.1541950794556762E-3</v>
       </c>
       <c r="H11" s="178" t="s">
         <v>394</v>
       </c>
       <c r="I11" s="206">
         <f ca="1">DDM!C26</f>
-        <v>13.090639846979702</v>
+        <v>13.039630248795358</v>
       </c>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.2">
@@ -16624,7 +16624,7 @@
       </c>
       <c r="C13" s="203" cm="1">
         <f t="array" aca="1" ref="C13" ca="1">_FV(C3,"Beta")</f>
-        <v>1.069</v>
+        <v>1.0795999999999999</v>
       </c>
       <c r="E13" s="179" t="s">
         <v>101</v>
@@ -16647,7 +16647,7 @@
       </c>
       <c r="C14" s="204" cm="1">
         <f t="array" aca="1" ref="C14" ca="1">_FV(C3,"Volume average",TRUE)</f>
-        <v>41825512</v>
+        <v>41951159</v>
       </c>
       <c r="E14" s="180" t="s">
         <v>102</v>
@@ -16663,7 +16663,7 @@
       </c>
       <c r="F15" s="186">
         <f ca="1">Statement!AC166</f>
-        <v>1.2845186203610951E-2</v>
+        <v>1.2746017924169453E-2</v>
       </c>
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.2">
@@ -16773,7 +16773,7 @@
       </c>
       <c r="F26" s="213" cm="1">
         <f t="array" aca="1" ref="F26" ca="1">_FV(E26,"Price")</f>
-        <v>52.93</v>
+        <v>52.77</v>
       </c>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.2">
@@ -16788,7 +16788,7 @@
       </c>
       <c r="F27" s="214">
         <f ca="1">F26/1000</f>
-        <v>5.2929999999999998E-2</v>
+        <v>5.2770000000000004E-2</v>
       </c>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.2">
@@ -21049,12 +21049,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="C3:G3"/>
-    <mergeCell ref="H3:L3"/>
-    <mergeCell ref="P3:W3"/>
-    <mergeCell ref="X3:Z3"/>
-    <mergeCell ref="C5:L5"/>
-    <mergeCell ref="P5:Z5"/>
     <mergeCell ref="C40:L40"/>
     <mergeCell ref="C11:L11"/>
     <mergeCell ref="P11:Z11"/>
@@ -21062,6 +21056,12 @@
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="C26:L26"/>
     <mergeCell ref="C33:L33"/>
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="H3:L3"/>
+    <mergeCell ref="P3:W3"/>
+    <mergeCell ref="X3:Z3"/>
+    <mergeCell ref="C5:L5"/>
+    <mergeCell ref="P5:Z5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -22121,16 +22121,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="C31:L31"/>
+    <mergeCell ref="C25:L25"/>
+    <mergeCell ref="C2:G2"/>
+    <mergeCell ref="H2:L2"/>
+    <mergeCell ref="S2:Z2"/>
     <mergeCell ref="AA2:AC2"/>
     <mergeCell ref="C4:L4"/>
     <mergeCell ref="S4:AC4"/>
     <mergeCell ref="C13:L13"/>
     <mergeCell ref="C18:L18"/>
-    <mergeCell ref="C31:L31"/>
-    <mergeCell ref="C25:L25"/>
-    <mergeCell ref="C2:G2"/>
-    <mergeCell ref="H2:L2"/>
-    <mergeCell ref="S2:Z2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -22213,7 +22213,7 @@
       </c>
       <c r="C6" s="133">
         <f ca="1">Overview!C5</f>
-        <v>330.32</v>
+        <v>332.89</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22222,7 +22222,7 @@
       </c>
       <c r="C7" s="134">
         <f ca="1">C5*C6</f>
-        <v>4840178.96</v>
+        <v>4877837.17</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22240,7 +22240,7 @@
       </c>
       <c r="C9" s="135">
         <f ca="1">Overview!F27</f>
-        <v>5.2929999999999998E-2</v>
+        <v>5.2770000000000004E-2</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22249,7 +22249,7 @@
       </c>
       <c r="C10" s="133">
         <f ca="1">Overview!C13</f>
-        <v>1.069</v>
+        <v>1.0795999999999999</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22292,7 +22292,7 @@
       </c>
       <c r="C16" s="46">
         <f ca="1">C8/(C8+C7)</f>
-        <v>1.7127344249401166E-2</v>
+        <v>1.6997364084552359E-2</v>
       </c>
     </row>
     <row r="17" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22301,7 +22301,7 @@
       </c>
       <c r="C17" s="46">
         <f ca="1">C7/(C8+C7)</f>
-        <v>0.98287265575059879</v>
+        <v>0.98300263591544768</v>
       </c>
     </row>
     <row r="18" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22319,7 +22319,7 @@
       </c>
       <c r="C19" s="46">
         <f ca="1">C9+C10*C11</f>
-        <v>0.10103499999999999</v>
+        <v>0.101352</v>
       </c>
     </row>
     <row r="20" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22328,7 +22328,7 @@
       </c>
       <c r="C20" s="46">
         <f ca="1">(C17*C19)+(C16*C18)</f>
-        <v>9.9967538269656056E-2</v>
+        <v>0.10028725111901547</v>
       </c>
     </row>
   </sheetData>
@@ -22579,7 +22579,7 @@
       </c>
       <c r="L8" s="126">
         <f ca="1">L7*(1+C14)/(C15-C14)</f>
-        <v>1812668.3875956913</v>
+        <v>1805450.1385329245</v>
       </c>
       <c r="N8" s="91"/>
       <c r="O8" s="16"/>
@@ -22633,23 +22633,23 @@
       <c r="G10" s="138"/>
       <c r="H10" s="126">
         <f ca="1">H7/(1+$C$15)^H9</f>
-        <v>100329.33882403738</v>
+        <v>100300.18591078027</v>
       </c>
       <c r="I10" s="126">
         <f t="shared" ref="I10:L10" ca="1" si="0">I7/(1+$C$15)^I9</f>
-        <v>96907.925008476799</v>
+        <v>96851.615699354021</v>
       </c>
       <c r="J10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>93086.532266053357</v>
+        <v>93005.410776455916</v>
       </c>
       <c r="K10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>89005.203844455478</v>
+        <v>88901.799185814481</v>
       </c>
       <c r="L10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>88253.629002446542</v>
+        <v>88125.483254749459</v>
       </c>
       <c r="N10" s="91"/>
     </row>
@@ -22668,7 +22668,7 @@
       <c r="K11" s="137"/>
       <c r="L11" s="126">
         <f ca="1">L8/(1+C15)^L9</f>
-        <v>1125690.5430669405</v>
+        <v>1119579.904244039</v>
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.2">
@@ -22691,7 +22691,7 @@
       </c>
       <c r="C15" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.9967538269656056E-2</v>
+        <v>0.10028725111901547</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.2">
@@ -22706,7 +22706,7 @@
       </c>
       <c r="C19" s="64">
         <f ca="1">SUM(H10:L10)</f>
-        <v>467582.62894546957</v>
+        <v>467184.49482715409</v>
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.2">
@@ -22715,7 +22715,7 @@
       </c>
       <c r="C20" s="64">
         <f ca="1">L11</f>
-        <v>1125690.5430669405</v>
+        <v>1119579.904244039</v>
       </c>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.2">
@@ -22724,7 +22724,7 @@
       </c>
       <c r="C21" s="94">
         <f ca="1">C19+C20</f>
-        <v>1593273.1720124101</v>
+        <v>1586764.3990711931</v>
       </c>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.2">
@@ -22751,7 +22751,7 @@
       </c>
       <c r="C24" s="94">
         <f ca="1">C21+C22-C23</f>
-        <v>1655446.1720124101</v>
+        <v>1648937.3990711931</v>
       </c>
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.2">
@@ -22769,7 +22769,7 @@
       </c>
       <c r="C26" s="235">
         <f ca="1">C24/C25</f>
-        <v>112.97660356325736</v>
+        <v>112.5324096820578</v>
       </c>
     </row>
   </sheetData>
@@ -23038,23 +23038,23 @@
       <c r="G9" s="138"/>
       <c r="H9" s="92">
         <f ca="1">DCF!H10</f>
-        <v>100329.33882403738</v>
+        <v>100300.18591078027</v>
       </c>
       <c r="I9" s="92">
         <f ca="1">DCF!I10</f>
-        <v>96907.925008476799</v>
+        <v>96851.615699354021</v>
       </c>
       <c r="J9" s="92">
         <f ca="1">DCF!J10</f>
-        <v>93086.532266053357</v>
+        <v>93005.410776455916</v>
       </c>
       <c r="K9" s="92">
         <f ca="1">DCF!K10</f>
-        <v>89005.203844455478</v>
+        <v>88901.799185814481</v>
       </c>
       <c r="L9" s="92">
         <f ca="1">DCF!L10</f>
-        <v>88253.629002446542</v>
+        <v>88125.483254749459</v>
       </c>
       <c r="N9" s="91"/>
     </row>
@@ -23840,7 +23840,7 @@
       </c>
       <c r="C41" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.9967538269656056E-2</v>
+        <v>0.10028725111901547</v>
       </c>
     </row>
     <row r="42" spans="2:14" x14ac:dyDescent="0.2">
@@ -23866,7 +23866,7 @@
       </c>
       <c r="C44" s="24">
         <f ca="1">C43/(1+C41)^5</f>
-        <v>2908149.6669631819</v>
+        <v>2903926.9849307216</v>
       </c>
     </row>
     <row r="45" spans="2:14" x14ac:dyDescent="0.2">
@@ -23875,7 +23875,7 @@
       </c>
       <c r="C45" s="108">
         <f ca="1">SUM(H9:K9)+C44</f>
-        <v>3287478.666906205</v>
+        <v>3282985.9965031263</v>
       </c>
     </row>
     <row r="46" spans="2:14" x14ac:dyDescent="0.2">
@@ -23902,7 +23902,7 @@
       </c>
       <c r="C48" s="94">
         <f ca="1">C45+C46-C47</f>
-        <v>3349651.666906205</v>
+        <v>3345158.9965031263</v>
       </c>
     </row>
     <row r="49" spans="2:3" x14ac:dyDescent="0.2">
@@ -23920,7 +23920,7 @@
       </c>
       <c r="C50" s="235">
         <f ca="1">C48/C49</f>
-        <v>228.59835302710741</v>
+        <v>228.29174889122544</v>
       </c>
     </row>
     <row r="52" spans="2:3" x14ac:dyDescent="0.2">
@@ -23944,7 +23944,7 @@
       </c>
       <c r="C54" s="135">
         <f ca="1">IF(Overview!C29&gt;0,Overview!C29,WACC!C19)</f>
-        <v>0.10103499999999999</v>
+        <v>0.101352</v>
       </c>
     </row>
     <row r="55" spans="2:3" x14ac:dyDescent="0.2">
@@ -23979,7 +23979,7 @@
       </c>
       <c r="C58" s="235">
         <f ca="1">C57/(1+C54)^5</f>
-        <v>200.17486407506783</v>
+        <v>199.8869501569128</v>
       </c>
     </row>
     <row r="60" spans="2:3" x14ac:dyDescent="0.2">
@@ -24003,7 +24003,7 @@
       </c>
       <c r="C62" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.9967538269656056E-2</v>
+        <v>0.10028725111901547</v>
       </c>
     </row>
     <row r="63" spans="2:3" x14ac:dyDescent="0.2">
@@ -24029,7 +24029,7 @@
       </c>
       <c r="C65" s="24">
         <f ca="1">C64/(1+C62)^5</f>
-        <v>2471101.6120685032</v>
+        <v>2467513.5311329844</v>
       </c>
     </row>
     <row r="66" spans="2:3" x14ac:dyDescent="0.2">
@@ -24038,7 +24038,7 @@
       </c>
       <c r="C66" s="108">
         <f ca="1">SUM(H9:K9)+C65</f>
-        <v>2850430.6120115262</v>
+        <v>2846572.5427053892</v>
       </c>
     </row>
     <row r="67" spans="2:3" x14ac:dyDescent="0.2">
@@ -24065,7 +24065,7 @@
       </c>
       <c r="C69" s="94">
         <f ca="1">C66+C67-C68</f>
-        <v>2912603.6120115262</v>
+        <v>2908745.5427053892</v>
       </c>
     </row>
     <row r="70" spans="2:3" x14ac:dyDescent="0.2">
@@ -24083,7 +24083,7 @@
       </c>
       <c r="C71" s="235">
         <f ca="1">C69/C70</f>
-        <v>198.77182911427875</v>
+        <v>198.50853359075884</v>
       </c>
     </row>
     <row r="73" spans="2:3" x14ac:dyDescent="0.2">
@@ -24107,7 +24107,7 @@
       </c>
       <c r="C75" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.9967538269656056E-2</v>
+        <v>0.10028725111901547</v>
       </c>
     </row>
     <row r="76" spans="2:3" x14ac:dyDescent="0.2">
@@ -24133,7 +24133,7 @@
       </c>
       <c r="C78" s="24">
         <f ca="1">C77/(1+C75)^5</f>
-        <v>2675742.332905136</v>
+        <v>2671857.1102149123</v>
       </c>
     </row>
     <row r="79" spans="2:3" x14ac:dyDescent="0.2">
@@ -24142,7 +24142,7 @@
       </c>
       <c r="C79" s="108">
         <f ca="1">SUM(H9:K9)+C78</f>
-        <v>3055071.3328481591</v>
+        <v>3050916.1217873171</v>
       </c>
     </row>
     <row r="80" spans="2:3" x14ac:dyDescent="0.2">
@@ -24169,7 +24169,7 @@
       </c>
       <c r="C82" s="94">
         <f ca="1">C79+C80-C81</f>
-        <v>3117244.3328481591</v>
+        <v>3113089.1217873171</v>
       </c>
     </row>
     <row r="83" spans="2:3" x14ac:dyDescent="0.2">
@@ -24187,22 +24187,22 @@
       </c>
       <c r="C84" s="235">
         <f ca="1">C82/C83</f>
-        <v>212.73761911200157</v>
+        <v>212.45404502745629</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B73:C73"/>
-    <mergeCell ref="C27:L27"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="B60:C60"/>
     <mergeCell ref="C22:L22"/>
     <mergeCell ref="C2:G2"/>
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="C4:L4"/>
     <mergeCell ref="C11:L11"/>
     <mergeCell ref="C17:L17"/>
+    <mergeCell ref="B73:C73"/>
+    <mergeCell ref="C27:L27"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="B60:C60"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -24252,7 +24252,7 @@
       </c>
       <c r="C5" s="133">
         <f ca="1">DCF!C26</f>
-        <v>112.97660356325736</v>
+        <v>112.5324096820578</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -24261,7 +24261,7 @@
       </c>
       <c r="C6" s="133">
         <f ca="1">Multiples!C50</f>
-        <v>228.59835302710741</v>
+        <v>228.29174889122544</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
@@ -24270,7 +24270,7 @@
       </c>
       <c r="C7" s="133">
         <f ca="1">Multiples!C58</f>
-        <v>200.17486407506783</v>
+        <v>199.8869501569128</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
@@ -24279,7 +24279,7 @@
       </c>
       <c r="C8" s="133">
         <f ca="1">Multiples!C71</f>
-        <v>198.77182911427875</v>
+        <v>198.50853359075884</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
@@ -24288,7 +24288,7 @@
       </c>
       <c r="C9" s="133">
         <f ca="1">Multiples!C84</f>
-        <v>212.73761911200157</v>
+        <v>212.45404502745629</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
@@ -24297,7 +24297,7 @@
       </c>
       <c r="C10" s="235">
         <f ca="1">AVERAGE(C5:C9)</f>
-        <v>190.65185377834257</v>
+        <v>190.33473746968221</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
@@ -24306,7 +24306,7 @@
       </c>
       <c r="C11" s="133">
         <f ca="1">Overview!C5</f>
-        <v>330.32</v>
+        <v>332.89</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.2">
@@ -24315,7 +24315,7 @@
       </c>
       <c r="C12" s="149">
         <f ca="1">(C10-C11)/C11</f>
-        <v>-0.42282679287254005</v>
+        <v>-0.4282353405939433</v>
       </c>
     </row>
   </sheetData>
@@ -24785,7 +24785,7 @@
       </c>
       <c r="C24" s="135">
         <f ca="1">IF(Overview!C29&gt;0,Overview!C29,WACC!C19)</f>
-        <v>0.10103499999999999</v>
+        <v>0.101352</v>
       </c>
     </row>
     <row r="25" spans="2:14" x14ac:dyDescent="0.2">
@@ -24802,7 +24802,7 @@
       </c>
       <c r="C26" s="235">
         <f ca="1">C23/(C24-C25)</f>
-        <v>13.090639846979702</v>
+        <v>13.039630248795358</v>
       </c>
     </row>
   </sheetData>
@@ -25039,7 +25039,7 @@
       <c r="K8" s="137"/>
       <c r="L8" s="126">
         <f ca="1">L7*(1+C20)/(C21-C20)</f>
-        <v>6241625.2826948576</v>
+        <v>6216770.4299511006</v>
       </c>
       <c r="N8" s="91"/>
       <c r="O8" s="16"/>
@@ -25093,23 +25093,23 @@
       <c r="G10" s="138"/>
       <c r="H10" s="126">
         <f ca="1">H7/(1+$C$21)^H9</f>
-        <v>110970.00846034756</v>
+        <v>110937.76366467061</v>
       </c>
       <c r="I10" s="126">
         <f t="shared" ref="I10:L10" ca="1" si="1">I7/(1+$C$21)^I9</f>
-        <v>142751.99631654753</v>
+        <v>142669.04885597836</v>
       </c>
       <c r="J10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>183636.39631190285</v>
+        <v>183476.36394577549</v>
       </c>
       <c r="K10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>236230.15383717773</v>
+        <v>235955.70585702444</v>
       </c>
       <c r="L10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>303886.8476113716</v>
+        <v>303445.59881806257</v>
       </c>
       <c r="N10" s="91"/>
     </row>
@@ -25128,15 +25128,15 @@
       <c r="K11" s="137"/>
       <c r="L11" s="126">
         <f ca="1">L8/(1+C21)^L9</f>
-        <v>3876130.1306834915</v>
+        <v>3855089.1515218099</v>
       </c>
     </row>
     <row r="13" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="14" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="B14" s="252" t="s">
+      <c r="B14" s="251" t="s">
         <v>219</v>
       </c>
-      <c r="C14" s="253"/>
+      <c r="C14" s="252"/>
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B15" s="150" t="s">
@@ -25144,7 +25144,7 @@
       </c>
       <c r="C15" s="151">
         <f ca="1">Overview!C5</f>
-        <v>330.32</v>
+        <v>332.89</v>
       </c>
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.2">
@@ -25153,7 +25153,7 @@
       </c>
       <c r="C16" s="151">
         <f ca="1">C36</f>
-        <v>336.83558539268461</v>
+        <v>335.3259307018858</v>
       </c>
     </row>
     <row r="17" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -25163,20 +25163,20 @@
       <c r="C17" s="153">
         <v>0.41499999999999998</v>
       </c>
-      <c r="E17" s="251" t="s">
+      <c r="E17" s="253" t="s">
         <v>222</v>
       </c>
-      <c r="F17" s="251"/>
-      <c r="G17" s="251"/>
-      <c r="H17" s="251"/>
-      <c r="I17" s="251"/>
+      <c r="F17" s="253"/>
+      <c r="G17" s="253"/>
+      <c r="H17" s="253"/>
+      <c r="I17" s="253"/>
     </row>
     <row r="18" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B19" s="252" t="s">
+      <c r="B19" s="251" t="s">
         <v>181</v>
       </c>
-      <c r="C19" s="253"/>
+      <c r="C19" s="252"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B20" s="154" t="s">
@@ -25192,7 +25192,7 @@
       </c>
       <c r="C21" s="216">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.9967538269656056E-2</v>
+        <v>0.10028725111901547</v>
       </c>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.2">
@@ -25210,7 +25210,7 @@
       </c>
       <c r="C23" s="156">
         <f ca="1">C15*C22</f>
-        <v>4820690.08</v>
+        <v>4858196.66</v>
       </c>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.2">
@@ -25237,15 +25237,15 @@
       </c>
       <c r="C26" s="157">
         <f ca="1">C23+C25-C24</f>
-        <v>4758517.08</v>
+        <v>4796023.66</v>
       </c>
     </row>
     <row r="27" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="28" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B28" s="252" t="s">
+      <c r="B28" s="251" t="s">
         <v>183</v>
       </c>
-      <c r="C28" s="253"/>
+      <c r="C28" s="252"/>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B29" s="154" t="s">
@@ -25253,7 +25253,7 @@
       </c>
       <c r="C29" s="156">
         <f ca="1">SUM(H10:L10)</f>
-        <v>977475.40253734728</v>
+        <v>976484.48114151147</v>
       </c>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
@@ -25262,7 +25262,7 @@
       </c>
       <c r="C30" s="156">
         <f ca="1">L11</f>
-        <v>3876130.1306834915</v>
+        <v>3855089.1515218099</v>
       </c>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.2">
@@ -25271,7 +25271,7 @@
       </c>
       <c r="C31" s="159">
         <f ca="1">C29+C30</f>
-        <v>4853605.5332208388</v>
+        <v>4831573.6326633217</v>
       </c>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.2">
@@ -25298,7 +25298,7 @@
       </c>
       <c r="C34" s="159">
         <f ca="1">C31+C32-C33</f>
-        <v>4915778.5332208388</v>
+        <v>4893746.6326633217</v>
       </c>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.2">
@@ -25316,21 +25316,21 @@
       </c>
       <c r="C36" s="162">
         <f ca="1">C34/C35</f>
-        <v>336.83558539268461</v>
+        <v>335.3259307018858</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="E17:I17"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="H3:L3"/>
     <mergeCell ref="P3:W3"/>
     <mergeCell ref="X3:Z3"/>
     <mergeCell ref="C5:L5"/>
     <mergeCell ref="P5:Z5"/>
     <mergeCell ref="B14:C14"/>
-    <mergeCell ref="E17:I17"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="C3:G3"/>
-    <mergeCell ref="H3:L3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -31835,7 +31835,7 @@
       </c>
       <c r="AC114" s="63">
         <f ca="1">Overview!C5</f>
-        <v>330.32</v>
+        <v>332.89</v>
       </c>
     </row>
     <row r="115" spans="1:31" x14ac:dyDescent="0.2">
@@ -31906,7 +31906,7 @@
       </c>
       <c r="AC115" s="65">
         <f ca="1">AC114/AC84</f>
-        <v>330.32</v>
+        <v>332.89</v>
       </c>
     </row>
     <row r="117" spans="1:31" x14ac:dyDescent="0.2">
@@ -32820,7 +32820,7 @@
       <c r="AA140" s="49"/>
       <c r="AC140" s="72">
         <f ca="1">AC115/Statement!AC25</f>
-        <v>37.88073394495413</v>
+        <v>38.175458715596335</v>
       </c>
     </row>
     <row r="141" spans="2:29" x14ac:dyDescent="0.2">
@@ -32857,7 +32857,7 @@
       <c r="AA141" s="49"/>
       <c r="AC141" s="72">
         <f ca="1">AC115/(Statement!AC5/Statement!AC21)</f>
-        <v>10.457318298370046</v>
+        <v>10.53867972979052</v>
       </c>
     </row>
     <row r="142" spans="2:29" x14ac:dyDescent="0.2">
@@ -32918,7 +32918,7 @@
       </c>
       <c r="AC142" s="72">
         <f ca="1">AC115/(Statement!AC48/Statement!AC74)</f>
-        <v>44.835287202380947</v>
+        <v>45.184120721726188</v>
       </c>
     </row>
     <row r="143" spans="2:29" x14ac:dyDescent="0.2">
@@ -32979,7 +32979,7 @@
       </c>
       <c r="AC143" s="141">
         <f ca="1">Statement!AC115*Statement!AC77</f>
-        <v>4840178.96</v>
+        <v>4877837.17</v>
       </c>
     </row>
     <row r="144" spans="2:29" x14ac:dyDescent="0.2">
@@ -33040,7 +33040,7 @@
       </c>
       <c r="AC144" s="141">
         <f ca="1">AC143+AC106-AC105+AC47+AC44</f>
-        <v>4778005.96</v>
+        <v>4815664.17</v>
       </c>
     </row>
     <row r="145" spans="2:29" x14ac:dyDescent="0.2">
@@ -33077,7 +33077,7 @@
       <c r="AA145" s="49"/>
       <c r="AC145" s="177">
         <f ca="1">AC144/AC5</f>
-        <v>10.235155422933317</v>
+        <v>10.31582456305709</v>
       </c>
     </row>
     <row r="146" spans="2:29" x14ac:dyDescent="0.2">
@@ -33114,7 +33114,7 @@
       <c r="AA146" s="49"/>
       <c r="AC146" s="177">
         <f ca="1">AC144/AC11</f>
-        <v>30.853912010280318</v>
+        <v>31.097089416824335</v>
       </c>
     </row>
     <row r="147" spans="2:29" x14ac:dyDescent="0.2">
@@ -33211,8 +33211,8 @@
       <c r="Z148" s="49"/>
       <c r="AA148" s="49"/>
       <c r="AC148" s="64">
-        <f>AC107+AC52+AC108+AC54+AC56+AC57</f>
-        <v>127773.1596218234</v>
+        <f>AC107+AC52+AC108+AC54+AC56+AC57+AC55</f>
+        <v>122489.1596218234</v>
       </c>
     </row>
     <row r="149" spans="2:29" x14ac:dyDescent="0.2">
@@ -33249,7 +33249,7 @@
       <c r="AA149" s="49"/>
       <c r="AC149" s="72">
         <f t="shared" ref="AC149:AC150" ca="1" si="137">AC143/AC147</f>
-        <v>39.358408157622968</v>
+        <v>39.664629727510018</v>
       </c>
     </row>
     <row r="150" spans="2:29" x14ac:dyDescent="0.2">
@@ -33286,7 +33286,7 @@
       <c r="AA150" s="49"/>
       <c r="AC150" s="72">
         <f t="shared" ca="1" si="137"/>
-        <v>37.39444163501711</v>
+        <v>39.31502334466186</v>
       </c>
     </row>
     <row r="151" spans="2:29" x14ac:dyDescent="0.2">
@@ -33323,7 +33323,7 @@
       <c r="AA151" s="49"/>
       <c r="AC151" s="74">
         <f t="shared" ref="AC151" ca="1" si="140">AC147/AC143</f>
-        <v>2.5407531625648818E-2</v>
+        <v>2.521137867338856E-2</v>
       </c>
     </row>
     <row r="152" spans="2:29" x14ac:dyDescent="0.2">
@@ -33360,7 +33360,7 @@
       <c r="AA152" s="49"/>
       <c r="AC152" s="74">
         <f ca="1">AC25/AC115</f>
-        <v>2.6398643739404211E-2</v>
+        <v>2.6194839136050946E-2</v>
       </c>
     </row>
     <row r="153" spans="2:29" x14ac:dyDescent="0.2">
@@ -33397,7 +33397,7 @@
       <c r="AA153" s="49"/>
       <c r="AC153" s="149">
         <f ca="1">AC81/AC115</f>
-        <v>3.1787357713732142E-3</v>
+        <v>3.1541950794556762E-3</v>
       </c>
     </row>
     <row r="154" spans="2:29" x14ac:dyDescent="0.2">
@@ -33434,7 +33434,7 @@
       <c r="AA154" s="49"/>
       <c r="AC154" s="149">
         <f ca="1">-AC62/AC143</f>
-        <v>1.6988214832453219E-2</v>
+        <v>1.68570612618461E-2</v>
       </c>
     </row>
     <row r="155" spans="2:29" x14ac:dyDescent="0.2">
@@ -33471,7 +33471,7 @@
       <c r="AA155" s="49"/>
       <c r="AC155" s="149">
         <f ca="1">-(AC62+AC63)/AC143</f>
-        <v>2.0219500313682616E-2</v>
+        <v>2.0063400353316836E-2</v>
       </c>
     </row>
     <row r="156" spans="2:29" x14ac:dyDescent="0.2">
@@ -33508,7 +33508,7 @@
       <c r="AA156" s="49"/>
       <c r="AC156" s="149">
         <f>AC148/AC5</f>
-        <v>0.2737079356026233</v>
+        <v>0.26238887034662689</v>
       </c>
     </row>
     <row r="157" spans="2:29" x14ac:dyDescent="0.2">
@@ -33974,7 +33974,7 @@
       <c r="AA166" s="49"/>
       <c r="AC166" s="149">
         <f ca="1">(AC105-AC106)/AC143</f>
-        <v>1.2845186203610951E-2</v>
+        <v>1.2746017924169453E-2</v>
       </c>
     </row>
     <row r="167" spans="1:31" x14ac:dyDescent="0.2">
@@ -35987,7 +35987,7 @@
       </c>
       <c r="C5" s="166">
         <f ca="1">Overview!C5</f>
-        <v>330.32</v>
+        <v>332.89</v>
       </c>
       <c r="E5" s="12"/>
       <c r="F5" s="132" t="s">
@@ -36003,7 +36003,7 @@
       </c>
       <c r="C6" s="167">
         <f ca="1">Statement!AC143</f>
-        <v>4840178.96</v>
+        <v>4877837.17</v>
       </c>
       <c r="E6" s="20" t="s">
         <v>19</v>
@@ -36023,7 +36023,7 @@
       </c>
       <c r="C7" s="167">
         <f ca="1">Statement!AC144</f>
-        <v>4778005.96</v>
+        <v>4815664.17</v>
       </c>
       <c r="E7" s="20" t="s">
         <v>29</v>
@@ -36043,7 +36043,7 @@
       </c>
       <c r="C8" s="168">
         <f ca="1">Statement!AC140</f>
-        <v>37.88073394495413</v>
+        <v>38.175458715596335</v>
       </c>
       <c r="E8" s="20" t="s">
         <v>237</v>
@@ -36063,7 +36063,7 @@
       </c>
       <c r="C9" s="168">
         <f ca="1">Statement!AC141</f>
-        <v>10.457318298370046</v>
+        <v>10.53867972979052</v>
       </c>
       <c r="E9" s="20" t="s">
         <v>238</v>
@@ -36083,7 +36083,7 @@
       </c>
       <c r="C10" s="168">
         <f ca="1">Statement!AC142</f>
-        <v>44.835287202380947</v>
+        <v>45.184120721726188</v>
       </c>
       <c r="E10" s="20" t="s">
         <v>1</v>
@@ -36103,7 +36103,7 @@
       </c>
       <c r="C11" s="168">
         <f ca="1">Statement!AC145</f>
-        <v>10.235155422933317</v>
+        <v>10.31582456305709</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.2">
@@ -36112,7 +36112,7 @@
       </c>
       <c r="C12" s="168">
         <f ca="1">Statement!AC146</f>
-        <v>30.853912010280318</v>
+        <v>31.097089416824335</v>
       </c>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.2">
@@ -36348,7 +36348,7 @@
       </c>
       <c r="C38" s="169">
         <f ca="1">Statement!AC152</f>
-        <v>2.6398643739404211E-2</v>
+        <v>2.6194839136050946E-2</v>
       </c>
       <c r="E38" s="20" t="s">
         <v>264</v>
@@ -36364,7 +36364,7 @@
       </c>
       <c r="C39" s="209">
         <f ca="1">Statement!AC151</f>
-        <v>2.5407531625648818E-2</v>
+        <v>2.521137867338856E-2</v>
       </c>
       <c r="E39" s="20" t="s">
         <v>266</v>
@@ -36380,7 +36380,7 @@
       </c>
       <c r="C40" s="169">
         <f ca="1">Statement!AC153</f>
-        <v>3.1787357713732142E-3</v>
+        <v>3.1541950794556762E-3</v>
       </c>
       <c r="E40" s="20" t="s">
         <v>267</v>
@@ -36396,7 +36396,7 @@
       </c>
       <c r="C41" s="169">
         <f ca="1">Statement!AC154</f>
-        <v>1.6988214832453219E-2</v>
+        <v>1.68570612618461E-2</v>
       </c>
     </row>
     <row r="42" spans="2:6" x14ac:dyDescent="0.2">
@@ -36405,7 +36405,7 @@
       </c>
       <c r="C42" s="169">
         <f ca="1">Statement!AC155</f>
-        <v>2.0219500313682616E-2</v>
+        <v>2.0063400353316836E-2</v>
       </c>
     </row>
     <row r="45" spans="2:6" x14ac:dyDescent="0.2">
@@ -36449,7 +36449,7 @@
       </c>
       <c r="F48" s="169">
         <f ca="1">Statement!AC166</f>
-        <v>1.2845186203610951E-2</v>
+        <v>1.2746017924169453E-2</v>
       </c>
     </row>
     <row r="51" spans="2:6" x14ac:dyDescent="0.2">
@@ -36628,7 +36628,7 @@
       </c>
       <c r="I6" s="166">
         <f ca="1">Statement!AC114</f>
-        <v>330.32</v>
+        <v>332.89</v>
       </c>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.2">
@@ -36657,7 +36657,7 @@
       </c>
       <c r="I7" s="167">
         <f ca="1">Statement!AC143</f>
-        <v>4840178.96</v>
+        <v>4877837.17</v>
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
@@ -36686,7 +36686,7 @@
       </c>
       <c r="I8" s="167">
         <f ca="1">Statement!AC144</f>
-        <v>4778005.96</v>
+        <v>4815664.17</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
@@ -36715,7 +36715,7 @@
       </c>
       <c r="I9" s="168">
         <f ca="1">Statement!AC140</f>
-        <v>37.88073394495413</v>
+        <v>38.175458715596335</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.2">
@@ -36744,7 +36744,7 @@
       </c>
       <c r="I10" s="168">
         <f ca="1">Statement!AC141</f>
-        <v>10.457318298370046</v>
+        <v>10.53867972979052</v>
       </c>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.2">
@@ -36773,7 +36773,7 @@
       </c>
       <c r="I11" s="168">
         <f ca="1">Statement!AC142</f>
-        <v>44.835287202380947</v>
+        <v>45.184120721726188</v>
       </c>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.2">
@@ -36802,7 +36802,7 @@
       </c>
       <c r="I12" s="168">
         <f ca="1">Statement!AC145</f>
-        <v>10.235155422933317</v>
+        <v>10.31582456305709</v>
       </c>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
@@ -36831,7 +36831,7 @@
       </c>
       <c r="I13" s="168">
         <f ca="1">Statement!AC146</f>
-        <v>30.853912010280318</v>
+        <v>31.097089416824335</v>
       </c>
     </row>
     <row r="15" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -37604,7 +37604,7 @@
       </c>
       <c r="I51" s="169">
         <f ca="1">Statement!AC152</f>
-        <v>2.6398643739404211E-2</v>
+        <v>2.6194839136050946E-2</v>
       </c>
     </row>
     <row r="52" spans="2:9" x14ac:dyDescent="0.2">
@@ -37633,7 +37633,7 @@
       </c>
       <c r="I52" s="169">
         <f ca="1">Statement!AC151</f>
-        <v>2.5407531625648818E-2</v>
+        <v>2.521137867338856E-2</v>
       </c>
     </row>
     <row r="53" spans="2:9" x14ac:dyDescent="0.2">
@@ -37662,7 +37662,7 @@
       </c>
       <c r="I53" s="169">
         <f ca="1">Statement!AC153</f>
-        <v>3.1787357713732142E-3</v>
+        <v>3.1541950794556762E-3</v>
       </c>
     </row>
     <row r="54" spans="2:9" x14ac:dyDescent="0.2">
@@ -37691,7 +37691,7 @@
       </c>
       <c r="I54" s="169">
         <f ca="1">Statement!AC154</f>
-        <v>1.6988214832453219E-2</v>
+        <v>1.68570612618461E-2</v>
       </c>
     </row>
     <row r="55" spans="2:9" x14ac:dyDescent="0.2">
@@ -37720,7 +37720,7 @@
       </c>
       <c r="I55" s="169">
         <f ca="1">Statement!AC155</f>
-        <v>2.0219500313682616E-2</v>
+        <v>2.0063400353316836E-2</v>
       </c>
     </row>
     <row r="57" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -37956,7 +37956,7 @@
       </c>
       <c r="I68" s="190">
         <f ca="1">Statement!AC166</f>
-        <v>1.2845186203610951E-2</v>
+        <v>1.2746017924169453E-2</v>
       </c>
     </row>
     <row r="70" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -38648,14 +38648,14 @@
     <row r="1" spans="2:7" ht="12" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="3" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B3" s="8"/>
-      <c r="C3" s="242" t="s">
+      <c r="C3" s="240" t="s">
         <v>307</v>
       </c>
-      <c r="D3" s="243"/>
-      <c r="F3" s="244" t="s">
+      <c r="D3" s="241"/>
+      <c r="F3" s="242" t="s">
         <v>308</v>
       </c>
-      <c r="G3" s="243"/>
+      <c r="G3" s="241"/>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B4" s="8"/>
@@ -38722,19 +38722,19 @@
       <c r="B7" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C7" s="240">
+      <c r="C7" s="243">
         <f>Statement!AA88</f>
         <v>-1.5892574471146927E-2</v>
       </c>
-      <c r="D7" s="241"/>
-      <c r="F7" s="240">
+      <c r="D7" s="244"/>
+      <c r="F7" s="243">
         <f>IF(F6=0,
 IF(G6=0,0,IF(G6&gt;0,1,-1)),
 (G6-F6)/ABS(F6)
 )</f>
         <v>0.16356501765281381</v>
       </c>
-      <c r="G7" s="241"/>
+      <c r="G7" s="244"/>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B8" s="201" t="s">
@@ -38761,19 +38761,19 @@
       <c r="B9" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C9" s="240">
+      <c r="C9" s="243">
         <f>Statement!AA89</f>
         <v>-3.1133095757317875E-2</v>
       </c>
-      <c r="D9" s="241"/>
-      <c r="F9" s="240">
+      <c r="D9" s="244"/>
+      <c r="F9" s="243">
         <f>IF(F8=0,
 IF(G8=0,0,IF(G8&gt;0,1,-1)),
 (G8-F8)/ABS(F8)
 )</f>
         <v>8.6032831193608647E-2</v>
       </c>
-      <c r="G9" s="241"/>
+      <c r="G9" s="244"/>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B10" s="201" t="s">
@@ -38800,19 +38800,19 @@
       <c r="B11" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C11" s="240">
+      <c r="C11" s="243">
         <f>Statement!AA90</f>
         <v>-2.0079954728829339E-4</v>
       </c>
-      <c r="D11" s="241"/>
-      <c r="F11" s="240">
+      <c r="D11" s="244"/>
+      <c r="F11" s="243">
         <f>IF(F10=0,
 IF(G10=0,0,IF(G10&gt;0,1,-1)),
 (G10-F10)/ABS(F10)
 )</f>
         <v>0.25280204949906215</v>
       </c>
-      <c r="G11" s="241"/>
+      <c r="G11" s="244"/>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B12" s="201" t="s">
@@ -38839,19 +38839,19 @@
       <c r="B13" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C13" s="240">
+      <c r="C13" s="243">
         <f>Statement!AA93</f>
         <v>9.4729043183742583E-3</v>
       </c>
-      <c r="D13" s="241"/>
-      <c r="F13" s="240">
+      <c r="D13" s="244"/>
+      <c r="F13" s="243">
         <f>IF(F12=0,
 IF(G12=0,0,IF(G12&gt;0,1,-1)),
 (G12-F12)/ABS(F12)
 )</f>
         <v>0.22937612786800721</v>
       </c>
-      <c r="G13" s="241"/>
+      <c r="G13" s="244"/>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B14" s="201" t="s">
@@ -38878,19 +38878,19 @@
       <c r="B15" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C15" s="240">
+      <c r="C15" s="243">
         <f>Statement!AA94</f>
         <v>-5.2946913752264175E-3</v>
       </c>
-      <c r="D15" s="241"/>
-      <c r="F15" s="240">
+      <c r="D15" s="244"/>
+      <c r="F15" s="243">
         <f>IF(F14=0,
 IF(G14=0,0,IF(G14&gt;0,1,-1)),
 (G14-F14)/ABS(F14)
 )</f>
         <v>0.26569037656903766</v>
       </c>
-      <c r="G15" s="241"/>
+      <c r="G15" s="244"/>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B16" s="201" t="s">
@@ -38917,19 +38917,19 @@
       <c r="B17" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C17" s="240">
+      <c r="C17" s="243">
         <f>Statement!AA96</f>
         <v>7.1336804381635002E-3</v>
       </c>
-      <c r="D17" s="241"/>
-      <c r="F17" s="240">
+      <c r="D17" s="244"/>
+      <c r="F17" s="243">
         <f>IF(F16=0,
 IF(G16=0,0,IF(G16&gt;0,1,-1)),
 (G16-F16)/ABS(F16)
 )</f>
         <v>0.27118716394981651</v>
       </c>
-      <c r="G17" s="241"/>
+      <c r="G17" s="244"/>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B18" s="201" t="s">
@@ -38956,22 +38956,22 @@
       <c r="B19" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C19" s="240">
+      <c r="C19" s="243">
         <f>IF(C18=0,
 IF(D18=0,0,IF(D18&gt;0,1,-1)),
 (D18-C18)/ABS(C18)
 )</f>
         <v>-7.4697813391280731E-4</v>
       </c>
-      <c r="D19" s="241"/>
-      <c r="F19" s="240">
+      <c r="D19" s="244"/>
+      <c r="F19" s="243">
         <f>IF(F18=0,
 IF(G18=0,0,IF(G18&gt;0,1,-1)),
 (G18-F18)/ABS(F18)
 )</f>
         <v>-1.5587369547765587E-2</v>
       </c>
-      <c r="G19" s="241"/>
+      <c r="G19" s="244"/>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B20" s="201" t="s">
@@ -38998,22 +38998,22 @@
       <c r="B21" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C21" s="240">
+      <c r="C21" s="243">
         <f>IF(C20=0,
 IF(D20=0,0,IF(D20&gt;0,1,-1)),
 (D20-C20)/ABS(C20)
 )</f>
         <v>4.975124378109568E-3</v>
       </c>
-      <c r="D21" s="241"/>
-      <c r="F21" s="240">
+      <c r="D21" s="244"/>
+      <c r="F21" s="243">
         <f>IF(F20=0,
 IF(G20=0,0,IF(G20&gt;0,1,-1)),
 (G20-F20)/ABS(F20)
 )</f>
         <v>0.28662420382165599</v>
       </c>
-      <c r="G21" s="241"/>
+      <c r="G21" s="244"/>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23" s="8" t="s">
@@ -39061,22 +39061,22 @@
       <c r="B25" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C25" s="240">
+      <c r="C25" s="243">
         <f>IF(C24=0,
 IF(D24=0,0,IF(D24&gt;0,1,-1)),
 (D24-C24)/ABS(C24)
 )</f>
         <v>1.5257357017718937E-2</v>
       </c>
-      <c r="D25" s="241"/>
-      <c r="F25" s="240">
+      <c r="D25" s="244"/>
+      <c r="F25" s="243">
         <f>IF(F24=0,
 IF(G24=0,0,IF(G24&gt;0,1,-1)),
 (G24-F24)/ABS(F24)
 )</f>
         <v>0.11124326423612797</v>
       </c>
-      <c r="G25" s="241"/>
+      <c r="G25" s="244"/>
     </row>
     <row r="26" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B26" s="20" t="s">
@@ -39103,22 +39103,22 @@
       <c r="B27" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C27" s="240">
+      <c r="C27" s="243">
         <f>IF(C26=0,
 IF(D26=0,0,IF(D26&gt;0,1,-1)),
 (D26-C26)/ABS(C26)
 )</f>
         <v>4.7692033505613969E-2</v>
       </c>
-      <c r="D27" s="241"/>
-      <c r="F27" s="240">
+      <c r="D27" s="244"/>
+      <c r="F27" s="243">
         <f>IF(F26=0,
 IF(G26=0,0,IF(G26&gt;0,1,-1)),
 (G26-F26)/ABS(F26)
 )</f>
         <v>0.22399433663696178</v>
       </c>
-      <c r="G27" s="241"/>
+      <c r="G27" s="244"/>
     </row>
     <row r="28" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B28" s="20" t="s">
@@ -39145,22 +39145,22 @@
       <c r="B29" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C29" s="240">
+      <c r="C29" s="243">
         <f>IF(C28=0,
 IF(D28=0,0,IF(D28&gt;0,1,-1)),
 (D28-C28)/ABS(C28)
 )</f>
         <v>-8.2012001756354591E-2</v>
       </c>
-      <c r="D29" s="241"/>
-      <c r="F29" s="240">
+      <c r="D29" s="244"/>
+      <c r="F29" s="243">
         <f>IF(F28=0,
 IF(G28=0,0,IF(G28&gt;0,1,-1)),
 (G28-F28)/ABS(F28)
 )</f>
         <v>0.22428264688658989</v>
       </c>
-      <c r="G29" s="241"/>
+      <c r="G29" s="244"/>
     </row>
     <row r="30" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B30" s="20" t="s">
@@ -39187,22 +39187,22 @@
       <c r="B31" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C31" s="240">
+      <c r="C31" s="243">
         <f>IF(C30=0,
 IF(D30=0,0,IF(D30&gt;0,1,-1)),
 (D30-C30)/ABS(C30)
 )</f>
         <v>-0.21985477919295321</v>
       </c>
-      <c r="D31" s="241"/>
-      <c r="F31" s="240">
+      <c r="D31" s="244"/>
+      <c r="F31" s="243">
         <f>IF(F30=0,
 IF(G30=0,0,IF(G30&gt;0,1,-1)),
 (G30-F30)/ABS(F30)
 )</f>
         <v>0.1335178139052231</v>
       </c>
-      <c r="G31" s="241"/>
+      <c r="G31" s="244"/>
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B32" s="20" t="s">
@@ -39229,22 +39229,22 @@
       <c r="B33" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C33" s="240">
+      <c r="C33" s="243">
         <f>IF(C32=0,
 IF(D32=0,0,IF(D32&gt;0,1,-1)),
 (D32-C32)/ABS(C32)
 )</f>
         <v>-2.9218647406434668E-2</v>
       </c>
-      <c r="D33" s="241"/>
-      <c r="F33" s="240">
+      <c r="D33" s="244"/>
+      <c r="F33" s="243">
         <f>IF(F32=0,
 IF(G32=0,0,IF(G32&gt;0,1,-1)),
 (G32-F32)/ABS(F32)
 )</f>
         <v>0.15613189104652678</v>
       </c>
-      <c r="G33" s="241"/>
+      <c r="G33" s="244"/>
     </row>
     <row r="35" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B35" s="224" t="s">
@@ -39271,22 +39271,22 @@
       <c r="B36" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C36" s="240">
+      <c r="C36" s="243">
         <f>IF(C35=0,
 IF(D35=0,0,IF(D35&gt;0,1,-1)),
 (D35-C35)/ABS(C35)
 )</f>
         <v>-4.8110327402884512E-2</v>
       </c>
-      <c r="D36" s="241"/>
-      <c r="F36" s="240">
+      <c r="D36" s="244"/>
+      <c r="F36" s="243">
         <f>IF(F35=0,
 IF(G35=0,0,IF(G35&gt;0,1,-1)),
 (G35-F35)/ABS(F35)
 )</f>
         <v>0.21690368310080302</v>
       </c>
-      <c r="G36" s="241"/>
+      <c r="G36" s="244"/>
     </row>
     <row r="37" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B37" s="224" t="s">
@@ -39313,22 +39313,22 @@
       <c r="B38" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C38" s="240">
+      <c r="C38" s="243">
         <f>IF(C37=0,
 IF(D37=0,0,IF(D37&gt;0,1,-1)),
 (D37-C37)/ABS(C37)
 )</f>
         <v>0.23252768186688891</v>
       </c>
-      <c r="D38" s="241"/>
-      <c r="F38" s="240">
+      <c r="D38" s="244"/>
+      <c r="F38" s="243">
         <f>IF(F37=0,
 IF(G37=0,0,IF(G37&gt;0,1,-1)),
 (G37-F37)/ABS(F37)
 )</f>
         <v>0.28660203827989061</v>
       </c>
-      <c r="G38" s="241"/>
+      <c r="G38" s="244"/>
     </row>
     <row r="39" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B39" s="224" t="s">
@@ -39355,22 +39355,22 @@
       <c r="B40" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C40" s="240">
+      <c r="C40" s="243">
         <f>IF(C39=0,
 IF(D39=0,0,IF(D39&gt;0,1,-1)),
 (D39-C39)/ABS(C39)
 )</f>
         <v>-0.10457043679490888</v>
       </c>
-      <c r="D40" s="241"/>
-      <c r="F40" s="240">
+      <c r="D40" s="244"/>
+      <c r="F40" s="243">
         <f>IF(F39=0,
 IF(G39=0,0,IF(G39&gt;0,1,-1)),
 (G39-F39)/ABS(F39)
 )</f>
         <v>-5.9261510408752466E-2</v>
       </c>
-      <c r="G40" s="241"/>
+      <c r="G40" s="244"/>
     </row>
     <row r="41" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B41" s="224" t="s">
@@ -39397,22 +39397,22 @@
       <c r="B42" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C42" s="240">
+      <c r="C42" s="243">
         <f>IF(C41=0,
 IF(D41=0,0,IF(D41&gt;0,1,-1)),
 (D41-C41)/ABS(C41)
 )</f>
         <v>-2.2781926338438173E-3</v>
       </c>
-      <c r="D42" s="241"/>
-      <c r="F42" s="240">
+      <c r="D42" s="244"/>
+      <c r="F42" s="243">
         <f>IF(F41=0,
 IF(G41=0,0,IF(G41&gt;0,1,-1)),
 (G41-F41)/ABS(F41)
 )</f>
         <v>6.4694759589411135E-2</v>
       </c>
-      <c r="G42" s="241"/>
+      <c r="G42" s="244"/>
     </row>
     <row r="43" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B43" s="224" t="s">
@@ -39439,55 +39439,25 @@
       <c r="B44" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C44" s="240">
+      <c r="C44" s="243">
         <f>IF(C43=0,
 IF(D43=0,0,IF(D43&gt;0,1,-1)),
 (D43-C43)/ABS(C43)
 )</f>
         <v>-7.6510847107438013E-3</v>
       </c>
-      <c r="D44" s="241"/>
-      <c r="F44" s="240">
+      <c r="D44" s="244"/>
+      <c r="F44" s="243">
         <f>IF(F43=0,
 IF(G43=0,0,IF(G43&gt;0,1,-1)),
 (G43-F43)/ABS(F43)
 )</f>
         <v>0.12092039528862633</v>
       </c>
-      <c r="G44" s="241"/>
+      <c r="G44" s="244"/>
     </row>
   </sheetData>
   <mergeCells count="38">
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="F36:G36"/>
     <mergeCell ref="C44:D44"/>
     <mergeCell ref="F44:G44"/>
     <mergeCell ref="C38:D38"/>
@@ -39496,6 +39466,36 @@
     <mergeCell ref="F40:G40"/>
     <mergeCell ref="C42:D42"/>
     <mergeCell ref="F42:G42"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="F36:G36"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="F9:G9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>

</xml_diff>

<commit_message>
Updated models with latest marlet data and added a discount rate widget to VRT Overview page
</commit_message>
<xml_diff>
--- a/AAPL.xlsx
+++ b/AAPL.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/KINGSTON/MyStockData/Finance-StockLists/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F62E2388-65B4-0E4B-B5A6-9C27A724E166}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8937088-2595-D24F-965C-D633922907AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14400" activeTab="2" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14400" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -2344,6 +2344,12 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="168" fontId="18" fillId="17" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="18" fillId="17" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2351,12 +2357,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="18" fillId="17" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="18" fillId="17" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2377,14 +2377,14 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -15523,11 +15523,11 @@
     <v>Powered by Refinitiv</v>
     <v>345.34</v>
     <v>243.42</v>
-    <v>1.0795999999999999</v>
-    <v>-0.8</v>
-    <v>-2.3969999999999998E-3</v>
-    <v>7.4999999999999997E-3</v>
-    <v>2.2529999999999999E-5</v>
+    <v>1.0779000000000001</v>
+    <v>-3.78</v>
+    <v>-1.1104000000000001E-2</v>
+    <v>-0.59</v>
+    <v>-1.7530000000000002E-3</v>
     <v>USD</v>
     <v>Apple Inc. designs, manufactures and markets smartphones, personal computers, tablets, wearables and accessories, and sells a variety of related services. Its product categories include iPhone, Mac, iPad, Wearables, Home and Accessories. Its services include advertising, AppleCare, cloud services, digital content, and payment services. The Company operates various platforms, including the App Store, that allow customers to discover and download applications and digital content, such as books, music, video, games and podcasts. It also offers digital content through subscription-based services, including Apple Arcade, Apple Fitness+, Apple Music, Apple News+, and Apple TV+. Its wearables include smartwatches, wireless headphones, and spatial computers. Its products include iPhone 16 Pro, iPhone 16, iPhone 15, iPhone 14, iPhone SE, MacBook Air, MacBook Pro, iMac, Mac mini, Mac Studio, Mac Pro, iPad Pro, iPad Air, AirPods, AirPods Pro, AirPods Max, Apple TV, Apple Vision Pro and others.</v>
     <v>166000</v>
@@ -15535,25 +15535,25 @@
     <v>XNAS</v>
     <v>XNAS</v>
     <v>One Apple Park Way, CUPERTINO, CA, 95014 US</v>
-    <v>336.21</v>
+    <v>338.61</v>
     <v>Computers, Phones &amp; Household Electronics</v>
     <v>Stock</v>
-    <v>46300.889066863281</v>
+    <v>46304.999846180472</v>
     <v>0</v>
-    <v>331.65</v>
-    <v>4858256580200</v>
+    <v>330.7</v>
+    <v>4912984755200</v>
     <v>APPLE INC.</v>
     <v>APPLE INC.</v>
-    <v>332.815</v>
-    <v>38.396700000000003</v>
-    <v>333.69</v>
-    <v>332.89</v>
-    <v>332.89749999999998</v>
+    <v>331.69499999999999</v>
+    <v>39.171100000000003</v>
+    <v>340.42</v>
+    <v>336.64</v>
+    <v>336.05</v>
     <v>14594180000</v>
     <v>AAPL</v>
     <v>APPLE INC. (XNAS:AAPL)</v>
-    <v>34335686</v>
-    <v>41951159</v>
+    <v>37881199</v>
+    <v>40650930</v>
     <v>1977</v>
   </rv>
   <rv s="2">
@@ -15575,19 +15575,19 @@
     <v>268435456</v>
     <v>1</v>
     <v>Powered by Refinitiv</v>
-    <v>53.42</v>
+    <v>53.64</v>
     <v>39.47</v>
-    <v>0.4</v>
-    <v>7.6380000000000007E-3</v>
+    <v>0.13</v>
+    <v>2.4849999999999998E-3</v>
     <v>US</v>
-    <v>52.98</v>
+    <v>52.8</v>
     <v>Index</v>
     <v>3</v>
-    <v>51.57</v>
+    <v>52.34</v>
     <v>10 Y TSY YLD NDX</v>
-    <v>52.16</v>
-    <v>52.37</v>
-    <v>52.77</v>
+    <v>52.36</v>
+    <v>52.31</v>
+    <v>52.44</v>
     <v>TNX</v>
     <v>10 Y TSY YLD NDX</v>
   </rv>
@@ -15809,9 +15809,9 @@
       <v>at close</v>
       <v>from previous close</v>
       <v>from previous close</v>
-      <v>Source: Nasdaq Last Sale</v>
+      <v>Source: Nasdaq</v>
       <v>GMT</v>
-      <v>Real-Time Nasdaq Last Sale</v>
+      <v>Delayed 15 minutes</v>
       <v>from close</v>
       <v>from close</v>
     </spb>
@@ -16408,7 +16408,7 @@
       </c>
       <c r="F3" s="181">
         <f ca="1">Statement!AC143</f>
-        <v>4877837.17</v>
+        <v>4932785.92</v>
       </c>
       <c r="H3" s="179" t="str">
         <f>'AVG target price'!B5</f>
@@ -16416,7 +16416,7 @@
       </c>
       <c r="I3" s="205">
         <f ca="1">'AVG target price'!C5</f>
-        <v>112.5324096820578</v>
+        <v>113.07194781276988</v>
       </c>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.2">
@@ -16432,7 +16432,7 @@
       </c>
       <c r="F4" s="182">
         <f ca="1">Statement!AC144</f>
-        <v>4815664.17</v>
+        <v>4870612.92</v>
       </c>
       <c r="H4" s="179" t="str">
         <f>'AVG target price'!B6</f>
@@ -16440,7 +16440,7 @@
       </c>
       <c r="I4" s="205">
         <f ca="1">'AVG target price'!C6</f>
-        <v>228.29174889122544</v>
+        <v>228.66391288445607</v>
       </c>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.2">
@@ -16449,7 +16449,7 @@
       </c>
       <c r="C5" s="202" cm="1">
         <f t="array" aca="1" ref="C5" ca="1">_FV(C3,"Price",TRUE)</f>
-        <v>332.89</v>
+        <v>336.64</v>
       </c>
       <c r="E5" s="179" t="s">
         <v>237</v>
@@ -16464,7 +16464,7 @@
       </c>
       <c r="I5" s="205">
         <f ca="1">'AVG target price'!C7</f>
-        <v>199.8869501569128</v>
+        <v>200.25624214252309</v>
       </c>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.2">
@@ -16473,14 +16473,14 @@
       </c>
       <c r="C6" s="202" cm="1">
         <f t="array" aca="1" ref="C6" ca="1">_FV(C3,"Price (Extended hours)",TRUE)</f>
-        <v>332.89749999999998</v>
+        <v>336.05</v>
       </c>
       <c r="E6" s="179" t="s">
         <v>231</v>
       </c>
       <c r="F6" s="184">
         <f ca="1">Statement!AC140</f>
-        <v>38.175458715596335</v>
+        <v>38.60550458715597</v>
       </c>
       <c r="H6" s="179" t="str">
         <f>'AVG target price'!B8</f>
@@ -16488,7 +16488,7 @@
       </c>
       <c r="I6" s="205">
         <f ca="1">'AVG target price'!C8</f>
-        <v>198.50853359075884</v>
+        <v>198.82812827509545</v>
       </c>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.2">
@@ -16497,14 +16497,14 @@
       </c>
       <c r="C7" s="6" cm="1">
         <f t="array" aca="1" ref="C7" ca="1">_FV(C3,"Change")</f>
-        <v>-0.8</v>
+        <v>-3.78</v>
       </c>
       <c r="E7" s="180" t="s">
         <v>198</v>
       </c>
       <c r="F7" s="185">
         <f ca="1">Statement!AC141</f>
-        <v>10.53867972979052</v>
+        <v>10.657397771746464</v>
       </c>
       <c r="H7" s="179" t="str">
         <f>'AVG target price'!B9</f>
@@ -16512,7 +16512,7 @@
       </c>
       <c r="I7" s="205">
         <f ca="1">'AVG target price'!C9</f>
-        <v>212.45404502745629</v>
+        <v>212.79825444499096</v>
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
@@ -16521,14 +16521,14 @@
       </c>
       <c r="C8" s="6" cm="1">
         <f t="array" aca="1" ref="C8" ca="1">_FV(C3,"Change (extended hours)",TRUE)</f>
-        <v>7.4999999999999997E-3</v>
+        <v>-0.59</v>
       </c>
       <c r="E8" s="179" t="s">
         <v>259</v>
       </c>
       <c r="F8" s="186">
         <f ca="1">Statement!AC151</f>
-        <v>2.521137867338856E-2</v>
+        <v>2.4930536616517101E-2</v>
       </c>
       <c r="H8" s="178" t="str">
         <f>'AVG target price'!B10</f>
@@ -16536,7 +16536,7 @@
       </c>
       <c r="I8" s="206">
         <f ca="1">'AVG target price'!C10</f>
-        <v>190.33473746968221</v>
+        <v>190.72369711196706</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
@@ -16545,14 +16545,14 @@
       </c>
       <c r="C9" s="73" cm="1">
         <f t="array" aca="1" ref="C9" ca="1">_FV(C3,"Change (%)",TRUE)</f>
-        <v>-2.3969999999999998E-3</v>
+        <v>-1.1104000000000001E-2</v>
       </c>
       <c r="E9" s="179" t="s">
         <v>282</v>
       </c>
       <c r="F9" s="186">
         <f ca="1">Statement!AC152</f>
-        <v>2.6194839136050946E-2</v>
+        <v>2.5903041825095056E-2</v>
       </c>
       <c r="H9" s="178" t="str">
         <f>'AVG target price'!B12</f>
@@ -16560,7 +16560,7 @@
       </c>
       <c r="I9" s="207">
         <f ca="1">'AVG target price'!C12</f>
-        <v>-0.4282353405939433</v>
+        <v>-0.43344909365504081</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.2">
@@ -16569,14 +16569,14 @@
       </c>
       <c r="C10" s="73" cm="1">
         <f t="array" aca="1" ref="C10" ca="1">_FV(C3,"Change % (extended hours)",TRUE)</f>
-        <v>2.2529999999999999E-5</v>
+        <v>-1.7530000000000002E-3</v>
       </c>
       <c r="E10" s="179" t="s">
         <v>287</v>
       </c>
       <c r="F10" s="186">
         <f ca="1">Statement!AC154</f>
-        <v>1.68570612618461E-2</v>
+        <v>1.6669282092015052E-2</v>
       </c>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.2">
@@ -16592,14 +16592,14 @@
       </c>
       <c r="F11" s="187">
         <f ca="1">Statement!AC153</f>
-        <v>3.1541950794556762E-3</v>
+        <v>3.1190589353612169E-3</v>
       </c>
       <c r="H11" s="178" t="s">
         <v>394</v>
       </c>
       <c r="I11" s="206">
         <f ca="1">DDM!C26</f>
-        <v>13.039630248795358</v>
+        <v>13.10511393468445</v>
       </c>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.2">
@@ -16624,7 +16624,7 @@
       </c>
       <c r="C13" s="203" cm="1">
         <f t="array" aca="1" ref="C13" ca="1">_FV(C3,"Beta")</f>
-        <v>1.0795999999999999</v>
+        <v>1.0779000000000001</v>
       </c>
       <c r="E13" s="179" t="s">
         <v>101</v>
@@ -16647,7 +16647,7 @@
       </c>
       <c r="C14" s="204" cm="1">
         <f t="array" aca="1" ref="C14" ca="1">_FV(C3,"Volume average",TRUE)</f>
-        <v>41951159</v>
+        <v>40650930</v>
       </c>
       <c r="E14" s="180" t="s">
         <v>102</v>
@@ -16663,7 +16663,7 @@
       </c>
       <c r="F15" s="186">
         <f ca="1">Statement!AC166</f>
-        <v>1.2746017924169453E-2</v>
+        <v>1.2604033705967113E-2</v>
       </c>
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.2">
@@ -16773,7 +16773,7 @@
       </c>
       <c r="F26" s="213" cm="1">
         <f t="array" aca="1" ref="F26" ca="1">_FV(E26,"Price")</f>
-        <v>52.77</v>
+        <v>52.44</v>
       </c>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.2">
@@ -16788,7 +16788,7 @@
       </c>
       <c r="F27" s="214">
         <f ca="1">F26/1000</f>
-        <v>5.2770000000000004E-2</v>
+        <v>5.2440000000000001E-2</v>
       </c>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.2">
@@ -21049,6 +21049,12 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="H3:L3"/>
+    <mergeCell ref="P3:W3"/>
+    <mergeCell ref="X3:Z3"/>
+    <mergeCell ref="C5:L5"/>
+    <mergeCell ref="P5:Z5"/>
     <mergeCell ref="C40:L40"/>
     <mergeCell ref="C11:L11"/>
     <mergeCell ref="P11:Z11"/>
@@ -21056,12 +21062,6 @@
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="C26:L26"/>
     <mergeCell ref="C33:L33"/>
-    <mergeCell ref="C3:G3"/>
-    <mergeCell ref="H3:L3"/>
-    <mergeCell ref="P3:W3"/>
-    <mergeCell ref="X3:Z3"/>
-    <mergeCell ref="C5:L5"/>
-    <mergeCell ref="P5:Z5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -22121,16 +22121,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="AA2:AC2"/>
+    <mergeCell ref="C4:L4"/>
+    <mergeCell ref="S4:AC4"/>
+    <mergeCell ref="C13:L13"/>
+    <mergeCell ref="C18:L18"/>
     <mergeCell ref="C31:L31"/>
     <mergeCell ref="C25:L25"/>
     <mergeCell ref="C2:G2"/>
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="S2:Z2"/>
-    <mergeCell ref="AA2:AC2"/>
-    <mergeCell ref="C4:L4"/>
-    <mergeCell ref="S4:AC4"/>
-    <mergeCell ref="C13:L13"/>
-    <mergeCell ref="C18:L18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -22213,7 +22213,7 @@
       </c>
       <c r="C6" s="133">
         <f ca="1">Overview!C5</f>
-        <v>332.89</v>
+        <v>336.64</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22222,7 +22222,7 @@
       </c>
       <c r="C7" s="134">
         <f ca="1">C5*C6</f>
-        <v>4877837.17</v>
+        <v>4932785.92</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22240,7 +22240,7 @@
       </c>
       <c r="C9" s="135">
         <f ca="1">Overview!F27</f>
-        <v>5.2770000000000004E-2</v>
+        <v>5.2440000000000001E-2</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22249,7 +22249,7 @@
       </c>
       <c r="C10" s="133">
         <f ca="1">Overview!C13</f>
-        <v>1.0795999999999999</v>
+        <v>1.0779000000000001</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22292,7 +22292,7 @@
       </c>
       <c r="C16" s="46">
         <f ca="1">C8/(C8+C7)</f>
-        <v>1.6997364084552359E-2</v>
+        <v>1.6811205080373922E-2</v>
       </c>
     </row>
     <row r="17" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22301,7 +22301,7 @@
       </c>
       <c r="C17" s="46">
         <f ca="1">C7/(C8+C7)</f>
-        <v>0.98300263591544768</v>
+        <v>0.98318879491962607</v>
       </c>
     </row>
     <row r="18" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22319,7 +22319,7 @@
       </c>
       <c r="C19" s="46">
         <f ca="1">C9+C10*C11</f>
-        <v>0.101352</v>
+        <v>0.10094549999999999</v>
       </c>
     </row>
     <row r="20" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22328,7 +22328,7 @@
       </c>
       <c r="C20" s="46">
         <f ca="1">(C17*C19)+(C16*C18)</f>
-        <v>0.10028725111901547</v>
+        <v>9.9899246246220375E-2</v>
       </c>
     </row>
   </sheetData>
@@ -22579,7 +22579,7 @@
       </c>
       <c r="L8" s="126">
         <f ca="1">L7*(1+C14)/(C15-C14)</f>
-        <v>1805450.1385329245</v>
+        <v>1814217.7237637113</v>
       </c>
       <c r="N8" s="91"/>
       <c r="O8" s="16"/>
@@ -22633,23 +22633,23 @@
       <c r="G10" s="138"/>
       <c r="H10" s="126">
         <f ca="1">H7/(1+$C$15)^H9</f>
-        <v>100300.18591078027</v>
+        <v>100335.56820693916</v>
       </c>
       <c r="I10" s="126">
         <f t="shared" ref="I10:L10" ca="1" si="0">I7/(1+$C$15)^I9</f>
-        <v>96851.615699354021</v>
+        <v>96919.959281185322</v>
       </c>
       <c r="J10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>93005.410776455916</v>
+        <v>93103.872388012038</v>
       </c>
       <c r="K10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>88901.799185814481</v>
+        <v>89027.311002403832</v>
       </c>
       <c r="L10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>88125.483254749459</v>
+        <v>88281.030454872627</v>
       </c>
       <c r="N10" s="91"/>
     </row>
@@ -22668,7 +22668,7 @@
       <c r="K11" s="137"/>
       <c r="L11" s="126">
         <f ca="1">L8/(1+C15)^L9</f>
-        <v>1119579.904244039</v>
+        <v>1127002.5099671041</v>
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.2">
@@ -22691,7 +22691,7 @@
       </c>
       <c r="C15" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>0.10028725111901547</v>
+        <v>9.9899246246220375E-2</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.2">
@@ -22706,7 +22706,7 @@
       </c>
       <c r="C19" s="64">
         <f ca="1">SUM(H10:L10)</f>
-        <v>467184.49482715409</v>
+        <v>467667.74133341305</v>
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.2">
@@ -22715,7 +22715,7 @@
       </c>
       <c r="C20" s="64">
         <f ca="1">L11</f>
-        <v>1119579.904244039</v>
+        <v>1127002.5099671041</v>
       </c>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.2">
@@ -22724,7 +22724,7 @@
       </c>
       <c r="C21" s="94">
         <f ca="1">C19+C20</f>
-        <v>1586764.3990711931</v>
+        <v>1594670.251300517</v>
       </c>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.2">
@@ -22751,7 +22751,7 @@
       </c>
       <c r="C24" s="94">
         <f ca="1">C21+C22-C23</f>
-        <v>1648937.3990711931</v>
+        <v>1656843.251300517</v>
       </c>
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.2">
@@ -22769,7 +22769,7 @@
       </c>
       <c r="C26" s="235">
         <f ca="1">C24/C25</f>
-        <v>112.5324096820578</v>
+        <v>113.07194781276988</v>
       </c>
     </row>
   </sheetData>
@@ -23038,23 +23038,23 @@
       <c r="G9" s="138"/>
       <c r="H9" s="92">
         <f ca="1">DCF!H10</f>
-        <v>100300.18591078027</v>
+        <v>100335.56820693916</v>
       </c>
       <c r="I9" s="92">
         <f ca="1">DCF!I10</f>
-        <v>96851.615699354021</v>
+        <v>96919.959281185322</v>
       </c>
       <c r="J9" s="92">
         <f ca="1">DCF!J10</f>
-        <v>93005.410776455916</v>
+        <v>93103.872388012038</v>
       </c>
       <c r="K9" s="92">
         <f ca="1">DCF!K10</f>
-        <v>88901.799185814481</v>
+        <v>89027.311002403832</v>
       </c>
       <c r="L9" s="92">
         <f ca="1">DCF!L10</f>
-        <v>88125.483254749459</v>
+        <v>88281.030454872627</v>
       </c>
       <c r="N9" s="91"/>
     </row>
@@ -23840,7 +23840,7 @@
       </c>
       <c r="C41" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>0.10028725111901547</v>
+        <v>9.9899246246220375E-2</v>
       </c>
     </row>
     <row r="42" spans="2:14" x14ac:dyDescent="0.2">
@@ -23866,7 +23866,7 @@
       </c>
       <c r="C44" s="24">
         <f ca="1">C43/(1+C41)^5</f>
-        <v>2903926.9849307216</v>
+        <v>2909052.6046173945</v>
       </c>
     </row>
     <row r="45" spans="2:14" x14ac:dyDescent="0.2">
@@ -23875,7 +23875,7 @@
       </c>
       <c r="C45" s="108">
         <f ca="1">SUM(H9:K9)+C44</f>
-        <v>3282985.9965031263</v>
+        <v>3288439.3154959348</v>
       </c>
     </row>
     <row r="46" spans="2:14" x14ac:dyDescent="0.2">
@@ -23902,7 +23902,7 @@
       </c>
       <c r="C48" s="94">
         <f ca="1">C45+C46-C47</f>
-        <v>3345158.9965031263</v>
+        <v>3350612.3154959348</v>
       </c>
     </row>
     <row r="49" spans="2:3" x14ac:dyDescent="0.2">
@@ -23920,7 +23920,7 @@
       </c>
       <c r="C50" s="235">
         <f ca="1">C48/C49</f>
-        <v>228.29174889122544</v>
+        <v>228.66391288445607</v>
       </c>
     </row>
     <row r="52" spans="2:3" x14ac:dyDescent="0.2">
@@ -23944,7 +23944,7 @@
       </c>
       <c r="C54" s="135">
         <f ca="1">IF(Overview!C29&gt;0,Overview!C29,WACC!C19)</f>
-        <v>0.101352</v>
+        <v>0.10094549999999999</v>
       </c>
     </row>
     <row r="55" spans="2:3" x14ac:dyDescent="0.2">
@@ -23979,7 +23979,7 @@
       </c>
       <c r="C58" s="235">
         <f ca="1">C57/(1+C54)^5</f>
-        <v>199.8869501569128</v>
+        <v>200.25624214252309</v>
       </c>
     </row>
     <row r="60" spans="2:3" x14ac:dyDescent="0.2">
@@ -24003,7 +24003,7 @@
       </c>
       <c r="C62" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>0.10028725111901547</v>
+        <v>9.9899246246220375E-2</v>
       </c>
     </row>
     <row r="63" spans="2:3" x14ac:dyDescent="0.2">
@@ -24029,7 +24029,7 @@
       </c>
       <c r="C65" s="24">
         <f ca="1">C64/(1+C62)^5</f>
-        <v>2467513.5311329844</v>
+        <v>2471868.8527364335</v>
       </c>
     </row>
     <row r="66" spans="2:3" x14ac:dyDescent="0.2">
@@ -24038,7 +24038,7 @@
       </c>
       <c r="C66" s="108">
         <f ca="1">SUM(H9:K9)+C65</f>
-        <v>2846572.5427053892</v>
+        <v>2851255.5636149738</v>
       </c>
     </row>
     <row r="67" spans="2:3" x14ac:dyDescent="0.2">
@@ -24065,7 +24065,7 @@
       </c>
       <c r="C69" s="94">
         <f ca="1">C66+C67-C68</f>
-        <v>2908745.5427053892</v>
+        <v>2913428.5636149738</v>
       </c>
     </row>
     <row r="70" spans="2:3" x14ac:dyDescent="0.2">
@@ -24083,7 +24083,7 @@
       </c>
       <c r="C71" s="235">
         <f ca="1">C69/C70</f>
-        <v>198.50853359075884</v>
+        <v>198.82812827509545</v>
       </c>
     </row>
     <row r="73" spans="2:3" x14ac:dyDescent="0.2">
@@ -24107,7 +24107,7 @@
       </c>
       <c r="C75" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>0.10028725111901547</v>
+        <v>9.9899246246220375E-2</v>
       </c>
     </row>
     <row r="76" spans="2:3" x14ac:dyDescent="0.2">
@@ -24133,7 +24133,7 @@
       </c>
       <c r="C78" s="24">
         <f ca="1">C77/(1+C75)^5</f>
-        <v>2671857.1102149123</v>
+        <v>2676573.1115039121</v>
       </c>
     </row>
     <row r="79" spans="2:3" x14ac:dyDescent="0.2">
@@ -24142,7 +24142,7 @@
       </c>
       <c r="C79" s="108">
         <f ca="1">SUM(H9:K9)+C78</f>
-        <v>3050916.1217873171</v>
+        <v>3055959.8223824524</v>
       </c>
     </row>
     <row r="80" spans="2:3" x14ac:dyDescent="0.2">
@@ -24169,7 +24169,7 @@
       </c>
       <c r="C82" s="94">
         <f ca="1">C79+C80-C81</f>
-        <v>3113089.1217873171</v>
+        <v>3118132.8223824524</v>
       </c>
     </row>
     <row r="83" spans="2:3" x14ac:dyDescent="0.2">
@@ -24187,22 +24187,22 @@
       </c>
       <c r="C84" s="235">
         <f ca="1">C82/C83</f>
-        <v>212.45404502745629</v>
+        <v>212.79825444499096</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="B73:C73"/>
+    <mergeCell ref="C27:L27"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="B60:C60"/>
     <mergeCell ref="C22:L22"/>
     <mergeCell ref="C2:G2"/>
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="C4:L4"/>
     <mergeCell ref="C11:L11"/>
     <mergeCell ref="C17:L17"/>
-    <mergeCell ref="B73:C73"/>
-    <mergeCell ref="C27:L27"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="B60:C60"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -24252,7 +24252,7 @@
       </c>
       <c r="C5" s="133">
         <f ca="1">DCF!C26</f>
-        <v>112.5324096820578</v>
+        <v>113.07194781276988</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -24261,7 +24261,7 @@
       </c>
       <c r="C6" s="133">
         <f ca="1">Multiples!C50</f>
-        <v>228.29174889122544</v>
+        <v>228.66391288445607</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
@@ -24270,7 +24270,7 @@
       </c>
       <c r="C7" s="133">
         <f ca="1">Multiples!C58</f>
-        <v>199.8869501569128</v>
+        <v>200.25624214252309</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
@@ -24279,7 +24279,7 @@
       </c>
       <c r="C8" s="133">
         <f ca="1">Multiples!C71</f>
-        <v>198.50853359075884</v>
+        <v>198.82812827509545</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
@@ -24288,7 +24288,7 @@
       </c>
       <c r="C9" s="133">
         <f ca="1">Multiples!C84</f>
-        <v>212.45404502745629</v>
+        <v>212.79825444499096</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
@@ -24297,7 +24297,7 @@
       </c>
       <c r="C10" s="235">
         <f ca="1">AVERAGE(C5:C9)</f>
-        <v>190.33473746968221</v>
+        <v>190.72369711196706</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
@@ -24306,7 +24306,7 @@
       </c>
       <c r="C11" s="133">
         <f ca="1">Overview!C5</f>
-        <v>332.89</v>
+        <v>336.64</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.2">
@@ -24315,7 +24315,7 @@
       </c>
       <c r="C12" s="149">
         <f ca="1">(C10-C11)/C11</f>
-        <v>-0.4282353405939433</v>
+        <v>-0.43344909365504081</v>
       </c>
     </row>
   </sheetData>
@@ -24785,7 +24785,7 @@
       </c>
       <c r="C24" s="135">
         <f ca="1">IF(Overview!C29&gt;0,Overview!C29,WACC!C19)</f>
-        <v>0.101352</v>
+        <v>0.10094549999999999</v>
       </c>
     </row>
     <row r="25" spans="2:14" x14ac:dyDescent="0.2">
@@ -24802,7 +24802,7 @@
       </c>
       <c r="C26" s="235">
         <f ca="1">C23/(C24-C25)</f>
-        <v>13.039630248795358</v>
+        <v>13.10511393468445</v>
       </c>
     </row>
   </sheetData>
@@ -25039,7 +25039,7 @@
       <c r="K8" s="137"/>
       <c r="L8" s="126">
         <f ca="1">L7*(1+C20)/(C21-C20)</f>
-        <v>6216770.4299511006</v>
+        <v>6246960.166815904</v>
       </c>
       <c r="N8" s="91"/>
       <c r="O8" s="16"/>
@@ -25093,23 +25093,23 @@
       <c r="G10" s="138"/>
       <c r="H10" s="126">
         <f ca="1">H7/(1+$C$21)^H9</f>
-        <v>110937.76366467061</v>
+        <v>110976.89851545423</v>
       </c>
       <c r="I10" s="126">
         <f t="shared" ref="I10:L10" ca="1" si="1">I7/(1+$C$21)^I9</f>
-        <v>142669.04885597836</v>
+        <v>142769.72362268073</v>
       </c>
       <c r="J10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>183476.36394577549</v>
+        <v>183670.60402627985</v>
       </c>
       <c r="K10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>235955.70585702444</v>
+        <v>236288.82880333104</v>
       </c>
       <c r="L10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>303445.59881806257</v>
+        <v>303981.20000335656</v>
       </c>
       <c r="N10" s="91"/>
     </row>
@@ -25128,15 +25128,15 @@
       <c r="K11" s="137"/>
       <c r="L11" s="126">
         <f ca="1">L8/(1+C21)^L9</f>
-        <v>3855089.1515218099</v>
+        <v>3880647.672794424</v>
       </c>
     </row>
     <row r="13" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="14" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="B14" s="251" t="s">
+      <c r="B14" s="252" t="s">
         <v>219</v>
       </c>
-      <c r="C14" s="252"/>
+      <c r="C14" s="253"/>
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B15" s="150" t="s">
@@ -25144,7 +25144,7 @@
       </c>
       <c r="C15" s="151">
         <f ca="1">Overview!C5</f>
-        <v>332.89</v>
+        <v>336.64</v>
       </c>
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.2">
@@ -25153,7 +25153,7 @@
       </c>
       <c r="C16" s="151">
         <f ca="1">C36</f>
-        <v>335.3259307018858</v>
+        <v>337.15964970299615</v>
       </c>
     </row>
     <row r="17" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -25163,20 +25163,20 @@
       <c r="C17" s="153">
         <v>0.41499999999999998</v>
       </c>
-      <c r="E17" s="253" t="s">
+      <c r="E17" s="251" t="s">
         <v>222</v>
       </c>
-      <c r="F17" s="253"/>
-      <c r="G17" s="253"/>
-      <c r="H17" s="253"/>
-      <c r="I17" s="253"/>
+      <c r="F17" s="251"/>
+      <c r="G17" s="251"/>
+      <c r="H17" s="251"/>
+      <c r="I17" s="251"/>
     </row>
     <row r="18" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B19" s="251" t="s">
+      <c r="B19" s="252" t="s">
         <v>181</v>
       </c>
-      <c r="C19" s="252"/>
+      <c r="C19" s="253"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B20" s="154" t="s">
@@ -25192,7 +25192,7 @@
       </c>
       <c r="C21" s="216">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>0.10028725111901547</v>
+        <v>9.9899246246220375E-2</v>
       </c>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.2">
@@ -25210,7 +25210,7 @@
       </c>
       <c r="C23" s="156">
         <f ca="1">C15*C22</f>
-        <v>4858196.66</v>
+        <v>4912924.16</v>
       </c>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.2">
@@ -25237,15 +25237,15 @@
       </c>
       <c r="C26" s="157">
         <f ca="1">C23+C25-C24</f>
-        <v>4796023.66</v>
+        <v>4850751.16</v>
       </c>
     </row>
     <row r="27" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="28" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B28" s="251" t="s">
+      <c r="B28" s="252" t="s">
         <v>183</v>
       </c>
-      <c r="C28" s="252"/>
+      <c r="C28" s="253"/>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B29" s="154" t="s">
@@ -25253,7 +25253,7 @@
       </c>
       <c r="C29" s="156">
         <f ca="1">SUM(H10:L10)</f>
-        <v>976484.48114151147</v>
+        <v>977687.25497110235</v>
       </c>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
@@ -25262,7 +25262,7 @@
       </c>
       <c r="C30" s="156">
         <f ca="1">L11</f>
-        <v>3855089.1515218099</v>
+        <v>3880647.672794424</v>
       </c>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.2">
@@ -25271,7 +25271,7 @@
       </c>
       <c r="C31" s="159">
         <f ca="1">C29+C30</f>
-        <v>4831573.6326633217</v>
+        <v>4858334.9277655259</v>
       </c>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.2">
@@ -25298,7 +25298,7 @@
       </c>
       <c r="C34" s="159">
         <f ca="1">C31+C32-C33</f>
-        <v>4893746.6326633217</v>
+        <v>4920507.9277655259</v>
       </c>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.2">
@@ -25316,21 +25316,21 @@
       </c>
       <c r="C36" s="162">
         <f ca="1">C34/C35</f>
-        <v>335.3259307018858</v>
+        <v>337.15964970299615</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="P3:W3"/>
+    <mergeCell ref="X3:Z3"/>
+    <mergeCell ref="C5:L5"/>
+    <mergeCell ref="P5:Z5"/>
+    <mergeCell ref="B14:C14"/>
     <mergeCell ref="E17:I17"/>
     <mergeCell ref="B19:C19"/>
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="C3:G3"/>
     <mergeCell ref="H3:L3"/>
-    <mergeCell ref="P3:W3"/>
-    <mergeCell ref="X3:Z3"/>
-    <mergeCell ref="C5:L5"/>
-    <mergeCell ref="P5:Z5"/>
-    <mergeCell ref="B14:C14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -31835,7 +31835,7 @@
       </c>
       <c r="AC114" s="63">
         <f ca="1">Overview!C5</f>
-        <v>332.89</v>
+        <v>336.64</v>
       </c>
     </row>
     <row r="115" spans="1:31" x14ac:dyDescent="0.2">
@@ -31906,7 +31906,7 @@
       </c>
       <c r="AC115" s="65">
         <f ca="1">AC114/AC84</f>
-        <v>332.89</v>
+        <v>336.64</v>
       </c>
     </row>
     <row r="117" spans="1:31" x14ac:dyDescent="0.2">
@@ -32820,7 +32820,7 @@
       <c r="AA140" s="49"/>
       <c r="AC140" s="72">
         <f ca="1">AC115/Statement!AC25</f>
-        <v>38.175458715596335</v>
+        <v>38.60550458715597</v>
       </c>
     </row>
     <row r="141" spans="2:29" x14ac:dyDescent="0.2">
@@ -32857,7 +32857,7 @@
       <c r="AA141" s="49"/>
       <c r="AC141" s="72">
         <f ca="1">AC115/(Statement!AC5/Statement!AC21)</f>
-        <v>10.53867972979052</v>
+        <v>10.657397771746464</v>
       </c>
     </row>
     <row r="142" spans="2:29" x14ac:dyDescent="0.2">
@@ -32918,7 +32918,7 @@
       </c>
       <c r="AC142" s="72">
         <f ca="1">AC115/(Statement!AC48/Statement!AC74)</f>
-        <v>45.184120721726188</v>
+        <v>45.693119047619042</v>
       </c>
     </row>
     <row r="143" spans="2:29" x14ac:dyDescent="0.2">
@@ -32979,7 +32979,7 @@
       </c>
       <c r="AC143" s="141">
         <f ca="1">Statement!AC115*Statement!AC77</f>
-        <v>4877837.17</v>
+        <v>4932785.92</v>
       </c>
     </row>
     <row r="144" spans="2:29" x14ac:dyDescent="0.2">
@@ -33040,7 +33040,7 @@
       </c>
       <c r="AC144" s="141">
         <f ca="1">AC143+AC106-AC105+AC47+AC44</f>
-        <v>4815664.17</v>
+        <v>4870612.92</v>
       </c>
     </row>
     <row r="145" spans="2:29" x14ac:dyDescent="0.2">
@@ -33077,7 +33077,7 @@
       <c r="AA145" s="49"/>
       <c r="AC145" s="177">
         <f ca="1">AC144/AC5</f>
-        <v>10.31582456305709</v>
+        <v>10.433532452342751</v>
       </c>
     </row>
     <row r="146" spans="2:29" x14ac:dyDescent="0.2">
@@ -33114,7 +33114,7 @@
       <c r="AA146" s="49"/>
       <c r="AC146" s="177">
         <f ca="1">AC144/AC11</f>
-        <v>31.097089416824335</v>
+        <v>31.451920262948875</v>
       </c>
     </row>
     <row r="147" spans="2:29" x14ac:dyDescent="0.2">
@@ -33249,7 +33249,7 @@
       <c r="AA149" s="49"/>
       <c r="AC149" s="72">
         <f t="shared" ref="AC149:AC150" ca="1" si="137">AC143/AC147</f>
-        <v>39.664629727510018</v>
+        <v>40.111451084349106</v>
       </c>
     </row>
     <row r="150" spans="2:29" x14ac:dyDescent="0.2">
@@ -33286,7 +33286,7 @@
       <c r="AA150" s="49"/>
       <c r="AC150" s="72">
         <f t="shared" ca="1" si="137"/>
-        <v>39.31502334466186</v>
+        <v>39.763624267140635</v>
       </c>
     </row>
     <row r="151" spans="2:29" x14ac:dyDescent="0.2">
@@ -33323,7 +33323,7 @@
       <c r="AA151" s="49"/>
       <c r="AC151" s="74">
         <f t="shared" ref="AC151" ca="1" si="140">AC147/AC143</f>
-        <v>2.521137867338856E-2</v>
+        <v>2.4930536616517101E-2</v>
       </c>
     </row>
     <row r="152" spans="2:29" x14ac:dyDescent="0.2">
@@ -33360,7 +33360,7 @@
       <c r="AA152" s="49"/>
       <c r="AC152" s="74">
         <f ca="1">AC25/AC115</f>
-        <v>2.6194839136050946E-2</v>
+        <v>2.5903041825095056E-2</v>
       </c>
     </row>
     <row r="153" spans="2:29" x14ac:dyDescent="0.2">
@@ -33397,7 +33397,7 @@
       <c r="AA153" s="49"/>
       <c r="AC153" s="149">
         <f ca="1">AC81/AC115</f>
-        <v>3.1541950794556762E-3</v>
+        <v>3.1190589353612169E-3</v>
       </c>
     </row>
     <row r="154" spans="2:29" x14ac:dyDescent="0.2">
@@ -33434,7 +33434,7 @@
       <c r="AA154" s="49"/>
       <c r="AC154" s="149">
         <f ca="1">-AC62/AC143</f>
-        <v>1.68570612618461E-2</v>
+        <v>1.6669282092015052E-2</v>
       </c>
     </row>
     <row r="155" spans="2:29" x14ac:dyDescent="0.2">
@@ -33471,7 +33471,7 @@
       <c r="AA155" s="49"/>
       <c r="AC155" s="149">
         <f ca="1">-(AC62+AC63)/AC143</f>
-        <v>2.0063400353316836E-2</v>
+        <v>1.9839904181367756E-2</v>
       </c>
     </row>
     <row r="156" spans="2:29" x14ac:dyDescent="0.2">
@@ -33974,7 +33974,7 @@
       <c r="AA166" s="49"/>
       <c r="AC166" s="149">
         <f ca="1">(AC105-AC106)/AC143</f>
-        <v>1.2746017924169453E-2</v>
+        <v>1.2604033705967113E-2</v>
       </c>
     </row>
     <row r="167" spans="1:31" x14ac:dyDescent="0.2">
@@ -35987,7 +35987,7 @@
       </c>
       <c r="C5" s="166">
         <f ca="1">Overview!C5</f>
-        <v>332.89</v>
+        <v>336.64</v>
       </c>
       <c r="E5" s="12"/>
       <c r="F5" s="132" t="s">
@@ -36003,7 +36003,7 @@
       </c>
       <c r="C6" s="167">
         <f ca="1">Statement!AC143</f>
-        <v>4877837.17</v>
+        <v>4932785.92</v>
       </c>
       <c r="E6" s="20" t="s">
         <v>19</v>
@@ -36023,7 +36023,7 @@
       </c>
       <c r="C7" s="167">
         <f ca="1">Statement!AC144</f>
-        <v>4815664.17</v>
+        <v>4870612.92</v>
       </c>
       <c r="E7" s="20" t="s">
         <v>29</v>
@@ -36043,7 +36043,7 @@
       </c>
       <c r="C8" s="168">
         <f ca="1">Statement!AC140</f>
-        <v>38.175458715596335</v>
+        <v>38.60550458715597</v>
       </c>
       <c r="E8" s="20" t="s">
         <v>237</v>
@@ -36063,7 +36063,7 @@
       </c>
       <c r="C9" s="168">
         <f ca="1">Statement!AC141</f>
-        <v>10.53867972979052</v>
+        <v>10.657397771746464</v>
       </c>
       <c r="E9" s="20" t="s">
         <v>238</v>
@@ -36083,7 +36083,7 @@
       </c>
       <c r="C10" s="168">
         <f ca="1">Statement!AC142</f>
-        <v>45.184120721726188</v>
+        <v>45.693119047619042</v>
       </c>
       <c r="E10" s="20" t="s">
         <v>1</v>
@@ -36103,7 +36103,7 @@
       </c>
       <c r="C11" s="168">
         <f ca="1">Statement!AC145</f>
-        <v>10.31582456305709</v>
+        <v>10.433532452342751</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.2">
@@ -36112,7 +36112,7 @@
       </c>
       <c r="C12" s="168">
         <f ca="1">Statement!AC146</f>
-        <v>31.097089416824335</v>
+        <v>31.451920262948875</v>
       </c>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.2">
@@ -36348,7 +36348,7 @@
       </c>
       <c r="C38" s="169">
         <f ca="1">Statement!AC152</f>
-        <v>2.6194839136050946E-2</v>
+        <v>2.5903041825095056E-2</v>
       </c>
       <c r="E38" s="20" t="s">
         <v>264</v>
@@ -36364,7 +36364,7 @@
       </c>
       <c r="C39" s="209">
         <f ca="1">Statement!AC151</f>
-        <v>2.521137867338856E-2</v>
+        <v>2.4930536616517101E-2</v>
       </c>
       <c r="E39" s="20" t="s">
         <v>266</v>
@@ -36380,7 +36380,7 @@
       </c>
       <c r="C40" s="169">
         <f ca="1">Statement!AC153</f>
-        <v>3.1541950794556762E-3</v>
+        <v>3.1190589353612169E-3</v>
       </c>
       <c r="E40" s="20" t="s">
         <v>267</v>
@@ -36396,7 +36396,7 @@
       </c>
       <c r="C41" s="169">
         <f ca="1">Statement!AC154</f>
-        <v>1.68570612618461E-2</v>
+        <v>1.6669282092015052E-2</v>
       </c>
     </row>
     <row r="42" spans="2:6" x14ac:dyDescent="0.2">
@@ -36405,7 +36405,7 @@
       </c>
       <c r="C42" s="169">
         <f ca="1">Statement!AC155</f>
-        <v>2.0063400353316836E-2</v>
+        <v>1.9839904181367756E-2</v>
       </c>
     </row>
     <row r="45" spans="2:6" x14ac:dyDescent="0.2">
@@ -36449,7 +36449,7 @@
       </c>
       <c r="F48" s="169">
         <f ca="1">Statement!AC166</f>
-        <v>1.2746017924169453E-2</v>
+        <v>1.2604033705967113E-2</v>
       </c>
     </row>
     <row r="51" spans="2:6" x14ac:dyDescent="0.2">
@@ -36628,7 +36628,7 @@
       </c>
       <c r="I6" s="166">
         <f ca="1">Statement!AC114</f>
-        <v>332.89</v>
+        <v>336.64</v>
       </c>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.2">
@@ -36657,7 +36657,7 @@
       </c>
       <c r="I7" s="167">
         <f ca="1">Statement!AC143</f>
-        <v>4877837.17</v>
+        <v>4932785.92</v>
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
@@ -36686,7 +36686,7 @@
       </c>
       <c r="I8" s="167">
         <f ca="1">Statement!AC144</f>
-        <v>4815664.17</v>
+        <v>4870612.92</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
@@ -36715,7 +36715,7 @@
       </c>
       <c r="I9" s="168">
         <f ca="1">Statement!AC140</f>
-        <v>38.175458715596335</v>
+        <v>38.60550458715597</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.2">
@@ -36744,7 +36744,7 @@
       </c>
       <c r="I10" s="168">
         <f ca="1">Statement!AC141</f>
-        <v>10.53867972979052</v>
+        <v>10.657397771746464</v>
       </c>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.2">
@@ -36773,7 +36773,7 @@
       </c>
       <c r="I11" s="168">
         <f ca="1">Statement!AC142</f>
-        <v>45.184120721726188</v>
+        <v>45.693119047619042</v>
       </c>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.2">
@@ -36802,7 +36802,7 @@
       </c>
       <c r="I12" s="168">
         <f ca="1">Statement!AC145</f>
-        <v>10.31582456305709</v>
+        <v>10.433532452342751</v>
       </c>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
@@ -36831,7 +36831,7 @@
       </c>
       <c r="I13" s="168">
         <f ca="1">Statement!AC146</f>
-        <v>31.097089416824335</v>
+        <v>31.451920262948875</v>
       </c>
     </row>
     <row r="15" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -37604,7 +37604,7 @@
       </c>
       <c r="I51" s="169">
         <f ca="1">Statement!AC152</f>
-        <v>2.6194839136050946E-2</v>
+        <v>2.5903041825095056E-2</v>
       </c>
     </row>
     <row r="52" spans="2:9" x14ac:dyDescent="0.2">
@@ -37633,7 +37633,7 @@
       </c>
       <c r="I52" s="169">
         <f ca="1">Statement!AC151</f>
-        <v>2.521137867338856E-2</v>
+        <v>2.4930536616517101E-2</v>
       </c>
     </row>
     <row r="53" spans="2:9" x14ac:dyDescent="0.2">
@@ -37662,7 +37662,7 @@
       </c>
       <c r="I53" s="169">
         <f ca="1">Statement!AC153</f>
-        <v>3.1541950794556762E-3</v>
+        <v>3.1190589353612169E-3</v>
       </c>
     </row>
     <row r="54" spans="2:9" x14ac:dyDescent="0.2">
@@ -37691,7 +37691,7 @@
       </c>
       <c r="I54" s="169">
         <f ca="1">Statement!AC154</f>
-        <v>1.68570612618461E-2</v>
+        <v>1.6669282092015052E-2</v>
       </c>
     </row>
     <row r="55" spans="2:9" x14ac:dyDescent="0.2">
@@ -37720,7 +37720,7 @@
       </c>
       <c r="I55" s="169">
         <f ca="1">Statement!AC155</f>
-        <v>2.0063400353316836E-2</v>
+        <v>1.9839904181367756E-2</v>
       </c>
     </row>
     <row r="57" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -37956,7 +37956,7 @@
       </c>
       <c r="I68" s="190">
         <f ca="1">Statement!AC166</f>
-        <v>1.2746017924169453E-2</v>
+        <v>1.2604033705967113E-2</v>
       </c>
     </row>
     <row r="70" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -38648,14 +38648,14 @@
     <row r="1" spans="2:7" ht="12" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="3" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B3" s="8"/>
-      <c r="C3" s="240" t="s">
+      <c r="C3" s="242" t="s">
         <v>307</v>
       </c>
-      <c r="D3" s="241"/>
-      <c r="F3" s="242" t="s">
+      <c r="D3" s="243"/>
+      <c r="F3" s="244" t="s">
         <v>308</v>
       </c>
-      <c r="G3" s="241"/>
+      <c r="G3" s="243"/>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B4" s="8"/>
@@ -38722,19 +38722,19 @@
       <c r="B7" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C7" s="243">
+      <c r="C7" s="240">
         <f>Statement!AA88</f>
         <v>-1.5892574471146927E-2</v>
       </c>
-      <c r="D7" s="244"/>
-      <c r="F7" s="243">
+      <c r="D7" s="241"/>
+      <c r="F7" s="240">
         <f>IF(F6=0,
 IF(G6=0,0,IF(G6&gt;0,1,-1)),
 (G6-F6)/ABS(F6)
 )</f>
         <v>0.16356501765281381</v>
       </c>
-      <c r="G7" s="244"/>
+      <c r="G7" s="241"/>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B8" s="201" t="s">
@@ -38761,19 +38761,19 @@
       <c r="B9" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C9" s="243">
+      <c r="C9" s="240">
         <f>Statement!AA89</f>
         <v>-3.1133095757317875E-2</v>
       </c>
-      <c r="D9" s="244"/>
-      <c r="F9" s="243">
+      <c r="D9" s="241"/>
+      <c r="F9" s="240">
         <f>IF(F8=0,
 IF(G8=0,0,IF(G8&gt;0,1,-1)),
 (G8-F8)/ABS(F8)
 )</f>
         <v>8.6032831193608647E-2</v>
       </c>
-      <c r="G9" s="244"/>
+      <c r="G9" s="241"/>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B10" s="201" t="s">
@@ -38800,19 +38800,19 @@
       <c r="B11" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C11" s="243">
+      <c r="C11" s="240">
         <f>Statement!AA90</f>
         <v>-2.0079954728829339E-4</v>
       </c>
-      <c r="D11" s="244"/>
-      <c r="F11" s="243">
+      <c r="D11" s="241"/>
+      <c r="F11" s="240">
         <f>IF(F10=0,
 IF(G10=0,0,IF(G10&gt;0,1,-1)),
 (G10-F10)/ABS(F10)
 )</f>
         <v>0.25280204949906215</v>
       </c>
-      <c r="G11" s="244"/>
+      <c r="G11" s="241"/>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B12" s="201" t="s">
@@ -38839,19 +38839,19 @@
       <c r="B13" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C13" s="243">
+      <c r="C13" s="240">
         <f>Statement!AA93</f>
         <v>9.4729043183742583E-3</v>
       </c>
-      <c r="D13" s="244"/>
-      <c r="F13" s="243">
+      <c r="D13" s="241"/>
+      <c r="F13" s="240">
         <f>IF(F12=0,
 IF(G12=0,0,IF(G12&gt;0,1,-1)),
 (G12-F12)/ABS(F12)
 )</f>
         <v>0.22937612786800721</v>
       </c>
-      <c r="G13" s="244"/>
+      <c r="G13" s="241"/>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B14" s="201" t="s">
@@ -38878,19 +38878,19 @@
       <c r="B15" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C15" s="243">
+      <c r="C15" s="240">
         <f>Statement!AA94</f>
         <v>-5.2946913752264175E-3</v>
       </c>
-      <c r="D15" s="244"/>
-      <c r="F15" s="243">
+      <c r="D15" s="241"/>
+      <c r="F15" s="240">
         <f>IF(F14=0,
 IF(G14=0,0,IF(G14&gt;0,1,-1)),
 (G14-F14)/ABS(F14)
 )</f>
         <v>0.26569037656903766</v>
       </c>
-      <c r="G15" s="244"/>
+      <c r="G15" s="241"/>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B16" s="201" t="s">
@@ -38917,19 +38917,19 @@
       <c r="B17" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C17" s="243">
+      <c r="C17" s="240">
         <f>Statement!AA96</f>
         <v>7.1336804381635002E-3</v>
       </c>
-      <c r="D17" s="244"/>
-      <c r="F17" s="243">
+      <c r="D17" s="241"/>
+      <c r="F17" s="240">
         <f>IF(F16=0,
 IF(G16=0,0,IF(G16&gt;0,1,-1)),
 (G16-F16)/ABS(F16)
 )</f>
         <v>0.27118716394981651</v>
       </c>
-      <c r="G17" s="244"/>
+      <c r="G17" s="241"/>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B18" s="201" t="s">
@@ -38956,22 +38956,22 @@
       <c r="B19" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C19" s="243">
+      <c r="C19" s="240">
         <f>IF(C18=0,
 IF(D18=0,0,IF(D18&gt;0,1,-1)),
 (D18-C18)/ABS(C18)
 )</f>
         <v>-7.4697813391280731E-4</v>
       </c>
-      <c r="D19" s="244"/>
-      <c r="F19" s="243">
+      <c r="D19" s="241"/>
+      <c r="F19" s="240">
         <f>IF(F18=0,
 IF(G18=0,0,IF(G18&gt;0,1,-1)),
 (G18-F18)/ABS(F18)
 )</f>
         <v>-1.5587369547765587E-2</v>
       </c>
-      <c r="G19" s="244"/>
+      <c r="G19" s="241"/>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B20" s="201" t="s">
@@ -38998,22 +38998,22 @@
       <c r="B21" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C21" s="243">
+      <c r="C21" s="240">
         <f>IF(C20=0,
 IF(D20=0,0,IF(D20&gt;0,1,-1)),
 (D20-C20)/ABS(C20)
 )</f>
         <v>4.975124378109568E-3</v>
       </c>
-      <c r="D21" s="244"/>
-      <c r="F21" s="243">
+      <c r="D21" s="241"/>
+      <c r="F21" s="240">
         <f>IF(F20=0,
 IF(G20=0,0,IF(G20&gt;0,1,-1)),
 (G20-F20)/ABS(F20)
 )</f>
         <v>0.28662420382165599</v>
       </c>
-      <c r="G21" s="244"/>
+      <c r="G21" s="241"/>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23" s="8" t="s">
@@ -39061,22 +39061,22 @@
       <c r="B25" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C25" s="243">
+      <c r="C25" s="240">
         <f>IF(C24=0,
 IF(D24=0,0,IF(D24&gt;0,1,-1)),
 (D24-C24)/ABS(C24)
 )</f>
         <v>1.5257357017718937E-2</v>
       </c>
-      <c r="D25" s="244"/>
-      <c r="F25" s="243">
+      <c r="D25" s="241"/>
+      <c r="F25" s="240">
         <f>IF(F24=0,
 IF(G24=0,0,IF(G24&gt;0,1,-1)),
 (G24-F24)/ABS(F24)
 )</f>
         <v>0.11124326423612797</v>
       </c>
-      <c r="G25" s="244"/>
+      <c r="G25" s="241"/>
     </row>
     <row r="26" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B26" s="20" t="s">
@@ -39103,22 +39103,22 @@
       <c r="B27" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C27" s="243">
+      <c r="C27" s="240">
         <f>IF(C26=0,
 IF(D26=0,0,IF(D26&gt;0,1,-1)),
 (D26-C26)/ABS(C26)
 )</f>
         <v>4.7692033505613969E-2</v>
       </c>
-      <c r="D27" s="244"/>
-      <c r="F27" s="243">
+      <c r="D27" s="241"/>
+      <c r="F27" s="240">
         <f>IF(F26=0,
 IF(G26=0,0,IF(G26&gt;0,1,-1)),
 (G26-F26)/ABS(F26)
 )</f>
         <v>0.22399433663696178</v>
       </c>
-      <c r="G27" s="244"/>
+      <c r="G27" s="241"/>
     </row>
     <row r="28" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B28" s="20" t="s">
@@ -39145,22 +39145,22 @@
       <c r="B29" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C29" s="243">
+      <c r="C29" s="240">
         <f>IF(C28=0,
 IF(D28=0,0,IF(D28&gt;0,1,-1)),
 (D28-C28)/ABS(C28)
 )</f>
         <v>-8.2012001756354591E-2</v>
       </c>
-      <c r="D29" s="244"/>
-      <c r="F29" s="243">
+      <c r="D29" s="241"/>
+      <c r="F29" s="240">
         <f>IF(F28=0,
 IF(G28=0,0,IF(G28&gt;0,1,-1)),
 (G28-F28)/ABS(F28)
 )</f>
         <v>0.22428264688658989</v>
       </c>
-      <c r="G29" s="244"/>
+      <c r="G29" s="241"/>
     </row>
     <row r="30" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B30" s="20" t="s">
@@ -39187,22 +39187,22 @@
       <c r="B31" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C31" s="243">
+      <c r="C31" s="240">
         <f>IF(C30=0,
 IF(D30=0,0,IF(D30&gt;0,1,-1)),
 (D30-C30)/ABS(C30)
 )</f>
         <v>-0.21985477919295321</v>
       </c>
-      <c r="D31" s="244"/>
-      <c r="F31" s="243">
+      <c r="D31" s="241"/>
+      <c r="F31" s="240">
         <f>IF(F30=0,
 IF(G30=0,0,IF(G30&gt;0,1,-1)),
 (G30-F30)/ABS(F30)
 )</f>
         <v>0.1335178139052231</v>
       </c>
-      <c r="G31" s="244"/>
+      <c r="G31" s="241"/>
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B32" s="20" t="s">
@@ -39229,22 +39229,22 @@
       <c r="B33" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C33" s="243">
+      <c r="C33" s="240">
         <f>IF(C32=0,
 IF(D32=0,0,IF(D32&gt;0,1,-1)),
 (D32-C32)/ABS(C32)
 )</f>
         <v>-2.9218647406434668E-2</v>
       </c>
-      <c r="D33" s="244"/>
-      <c r="F33" s="243">
+      <c r="D33" s="241"/>
+      <c r="F33" s="240">
         <f>IF(F32=0,
 IF(G32=0,0,IF(G32&gt;0,1,-1)),
 (G32-F32)/ABS(F32)
 )</f>
         <v>0.15613189104652678</v>
       </c>
-      <c r="G33" s="244"/>
+      <c r="G33" s="241"/>
     </row>
     <row r="35" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B35" s="224" t="s">
@@ -39271,22 +39271,22 @@
       <c r="B36" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C36" s="243">
+      <c r="C36" s="240">
         <f>IF(C35=0,
 IF(D35=0,0,IF(D35&gt;0,1,-1)),
 (D35-C35)/ABS(C35)
 )</f>
         <v>-4.8110327402884512E-2</v>
       </c>
-      <c r="D36" s="244"/>
-      <c r="F36" s="243">
+      <c r="D36" s="241"/>
+      <c r="F36" s="240">
         <f>IF(F35=0,
 IF(G35=0,0,IF(G35&gt;0,1,-1)),
 (G35-F35)/ABS(F35)
 )</f>
         <v>0.21690368310080302</v>
       </c>
-      <c r="G36" s="244"/>
+      <c r="G36" s="241"/>
     </row>
     <row r="37" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B37" s="224" t="s">
@@ -39313,22 +39313,22 @@
       <c r="B38" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C38" s="243">
+      <c r="C38" s="240">
         <f>IF(C37=0,
 IF(D37=0,0,IF(D37&gt;0,1,-1)),
 (D37-C37)/ABS(C37)
 )</f>
         <v>0.23252768186688891</v>
       </c>
-      <c r="D38" s="244"/>
-      <c r="F38" s="243">
+      <c r="D38" s="241"/>
+      <c r="F38" s="240">
         <f>IF(F37=0,
 IF(G37=0,0,IF(G37&gt;0,1,-1)),
 (G37-F37)/ABS(F37)
 )</f>
         <v>0.28660203827989061</v>
       </c>
-      <c r="G38" s="244"/>
+      <c r="G38" s="241"/>
     </row>
     <row r="39" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B39" s="224" t="s">
@@ -39355,22 +39355,22 @@
       <c r="B40" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C40" s="243">
+      <c r="C40" s="240">
         <f>IF(C39=0,
 IF(D39=0,0,IF(D39&gt;0,1,-1)),
 (D39-C39)/ABS(C39)
 )</f>
         <v>-0.10457043679490888</v>
       </c>
-      <c r="D40" s="244"/>
-      <c r="F40" s="243">
+      <c r="D40" s="241"/>
+      <c r="F40" s="240">
         <f>IF(F39=0,
 IF(G39=0,0,IF(G39&gt;0,1,-1)),
 (G39-F39)/ABS(F39)
 )</f>
         <v>-5.9261510408752466E-2</v>
       </c>
-      <c r="G40" s="244"/>
+      <c r="G40" s="241"/>
     </row>
     <row r="41" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B41" s="224" t="s">
@@ -39397,22 +39397,22 @@
       <c r="B42" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C42" s="243">
+      <c r="C42" s="240">
         <f>IF(C41=0,
 IF(D41=0,0,IF(D41&gt;0,1,-1)),
 (D41-C41)/ABS(C41)
 )</f>
         <v>-2.2781926338438173E-3</v>
       </c>
-      <c r="D42" s="244"/>
-      <c r="F42" s="243">
+      <c r="D42" s="241"/>
+      <c r="F42" s="240">
         <f>IF(F41=0,
 IF(G41=0,0,IF(G41&gt;0,1,-1)),
 (G41-F41)/ABS(F41)
 )</f>
         <v>6.4694759589411135E-2</v>
       </c>
-      <c r="G42" s="244"/>
+      <c r="G42" s="241"/>
     </row>
     <row r="43" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B43" s="224" t="s">
@@ -39439,25 +39439,55 @@
       <c r="B44" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C44" s="243">
+      <c r="C44" s="240">
         <f>IF(C43=0,
 IF(D43=0,0,IF(D43&gt;0,1,-1)),
 (D43-C43)/ABS(C43)
 )</f>
         <v>-7.6510847107438013E-3</v>
       </c>
-      <c r="D44" s="244"/>
-      <c r="F44" s="243">
+      <c r="D44" s="241"/>
+      <c r="F44" s="240">
         <f>IF(F43=0,
 IF(G43=0,0,IF(G43&gt;0,1,-1)),
 (G43-F43)/ABS(F43)
 )</f>
         <v>0.12092039528862633</v>
       </c>
-      <c r="G44" s="244"/>
+      <c r="G44" s="241"/>
     </row>
   </sheetData>
   <mergeCells count="38">
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="F36:G36"/>
     <mergeCell ref="C44:D44"/>
     <mergeCell ref="F44:G44"/>
     <mergeCell ref="C38:D38"/>
@@ -39466,36 +39496,6 @@
     <mergeCell ref="F40:G40"/>
     <mergeCell ref="C42:D42"/>
     <mergeCell ref="F42:G42"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="F36:G36"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="F9:G9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>

</xml_diff>

<commit_message>
Added links on all sections
</commit_message>
<xml_diff>
--- a/AAPL.xlsx
+++ b/AAPL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/KINGSTON/MyStockData/Finance-StockLists/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8937088-2595-D24F-965C-D633922907AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AB53D8D-1CCB-7C45-8DD5-BABDB1093D1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14400" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
   </bookViews>
@@ -152,7 +152,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="801" uniqueCount="419">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="833" uniqueCount="427">
   <si>
     <t>Ticker</t>
   </si>
@@ -1409,6 +1409,30 @@
   </si>
   <si>
     <t>Reverse DCF rate</t>
+  </si>
+  <si>
+    <t>Discount rates used</t>
+  </si>
+  <si>
+    <t>Cost of Equity</t>
+  </si>
+  <si>
+    <t>Links</t>
+  </si>
+  <si>
+    <t>Financials -&gt;'!B13</t>
+  </si>
+  <si>
+    <t>Analysis -&gt;'!B13</t>
+  </si>
+  <si>
+    <t>Forecast -&gt;'!B13</t>
+  </si>
+  <si>
+    <t>Valuation -&gt;'!B13</t>
+  </si>
+  <si>
+    <t>Overview'!B3</t>
   </si>
 </sst>
 </file>
@@ -1425,7 +1449,7 @@
     <numFmt numFmtId="169" formatCode="#,##0.0_);\(#,##0.0\)"/>
     <numFmt numFmtId="170" formatCode="0.0"/>
   </numFmts>
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1591,6 +1615,14 @@
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -2017,11 +2049,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="254">
+  <cellXfs count="258">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
@@ -2332,6 +2365,8 @@
     <xf numFmtId="39" fontId="10" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="7" fillId="9" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="17" borderId="25" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="17" borderId="26" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2386,8 +2421,15 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="25" xfId="2" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="26" xfId="2" quotePrefix="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
@@ -15524,10 +15566,10 @@
     <v>345.34</v>
     <v>243.42</v>
     <v>1.0779000000000001</v>
-    <v>-3.78</v>
-    <v>-1.1104000000000001E-2</v>
-    <v>-0.59</v>
-    <v>-1.7530000000000002E-3</v>
+    <v>4.33</v>
+    <v>1.2862E-2</v>
+    <v>-0.26829999999999998</v>
+    <v>-7.8689999999999999E-4</v>
     <v>USD</v>
     <v>Apple Inc. designs, manufactures and markets smartphones, personal computers, tablets, wearables and accessories, and sells a variety of related services. Its product categories include iPhone, Mac, iPad, Wearables, Home and Accessories. Its services include advertising, AppleCare, cloud services, digital content, and payment services. The Company operates various platforms, including the App Store, that allow customers to discover and download applications and digital content, such as books, music, video, games and podcasts. It also offers digital content through subscription-based services, including Apple Arcade, Apple Fitness+, Apple Music, Apple News+, and Apple TV+. Its wearables include smartwatches, wireless headphones, and spatial computers. Its products include iPhone 16 Pro, iPhone 16, iPhone 15, iPhone 14, iPhone SE, MacBook Air, MacBook Pro, iMac, Mac mini, Mac Studio, Mac Pro, iPad Pro, iPad Air, AirPods, AirPods Pro, AirPods Max, Apple TV, Apple Vision Pro and others.</v>
     <v>166000</v>
@@ -15535,25 +15577,25 @@
     <v>XNAS</v>
     <v>XNAS</v>
     <v>One Apple Park Way, CUPERTINO, CA, 95014 US</v>
-    <v>338.61</v>
+    <v>342.63</v>
     <v>Computers, Phones &amp; Household Electronics</v>
     <v>Stock</v>
-    <v>46304.999846180472</v>
+    <v>46307.864467488282</v>
     <v>0</v>
-    <v>330.7</v>
-    <v>4912984755200</v>
+    <v>337.6</v>
+    <v>4976177554600</v>
     <v>APPLE INC.</v>
     <v>APPLE INC.</v>
-    <v>331.69499999999999</v>
-    <v>39.171100000000003</v>
-    <v>340.42</v>
+    <v>338.21499999999997</v>
+    <v>39.234299999999998</v>
     <v>336.64</v>
-    <v>336.05</v>
+    <v>340.97</v>
+    <v>340.70170000000002</v>
     <v>14594180000</v>
     <v>AAPL</v>
     <v>APPLE INC. (XNAS:AAPL)</v>
-    <v>37881199</v>
-    <v>40650930</v>
+    <v>25792513</v>
+    <v>40677145</v>
     <v>1977</v>
   </rv>
   <rv s="2">
@@ -15809,9 +15851,9 @@
       <v>at close</v>
       <v>from previous close</v>
       <v>from previous close</v>
-      <v>Source: Nasdaq</v>
+      <v>Source: Nasdaq Last Sale</v>
       <v>GMT</v>
-      <v>Delayed 15 minutes</v>
+      <v>Real-Time Nasdaq Last Sale</v>
       <v>from close</v>
       <v>from close</v>
     </spb>
@@ -16365,7 +16407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{825B172E-7ADE-4B4A-B533-F037BCFCDCB0}">
-  <dimension ref="B1:I59"/>
+  <dimension ref="B1:K59"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2" style="1" customWidth="1"/>
@@ -16377,25 +16419,30 @@
     <col min="7" max="7" width="1.6640625" style="1" customWidth="1"/>
     <col min="8" max="8" width="15.1640625" style="1" customWidth="1"/>
     <col min="9" max="9" width="8.6640625" style="1" customWidth="1"/>
-    <col min="10" max="16384" width="10.83203125" style="1"/>
+    <col min="10" max="10" width="2" style="1" customWidth="1"/>
+    <col min="11" max="11" width="16.5" style="1" customWidth="1"/>
+    <col min="12" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:9" ht="11" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B2" s="236" t="s">
+    <row r="1" spans="2:11" ht="11" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="2" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B2" s="238" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="237"/>
-      <c r="E2" s="236" t="s">
+      <c r="C2" s="239"/>
+      <c r="E2" s="238" t="s">
         <v>281</v>
       </c>
-      <c r="F2" s="237"/>
-      <c r="H2" s="236" t="s">
+      <c r="F2" s="239"/>
+      <c r="H2" s="238" t="s">
         <v>319</v>
       </c>
-      <c r="I2" s="237"/>
-    </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="I2" s="239"/>
+      <c r="K2" s="132" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="3" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B3" s="179" t="s">
         <v>11</v>
       </c>
@@ -16408,7 +16455,7 @@
       </c>
       <c r="F3" s="181">
         <f ca="1">Statement!AC143</f>
-        <v>4932785.92</v>
+        <v>4996233.41</v>
       </c>
       <c r="H3" s="179" t="str">
         <f>'AVG target price'!B5</f>
@@ -16416,10 +16463,13 @@
       </c>
       <c r="I3" s="205">
         <f ca="1">'AVG target price'!C5</f>
-        <v>113.07194781276988</v>
-      </c>
-    </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.2">
+        <v>113.05369355770794</v>
+      </c>
+      <c r="K3" s="256" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="4" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B4" s="179" t="s">
         <v>0</v>
       </c>
@@ -16432,7 +16482,7 @@
       </c>
       <c r="F4" s="182">
         <f ca="1">Statement!AC144</f>
-        <v>4870612.92</v>
+        <v>4934060.41</v>
       </c>
       <c r="H4" s="179" t="str">
         <f>'AVG target price'!B6</f>
@@ -16440,16 +16490,19 @@
       </c>
       <c r="I4" s="205">
         <f ca="1">'AVG target price'!C6</f>
-        <v>228.66391288445607</v>
-      </c>
-    </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.2">
+        <v>228.65136788928197</v>
+      </c>
+      <c r="K4" s="256" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="5" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B5" s="179" t="s">
         <v>1</v>
       </c>
       <c r="C5" s="202" cm="1">
         <f t="array" aca="1" ref="C5" ca="1">_FV(C3,"Price",TRUE)</f>
-        <v>336.64</v>
+        <v>340.97</v>
       </c>
       <c r="E5" s="179" t="s">
         <v>237</v>
@@ -16466,21 +16519,24 @@
         <f ca="1">'AVG target price'!C7</f>
         <v>200.25624214252309</v>
       </c>
-    </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="K5" s="256" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="6" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B6" s="179" t="s">
         <v>2</v>
       </c>
       <c r="C6" s="202" cm="1">
         <f t="array" aca="1" ref="C6" ca="1">_FV(C3,"Price (Extended hours)",TRUE)</f>
-        <v>336.05</v>
+        <v>340.70170000000002</v>
       </c>
       <c r="E6" s="179" t="s">
         <v>231</v>
       </c>
       <c r="F6" s="184">
         <f ca="1">Statement!AC140</f>
-        <v>38.60550458715597</v>
+        <v>39.102064220183493</v>
       </c>
       <c r="H6" s="179" t="str">
         <f>'AVG target price'!B8</f>
@@ -16488,23 +16544,26 @@
       </c>
       <c r="I6" s="205">
         <f ca="1">'AVG target price'!C8</f>
-        <v>198.82812827509545</v>
-      </c>
-    </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.2">
+        <v>198.8173553361099</v>
+      </c>
+      <c r="K6" s="257" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="7" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B7" s="179" t="s">
         <v>3</v>
       </c>
       <c r="C7" s="6" cm="1">
         <f t="array" aca="1" ref="C7" ca="1">_FV(C3,"Change")</f>
-        <v>-3.78</v>
+        <v>4.33</v>
       </c>
       <c r="E7" s="180" t="s">
         <v>198</v>
       </c>
       <c r="F7" s="185">
         <f ca="1">Statement!AC141</f>
-        <v>10.657397771746464</v>
+        <v>10.79447753752493</v>
       </c>
       <c r="H7" s="179" t="str">
         <f>'AVG target price'!B9</f>
@@ -16512,23 +16571,23 @@
       </c>
       <c r="I7" s="205">
         <f ca="1">'AVG target price'!C9</f>
-        <v>212.79825444499096</v>
-      </c>
-    </row>
-    <row r="8" spans="2:9" x14ac:dyDescent="0.2">
+        <v>212.78665176920245</v>
+      </c>
+    </row>
+    <row r="8" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B8" s="179" t="s">
         <v>4</v>
       </c>
       <c r="C8" s="6" cm="1">
         <f t="array" aca="1" ref="C8" ca="1">_FV(C3,"Change (extended hours)",TRUE)</f>
-        <v>-0.59</v>
+        <v>-0.26829999999999998</v>
       </c>
       <c r="E8" s="179" t="s">
         <v>259</v>
       </c>
       <c r="F8" s="186">
         <f ca="1">Statement!AC151</f>
-        <v>2.4930536616517101E-2</v>
+        <v>2.4613942125654212E-2</v>
       </c>
       <c r="H8" s="178" t="str">
         <f>'AVG target price'!B10</f>
@@ -16536,23 +16595,23 @@
       </c>
       <c r="I8" s="206">
         <f ca="1">'AVG target price'!C10</f>
-        <v>190.72369711196706</v>
-      </c>
-    </row>
-    <row r="9" spans="2:9" x14ac:dyDescent="0.2">
+        <v>190.71306213896509</v>
+      </c>
+    </row>
+    <row r="9" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B9" s="179" t="s">
         <v>5</v>
       </c>
       <c r="C9" s="73" cm="1">
         <f t="array" aca="1" ref="C9" ca="1">_FV(C3,"Change (%)",TRUE)</f>
-        <v>-1.1104000000000001E-2</v>
+        <v>1.2862E-2</v>
       </c>
       <c r="E9" s="179" t="s">
         <v>282</v>
       </c>
       <c r="F9" s="186">
         <f ca="1">Statement!AC152</f>
-        <v>2.5903041825095056E-2</v>
+        <v>2.5574097427926205E-2</v>
       </c>
       <c r="H9" s="178" t="str">
         <f>'AVG target price'!B12</f>
@@ -16560,26 +16619,26 @@
       </c>
       <c r="I9" s="207">
         <f ca="1">'AVG target price'!C12</f>
-        <v>-0.43344909365504081</v>
-      </c>
-    </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.2">
+        <v>-0.44067495046788552</v>
+      </c>
+    </row>
+    <row r="10" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B10" s="179" t="s">
         <v>6</v>
       </c>
       <c r="C10" s="73" cm="1">
         <f t="array" aca="1" ref="C10" ca="1">_FV(C3,"Change % (extended hours)",TRUE)</f>
-        <v>-1.7530000000000002E-3</v>
+        <v>-7.8689999999999999E-4</v>
       </c>
       <c r="E10" s="179" t="s">
         <v>287</v>
       </c>
       <c r="F10" s="186">
         <f ca="1">Statement!AC154</f>
-        <v>1.6669282092015052E-2</v>
-      </c>
-    </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.2">
+        <v>1.6457597804663014E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B11" s="179" t="s">
         <v>7</v>
       </c>
@@ -16592,7 +16651,7 @@
       </c>
       <c r="F11" s="187">
         <f ca="1">Statement!AC153</f>
-        <v>3.1190589353612169E-3</v>
+        <v>3.0794498049681791E-3</v>
       </c>
       <c r="H11" s="178" t="s">
         <v>394</v>
@@ -16602,7 +16661,7 @@
         <v>13.10511393468445</v>
       </c>
     </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B12" s="179" t="s">
         <v>8</v>
       </c>
@@ -16618,7 +16677,7 @@
         <v>0.33639821951334065</v>
       </c>
     </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B13" s="179" t="s">
         <v>9</v>
       </c>
@@ -16641,13 +16700,13 @@
         <v>0.41499999999999998</v>
       </c>
     </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B14" s="180" t="s">
         <v>10</v>
       </c>
       <c r="C14" s="204" cm="1">
         <f t="array" aca="1" ref="C14" ca="1">_FV(C3,"Volume average",TRUE)</f>
-        <v>40650930</v>
+        <v>40677145</v>
       </c>
       <c r="E14" s="180" t="s">
         <v>102</v>
@@ -16657,16 +16716,16 @@
         <v>2.8240933164668753</v>
       </c>
     </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:11" x14ac:dyDescent="0.2">
       <c r="E15" s="179" t="s">
         <v>284</v>
       </c>
       <c r="F15" s="186">
         <f ca="1">Statement!AC166</f>
-        <v>1.2604033705967113E-2</v>
-      </c>
-    </row>
-    <row r="16" spans="2:9" x14ac:dyDescent="0.2">
+        <v>1.2443974269808984E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="2:11" x14ac:dyDescent="0.2">
       <c r="E16" s="180" t="s">
         <v>289</v>
       </c>
@@ -16674,12 +16733,16 @@
         <f>Statement!AC165</f>
         <v>4.2601754145539266</v>
       </c>
+      <c r="H16" s="238" t="s">
+        <v>419</v>
+      </c>
+      <c r="I16" s="239"/>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B17" s="238" t="s">
+      <c r="B17" s="240" t="s">
         <v>88</v>
       </c>
-      <c r="C17" s="238"/>
+      <c r="C17" s="240"/>
       <c r="E17" s="178" t="s">
         <v>290</v>
       </c>
@@ -16687,6 +16750,13 @@
         <f>Statement!AC161</f>
         <v>6.1420869446529721E-4</v>
       </c>
+      <c r="H17" s="179" t="s">
+        <v>162</v>
+      </c>
+      <c r="I17" s="236">
+        <f ca="1">DCF!C15</f>
+        <v>9.991231211830999E-2</v>
+      </c>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B18" s="178" t="s">
@@ -16702,6 +16772,13 @@
         <f>Statement!AC134</f>
         <v>-56.814895644278849</v>
       </c>
+      <c r="H18" s="180" t="s">
+        <v>420</v>
+      </c>
+      <c r="I18" s="237">
+        <f ca="1">Multiples!C54</f>
+        <v>0.10094549999999999</v>
+      </c>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B19" s="178" t="s">
@@ -16752,14 +16829,14 @@
       <c r="I22" s="50"/>
     </row>
     <row r="25" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B25" s="238" t="s">
+      <c r="B25" s="240" t="s">
         <v>104</v>
       </c>
-      <c r="C25" s="238"/>
-      <c r="E25" s="236" t="s">
+      <c r="C25" s="240"/>
+      <c r="E25" s="238" t="s">
         <v>332</v>
       </c>
-      <c r="F25" s="237"/>
+      <c r="F25" s="239"/>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B26" s="178" t="s">
@@ -16908,13 +16985,14 @@
       <c r="H59" s="132"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B17:C17"/>
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="E25:F25"/>
+    <mergeCell ref="H16:I16"/>
   </mergeCells>
   <conditionalFormatting sqref="C7:C10">
     <cfRule type="cellIs" dxfId="2" priority="4" operator="lessThan">
@@ -16927,6 +17005,12 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
+  <hyperlinks>
+    <hyperlink ref="K3" location="'Financials -&gt;'!B13" display="'Financials -&gt;'!B13" xr:uid="{AE234545-B8DD-1441-A2D8-05C594C6DF05}"/>
+    <hyperlink ref="K4" location="'Analysis -&gt;'!B13" display="'Analysis -&gt;'!B13" xr:uid="{21F3FBA0-B697-A143-B77C-174BC5D52ED7}"/>
+    <hyperlink ref="K5" location="'Forecast -&gt;'!B13" display="'Forecast -&gt;'!B13" xr:uid="{9399ACBE-A298-674C-921C-C96C9A4475C7}"/>
+    <hyperlink ref="K6" location="'Valuation -&gt;'!B13" display="'Valuation -&gt;'!B13" xr:uid="{AFC00F09-27F9-8A49-AFE6-BCBC83F7D2CE}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -16936,18 +17020,57 @@
   <sheetPr>
     <tabColor theme="6" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="B13"/>
+  <dimension ref="B5:H13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="16384" width="10.83203125" style="1"/>
+    <col min="1" max="7" width="10.83203125" style="1"/>
+    <col min="8" max="8" width="15.83203125" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="13" spans="2:2" s="4" customFormat="1" ht="49" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="H5" s="132" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="H6" s="256" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="H7" s="256" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="H8" s="256" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="H9" s="256" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="H10" s="257" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8" s="4" customFormat="1" ht="49" x14ac:dyDescent="0.2">
       <c r="B13" s="3" t="s">
         <v>108</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="H6" location="Overview!B3" display="Overview'!B3" xr:uid="{43E9F232-9BA2-E847-9E40-BB10D84B4FCB}"/>
+    <hyperlink ref="H8" location="'Analysis -&gt;'!B13" display="'Analysis -&gt;'!B13" xr:uid="{549E473E-F154-C142-B126-E3EED41DED4E}"/>
+    <hyperlink ref="H9" location="'Forecast -&gt;'!B13" display="'Forecast -&gt;'!B13" xr:uid="{56DA308D-4269-B544-8691-FA8EA4BC7D01}"/>
+    <hyperlink ref="H10" location="'Valuation -&gt;'!B13" display="'Valuation -&gt;'!B13" xr:uid="{21C251FC-5BC6-C545-9606-991F5FBB8C27}"/>
+    <hyperlink ref="H7" location="'Financials -&gt;'!B13" display="'Financials -&gt;'!B13" xr:uid="{3C83CC8C-4C84-B042-BAAE-7986AE014593}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -16984,36 +17107,36 @@
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
-      <c r="C2" s="239" t="s">
+      <c r="C2" s="241" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="239"/>
-      <c r="E2" s="239"/>
-      <c r="F2" s="239"/>
-      <c r="G2" s="248"/>
-      <c r="H2" s="249" t="s">
+      <c r="D2" s="241"/>
+      <c r="E2" s="241"/>
+      <c r="F2" s="241"/>
+      <c r="G2" s="250"/>
+      <c r="H2" s="251" t="s">
         <v>111</v>
       </c>
-      <c r="I2" s="239"/>
-      <c r="J2" s="239"/>
-      <c r="K2" s="239"/>
-      <c r="L2" s="239"/>
+      <c r="I2" s="241"/>
+      <c r="J2" s="241"/>
+      <c r="K2" s="241"/>
+      <c r="L2" s="241"/>
       <c r="O2" s="5"/>
-      <c r="S2" s="239" t="s">
+      <c r="S2" s="241" t="s">
         <v>110</v>
       </c>
-      <c r="T2" s="239"/>
-      <c r="U2" s="239"/>
-      <c r="V2" s="239"/>
-      <c r="W2" s="239"/>
-      <c r="X2" s="239"/>
-      <c r="Y2" s="239"/>
-      <c r="Z2" s="239"/>
-      <c r="AA2" s="239" t="s">
+      <c r="T2" s="241"/>
+      <c r="U2" s="241"/>
+      <c r="V2" s="241"/>
+      <c r="W2" s="241"/>
+      <c r="X2" s="241"/>
+      <c r="Y2" s="241"/>
+      <c r="Z2" s="241"/>
+      <c r="AA2" s="241" t="s">
         <v>111</v>
       </c>
-      <c r="AB2" s="239"/>
-      <c r="AC2" s="239"/>
+      <c r="AB2" s="241"/>
+      <c r="AC2" s="241"/>
       <c r="AE2" s="85" t="s">
         <v>112</v>
       </c>
@@ -17024,32 +17147,32 @@
     <row r="4" spans="1:31" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="86"/>
       <c r="B4" s="60"/>
-      <c r="C4" s="245" t="s">
+      <c r="C4" s="247" t="s">
         <v>113</v>
       </c>
-      <c r="D4" s="245"/>
-      <c r="E4" s="245"/>
-      <c r="F4" s="245"/>
-      <c r="G4" s="245"/>
-      <c r="H4" s="245"/>
-      <c r="I4" s="245"/>
-      <c r="J4" s="245"/>
-      <c r="K4" s="245"/>
-      <c r="L4" s="245"/>
+      <c r="D4" s="247"/>
+      <c r="E4" s="247"/>
+      <c r="F4" s="247"/>
+      <c r="G4" s="247"/>
+      <c r="H4" s="247"/>
+      <c r="I4" s="247"/>
+      <c r="J4" s="247"/>
+      <c r="K4" s="247"/>
+      <c r="L4" s="247"/>
       <c r="O4" s="5"/>
-      <c r="S4" s="246" t="s">
+      <c r="S4" s="248" t="s">
         <v>113</v>
       </c>
-      <c r="T4" s="247"/>
-      <c r="U4" s="247"/>
-      <c r="V4" s="247"/>
-      <c r="W4" s="247"/>
-      <c r="X4" s="247"/>
-      <c r="Y4" s="247"/>
-      <c r="Z4" s="247"/>
-      <c r="AA4" s="247"/>
-      <c r="AB4" s="247"/>
-      <c r="AC4" s="247"/>
+      <c r="T4" s="249"/>
+      <c r="U4" s="249"/>
+      <c r="V4" s="249"/>
+      <c r="W4" s="249"/>
+      <c r="X4" s="249"/>
+      <c r="Y4" s="249"/>
+      <c r="Z4" s="249"/>
+      <c r="AA4" s="249"/>
+      <c r="AB4" s="249"/>
+      <c r="AC4" s="249"/>
       <c r="AE4" s="87"/>
     </row>
     <row r="5" spans="1:31" x14ac:dyDescent="0.2">
@@ -17737,33 +17860,33 @@
       <c r="Q12" s="91"/>
     </row>
     <row r="13" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="C13" s="245" t="s">
+      <c r="C13" s="247" t="s">
         <v>119</v>
       </c>
-      <c r="D13" s="245"/>
-      <c r="E13" s="245"/>
-      <c r="F13" s="245"/>
-      <c r="G13" s="245"/>
-      <c r="H13" s="245"/>
-      <c r="I13" s="245"/>
-      <c r="J13" s="245"/>
-      <c r="K13" s="245"/>
-      <c r="L13" s="245"/>
+      <c r="D13" s="247"/>
+      <c r="E13" s="247"/>
+      <c r="F13" s="247"/>
+      <c r="G13" s="247"/>
+      <c r="H13" s="247"/>
+      <c r="I13" s="247"/>
+      <c r="J13" s="247"/>
+      <c r="K13" s="247"/>
+      <c r="L13" s="247"/>
       <c r="O13" s="5"/>
       <c r="Q13" s="91"/>
-      <c r="S13" s="246" t="s">
+      <c r="S13" s="248" t="s">
         <v>119</v>
       </c>
-      <c r="T13" s="247"/>
-      <c r="U13" s="247"/>
-      <c r="V13" s="247"/>
-      <c r="W13" s="247"/>
-      <c r="X13" s="247"/>
-      <c r="Y13" s="247"/>
-      <c r="Z13" s="247"/>
-      <c r="AA13" s="247"/>
-      <c r="AB13" s="247"/>
-      <c r="AC13" s="247"/>
+      <c r="T13" s="249"/>
+      <c r="U13" s="249"/>
+      <c r="V13" s="249"/>
+      <c r="W13" s="249"/>
+      <c r="X13" s="249"/>
+      <c r="Y13" s="249"/>
+      <c r="Z13" s="249"/>
+      <c r="AA13" s="249"/>
+      <c r="AB13" s="249"/>
+      <c r="AC13" s="249"/>
     </row>
     <row r="14" spans="1:31" x14ac:dyDescent="0.2">
       <c r="B14" s="16" t="s">
@@ -18384,35 +18507,35 @@
     </row>
     <row r="2" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
-      <c r="C2" s="239" t="s">
+      <c r="C2" s="241" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="239"/>
-      <c r="E2" s="239"/>
-      <c r="F2" s="239"/>
-      <c r="G2" s="248"/>
-      <c r="H2" s="249" t="s">
+      <c r="D2" s="241"/>
+      <c r="E2" s="241"/>
+      <c r="F2" s="241"/>
+      <c r="G2" s="250"/>
+      <c r="H2" s="251" t="s">
         <v>111</v>
       </c>
-      <c r="I2" s="239"/>
-      <c r="J2" s="239"/>
-      <c r="K2" s="239"/>
-      <c r="L2" s="239"/>
-      <c r="P2" s="239" t="s">
+      <c r="I2" s="241"/>
+      <c r="J2" s="241"/>
+      <c r="K2" s="241"/>
+      <c r="L2" s="241"/>
+      <c r="P2" s="241" t="s">
         <v>110</v>
       </c>
-      <c r="Q2" s="239"/>
-      <c r="R2" s="239"/>
-      <c r="S2" s="239"/>
-      <c r="T2" s="239"/>
-      <c r="U2" s="239"/>
-      <c r="V2" s="239"/>
-      <c r="W2" s="239"/>
-      <c r="X2" s="239" t="s">
+      <c r="Q2" s="241"/>
+      <c r="R2" s="241"/>
+      <c r="S2" s="241"/>
+      <c r="T2" s="241"/>
+      <c r="U2" s="241"/>
+      <c r="V2" s="241"/>
+      <c r="W2" s="241"/>
+      <c r="X2" s="241" t="s">
         <v>111</v>
       </c>
-      <c r="Y2" s="239"/>
-      <c r="Z2" s="239"/>
+      <c r="Y2" s="241"/>
+      <c r="Z2" s="241"/>
       <c r="AB2" s="85" t="s">
         <v>112</v>
       </c>
@@ -18421,31 +18544,31 @@
     <row r="4" spans="1:28" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="86"/>
       <c r="B4" s="60"/>
-      <c r="C4" s="245" t="s">
+      <c r="C4" s="247" t="s">
         <v>113</v>
       </c>
-      <c r="D4" s="245"/>
-      <c r="E4" s="245"/>
-      <c r="F4" s="245"/>
-      <c r="G4" s="245"/>
-      <c r="H4" s="245"/>
-      <c r="I4" s="245"/>
-      <c r="J4" s="245"/>
-      <c r="K4" s="245"/>
-      <c r="L4" s="245"/>
-      <c r="P4" s="247" t="s">
+      <c r="D4" s="247"/>
+      <c r="E4" s="247"/>
+      <c r="F4" s="247"/>
+      <c r="G4" s="247"/>
+      <c r="H4" s="247"/>
+      <c r="I4" s="247"/>
+      <c r="J4" s="247"/>
+      <c r="K4" s="247"/>
+      <c r="L4" s="247"/>
+      <c r="P4" s="249" t="s">
         <v>113</v>
       </c>
-      <c r="Q4" s="247"/>
-      <c r="R4" s="247"/>
-      <c r="S4" s="247"/>
-      <c r="T4" s="247"/>
-      <c r="U4" s="247"/>
-      <c r="V4" s="247"/>
-      <c r="W4" s="247"/>
-      <c r="X4" s="247"/>
-      <c r="Y4" s="247"/>
-      <c r="Z4" s="247"/>
+      <c r="Q4" s="249"/>
+      <c r="R4" s="249"/>
+      <c r="S4" s="249"/>
+      <c r="T4" s="249"/>
+      <c r="U4" s="249"/>
+      <c r="V4" s="249"/>
+      <c r="W4" s="249"/>
+      <c r="X4" s="249"/>
+      <c r="Y4" s="249"/>
+      <c r="Z4" s="249"/>
       <c r="AB4" s="87"/>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.2">
@@ -18640,32 +18763,32 @@
       <c r="N8" s="91"/>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="C9" s="245" t="s">
+      <c r="C9" s="247" t="s">
         <v>122</v>
       </c>
-      <c r="D9" s="245"/>
-      <c r="E9" s="245"/>
-      <c r="F9" s="245"/>
-      <c r="G9" s="245"/>
-      <c r="H9" s="245"/>
-      <c r="I9" s="245"/>
-      <c r="J9" s="245"/>
-      <c r="K9" s="245"/>
-      <c r="L9" s="245"/>
+      <c r="D9" s="247"/>
+      <c r="E9" s="247"/>
+      <c r="F9" s="247"/>
+      <c r="G9" s="247"/>
+      <c r="H9" s="247"/>
+      <c r="I9" s="247"/>
+      <c r="J9" s="247"/>
+      <c r="K9" s="247"/>
+      <c r="L9" s="247"/>
       <c r="N9" s="91"/>
-      <c r="P9" s="247" t="s">
+      <c r="P9" s="249" t="s">
         <v>123</v>
       </c>
-      <c r="Q9" s="247"/>
-      <c r="R9" s="247"/>
-      <c r="S9" s="247"/>
-      <c r="T9" s="247"/>
-      <c r="U9" s="247"/>
-      <c r="V9" s="247"/>
-      <c r="W9" s="247"/>
-      <c r="X9" s="247"/>
-      <c r="Y9" s="247"/>
-      <c r="Z9" s="247"/>
+      <c r="Q9" s="249"/>
+      <c r="R9" s="249"/>
+      <c r="S9" s="249"/>
+      <c r="T9" s="249"/>
+      <c r="U9" s="249"/>
+      <c r="V9" s="249"/>
+      <c r="W9" s="249"/>
+      <c r="X9" s="249"/>
+      <c r="Y9" s="249"/>
+      <c r="Z9" s="249"/>
       <c r="AB9" s="87">
         <f>AB4</f>
         <v>0</v>
@@ -19141,31 +19264,31 @@
       </c>
     </row>
     <row r="17" spans="2:26" x14ac:dyDescent="0.2">
-      <c r="C17" s="245" t="s">
+      <c r="C17" s="247" t="s">
         <v>125</v>
       </c>
-      <c r="D17" s="245"/>
-      <c r="E17" s="245"/>
-      <c r="F17" s="245"/>
-      <c r="G17" s="245"/>
-      <c r="H17" s="245"/>
-      <c r="I17" s="245"/>
-      <c r="J17" s="245"/>
-      <c r="K17" s="245"/>
-      <c r="L17" s="245"/>
-      <c r="P17" s="247" t="s">
+      <c r="D17" s="247"/>
+      <c r="E17" s="247"/>
+      <c r="F17" s="247"/>
+      <c r="G17" s="247"/>
+      <c r="H17" s="247"/>
+      <c r="I17" s="247"/>
+      <c r="J17" s="247"/>
+      <c r="K17" s="247"/>
+      <c r="L17" s="247"/>
+      <c r="P17" s="249" t="s">
         <v>125</v>
       </c>
-      <c r="Q17" s="247"/>
-      <c r="R17" s="247"/>
-      <c r="S17" s="247"/>
-      <c r="T17" s="247"/>
-      <c r="U17" s="247"/>
-      <c r="V17" s="247"/>
-      <c r="W17" s="247"/>
-      <c r="X17" s="247"/>
-      <c r="Y17" s="247"/>
-      <c r="Z17" s="247"/>
+      <c r="Q17" s="249"/>
+      <c r="R17" s="249"/>
+      <c r="S17" s="249"/>
+      <c r="T17" s="249"/>
+      <c r="U17" s="249"/>
+      <c r="V17" s="249"/>
+      <c r="W17" s="249"/>
+      <c r="X17" s="249"/>
+      <c r="Y17" s="249"/>
+      <c r="Z17" s="249"/>
     </row>
     <row r="18" spans="2:26" x14ac:dyDescent="0.2">
       <c r="B18" s="16" t="s">
@@ -19643,60 +19766,60 @@
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A3" s="4"/>
-      <c r="C3" s="239" t="s">
+      <c r="C3" s="241" t="s">
         <v>110</v>
       </c>
-      <c r="D3" s="239"/>
-      <c r="E3" s="239"/>
-      <c r="F3" s="239"/>
-      <c r="G3" s="248"/>
-      <c r="H3" s="249" t="s">
+      <c r="D3" s="241"/>
+      <c r="E3" s="241"/>
+      <c r="F3" s="241"/>
+      <c r="G3" s="250"/>
+      <c r="H3" s="251" t="s">
         <v>111</v>
       </c>
-      <c r="I3" s="239"/>
-      <c r="J3" s="239"/>
-      <c r="K3" s="239"/>
-      <c r="L3" s="239"/>
-      <c r="P3" s="250"/>
-      <c r="Q3" s="250"/>
-      <c r="R3" s="250"/>
-      <c r="S3" s="250"/>
-      <c r="T3" s="250"/>
-      <c r="U3" s="250"/>
-      <c r="V3" s="250"/>
-      <c r="W3" s="250"/>
-      <c r="X3" s="250"/>
-      <c r="Y3" s="250"/>
-      <c r="Z3" s="250"/>
+      <c r="I3" s="241"/>
+      <c r="J3" s="241"/>
+      <c r="K3" s="241"/>
+      <c r="L3" s="241"/>
+      <c r="P3" s="252"/>
+      <c r="Q3" s="252"/>
+      <c r="R3" s="252"/>
+      <c r="S3" s="252"/>
+      <c r="T3" s="252"/>
+      <c r="U3" s="252"/>
+      <c r="V3" s="252"/>
+      <c r="W3" s="252"/>
+      <c r="X3" s="252"/>
+      <c r="Y3" s="252"/>
+      <c r="Z3" s="252"/>
       <c r="AB3" s="109"/>
     </row>
     <row r="4" spans="1:28" ht="10" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="5" spans="1:28" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="86"/>
       <c r="B5" s="60"/>
-      <c r="C5" s="245" t="s">
+      <c r="C5" s="247" t="s">
         <v>113</v>
       </c>
-      <c r="D5" s="245"/>
-      <c r="E5" s="245"/>
-      <c r="F5" s="245"/>
-      <c r="G5" s="245"/>
-      <c r="H5" s="245"/>
-      <c r="I5" s="245"/>
-      <c r="J5" s="245"/>
-      <c r="K5" s="245"/>
-      <c r="L5" s="245"/>
-      <c r="P5" s="250"/>
-      <c r="Q5" s="250"/>
-      <c r="R5" s="250"/>
-      <c r="S5" s="250"/>
-      <c r="T5" s="250"/>
-      <c r="U5" s="250"/>
-      <c r="V5" s="250"/>
-      <c r="W5" s="250"/>
-      <c r="X5" s="250"/>
-      <c r="Y5" s="250"/>
-      <c r="Z5" s="250"/>
+      <c r="D5" s="247"/>
+      <c r="E5" s="247"/>
+      <c r="F5" s="247"/>
+      <c r="G5" s="247"/>
+      <c r="H5" s="247"/>
+      <c r="I5" s="247"/>
+      <c r="J5" s="247"/>
+      <c r="K5" s="247"/>
+      <c r="L5" s="247"/>
+      <c r="P5" s="252"/>
+      <c r="Q5" s="252"/>
+      <c r="R5" s="252"/>
+      <c r="S5" s="252"/>
+      <c r="T5" s="252"/>
+      <c r="U5" s="252"/>
+      <c r="V5" s="252"/>
+      <c r="W5" s="252"/>
+      <c r="X5" s="252"/>
+      <c r="Y5" s="252"/>
+      <c r="Z5" s="252"/>
       <c r="AB5" s="110"/>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.2">
@@ -19882,30 +20005,30 @@
       <c r="N10" s="91"/>
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="C11" s="245" t="s">
+      <c r="C11" s="247" t="s">
         <v>129</v>
       </c>
-      <c r="D11" s="245"/>
-      <c r="E11" s="245"/>
-      <c r="F11" s="245"/>
-      <c r="G11" s="245"/>
-      <c r="H11" s="245"/>
-      <c r="I11" s="245"/>
-      <c r="J11" s="245"/>
-      <c r="K11" s="245"/>
-      <c r="L11" s="245"/>
+      <c r="D11" s="247"/>
+      <c r="E11" s="247"/>
+      <c r="F11" s="247"/>
+      <c r="G11" s="247"/>
+      <c r="H11" s="247"/>
+      <c r="I11" s="247"/>
+      <c r="J11" s="247"/>
+      <c r="K11" s="247"/>
+      <c r="L11" s="247"/>
       <c r="N11" s="91"/>
-      <c r="P11" s="250"/>
-      <c r="Q11" s="250"/>
-      <c r="R11" s="250"/>
-      <c r="S11" s="250"/>
-      <c r="T11" s="250"/>
-      <c r="U11" s="250"/>
-      <c r="V11" s="250"/>
-      <c r="W11" s="250"/>
-      <c r="X11" s="250"/>
-      <c r="Y11" s="250"/>
-      <c r="Z11" s="250"/>
+      <c r="P11" s="252"/>
+      <c r="Q11" s="252"/>
+      <c r="R11" s="252"/>
+      <c r="S11" s="252"/>
+      <c r="T11" s="252"/>
+      <c r="U11" s="252"/>
+      <c r="V11" s="252"/>
+      <c r="W11" s="252"/>
+      <c r="X11" s="252"/>
+      <c r="Y11" s="252"/>
+      <c r="Z11" s="252"/>
       <c r="AB11" s="110"/>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.2">
@@ -20147,18 +20270,18 @@
       <c r="D16" s="24"/>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="C18" s="245" t="s">
+      <c r="C18" s="247" t="s">
         <v>134</v>
       </c>
-      <c r="D18" s="245"/>
-      <c r="E18" s="245"/>
-      <c r="F18" s="245"/>
-      <c r="G18" s="245"/>
-      <c r="H18" s="245"/>
-      <c r="I18" s="245"/>
-      <c r="J18" s="245"/>
-      <c r="K18" s="245"/>
-      <c r="L18" s="245"/>
+      <c r="D18" s="247"/>
+      <c r="E18" s="247"/>
+      <c r="F18" s="247"/>
+      <c r="G18" s="247"/>
+      <c r="H18" s="247"/>
+      <c r="I18" s="247"/>
+      <c r="J18" s="247"/>
+      <c r="K18" s="247"/>
+      <c r="L18" s="247"/>
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B19" s="16" t="s">
@@ -20371,23 +20494,23 @@
       </c>
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="B25" s="250"/>
-      <c r="C25" s="250"/>
+      <c r="B25" s="252"/>
+      <c r="C25" s="252"/>
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B26" s="109"/>
-      <c r="C26" s="245" t="s">
+      <c r="C26" s="247" t="s">
         <v>140</v>
       </c>
-      <c r="D26" s="245"/>
-      <c r="E26" s="245"/>
-      <c r="F26" s="245"/>
-      <c r="G26" s="245"/>
-      <c r="H26" s="245"/>
-      <c r="I26" s="245"/>
-      <c r="J26" s="245"/>
-      <c r="K26" s="245"/>
-      <c r="L26" s="245"/>
+      <c r="D26" s="247"/>
+      <c r="E26" s="247"/>
+      <c r="F26" s="247"/>
+      <c r="G26" s="247"/>
+      <c r="H26" s="247"/>
+      <c r="I26" s="247"/>
+      <c r="J26" s="247"/>
+      <c r="K26" s="247"/>
+      <c r="L26" s="247"/>
     </row>
     <row r="27" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B27" s="16" t="s">
@@ -20579,18 +20702,18 @@
     </row>
     <row r="33" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B33" s="109"/>
-      <c r="C33" s="245" t="s">
+      <c r="C33" s="247" t="s">
         <v>144</v>
       </c>
-      <c r="D33" s="245"/>
-      <c r="E33" s="245"/>
-      <c r="F33" s="245"/>
-      <c r="G33" s="245"/>
-      <c r="H33" s="245"/>
-      <c r="I33" s="245"/>
-      <c r="J33" s="245"/>
-      <c r="K33" s="245"/>
-      <c r="L33" s="245"/>
+      <c r="D33" s="247"/>
+      <c r="E33" s="247"/>
+      <c r="F33" s="247"/>
+      <c r="G33" s="247"/>
+      <c r="H33" s="247"/>
+      <c r="I33" s="247"/>
+      <c r="J33" s="247"/>
+      <c r="K33" s="247"/>
+      <c r="L33" s="247"/>
     </row>
     <row r="34" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B34" s="16" t="s">
@@ -20774,18 +20897,18 @@
       <c r="C39" s="125"/>
     </row>
     <row r="40" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="C40" s="245" t="s">
+      <c r="C40" s="247" t="s">
         <v>147</v>
       </c>
-      <c r="D40" s="245"/>
-      <c r="E40" s="245"/>
-      <c r="F40" s="245"/>
-      <c r="G40" s="245"/>
-      <c r="H40" s="245"/>
-      <c r="I40" s="245"/>
-      <c r="J40" s="245"/>
-      <c r="K40" s="245"/>
-      <c r="L40" s="245"/>
+      <c r="D40" s="247"/>
+      <c r="E40" s="247"/>
+      <c r="F40" s="247"/>
+      <c r="G40" s="247"/>
+      <c r="H40" s="247"/>
+      <c r="I40" s="247"/>
+      <c r="J40" s="247"/>
+      <c r="K40" s="247"/>
+      <c r="L40" s="247"/>
     </row>
     <row r="41" spans="2:12" x14ac:dyDescent="0.2">
       <c r="B41" s="16" t="s">
@@ -21099,60 +21222,60 @@
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
-      <c r="C2" s="239" t="s">
+      <c r="C2" s="241" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="239"/>
-      <c r="E2" s="239"/>
-      <c r="F2" s="239"/>
-      <c r="G2" s="248"/>
-      <c r="H2" s="249" t="s">
+      <c r="D2" s="241"/>
+      <c r="E2" s="241"/>
+      <c r="F2" s="241"/>
+      <c r="G2" s="250"/>
+      <c r="H2" s="251" t="s">
         <v>111</v>
       </c>
-      <c r="I2" s="239"/>
-      <c r="J2" s="239"/>
-      <c r="K2" s="239"/>
-      <c r="L2" s="239"/>
-      <c r="S2" s="250"/>
-      <c r="T2" s="250"/>
-      <c r="U2" s="250"/>
-      <c r="V2" s="250"/>
-      <c r="W2" s="250"/>
-      <c r="X2" s="250"/>
-      <c r="Y2" s="250"/>
-      <c r="Z2" s="250"/>
-      <c r="AA2" s="250"/>
-      <c r="AB2" s="250"/>
-      <c r="AC2" s="250"/>
+      <c r="I2" s="241"/>
+      <c r="J2" s="241"/>
+      <c r="K2" s="241"/>
+      <c r="L2" s="241"/>
+      <c r="S2" s="252"/>
+      <c r="T2" s="252"/>
+      <c r="U2" s="252"/>
+      <c r="V2" s="252"/>
+      <c r="W2" s="252"/>
+      <c r="X2" s="252"/>
+      <c r="Y2" s="252"/>
+      <c r="Z2" s="252"/>
+      <c r="AA2" s="252"/>
+      <c r="AB2" s="252"/>
+      <c r="AC2" s="252"/>
       <c r="AE2" s="109"/>
     </row>
     <row r="3" spans="1:31" ht="10" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:31" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="86"/>
       <c r="B4" s="60"/>
-      <c r="C4" s="245" t="s">
+      <c r="C4" s="247" t="s">
         <v>18</v>
       </c>
-      <c r="D4" s="245"/>
-      <c r="E4" s="245"/>
-      <c r="F4" s="245"/>
-      <c r="G4" s="245"/>
-      <c r="H4" s="245"/>
-      <c r="I4" s="245"/>
-      <c r="J4" s="245"/>
-      <c r="K4" s="245"/>
-      <c r="L4" s="245"/>
-      <c r="S4" s="250"/>
-      <c r="T4" s="250"/>
-      <c r="U4" s="250"/>
-      <c r="V4" s="250"/>
-      <c r="W4" s="250"/>
-      <c r="X4" s="250"/>
-      <c r="Y4" s="250"/>
-      <c r="Z4" s="250"/>
-      <c r="AA4" s="250"/>
-      <c r="AB4" s="250"/>
-      <c r="AC4" s="250"/>
+      <c r="D4" s="247"/>
+      <c r="E4" s="247"/>
+      <c r="F4" s="247"/>
+      <c r="G4" s="247"/>
+      <c r="H4" s="247"/>
+      <c r="I4" s="247"/>
+      <c r="J4" s="247"/>
+      <c r="K4" s="247"/>
+      <c r="L4" s="247"/>
+      <c r="S4" s="252"/>
+      <c r="T4" s="252"/>
+      <c r="U4" s="252"/>
+      <c r="V4" s="252"/>
+      <c r="W4" s="252"/>
+      <c r="X4" s="252"/>
+      <c r="Y4" s="252"/>
+      <c r="Z4" s="252"/>
+      <c r="AA4" s="252"/>
+      <c r="AB4" s="252"/>
+      <c r="AC4" s="252"/>
       <c r="AE4" s="110"/>
     </row>
     <row r="5" spans="1:31" x14ac:dyDescent="0.2">
@@ -21515,18 +21638,18 @@
       <c r="AE10" s="64"/>
     </row>
     <row r="13" spans="1:31" x14ac:dyDescent="0.2">
-      <c r="C13" s="245" t="s">
+      <c r="C13" s="247" t="s">
         <v>155</v>
       </c>
-      <c r="D13" s="245"/>
-      <c r="E13" s="245"/>
-      <c r="F13" s="245"/>
-      <c r="G13" s="245"/>
-      <c r="H13" s="245"/>
-      <c r="I13" s="245"/>
-      <c r="J13" s="245"/>
-      <c r="K13" s="245"/>
-      <c r="L13" s="245"/>
+      <c r="D13" s="247"/>
+      <c r="E13" s="247"/>
+      <c r="F13" s="247"/>
+      <c r="G13" s="247"/>
+      <c r="H13" s="247"/>
+      <c r="I13" s="247"/>
+      <c r="J13" s="247"/>
+      <c r="K13" s="247"/>
+      <c r="L13" s="247"/>
     </row>
     <row r="14" spans="1:31" x14ac:dyDescent="0.2">
       <c r="C14" s="12">
@@ -21619,18 +21742,18 @@
       </c>
     </row>
     <row r="18" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="C18" s="245" t="s">
+      <c r="C18" s="247" t="s">
         <v>156</v>
       </c>
-      <c r="D18" s="245"/>
-      <c r="E18" s="245"/>
-      <c r="F18" s="245"/>
-      <c r="G18" s="245"/>
-      <c r="H18" s="245"/>
-      <c r="I18" s="245"/>
-      <c r="J18" s="245"/>
-      <c r="K18" s="245"/>
-      <c r="L18" s="245"/>
+      <c r="D18" s="247"/>
+      <c r="E18" s="247"/>
+      <c r="F18" s="247"/>
+      <c r="G18" s="247"/>
+      <c r="H18" s="247"/>
+      <c r="I18" s="247"/>
+      <c r="J18" s="247"/>
+      <c r="K18" s="247"/>
+      <c r="L18" s="247"/>
     </row>
     <row r="19" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B19" s="16" t="s">
@@ -21822,18 +21945,18 @@
       </c>
     </row>
     <row r="25" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="C25" s="245" t="s">
+      <c r="C25" s="247" t="s">
         <v>256</v>
       </c>
-      <c r="D25" s="245"/>
-      <c r="E25" s="245"/>
-      <c r="F25" s="245"/>
-      <c r="G25" s="245"/>
-      <c r="H25" s="245"/>
-      <c r="I25" s="245"/>
-      <c r="J25" s="245"/>
-      <c r="K25" s="245"/>
-      <c r="L25" s="245"/>
+      <c r="D25" s="247"/>
+      <c r="E25" s="247"/>
+      <c r="F25" s="247"/>
+      <c r="G25" s="247"/>
+      <c r="H25" s="247"/>
+      <c r="I25" s="247"/>
+      <c r="J25" s="247"/>
+      <c r="K25" s="247"/>
+      <c r="L25" s="247"/>
     </row>
     <row r="26" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B26" s="16" t="s">
@@ -21971,18 +22094,18 @@
       </c>
     </row>
     <row r="31" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="C31" s="245" t="s">
+      <c r="C31" s="247" t="s">
         <v>75</v>
       </c>
-      <c r="D31" s="245"/>
-      <c r="E31" s="245"/>
-      <c r="F31" s="245"/>
-      <c r="G31" s="245"/>
-      <c r="H31" s="245"/>
-      <c r="I31" s="245"/>
-      <c r="J31" s="245"/>
-      <c r="K31" s="245"/>
-      <c r="L31" s="245"/>
+      <c r="D31" s="247"/>
+      <c r="E31" s="247"/>
+      <c r="F31" s="247"/>
+      <c r="G31" s="247"/>
+      <c r="H31" s="247"/>
+      <c r="I31" s="247"/>
+      <c r="J31" s="247"/>
+      <c r="K31" s="247"/>
+      <c r="L31" s="247"/>
     </row>
     <row r="32" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B32" s="16" t="s">
@@ -22144,18 +22267,57 @@
   <sheetPr>
     <tabColor theme="6" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="B13"/>
+  <dimension ref="B5:H13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="16384" width="10.83203125" style="1"/>
+    <col min="1" max="7" width="10.83203125" style="1"/>
+    <col min="8" max="8" width="16.33203125" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="13" spans="2:2" s="4" customFormat="1" ht="49" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="H5" s="132" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="H6" s="256" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="H7" s="256" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="H8" s="256" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="H9" s="256" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="H10" s="257" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8" s="4" customFormat="1" ht="49" x14ac:dyDescent="0.2">
       <c r="B13" s="3" t="s">
         <v>161</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="H6" location="Overview!B3" display="Overview'!B3" xr:uid="{702C65B7-0DC1-1945-AD20-6DB846C06AF6}"/>
+    <hyperlink ref="H8" location="'Analysis -&gt;'!B13" display="'Analysis -&gt;'!B13" xr:uid="{F5D2F504-8FE9-7242-BDA8-545FF0614D91}"/>
+    <hyperlink ref="H9" location="'Forecast -&gt;'!B13" display="'Forecast -&gt;'!B13" xr:uid="{1FC82CE0-4B7E-CE42-BCD0-D7A6C18353B0}"/>
+    <hyperlink ref="H10" location="'Valuation -&gt;'!B13" display="'Valuation -&gt;'!B13" xr:uid="{A12E42FD-5CA7-BF40-8E34-014BB797E49B}"/>
+    <hyperlink ref="H7" location="'Financials -&gt;'!B13" display="'Financials -&gt;'!B13" xr:uid="{F50AA8E2-EDCE-4048-AC38-D5A6282DBC28}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -22193,10 +22355,10 @@
     </row>
     <row r="3" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="239" t="s">
+      <c r="B4" s="241" t="s">
         <v>163</v>
       </c>
-      <c r="C4" s="239"/>
+      <c r="C4" s="241"/>
     </row>
     <row r="5" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
@@ -22213,7 +22375,7 @@
       </c>
       <c r="C6" s="133">
         <f ca="1">Overview!C5</f>
-        <v>336.64</v>
+        <v>340.97</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22222,7 +22384,7 @@
       </c>
       <c r="C7" s="134">
         <f ca="1">C5*C6</f>
-        <v>4932785.92</v>
+        <v>4996233.41</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22281,10 +22443,10 @@
     </row>
     <row r="14" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="15" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="239" t="s">
+      <c r="B15" s="241" t="s">
         <v>170</v>
       </c>
-      <c r="C15" s="239"/>
+      <c r="C15" s="241"/>
     </row>
     <row r="16" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B16" s="1" t="s">
@@ -22292,7 +22454,7 @@
       </c>
       <c r="C16" s="46">
         <f ca="1">C8/(C8+C7)</f>
-        <v>1.6811205080373922E-2</v>
+        <v>1.6601262650577348E-2</v>
       </c>
     </row>
     <row r="17" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22301,7 +22463,7 @@
       </c>
       <c r="C17" s="46">
         <f ca="1">C7/(C8+C7)</f>
-        <v>0.98318879491962607</v>
+        <v>0.98339873734942262</v>
       </c>
     </row>
     <row r="18" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22328,7 +22490,7 @@
       </c>
       <c r="C20" s="46">
         <f ca="1">(C17*C19)+(C16*C18)</f>
-        <v>9.9899246246220375E-2</v>
+        <v>9.991231211830999E-2</v>
       </c>
     </row>
   </sheetData>
@@ -22373,60 +22535,60 @@
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A3" s="4"/>
-      <c r="C3" s="239" t="s">
+      <c r="C3" s="241" t="s">
         <v>110</v>
       </c>
-      <c r="D3" s="239"/>
-      <c r="E3" s="239"/>
-      <c r="F3" s="239"/>
-      <c r="G3" s="248"/>
-      <c r="H3" s="249" t="s">
+      <c r="D3" s="241"/>
+      <c r="E3" s="241"/>
+      <c r="F3" s="241"/>
+      <c r="G3" s="250"/>
+      <c r="H3" s="251" t="s">
         <v>111</v>
       </c>
-      <c r="I3" s="239"/>
-      <c r="J3" s="239"/>
-      <c r="K3" s="239"/>
-      <c r="L3" s="239"/>
-      <c r="P3" s="250"/>
-      <c r="Q3" s="250"/>
-      <c r="R3" s="250"/>
-      <c r="S3" s="250"/>
-      <c r="T3" s="250"/>
-      <c r="U3" s="250"/>
-      <c r="V3" s="250"/>
-      <c r="W3" s="250"/>
-      <c r="X3" s="250"/>
-      <c r="Y3" s="250"/>
-      <c r="Z3" s="250"/>
+      <c r="I3" s="241"/>
+      <c r="J3" s="241"/>
+      <c r="K3" s="241"/>
+      <c r="L3" s="241"/>
+      <c r="P3" s="252"/>
+      <c r="Q3" s="252"/>
+      <c r="R3" s="252"/>
+      <c r="S3" s="252"/>
+      <c r="T3" s="252"/>
+      <c r="U3" s="252"/>
+      <c r="V3" s="252"/>
+      <c r="W3" s="252"/>
+      <c r="X3" s="252"/>
+      <c r="Y3" s="252"/>
+      <c r="Z3" s="252"/>
       <c r="AB3" s="109"/>
     </row>
     <row r="4" spans="1:28" ht="10" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="5" spans="1:28" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="86"/>
       <c r="B5" s="60"/>
-      <c r="C5" s="245" t="s">
+      <c r="C5" s="247" t="s">
         <v>177</v>
       </c>
-      <c r="D5" s="245"/>
-      <c r="E5" s="245"/>
-      <c r="F5" s="245"/>
-      <c r="G5" s="245"/>
-      <c r="H5" s="245"/>
-      <c r="I5" s="245"/>
-      <c r="J5" s="245"/>
-      <c r="K5" s="245"/>
-      <c r="L5" s="245"/>
-      <c r="P5" s="250"/>
-      <c r="Q5" s="250"/>
-      <c r="R5" s="250"/>
-      <c r="S5" s="250"/>
-      <c r="T5" s="250"/>
-      <c r="U5" s="250"/>
-      <c r="V5" s="250"/>
-      <c r="W5" s="250"/>
-      <c r="X5" s="250"/>
-      <c r="Y5" s="250"/>
-      <c r="Z5" s="250"/>
+      <c r="D5" s="247"/>
+      <c r="E5" s="247"/>
+      <c r="F5" s="247"/>
+      <c r="G5" s="247"/>
+      <c r="H5" s="247"/>
+      <c r="I5" s="247"/>
+      <c r="J5" s="247"/>
+      <c r="K5" s="247"/>
+      <c r="L5" s="247"/>
+      <c r="P5" s="252"/>
+      <c r="Q5" s="252"/>
+      <c r="R5" s="252"/>
+      <c r="S5" s="252"/>
+      <c r="T5" s="252"/>
+      <c r="U5" s="252"/>
+      <c r="V5" s="252"/>
+      <c r="W5" s="252"/>
+      <c r="X5" s="252"/>
+      <c r="Y5" s="252"/>
+      <c r="Z5" s="252"/>
       <c r="AB5" s="110"/>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.2">
@@ -22579,7 +22741,7 @@
       </c>
       <c r="L8" s="126">
         <f ca="1">L7*(1+C14)/(C15-C14)</f>
-        <v>1814217.7237637113</v>
+        <v>1813921.0944197082</v>
       </c>
       <c r="N8" s="91"/>
       <c r="O8" s="16"/>
@@ -22633,23 +22795,23 @@
       <c r="G10" s="138"/>
       <c r="H10" s="126">
         <f ca="1">H7/(1+$C$15)^H9</f>
-        <v>100335.56820693916</v>
+        <v>100334.3763194716</v>
       </c>
       <c r="I10" s="126">
         <f t="shared" ref="I10:L10" ca="1" si="0">I7/(1+$C$15)^I9</f>
-        <v>96919.959281185322</v>
+        <v>96917.656668048818</v>
       </c>
       <c r="J10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>93103.872388012038</v>
+        <v>93100.554481237908</v>
       </c>
       <c r="K10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>89027.311002403832</v>
+        <v>89023.080851623468</v>
       </c>
       <c r="L10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>88281.030454872627</v>
+        <v>88275.787122129885</v>
       </c>
       <c r="N10" s="91"/>
     </row>
@@ -22668,14 +22830,14 @@
       <c r="K11" s="137"/>
       <c r="L11" s="126">
         <f ca="1">L8/(1+C15)^L9</f>
-        <v>1127002.5099671041</v>
+        <v>1126751.3162585828</v>
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="B13" s="239" t="s">
+      <c r="B13" s="241" t="s">
         <v>181</v>
       </c>
-      <c r="C13" s="239"/>
+      <c r="C13" s="241"/>
     </row>
     <row r="14" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B14" s="1" t="s">
@@ -22691,14 +22853,14 @@
       </c>
       <c r="C15" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.9899246246220375E-2</v>
+        <v>9.991231211830999E-2</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B18" s="239" t="s">
+      <c r="B18" s="241" t="s">
         <v>183</v>
       </c>
-      <c r="C18" s="239"/>
+      <c r="C18" s="241"/>
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B19" s="1" t="s">
@@ -22706,7 +22868,7 @@
       </c>
       <c r="C19" s="64">
         <f ca="1">SUM(H10:L10)</f>
-        <v>467667.74133341305</v>
+        <v>467651.45544251165</v>
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.2">
@@ -22715,7 +22877,7 @@
       </c>
       <c r="C20" s="64">
         <f ca="1">L11</f>
-        <v>1127002.5099671041</v>
+        <v>1126751.3162585828</v>
       </c>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.2">
@@ -22724,7 +22886,7 @@
       </c>
       <c r="C21" s="94">
         <f ca="1">C19+C20</f>
-        <v>1594670.251300517</v>
+        <v>1594402.7717010945</v>
       </c>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.2">
@@ -22751,7 +22913,7 @@
       </c>
       <c r="C24" s="94">
         <f ca="1">C21+C22-C23</f>
-        <v>1656843.251300517</v>
+        <v>1656575.7717010945</v>
       </c>
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.2">
@@ -22769,7 +22931,7 @@
       </c>
       <c r="C26" s="235">
         <f ca="1">C24/C25</f>
-        <v>113.07194781276988</v>
+        <v>113.05369355770794</v>
       </c>
     </row>
   </sheetData>
@@ -22812,37 +22974,37 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
-      <c r="C2" s="239" t="s">
+      <c r="C2" s="241" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="239"/>
-      <c r="E2" s="239"/>
-      <c r="F2" s="239"/>
-      <c r="G2" s="248"/>
-      <c r="H2" s="249" t="s">
+      <c r="D2" s="241"/>
+      <c r="E2" s="241"/>
+      <c r="F2" s="241"/>
+      <c r="G2" s="250"/>
+      <c r="H2" s="251" t="s">
         <v>111</v>
       </c>
-      <c r="I2" s="239"/>
-      <c r="J2" s="239"/>
-      <c r="K2" s="239"/>
-      <c r="L2" s="239"/>
+      <c r="I2" s="241"/>
+      <c r="J2" s="241"/>
+      <c r="K2" s="241"/>
+      <c r="L2" s="241"/>
     </row>
     <row r="3" spans="1:14" ht="10" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:14" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="86"/>
       <c r="B4" s="60"/>
-      <c r="C4" s="245" t="s">
+      <c r="C4" s="247" t="s">
         <v>191</v>
       </c>
-      <c r="D4" s="245"/>
-      <c r="E4" s="245"/>
-      <c r="F4" s="245"/>
-      <c r="G4" s="245"/>
-      <c r="H4" s="245"/>
-      <c r="I4" s="245"/>
-      <c r="J4" s="245"/>
-      <c r="K4" s="245"/>
-      <c r="L4" s="245"/>
+      <c r="D4" s="247"/>
+      <c r="E4" s="247"/>
+      <c r="F4" s="247"/>
+      <c r="G4" s="247"/>
+      <c r="H4" s="247"/>
+      <c r="I4" s="247"/>
+      <c r="J4" s="247"/>
+      <c r="K4" s="247"/>
+      <c r="L4" s="247"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B5" s="16" t="s">
@@ -23038,23 +23200,23 @@
       <c r="G9" s="138"/>
       <c r="H9" s="92">
         <f ca="1">DCF!H10</f>
-        <v>100335.56820693916</v>
+        <v>100334.3763194716</v>
       </c>
       <c r="I9" s="92">
         <f ca="1">DCF!I10</f>
-        <v>96919.959281185322</v>
+        <v>96917.656668048818</v>
       </c>
       <c r="J9" s="92">
         <f ca="1">DCF!J10</f>
-        <v>93103.872388012038</v>
+        <v>93100.554481237908</v>
       </c>
       <c r="K9" s="92">
         <f ca="1">DCF!K10</f>
-        <v>89027.311002403832</v>
+        <v>89023.080851623468</v>
       </c>
       <c r="L9" s="92">
         <f ca="1">DCF!L10</f>
-        <v>88281.030454872627</v>
+        <v>88275.787122129885</v>
       </c>
       <c r="N9" s="91"/>
     </row>
@@ -23062,18 +23224,18 @@
       <c r="N10" s="91"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="C11" s="245" t="s">
+      <c r="C11" s="247" t="s">
         <v>119</v>
       </c>
-      <c r="D11" s="245"/>
-      <c r="E11" s="245"/>
-      <c r="F11" s="245"/>
-      <c r="G11" s="245"/>
-      <c r="H11" s="245"/>
-      <c r="I11" s="245"/>
-      <c r="J11" s="245"/>
-      <c r="K11" s="245"/>
-      <c r="L11" s="245"/>
+      <c r="D11" s="247"/>
+      <c r="E11" s="247"/>
+      <c r="F11" s="247"/>
+      <c r="G11" s="247"/>
+      <c r="H11" s="247"/>
+      <c r="I11" s="247"/>
+      <c r="J11" s="247"/>
+      <c r="K11" s="247"/>
+      <c r="L11" s="247"/>
       <c r="N11" s="91"/>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.2">
@@ -23267,18 +23429,18 @@
       <c r="N16" s="91"/>
     </row>
     <row r="17" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="C17" s="245" t="s">
+      <c r="C17" s="247" t="s">
         <v>193</v>
       </c>
-      <c r="D17" s="245"/>
-      <c r="E17" s="245"/>
-      <c r="F17" s="245"/>
-      <c r="G17" s="245"/>
-      <c r="H17" s="245"/>
-      <c r="I17" s="245"/>
-      <c r="J17" s="245"/>
-      <c r="K17" s="245"/>
-      <c r="L17" s="245"/>
+      <c r="D17" s="247"/>
+      <c r="E17" s="247"/>
+      <c r="F17" s="247"/>
+      <c r="G17" s="247"/>
+      <c r="H17" s="247"/>
+      <c r="I17" s="247"/>
+      <c r="J17" s="247"/>
+      <c r="K17" s="247"/>
+      <c r="L17" s="247"/>
       <c r="N17" s="91"/>
     </row>
     <row r="18" spans="2:14" x14ac:dyDescent="0.2">
@@ -23412,18 +23574,18 @@
       <c r="N21" s="91"/>
     </row>
     <row r="22" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="C22" s="245" t="s">
+      <c r="C22" s="247" t="s">
         <v>196</v>
       </c>
-      <c r="D22" s="245"/>
-      <c r="E22" s="245"/>
-      <c r="F22" s="245"/>
-      <c r="G22" s="245"/>
-      <c r="H22" s="245"/>
-      <c r="I22" s="245"/>
-      <c r="J22" s="245"/>
-      <c r="K22" s="245"/>
-      <c r="L22" s="245"/>
+      <c r="D22" s="247"/>
+      <c r="E22" s="247"/>
+      <c r="F22" s="247"/>
+      <c r="G22" s="247"/>
+      <c r="H22" s="247"/>
+      <c r="I22" s="247"/>
+      <c r="J22" s="247"/>
+      <c r="K22" s="247"/>
+      <c r="L22" s="247"/>
       <c r="N22" s="91"/>
     </row>
     <row r="23" spans="2:14" x14ac:dyDescent="0.2">
@@ -23507,18 +23669,18 @@
       <c r="N26" s="91"/>
     </row>
     <row r="27" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="C27" s="245" t="s">
+      <c r="C27" s="247" t="s">
         <v>197</v>
       </c>
-      <c r="D27" s="245"/>
-      <c r="E27" s="245"/>
-      <c r="F27" s="245"/>
-      <c r="G27" s="245"/>
-      <c r="H27" s="245"/>
-      <c r="I27" s="245"/>
-      <c r="J27" s="245"/>
-      <c r="K27" s="245"/>
-      <c r="L27" s="245"/>
+      <c r="D27" s="247"/>
+      <c r="E27" s="247"/>
+      <c r="F27" s="247"/>
+      <c r="G27" s="247"/>
+      <c r="H27" s="247"/>
+      <c r="I27" s="247"/>
+      <c r="J27" s="247"/>
+      <c r="K27" s="247"/>
+      <c r="L27" s="247"/>
       <c r="N27" s="91"/>
     </row>
     <row r="28" spans="2:14" x14ac:dyDescent="0.2">
@@ -23819,10 +23981,10 @@
       <c r="N38" s="91"/>
     </row>
     <row r="39" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B39" s="239" t="s">
+      <c r="B39" s="241" t="s">
         <v>202</v>
       </c>
-      <c r="C39" s="239"/>
+      <c r="C39" s="241"/>
       <c r="N39" s="91"/>
     </row>
     <row r="40" spans="2:14" x14ac:dyDescent="0.2">
@@ -23840,7 +24002,7 @@
       </c>
       <c r="C41" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.9899246246220375E-2</v>
+        <v>9.991231211830999E-2</v>
       </c>
     </row>
     <row r="42" spans="2:14" x14ac:dyDescent="0.2">
@@ -23866,7 +24028,7 @@
       </c>
       <c r="C44" s="24">
         <f ca="1">C43/(1+C41)^5</f>
-        <v>2909052.6046173945</v>
+        <v>2908879.8253612672</v>
       </c>
     </row>
     <row r="45" spans="2:14" x14ac:dyDescent="0.2">
@@ -23875,7 +24037,7 @@
       </c>
       <c r="C45" s="108">
         <f ca="1">SUM(H9:K9)+C44</f>
-        <v>3288439.3154959348</v>
+        <v>3288255.4936816487</v>
       </c>
     </row>
     <row r="46" spans="2:14" x14ac:dyDescent="0.2">
@@ -23902,7 +24064,7 @@
       </c>
       <c r="C48" s="94">
         <f ca="1">C45+C46-C47</f>
-        <v>3350612.3154959348</v>
+        <v>3350428.4936816487</v>
       </c>
     </row>
     <row r="49" spans="2:3" x14ac:dyDescent="0.2">
@@ -23920,14 +24082,14 @@
       </c>
       <c r="C50" s="235">
         <f ca="1">C48/C49</f>
-        <v>228.66391288445607</v>
+        <v>228.65136788928197</v>
       </c>
     </row>
     <row r="52" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B52" s="239" t="s">
+      <c r="B52" s="241" t="s">
         <v>207</v>
       </c>
-      <c r="C52" s="239"/>
+      <c r="C52" s="241"/>
     </row>
     <row r="53" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B53" s="1" t="s">
@@ -23983,10 +24145,10 @@
       </c>
     </row>
     <row r="60" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B60" s="239" t="s">
+      <c r="B60" s="241" t="s">
         <v>316</v>
       </c>
-      <c r="C60" s="239"/>
+      <c r="C60" s="241"/>
     </row>
     <row r="61" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B61" s="1" t="s">
@@ -24003,7 +24165,7 @@
       </c>
       <c r="C62" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.9899246246220375E-2</v>
+        <v>9.991231211830999E-2</v>
       </c>
     </row>
     <row r="63" spans="2:3" x14ac:dyDescent="0.2">
@@ -24029,7 +24191,7 @@
       </c>
       <c r="C65" s="24">
         <f ca="1">C64/(1+C62)^5</f>
-        <v>2471868.8527364335</v>
+        <v>2471722.0394196366</v>
       </c>
     </row>
     <row r="66" spans="2:3" x14ac:dyDescent="0.2">
@@ -24038,7 +24200,7 @@
       </c>
       <c r="C66" s="108">
         <f ca="1">SUM(H9:K9)+C65</f>
-        <v>2851255.5636149738</v>
+        <v>2851097.7077400181</v>
       </c>
     </row>
     <row r="67" spans="2:3" x14ac:dyDescent="0.2">
@@ -24065,7 +24227,7 @@
       </c>
       <c r="C69" s="94">
         <f ca="1">C66+C67-C68</f>
-        <v>2913428.5636149738</v>
+        <v>2913270.7077400181</v>
       </c>
     </row>
     <row r="70" spans="2:3" x14ac:dyDescent="0.2">
@@ -24083,14 +24245,14 @@
       </c>
       <c r="C71" s="235">
         <f ca="1">C69/C70</f>
-        <v>198.82812827509545</v>
+        <v>198.8173553361099</v>
       </c>
     </row>
     <row r="73" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B73" s="239" t="s">
+      <c r="B73" s="241" t="s">
         <v>414</v>
       </c>
-      <c r="C73" s="239"/>
+      <c r="C73" s="241"/>
     </row>
     <row r="74" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B74" s="1" t="s">
@@ -24107,7 +24269,7 @@
       </c>
       <c r="C75" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.9899246246220375E-2</v>
+        <v>9.991231211830999E-2</v>
       </c>
     </row>
     <row r="76" spans="2:3" x14ac:dyDescent="0.2">
@@ -24133,7 +24295,7 @@
       </c>
       <c r="C78" s="24">
         <f ca="1">C77/(1+C75)^5</f>
-        <v>2676573.1115039121</v>
+        <v>2676414.1400537421</v>
       </c>
     </row>
     <row r="79" spans="2:3" x14ac:dyDescent="0.2">
@@ -24142,7 +24304,7 @@
       </c>
       <c r="C79" s="108">
         <f ca="1">SUM(H9:K9)+C78</f>
-        <v>3055959.8223824524</v>
+        <v>3055789.8083741236</v>
       </c>
     </row>
     <row r="80" spans="2:3" x14ac:dyDescent="0.2">
@@ -24169,7 +24331,7 @@
       </c>
       <c r="C82" s="94">
         <f ca="1">C79+C80-C81</f>
-        <v>3118132.8223824524</v>
+        <v>3117962.8083741236</v>
       </c>
     </row>
     <row r="83" spans="2:3" x14ac:dyDescent="0.2">
@@ -24187,7 +24349,7 @@
       </c>
       <c r="C84" s="235">
         <f ca="1">C82/C83</f>
-        <v>212.79825444499096</v>
+        <v>212.78665176920245</v>
       </c>
     </row>
   </sheetData>
@@ -24240,10 +24402,10 @@
       <c r="N3" s="91"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B4" s="239" t="s">
+      <c r="B4" s="241" t="s">
         <v>211</v>
       </c>
-      <c r="C4" s="239"/>
+      <c r="C4" s="241"/>
       <c r="N4" s="91"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
@@ -24252,7 +24414,7 @@
       </c>
       <c r="C5" s="133">
         <f ca="1">DCF!C26</f>
-        <v>113.07194781276988</v>
+        <v>113.05369355770794</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -24261,7 +24423,7 @@
       </c>
       <c r="C6" s="133">
         <f ca="1">Multiples!C50</f>
-        <v>228.66391288445607</v>
+        <v>228.65136788928197</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
@@ -24279,7 +24441,7 @@
       </c>
       <c r="C8" s="133">
         <f ca="1">Multiples!C71</f>
-        <v>198.82812827509545</v>
+        <v>198.8173553361099</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
@@ -24288,7 +24450,7 @@
       </c>
       <c r="C9" s="133">
         <f ca="1">Multiples!C84</f>
-        <v>212.79825444499096</v>
+        <v>212.78665176920245</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
@@ -24297,7 +24459,7 @@
       </c>
       <c r="C10" s="235">
         <f ca="1">AVERAGE(C5:C9)</f>
-        <v>190.72369711196706</v>
+        <v>190.71306213896509</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
@@ -24306,7 +24468,7 @@
       </c>
       <c r="C11" s="133">
         <f ca="1">Overview!C5</f>
-        <v>336.64</v>
+        <v>340.97</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.2">
@@ -24315,7 +24477,7 @@
       </c>
       <c r="C12" s="149">
         <f ca="1">(C10-C11)/C11</f>
-        <v>-0.43344909365504081</v>
+        <v>-0.44067495046788552</v>
       </c>
     </row>
   </sheetData>
@@ -24331,18 +24493,57 @@
   <sheetPr>
     <tabColor theme="6" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="B13"/>
+  <dimension ref="B5:H13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="16384" width="10.83203125" style="1"/>
+    <col min="1" max="7" width="10.83203125" style="1"/>
+    <col min="8" max="8" width="16.33203125" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="13" spans="2:2" s="4" customFormat="1" ht="49" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="H5" s="132" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="H6" s="256" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="H7" s="256" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="H8" s="256" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="H9" s="256" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="H10" s="257" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8" s="4" customFormat="1" ht="49" x14ac:dyDescent="0.2">
       <c r="B13" s="3" t="s">
         <v>14</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="H6" location="Overview!B3" display="Overview'!B3" xr:uid="{BFEE9001-6FF4-F648-BE8B-7653ADE21047}"/>
+    <hyperlink ref="H8" location="'Analysis -&gt;'!B13" display="'Analysis -&gt;'!B13" xr:uid="{78C2AB09-CE06-8C41-B9C8-8FA362F2C5FA}"/>
+    <hyperlink ref="H9" location="'Forecast -&gt;'!B13" display="'Forecast -&gt;'!B13" xr:uid="{E448F36E-1A10-C24C-8CE0-3533F5487BFF}"/>
+    <hyperlink ref="H10" location="'Valuation -&gt;'!B13" display="'Valuation -&gt;'!B13" xr:uid="{2C295BB6-FDE9-D04D-A867-57B3ACA53A98}"/>
+    <hyperlink ref="H7" location="'Financials -&gt;'!B13" display="'Financials -&gt;'!B13" xr:uid="{8132A921-D1D1-1848-8BC4-49C4E1A83BB7}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -24371,37 +24572,37 @@
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
-      <c r="C2" s="239" t="s">
+      <c r="C2" s="241" t="s">
         <v>110</v>
       </c>
-      <c r="D2" s="239"/>
-      <c r="E2" s="239"/>
-      <c r="F2" s="239"/>
-      <c r="G2" s="248"/>
-      <c r="H2" s="249" t="s">
+      <c r="D2" s="241"/>
+      <c r="E2" s="241"/>
+      <c r="F2" s="241"/>
+      <c r="G2" s="250"/>
+      <c r="H2" s="251" t="s">
         <v>111</v>
       </c>
-      <c r="I2" s="239"/>
-      <c r="J2" s="239"/>
-      <c r="K2" s="239"/>
-      <c r="L2" s="239"/>
+      <c r="I2" s="241"/>
+      <c r="J2" s="241"/>
+      <c r="K2" s="241"/>
+      <c r="L2" s="241"/>
     </row>
     <row r="3" spans="1:14" ht="10" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:14" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="86"/>
       <c r="B4" s="60"/>
-      <c r="C4" s="245" t="s">
+      <c r="C4" s="247" t="s">
         <v>191</v>
       </c>
-      <c r="D4" s="245"/>
-      <c r="E4" s="245"/>
-      <c r="F4" s="245"/>
-      <c r="G4" s="245"/>
-      <c r="H4" s="245"/>
-      <c r="I4" s="245"/>
-      <c r="J4" s="245"/>
-      <c r="K4" s="245"/>
-      <c r="L4" s="245"/>
+      <c r="D4" s="247"/>
+      <c r="E4" s="247"/>
+      <c r="F4" s="247"/>
+      <c r="G4" s="247"/>
+      <c r="H4" s="247"/>
+      <c r="I4" s="247"/>
+      <c r="J4" s="247"/>
+      <c r="K4" s="247"/>
+      <c r="L4" s="247"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="B5" s="16" t="s">
@@ -24514,18 +24715,18 @@
       <c r="N8" s="91"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="C9" s="245" t="s">
+      <c r="C9" s="247" t="s">
         <v>119</v>
       </c>
-      <c r="D9" s="245"/>
-      <c r="E9" s="245"/>
-      <c r="F9" s="245"/>
-      <c r="G9" s="245"/>
-      <c r="H9" s="245"/>
-      <c r="I9" s="245"/>
-      <c r="J9" s="245"/>
-      <c r="K9" s="245"/>
-      <c r="L9" s="245"/>
+      <c r="D9" s="247"/>
+      <c r="E9" s="247"/>
+      <c r="F9" s="247"/>
+      <c r="G9" s="247"/>
+      <c r="H9" s="247"/>
+      <c r="I9" s="247"/>
+      <c r="J9" s="247"/>
+      <c r="K9" s="247"/>
+      <c r="L9" s="247"/>
       <c r="N9" s="91"/>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
@@ -24646,18 +24847,18 @@
       <c r="N13" s="91"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="C14" s="245" t="s">
+      <c r="C14" s="247" t="s">
         <v>397</v>
       </c>
-      <c r="D14" s="245"/>
-      <c r="E14" s="245"/>
-      <c r="F14" s="245"/>
-      <c r="G14" s="245"/>
-      <c r="H14" s="245"/>
-      <c r="I14" s="245"/>
-      <c r="J14" s="245"/>
-      <c r="K14" s="245"/>
-      <c r="L14" s="245"/>
+      <c r="D14" s="247"/>
+      <c r="E14" s="247"/>
+      <c r="F14" s="247"/>
+      <c r="G14" s="247"/>
+      <c r="H14" s="247"/>
+      <c r="I14" s="247"/>
+      <c r="J14" s="247"/>
+      <c r="K14" s="247"/>
+      <c r="L14" s="247"/>
       <c r="N14" s="91"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.2">
@@ -24747,10 +24948,10 @@
       <c r="N19" s="91"/>
     </row>
     <row r="20" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B20" s="239" t="s">
+      <c r="B20" s="241" t="s">
         <v>399</v>
       </c>
-      <c r="C20" s="239"/>
+      <c r="C20" s="241"/>
       <c r="N20" s="91"/>
     </row>
     <row r="21" spans="2:14" x14ac:dyDescent="0.2">
@@ -24851,60 +25052,60 @@
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A3" s="4"/>
-      <c r="C3" s="239" t="s">
+      <c r="C3" s="241" t="s">
         <v>110</v>
       </c>
-      <c r="D3" s="239"/>
-      <c r="E3" s="239"/>
-      <c r="F3" s="239"/>
-      <c r="G3" s="248"/>
-      <c r="H3" s="249" t="s">
+      <c r="D3" s="241"/>
+      <c r="E3" s="241"/>
+      <c r="F3" s="241"/>
+      <c r="G3" s="250"/>
+      <c r="H3" s="251" t="s">
         <v>111</v>
       </c>
-      <c r="I3" s="239"/>
-      <c r="J3" s="239"/>
-      <c r="K3" s="239"/>
-      <c r="L3" s="239"/>
-      <c r="P3" s="250"/>
-      <c r="Q3" s="250"/>
-      <c r="R3" s="250"/>
-      <c r="S3" s="250"/>
-      <c r="T3" s="250"/>
-      <c r="U3" s="250"/>
-      <c r="V3" s="250"/>
-      <c r="W3" s="250"/>
-      <c r="X3" s="250"/>
-      <c r="Y3" s="250"/>
-      <c r="Z3" s="250"/>
+      <c r="I3" s="241"/>
+      <c r="J3" s="241"/>
+      <c r="K3" s="241"/>
+      <c r="L3" s="241"/>
+      <c r="P3" s="252"/>
+      <c r="Q3" s="252"/>
+      <c r="R3" s="252"/>
+      <c r="S3" s="252"/>
+      <c r="T3" s="252"/>
+      <c r="U3" s="252"/>
+      <c r="V3" s="252"/>
+      <c r="W3" s="252"/>
+      <c r="X3" s="252"/>
+      <c r="Y3" s="252"/>
+      <c r="Z3" s="252"/>
       <c r="AB3" s="109"/>
     </row>
     <row r="4" spans="1:28" ht="10" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="5" spans="1:28" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="86"/>
       <c r="B5" s="60"/>
-      <c r="C5" s="245" t="s">
+      <c r="C5" s="247" t="s">
         <v>177</v>
       </c>
-      <c r="D5" s="245"/>
-      <c r="E5" s="245"/>
-      <c r="F5" s="245"/>
-      <c r="G5" s="245"/>
-      <c r="H5" s="245"/>
-      <c r="I5" s="245"/>
-      <c r="J5" s="245"/>
-      <c r="K5" s="245"/>
-      <c r="L5" s="245"/>
-      <c r="P5" s="250"/>
-      <c r="Q5" s="250"/>
-      <c r="R5" s="250"/>
-      <c r="S5" s="250"/>
-      <c r="T5" s="250"/>
-      <c r="U5" s="250"/>
-      <c r="V5" s="250"/>
-      <c r="W5" s="250"/>
-      <c r="X5" s="250"/>
-      <c r="Y5" s="250"/>
-      <c r="Z5" s="250"/>
+      <c r="D5" s="247"/>
+      <c r="E5" s="247"/>
+      <c r="F5" s="247"/>
+      <c r="G5" s="247"/>
+      <c r="H5" s="247"/>
+      <c r="I5" s="247"/>
+      <c r="J5" s="247"/>
+      <c r="K5" s="247"/>
+      <c r="L5" s="247"/>
+      <c r="P5" s="252"/>
+      <c r="Q5" s="252"/>
+      <c r="R5" s="252"/>
+      <c r="S5" s="252"/>
+      <c r="T5" s="252"/>
+      <c r="U5" s="252"/>
+      <c r="V5" s="252"/>
+      <c r="W5" s="252"/>
+      <c r="X5" s="252"/>
+      <c r="Y5" s="252"/>
+      <c r="Z5" s="252"/>
       <c r="AB5" s="110"/>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.2">
@@ -25039,7 +25240,7 @@
       <c r="K8" s="137"/>
       <c r="L8" s="126">
         <f ca="1">L7*(1+C20)/(C21-C20)</f>
-        <v>6246960.166815904</v>
+        <v>6245938.7724859826</v>
       </c>
       <c r="N8" s="91"/>
       <c r="O8" s="16"/>
@@ -25093,23 +25294,23 @@
       <c r="G10" s="138"/>
       <c r="H10" s="126">
         <f ca="1">H7/(1+$C$21)^H9</f>
-        <v>110976.89851545423</v>
+        <v>110975.58021949106</v>
       </c>
       <c r="I10" s="126">
         <f t="shared" ref="I10:L10" ca="1" si="1">I7/(1+$C$21)^I9</f>
-        <v>142769.72362268073</v>
+        <v>142766.33171616792</v>
       </c>
       <c r="J10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>183670.60402627985</v>
+        <v>183664.05862783748</v>
       </c>
       <c r="K10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>236288.82880333104</v>
+        <v>236277.60149159603</v>
       </c>
       <c r="L10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>303981.20000335656</v>
+        <v>303963.14544994972</v>
       </c>
       <c r="N10" s="91"/>
     </row>
@@ -25128,15 +25329,15 @@
       <c r="K11" s="137"/>
       <c r="L11" s="126">
         <f ca="1">L8/(1+C21)^L9</f>
-        <v>3880647.672794424</v>
+        <v>3879782.7285979628</v>
       </c>
     </row>
     <row r="13" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="14" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="B14" s="252" t="s">
+      <c r="B14" s="254" t="s">
         <v>219</v>
       </c>
-      <c r="C14" s="253"/>
+      <c r="C14" s="255"/>
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B15" s="150" t="s">
@@ -25144,7 +25345,7 @@
       </c>
       <c r="C15" s="151">
         <f ca="1">Overview!C5</f>
-        <v>336.64</v>
+        <v>340.97</v>
       </c>
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.2">
@@ -25153,7 +25354,7 @@
       </c>
       <c r="C16" s="151">
         <f ca="1">C36</f>
-        <v>337.15964970299615</v>
+        <v>337.09760491318383</v>
       </c>
     </row>
     <row r="17" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -25163,20 +25364,20 @@
       <c r="C17" s="153">
         <v>0.41499999999999998</v>
       </c>
-      <c r="E17" s="251" t="s">
+      <c r="E17" s="253" t="s">
         <v>222</v>
       </c>
-      <c r="F17" s="251"/>
-      <c r="G17" s="251"/>
-      <c r="H17" s="251"/>
-      <c r="I17" s="251"/>
+      <c r="F17" s="253"/>
+      <c r="G17" s="253"/>
+      <c r="H17" s="253"/>
+      <c r="I17" s="253"/>
     </row>
     <row r="18" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B19" s="252" t="s">
+      <c r="B19" s="254" t="s">
         <v>181</v>
       </c>
-      <c r="C19" s="253"/>
+      <c r="C19" s="255"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B20" s="154" t="s">
@@ -25192,7 +25393,7 @@
       </c>
       <c r="C21" s="216">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.9899246246220375E-2</v>
+        <v>9.991231211830999E-2</v>
       </c>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.2">
@@ -25210,7 +25411,7 @@
       </c>
       <c r="C23" s="156">
         <f ca="1">C15*C22</f>
-        <v>4912924.16</v>
+        <v>4976116.1800000006</v>
       </c>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.2">
@@ -25237,15 +25438,15 @@
       </c>
       <c r="C26" s="157">
         <f ca="1">C23+C25-C24</f>
-        <v>4850751.16</v>
+        <v>4913943.1800000006</v>
       </c>
     </row>
     <row r="27" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="28" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B28" s="252" t="s">
+      <c r="B28" s="254" t="s">
         <v>183</v>
       </c>
-      <c r="C28" s="253"/>
+      <c r="C28" s="255"/>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B29" s="154" t="s">
@@ -25253,7 +25454,7 @@
       </c>
       <c r="C29" s="156">
         <f ca="1">SUM(H10:L10)</f>
-        <v>977687.25497110235</v>
+        <v>977646.71750504221</v>
       </c>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
@@ -25262,7 +25463,7 @@
       </c>
       <c r="C30" s="156">
         <f ca="1">L11</f>
-        <v>3880647.672794424</v>
+        <v>3879782.7285979628</v>
       </c>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.2">
@@ -25271,7 +25472,7 @@
       </c>
       <c r="C31" s="159">
         <f ca="1">C29+C30</f>
-        <v>4858334.9277655259</v>
+        <v>4857429.4461030047</v>
       </c>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.2">
@@ -25298,7 +25499,7 @@
       </c>
       <c r="C34" s="159">
         <f ca="1">C31+C32-C33</f>
-        <v>4920507.9277655259</v>
+        <v>4919602.4461030047</v>
       </c>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.2">
@@ -25316,7 +25517,7 @@
       </c>
       <c r="C36" s="162">
         <f ca="1">C34/C35</f>
-        <v>337.15964970299615</v>
+        <v>337.09760491318383</v>
       </c>
     </row>
   </sheetData>
@@ -31835,7 +32036,7 @@
       </c>
       <c r="AC114" s="63">
         <f ca="1">Overview!C5</f>
-        <v>336.64</v>
+        <v>340.97</v>
       </c>
     </row>
     <row r="115" spans="1:31" x14ac:dyDescent="0.2">
@@ -31906,7 +32107,7 @@
       </c>
       <c r="AC115" s="65">
         <f ca="1">AC114/AC84</f>
-        <v>336.64</v>
+        <v>340.97</v>
       </c>
     </row>
     <row r="117" spans="1:31" x14ac:dyDescent="0.2">
@@ -32820,7 +33021,7 @@
       <c r="AA140" s="49"/>
       <c r="AC140" s="72">
         <f ca="1">AC115/Statement!AC25</f>
-        <v>38.60550458715597</v>
+        <v>39.102064220183493</v>
       </c>
     </row>
     <row r="141" spans="2:29" x14ac:dyDescent="0.2">
@@ -32857,7 +33058,7 @@
       <c r="AA141" s="49"/>
       <c r="AC141" s="72">
         <f ca="1">AC115/(Statement!AC5/Statement!AC21)</f>
-        <v>10.657397771746464</v>
+        <v>10.79447753752493</v>
       </c>
     </row>
     <row r="142" spans="2:29" x14ac:dyDescent="0.2">
@@ -32918,7 +33119,7 @@
       </c>
       <c r="AC142" s="72">
         <f ca="1">AC115/(Statement!AC48/Statement!AC74)</f>
-        <v>45.693119047619042</v>
+        <v>46.280842447916669</v>
       </c>
     </row>
     <row r="143" spans="2:29" x14ac:dyDescent="0.2">
@@ -32979,7 +33180,7 @@
       </c>
       <c r="AC143" s="141">
         <f ca="1">Statement!AC115*Statement!AC77</f>
-        <v>4932785.92</v>
+        <v>4996233.41</v>
       </c>
     </row>
     <row r="144" spans="2:29" x14ac:dyDescent="0.2">
@@ -33040,7 +33241,7 @@
       </c>
       <c r="AC144" s="141">
         <f ca="1">AC143+AC106-AC105+AC47+AC44</f>
-        <v>4870612.92</v>
+        <v>4934060.41</v>
       </c>
     </row>
     <row r="145" spans="2:29" x14ac:dyDescent="0.2">
@@ -33077,7 +33278,7 @@
       <c r="AA145" s="49"/>
       <c r="AC145" s="177">
         <f ca="1">AC144/AC5</f>
-        <v>10.433532452342751</v>
+        <v>10.569445828504595</v>
       </c>
     </row>
     <row r="146" spans="2:29" x14ac:dyDescent="0.2">
@@ -33114,7 +33315,7 @@
       <c r="AA146" s="49"/>
       <c r="AC146" s="177">
         <f ca="1">AC144/AC11</f>
-        <v>31.451920262948875</v>
+        <v>31.86163161327401</v>
       </c>
     </row>
     <row r="147" spans="2:29" x14ac:dyDescent="0.2">
@@ -33249,7 +33450,7 @@
       <c r="AA149" s="49"/>
       <c r="AC149" s="72">
         <f t="shared" ref="AC149:AC150" ca="1" si="137">AC143/AC147</f>
-        <v>40.111451084349106</v>
+        <v>40.627380811045967</v>
       </c>
     </row>
     <row r="150" spans="2:29" x14ac:dyDescent="0.2">
@@ -33286,7 +33487,7 @@
       <c r="AA150" s="49"/>
       <c r="AC150" s="72">
         <f t="shared" ca="1" si="137"/>
-        <v>39.763624267140635</v>
+        <v>40.281608798962793</v>
       </c>
     </row>
     <row r="151" spans="2:29" x14ac:dyDescent="0.2">
@@ -33323,7 +33524,7 @@
       <c r="AA151" s="49"/>
       <c r="AC151" s="74">
         <f t="shared" ref="AC151" ca="1" si="140">AC147/AC143</f>
-        <v>2.4930536616517101E-2</v>
+        <v>2.4613942125654212E-2</v>
       </c>
     </row>
     <row r="152" spans="2:29" x14ac:dyDescent="0.2">
@@ -33360,7 +33561,7 @@
       <c r="AA152" s="49"/>
       <c r="AC152" s="74">
         <f ca="1">AC25/AC115</f>
-        <v>2.5903041825095056E-2</v>
+        <v>2.5574097427926205E-2</v>
       </c>
     </row>
     <row r="153" spans="2:29" x14ac:dyDescent="0.2">
@@ -33397,7 +33598,7 @@
       <c r="AA153" s="49"/>
       <c r="AC153" s="149">
         <f ca="1">AC81/AC115</f>
-        <v>3.1190589353612169E-3</v>
+        <v>3.0794498049681791E-3</v>
       </c>
     </row>
     <row r="154" spans="2:29" x14ac:dyDescent="0.2">
@@ -33434,7 +33635,7 @@
       <c r="AA154" s="49"/>
       <c r="AC154" s="149">
         <f ca="1">-AC62/AC143</f>
-        <v>1.6669282092015052E-2</v>
+        <v>1.6457597804663014E-2</v>
       </c>
     </row>
     <row r="155" spans="2:29" x14ac:dyDescent="0.2">
@@ -33471,7 +33672,7 @@
       <c r="AA155" s="49"/>
       <c r="AC155" s="149">
         <f ca="1">-(AC62+AC63)/AC143</f>
-        <v>1.9839904181367756E-2</v>
+        <v>1.958795595980773E-2</v>
       </c>
     </row>
     <row r="156" spans="2:29" x14ac:dyDescent="0.2">
@@ -33974,7 +34175,7 @@
       <c r="AA166" s="49"/>
       <c r="AC166" s="149">
         <f ca="1">(AC105-AC106)/AC143</f>
-        <v>1.2604033705967113E-2</v>
+        <v>1.2443974269808984E-2</v>
       </c>
     </row>
     <row r="167" spans="1:31" x14ac:dyDescent="0.2">
@@ -35936,18 +36137,57 @@
   <sheetPr>
     <tabColor theme="6" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="B13"/>
+  <dimension ref="B5:H13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="16384" width="10.83203125" style="1"/>
+    <col min="1" max="7" width="10.83203125" style="1"/>
+    <col min="8" max="8" width="15.33203125" style="1" customWidth="1"/>
+    <col min="9" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="13" spans="2:2" s="4" customFormat="1" ht="49" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="H5" s="132" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="H6" s="256" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="H7" s="256" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="H8" s="256" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="H9" s="256" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="H10" s="257" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8" s="4" customFormat="1" ht="49" x14ac:dyDescent="0.2">
       <c r="B13" s="3" t="s">
         <v>226</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="H6" location="Overview!B3" display="Overview'!B3" xr:uid="{A080AF01-DFE7-3744-909C-DBF9BFA33E62}"/>
+    <hyperlink ref="H8" location="'Analysis -&gt;'!B13" display="'Analysis -&gt;'!B13" xr:uid="{A031DF02-925C-E84E-9F77-697F34179C56}"/>
+    <hyperlink ref="H9" location="'Forecast -&gt;'!B13" display="'Forecast -&gt;'!B13" xr:uid="{D40DD6AD-121C-DA4E-9EA5-D10A20FFC96A}"/>
+    <hyperlink ref="H10" location="'Valuation -&gt;'!B13" display="'Valuation -&gt;'!B13" xr:uid="{1037D27B-0ADB-FB4A-8CB4-85CE0D3ABA2D}"/>
+    <hyperlink ref="H7" location="'Financials -&gt;'!B13" display="'Financials -&gt;'!B13" xr:uid="{24BEE560-CF54-994E-B69A-9DA0A678B7B6}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -35971,15 +36211,15 @@
       </c>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B4" s="239" t="s">
+      <c r="B4" s="241" t="s">
         <v>227</v>
       </c>
-      <c r="C4" s="239"/>
-      <c r="E4" s="239" t="s">
+      <c r="C4" s="241"/>
+      <c r="E4" s="241" t="s">
         <v>234</v>
       </c>
-      <c r="F4" s="239"/>
-      <c r="G4" s="239"/>
+      <c r="F4" s="241"/>
+      <c r="G4" s="241"/>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B5" s="20" t="s">
@@ -35987,7 +36227,7 @@
       </c>
       <c r="C5" s="166">
         <f ca="1">Overview!C5</f>
-        <v>336.64</v>
+        <v>340.97</v>
       </c>
       <c r="E5" s="12"/>
       <c r="F5" s="132" t="s">
@@ -36003,7 +36243,7 @@
       </c>
       <c r="C6" s="167">
         <f ca="1">Statement!AC143</f>
-        <v>4932785.92</v>
+        <v>4996233.41</v>
       </c>
       <c r="E6" s="20" t="s">
         <v>19</v>
@@ -36023,7 +36263,7 @@
       </c>
       <c r="C7" s="167">
         <f ca="1">Statement!AC144</f>
-        <v>4870612.92</v>
+        <v>4934060.41</v>
       </c>
       <c r="E7" s="20" t="s">
         <v>29</v>
@@ -36043,7 +36283,7 @@
       </c>
       <c r="C8" s="168">
         <f ca="1">Statement!AC140</f>
-        <v>38.60550458715597</v>
+        <v>39.102064220183493</v>
       </c>
       <c r="E8" s="20" t="s">
         <v>237</v>
@@ -36063,7 +36303,7 @@
       </c>
       <c r="C9" s="168">
         <f ca="1">Statement!AC141</f>
-        <v>10.657397771746464</v>
+        <v>10.79447753752493</v>
       </c>
       <c r="E9" s="20" t="s">
         <v>238</v>
@@ -36083,7 +36323,7 @@
       </c>
       <c r="C10" s="168">
         <f ca="1">Statement!AC142</f>
-        <v>45.693119047619042</v>
+        <v>46.280842447916669</v>
       </c>
       <c r="E10" s="20" t="s">
         <v>1</v>
@@ -36103,7 +36343,7 @@
       </c>
       <c r="C11" s="168">
         <f ca="1">Statement!AC145</f>
-        <v>10.433532452342751</v>
+        <v>10.569445828504595</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.2">
@@ -36112,18 +36352,18 @@
       </c>
       <c r="C12" s="168">
         <f ca="1">Statement!AC146</f>
-        <v>31.451920262948875</v>
+        <v>31.86163161327401</v>
       </c>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B15" s="239" t="s">
+      <c r="B15" s="241" t="s">
         <v>75</v>
       </c>
-      <c r="C15" s="239"/>
-      <c r="E15" s="239" t="s">
+      <c r="C15" s="241"/>
+      <c r="E15" s="241" t="s">
         <v>240</v>
       </c>
-      <c r="F15" s="239"/>
+      <c r="F15" s="241"/>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B16" s="20" t="s">
@@ -36174,14 +36414,14 @@
       </c>
     </row>
     <row r="21" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B21" s="239" t="s">
+      <c r="B21" s="241" t="s">
         <v>239</v>
       </c>
-      <c r="C21" s="239"/>
-      <c r="E21" s="239" t="s">
+      <c r="C21" s="241"/>
+      <c r="E21" s="241" t="s">
         <v>243</v>
       </c>
-      <c r="F21" s="239"/>
+      <c r="F21" s="241"/>
     </row>
     <row r="22" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B22" s="20" t="s">
@@ -36250,14 +36490,14 @@
       </c>
     </row>
     <row r="29" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B29" s="239" t="s">
+      <c r="B29" s="241" t="s">
         <v>244</v>
       </c>
-      <c r="C29" s="239"/>
-      <c r="E29" s="239" t="s">
+      <c r="C29" s="241"/>
+      <c r="E29" s="241" t="s">
         <v>250</v>
       </c>
-      <c r="F29" s="239"/>
+      <c r="F29" s="241"/>
     </row>
     <row r="30" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B30" s="20" t="s">
@@ -36333,14 +36573,14 @@
       </c>
     </row>
     <row r="37" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B37" s="239" t="s">
+      <c r="B37" s="241" t="s">
         <v>262</v>
       </c>
-      <c r="C37" s="239"/>
-      <c r="E37" s="239" t="s">
+      <c r="C37" s="241"/>
+      <c r="E37" s="241" t="s">
         <v>265</v>
       </c>
-      <c r="F37" s="239"/>
+      <c r="F37" s="241"/>
     </row>
     <row r="38" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B38" s="20" t="s">
@@ -36348,7 +36588,7 @@
       </c>
       <c r="C38" s="169">
         <f ca="1">Statement!AC152</f>
-        <v>2.5903041825095056E-2</v>
+        <v>2.5574097427926205E-2</v>
       </c>
       <c r="E38" s="20" t="s">
         <v>264</v>
@@ -36364,7 +36604,7 @@
       </c>
       <c r="C39" s="209">
         <f ca="1">Statement!AC151</f>
-        <v>2.4930536616517101E-2</v>
+        <v>2.4613942125654212E-2</v>
       </c>
       <c r="E39" s="20" t="s">
         <v>266</v>
@@ -36380,7 +36620,7 @@
       </c>
       <c r="C40" s="169">
         <f ca="1">Statement!AC153</f>
-        <v>3.1190589353612169E-3</v>
+        <v>3.0794498049681791E-3</v>
       </c>
       <c r="E40" s="20" t="s">
         <v>267</v>
@@ -36396,7 +36636,7 @@
       </c>
       <c r="C41" s="169">
         <f ca="1">Statement!AC154</f>
-        <v>1.6669282092015052E-2</v>
+        <v>1.6457597804663014E-2</v>
       </c>
     </row>
     <row r="42" spans="2:6" x14ac:dyDescent="0.2">
@@ -36405,18 +36645,18 @@
       </c>
       <c r="C42" s="169">
         <f ca="1">Statement!AC155</f>
-        <v>1.9839904181367756E-2</v>
+        <v>1.958795595980773E-2</v>
       </c>
     </row>
     <row r="45" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B45" s="239" t="s">
+      <c r="B45" s="241" t="s">
         <v>273</v>
       </c>
-      <c r="C45" s="239"/>
-      <c r="E45" s="239" t="s">
+      <c r="C45" s="241"/>
+      <c r="E45" s="241" t="s">
         <v>279</v>
       </c>
-      <c r="F45" s="239"/>
+      <c r="F45" s="241"/>
     </row>
     <row r="46" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B46" s="20" t="s">
@@ -36449,18 +36689,18 @@
       </c>
       <c r="F48" s="169">
         <f ca="1">Statement!AC166</f>
-        <v>1.2604033705967113E-2</v>
+        <v>1.2443974269808984E-2</v>
       </c>
     </row>
     <row r="51" spans="2:6" x14ac:dyDescent="0.2">
-      <c r="B51" s="239" t="s">
+      <c r="B51" s="241" t="s">
         <v>276</v>
       </c>
-      <c r="C51" s="239"/>
-      <c r="E51" s="239" t="s">
+      <c r="C51" s="241"/>
+      <c r="E51" s="241" t="s">
         <v>297</v>
       </c>
-      <c r="F51" s="239"/>
+      <c r="F51" s="241"/>
     </row>
     <row r="52" spans="2:6" x14ac:dyDescent="0.2">
       <c r="B52" s="20" t="s">
@@ -36628,7 +36868,7 @@
       </c>
       <c r="I6" s="166">
         <f ca="1">Statement!AC114</f>
-        <v>336.64</v>
+        <v>340.97</v>
       </c>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.2">
@@ -36657,7 +36897,7 @@
       </c>
       <c r="I7" s="167">
         <f ca="1">Statement!AC143</f>
-        <v>4932785.92</v>
+        <v>4996233.41</v>
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
@@ -36686,7 +36926,7 @@
       </c>
       <c r="I8" s="167">
         <f ca="1">Statement!AC144</f>
-        <v>4870612.92</v>
+        <v>4934060.41</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
@@ -36715,7 +36955,7 @@
       </c>
       <c r="I9" s="168">
         <f ca="1">Statement!AC140</f>
-        <v>38.60550458715597</v>
+        <v>39.102064220183493</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.2">
@@ -36744,7 +36984,7 @@
       </c>
       <c r="I10" s="168">
         <f ca="1">Statement!AC141</f>
-        <v>10.657397771746464</v>
+        <v>10.79447753752493</v>
       </c>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.2">
@@ -36773,7 +37013,7 @@
       </c>
       <c r="I11" s="168">
         <f ca="1">Statement!AC142</f>
-        <v>45.693119047619042</v>
+        <v>46.280842447916669</v>
       </c>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.2">
@@ -36802,7 +37042,7 @@
       </c>
       <c r="I12" s="168">
         <f ca="1">Statement!AC145</f>
-        <v>10.433532452342751</v>
+        <v>10.569445828504595</v>
       </c>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
@@ -36831,7 +37071,7 @@
       </c>
       <c r="I13" s="168">
         <f ca="1">Statement!AC146</f>
-        <v>31.451920262948875</v>
+        <v>31.86163161327401</v>
       </c>
     </row>
     <row r="15" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -37604,7 +37844,7 @@
       </c>
       <c r="I51" s="169">
         <f ca="1">Statement!AC152</f>
-        <v>2.5903041825095056E-2</v>
+        <v>2.5574097427926205E-2</v>
       </c>
     </row>
     <row r="52" spans="2:9" x14ac:dyDescent="0.2">
@@ -37633,7 +37873,7 @@
       </c>
       <c r="I52" s="169">
         <f ca="1">Statement!AC151</f>
-        <v>2.4930536616517101E-2</v>
+        <v>2.4613942125654212E-2</v>
       </c>
     </row>
     <row r="53" spans="2:9" x14ac:dyDescent="0.2">
@@ -37662,7 +37902,7 @@
       </c>
       <c r="I53" s="169">
         <f ca="1">Statement!AC153</f>
-        <v>3.1190589353612169E-3</v>
+        <v>3.0794498049681791E-3</v>
       </c>
     </row>
     <row r="54" spans="2:9" x14ac:dyDescent="0.2">
@@ -37691,7 +37931,7 @@
       </c>
       <c r="I54" s="169">
         <f ca="1">Statement!AC154</f>
-        <v>1.6669282092015052E-2</v>
+        <v>1.6457597804663014E-2</v>
       </c>
     </row>
     <row r="55" spans="2:9" x14ac:dyDescent="0.2">
@@ -37720,7 +37960,7 @@
       </c>
       <c r="I55" s="169">
         <f ca="1">Statement!AC155</f>
-        <v>1.9839904181367756E-2</v>
+        <v>1.958795595980773E-2</v>
       </c>
     </row>
     <row r="57" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -37956,7 +38196,7 @@
       </c>
       <c r="I68" s="190">
         <f ca="1">Statement!AC166</f>
-        <v>1.2604033705967113E-2</v>
+        <v>1.2443974269808984E-2</v>
       </c>
     </row>
     <row r="70" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -38648,14 +38888,14 @@
     <row r="1" spans="2:7" ht="12" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="3" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B3" s="8"/>
-      <c r="C3" s="242" t="s">
+      <c r="C3" s="244" t="s">
         <v>307</v>
       </c>
-      <c r="D3" s="243"/>
-      <c r="F3" s="244" t="s">
+      <c r="D3" s="245"/>
+      <c r="F3" s="246" t="s">
         <v>308</v>
       </c>
-      <c r="G3" s="243"/>
+      <c r="G3" s="245"/>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B4" s="8"/>
@@ -38722,19 +38962,19 @@
       <c r="B7" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C7" s="240">
+      <c r="C7" s="242">
         <f>Statement!AA88</f>
         <v>-1.5892574471146927E-2</v>
       </c>
-      <c r="D7" s="241"/>
-      <c r="F7" s="240">
+      <c r="D7" s="243"/>
+      <c r="F7" s="242">
         <f>IF(F6=0,
 IF(G6=0,0,IF(G6&gt;0,1,-1)),
 (G6-F6)/ABS(F6)
 )</f>
         <v>0.16356501765281381</v>
       </c>
-      <c r="G7" s="241"/>
+      <c r="G7" s="243"/>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B8" s="201" t="s">
@@ -38761,19 +39001,19 @@
       <c r="B9" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C9" s="240">
+      <c r="C9" s="242">
         <f>Statement!AA89</f>
         <v>-3.1133095757317875E-2</v>
       </c>
-      <c r="D9" s="241"/>
-      <c r="F9" s="240">
+      <c r="D9" s="243"/>
+      <c r="F9" s="242">
         <f>IF(F8=0,
 IF(G8=0,0,IF(G8&gt;0,1,-1)),
 (G8-F8)/ABS(F8)
 )</f>
         <v>8.6032831193608647E-2</v>
       </c>
-      <c r="G9" s="241"/>
+      <c r="G9" s="243"/>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B10" s="201" t="s">
@@ -38800,19 +39040,19 @@
       <c r="B11" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C11" s="240">
+      <c r="C11" s="242">
         <f>Statement!AA90</f>
         <v>-2.0079954728829339E-4</v>
       </c>
-      <c r="D11" s="241"/>
-      <c r="F11" s="240">
+      <c r="D11" s="243"/>
+      <c r="F11" s="242">
         <f>IF(F10=0,
 IF(G10=0,0,IF(G10&gt;0,1,-1)),
 (G10-F10)/ABS(F10)
 )</f>
         <v>0.25280204949906215</v>
       </c>
-      <c r="G11" s="241"/>
+      <c r="G11" s="243"/>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B12" s="201" t="s">
@@ -38839,19 +39079,19 @@
       <c r="B13" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C13" s="240">
+      <c r="C13" s="242">
         <f>Statement!AA93</f>
         <v>9.4729043183742583E-3</v>
       </c>
-      <c r="D13" s="241"/>
-      <c r="F13" s="240">
+      <c r="D13" s="243"/>
+      <c r="F13" s="242">
         <f>IF(F12=0,
 IF(G12=0,0,IF(G12&gt;0,1,-1)),
 (G12-F12)/ABS(F12)
 )</f>
         <v>0.22937612786800721</v>
       </c>
-      <c r="G13" s="241"/>
+      <c r="G13" s="243"/>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B14" s="201" t="s">
@@ -38878,19 +39118,19 @@
       <c r="B15" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C15" s="240">
+      <c r="C15" s="242">
         <f>Statement!AA94</f>
         <v>-5.2946913752264175E-3</v>
       </c>
-      <c r="D15" s="241"/>
-      <c r="F15" s="240">
+      <c r="D15" s="243"/>
+      <c r="F15" s="242">
         <f>IF(F14=0,
 IF(G14=0,0,IF(G14&gt;0,1,-1)),
 (G14-F14)/ABS(F14)
 )</f>
         <v>0.26569037656903766</v>
       </c>
-      <c r="G15" s="241"/>
+      <c r="G15" s="243"/>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B16" s="201" t="s">
@@ -38917,19 +39157,19 @@
       <c r="B17" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C17" s="240">
+      <c r="C17" s="242">
         <f>Statement!AA96</f>
         <v>7.1336804381635002E-3</v>
       </c>
-      <c r="D17" s="241"/>
-      <c r="F17" s="240">
+      <c r="D17" s="243"/>
+      <c r="F17" s="242">
         <f>IF(F16=0,
 IF(G16=0,0,IF(G16&gt;0,1,-1)),
 (G16-F16)/ABS(F16)
 )</f>
         <v>0.27118716394981651</v>
       </c>
-      <c r="G17" s="241"/>
+      <c r="G17" s="243"/>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B18" s="201" t="s">
@@ -38956,22 +39196,22 @@
       <c r="B19" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C19" s="240">
+      <c r="C19" s="242">
         <f>IF(C18=0,
 IF(D18=0,0,IF(D18&gt;0,1,-1)),
 (D18-C18)/ABS(C18)
 )</f>
         <v>-7.4697813391280731E-4</v>
       </c>
-      <c r="D19" s="241"/>
-      <c r="F19" s="240">
+      <c r="D19" s="243"/>
+      <c r="F19" s="242">
         <f>IF(F18=0,
 IF(G18=0,0,IF(G18&gt;0,1,-1)),
 (G18-F18)/ABS(F18)
 )</f>
         <v>-1.5587369547765587E-2</v>
       </c>
-      <c r="G19" s="241"/>
+      <c r="G19" s="243"/>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B20" s="201" t="s">
@@ -38998,22 +39238,22 @@
       <c r="B21" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C21" s="240">
+      <c r="C21" s="242">
         <f>IF(C20=0,
 IF(D20=0,0,IF(D20&gt;0,1,-1)),
 (D20-C20)/ABS(C20)
 )</f>
         <v>4.975124378109568E-3</v>
       </c>
-      <c r="D21" s="241"/>
-      <c r="F21" s="240">
+      <c r="D21" s="243"/>
+      <c r="F21" s="242">
         <f>IF(F20=0,
 IF(G20=0,0,IF(G20&gt;0,1,-1)),
 (G20-F20)/ABS(F20)
 )</f>
         <v>0.28662420382165599</v>
       </c>
-      <c r="G21" s="241"/>
+      <c r="G21" s="243"/>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23" s="8" t="s">
@@ -39061,22 +39301,22 @@
       <c r="B25" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C25" s="240">
+      <c r="C25" s="242">
         <f>IF(C24=0,
 IF(D24=0,0,IF(D24&gt;0,1,-1)),
 (D24-C24)/ABS(C24)
 )</f>
         <v>1.5257357017718937E-2</v>
       </c>
-      <c r="D25" s="241"/>
-      <c r="F25" s="240">
+      <c r="D25" s="243"/>
+      <c r="F25" s="242">
         <f>IF(F24=0,
 IF(G24=0,0,IF(G24&gt;0,1,-1)),
 (G24-F24)/ABS(F24)
 )</f>
         <v>0.11124326423612797</v>
       </c>
-      <c r="G25" s="241"/>
+      <c r="G25" s="243"/>
     </row>
     <row r="26" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B26" s="20" t="s">
@@ -39103,22 +39343,22 @@
       <c r="B27" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C27" s="240">
+      <c r="C27" s="242">
         <f>IF(C26=0,
 IF(D26=0,0,IF(D26&gt;0,1,-1)),
 (D26-C26)/ABS(C26)
 )</f>
         <v>4.7692033505613969E-2</v>
       </c>
-      <c r="D27" s="241"/>
-      <c r="F27" s="240">
+      <c r="D27" s="243"/>
+      <c r="F27" s="242">
         <f>IF(F26=0,
 IF(G26=0,0,IF(G26&gt;0,1,-1)),
 (G26-F26)/ABS(F26)
 )</f>
         <v>0.22399433663696178</v>
       </c>
-      <c r="G27" s="241"/>
+      <c r="G27" s="243"/>
     </row>
     <row r="28" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B28" s="20" t="s">
@@ -39145,22 +39385,22 @@
       <c r="B29" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C29" s="240">
+      <c r="C29" s="242">
         <f>IF(C28=0,
 IF(D28=0,0,IF(D28&gt;0,1,-1)),
 (D28-C28)/ABS(C28)
 )</f>
         <v>-8.2012001756354591E-2</v>
       </c>
-      <c r="D29" s="241"/>
-      <c r="F29" s="240">
+      <c r="D29" s="243"/>
+      <c r="F29" s="242">
         <f>IF(F28=0,
 IF(G28=0,0,IF(G28&gt;0,1,-1)),
 (G28-F28)/ABS(F28)
 )</f>
         <v>0.22428264688658989</v>
       </c>
-      <c r="G29" s="241"/>
+      <c r="G29" s="243"/>
     </row>
     <row r="30" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B30" s="20" t="s">
@@ -39187,22 +39427,22 @@
       <c r="B31" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C31" s="240">
+      <c r="C31" s="242">
         <f>IF(C30=0,
 IF(D30=0,0,IF(D30&gt;0,1,-1)),
 (D30-C30)/ABS(C30)
 )</f>
         <v>-0.21985477919295321</v>
       </c>
-      <c r="D31" s="241"/>
-      <c r="F31" s="240">
+      <c r="D31" s="243"/>
+      <c r="F31" s="242">
         <f>IF(F30=0,
 IF(G30=0,0,IF(G30&gt;0,1,-1)),
 (G30-F30)/ABS(F30)
 )</f>
         <v>0.1335178139052231</v>
       </c>
-      <c r="G31" s="241"/>
+      <c r="G31" s="243"/>
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B32" s="20" t="s">
@@ -39229,22 +39469,22 @@
       <c r="B33" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C33" s="240">
+      <c r="C33" s="242">
         <f>IF(C32=0,
 IF(D32=0,0,IF(D32&gt;0,1,-1)),
 (D32-C32)/ABS(C32)
 )</f>
         <v>-2.9218647406434668E-2</v>
       </c>
-      <c r="D33" s="241"/>
-      <c r="F33" s="240">
+      <c r="D33" s="243"/>
+      <c r="F33" s="242">
         <f>IF(F32=0,
 IF(G32=0,0,IF(G32&gt;0,1,-1)),
 (G32-F32)/ABS(F32)
 )</f>
         <v>0.15613189104652678</v>
       </c>
-      <c r="G33" s="241"/>
+      <c r="G33" s="243"/>
     </row>
     <row r="35" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B35" s="224" t="s">
@@ -39271,22 +39511,22 @@
       <c r="B36" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C36" s="240">
+      <c r="C36" s="242">
         <f>IF(C35=0,
 IF(D35=0,0,IF(D35&gt;0,1,-1)),
 (D35-C35)/ABS(C35)
 )</f>
         <v>-4.8110327402884512E-2</v>
       </c>
-      <c r="D36" s="241"/>
-      <c r="F36" s="240">
+      <c r="D36" s="243"/>
+      <c r="F36" s="242">
         <f>IF(F35=0,
 IF(G35=0,0,IF(G35&gt;0,1,-1)),
 (G35-F35)/ABS(F35)
 )</f>
         <v>0.21690368310080302</v>
       </c>
-      <c r="G36" s="241"/>
+      <c r="G36" s="243"/>
     </row>
     <row r="37" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B37" s="224" t="s">
@@ -39313,22 +39553,22 @@
       <c r="B38" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C38" s="240">
+      <c r="C38" s="242">
         <f>IF(C37=0,
 IF(D37=0,0,IF(D37&gt;0,1,-1)),
 (D37-C37)/ABS(C37)
 )</f>
         <v>0.23252768186688891</v>
       </c>
-      <c r="D38" s="241"/>
-      <c r="F38" s="240">
+      <c r="D38" s="243"/>
+      <c r="F38" s="242">
         <f>IF(F37=0,
 IF(G37=0,0,IF(G37&gt;0,1,-1)),
 (G37-F37)/ABS(F37)
 )</f>
         <v>0.28660203827989061</v>
       </c>
-      <c r="G38" s="241"/>
+      <c r="G38" s="243"/>
     </row>
     <row r="39" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B39" s="224" t="s">
@@ -39355,22 +39595,22 @@
       <c r="B40" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C40" s="240">
+      <c r="C40" s="242">
         <f>IF(C39=0,
 IF(D39=0,0,IF(D39&gt;0,1,-1)),
 (D39-C39)/ABS(C39)
 )</f>
         <v>-0.10457043679490888</v>
       </c>
-      <c r="D40" s="241"/>
-      <c r="F40" s="240">
+      <c r="D40" s="243"/>
+      <c r="F40" s="242">
         <f>IF(F39=0,
 IF(G39=0,0,IF(G39&gt;0,1,-1)),
 (G39-F39)/ABS(F39)
 )</f>
         <v>-5.9261510408752466E-2</v>
       </c>
-      <c r="G40" s="241"/>
+      <c r="G40" s="243"/>
     </row>
     <row r="41" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B41" s="224" t="s">
@@ -39397,22 +39637,22 @@
       <c r="B42" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C42" s="240">
+      <c r="C42" s="242">
         <f>IF(C41=0,
 IF(D41=0,0,IF(D41&gt;0,1,-1)),
 (D41-C41)/ABS(C41)
 )</f>
         <v>-2.2781926338438173E-3</v>
       </c>
-      <c r="D42" s="241"/>
-      <c r="F42" s="240">
+      <c r="D42" s="243"/>
+      <c r="F42" s="242">
         <f>IF(F41=0,
 IF(G41=0,0,IF(G41&gt;0,1,-1)),
 (G41-F41)/ABS(F41)
 )</f>
         <v>6.4694759589411135E-2</v>
       </c>
-      <c r="G42" s="241"/>
+      <c r="G42" s="243"/>
     </row>
     <row r="43" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B43" s="224" t="s">
@@ -39439,22 +39679,22 @@
       <c r="B44" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C44" s="240">
+      <c r="C44" s="242">
         <f>IF(C43=0,
 IF(D43=0,0,IF(D43&gt;0,1,-1)),
 (D43-C43)/ABS(C43)
 )</f>
         <v>-7.6510847107438013E-3</v>
       </c>
-      <c r="D44" s="241"/>
-      <c r="F44" s="240">
+      <c r="D44" s="243"/>
+      <c r="F44" s="242">
         <f>IF(F43=0,
 IF(G43=0,0,IF(G43&gt;0,1,-1)),
 (G43-F43)/ABS(F43)
 )</f>
         <v>0.12092039528862633</v>
       </c>
-      <c r="G44" s="241"/>
+      <c r="G44" s="243"/>
     </row>
   </sheetData>
   <mergeCells count="38">

</xml_diff>

<commit_message>
Updated data in files
</commit_message>
<xml_diff>
--- a/AAPL.xlsx
+++ b/AAPL.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11011"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11020"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/KINGSTON/MyStockData/Finance-StockLists/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEB38430-39CF-F34C-AD5A-3580BB2166AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28F5C13A-E116-8A49-A165-25B31C0AEF2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14400" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
   </bookViews>
@@ -119,7 +119,7 @@
       </extLst>
     </bk>
   </futureMetadata>
-  <futureMetadata name="XLRICHVALUE" count="5">
+  <futureMetadata name="XLRICHVALUE" count="2">
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
@@ -130,28 +130,7 @@
     <bk>
       <extLst>
         <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="3"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="4"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
           <xlrd:rvb i="5"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="8"/>
         </ext>
       </extLst>
     </bk>
@@ -161,21 +140,12 @@
       <rc t="1" v="0"/>
     </bk>
   </cellMetadata>
-  <valueMetadata count="5">
+  <valueMetadata count="2">
     <bk>
       <rc t="2" v="0"/>
     </bk>
     <bk>
       <rc t="2" v="1"/>
-    </bk>
-    <bk>
-      <rc t="2" v="2"/>
-    </bk>
-    <bk>
-      <rc t="2" v="3"/>
-    </bk>
-    <bk>
-      <rc t="2" v="4"/>
     </bk>
   </valueMetadata>
 </metadata>
@@ -2421,12 +2391,6 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="18" fillId="17" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="18" fillId="17" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2434,6 +2398,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="18" fillId="17" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="18" fillId="17" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2454,14 +2424,14 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -15582,7 +15552,7 @@
 </file>
 
 <file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="9">
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="6">
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a1mou2&amp;q=XNAS%3aAAPL&amp;form=skydnc</v>
     <v>Learn more on Bing</v>
@@ -15599,11 +15569,13 @@
     <v>268435456</v>
     <v>1</v>
     <v>Powered by Refinitiv</v>
-    <v>348.1499</v>
+    <v>351.73</v>
     <v>243.42</v>
-    <v>1.0789</v>
-    <v>-2.5049999999999999</v>
-    <v>-7.3040000000000006E-3</v>
+    <v>1.077</v>
+    <v>-0.495</v>
+    <v>-1.4219999999999999E-3</v>
+    <v>-0.185</v>
+    <v>-5.3199999999999992E-4</v>
     <v>USD</v>
     <v>Apple Inc. designs, manufactures and markets smartphones, personal computers, tablets, wearables and accessories, and sells a variety of related services. Its product categories include iPhone, Mac, iPad, Wearables, Home and Accessories. Its services include advertising, AppleCare, cloud services, digital content, and payment services. The Company operates various platforms, including the App Store, that allow customers to discover and download applications and digital content, such as books, music, video, games and podcasts. It also offers digital content through subscription-based services, including Apple Arcade, Apple Fitness+, Apple Music, Apple News+, and Apple TV+. Its wearables include smartwatches, wireless headphones, and spatial computers. Its products include iPhone 16 Pro, iPhone 16, iPhone 15, iPhone 14, iPhone SE, MacBook Air, MacBook Pro, iMac, Mac mini, Mac Studio, Mac Pro, iPad Pro, iPad Air, AirPods, AirPods Pro, AirPods Max, Apple TV, Apple Vision Pro and others.</v>
     <v>166000</v>
@@ -15611,49 +15583,35 @@
     <v>XNAS</v>
     <v>XNAS</v>
     <v>One Apple Park Way, CUPERTINO, CA, 95014 US</v>
-    <v>343.06</v>
+    <v>351.73</v>
     <v>Computers, Phones &amp; Household Electronics</v>
     <v>Stock</v>
-    <v>46315.716929988281</v>
+    <v>46318.958116758593</v>
     <v>0</v>
-    <v>338.7</v>
-    <v>4968369668300</v>
+    <v>345.75</v>
+    <v>5074761240500</v>
     <v>APPLE INC.</v>
     <v>APPLE INC.</v>
-    <v>339.62</v>
-    <v>39.172800000000002</v>
-    <v>342.94</v>
-    <v>340.435</v>
+    <v>349.11500000000001</v>
+    <v>40.0687</v>
+    <v>348.22</v>
+    <v>347.72500000000002</v>
+    <v>347.54</v>
     <v>14594180000</v>
     <v>AAPL</v>
     <v>APPLE INC. (XNAS:AAPL)</v>
-    <v>14058343</v>
-    <v>38617562</v>
+    <v>39502829</v>
+    <v>39174961</v>
     <v>1977</v>
   </rv>
   <rv s="2">
     <v>1</v>
   </rv>
-  <rv s="3">
-    <v>12</v>
-    <v>Price (Extended hours)</v>
-    <v>0</v>
-  </rv>
-  <rv s="3">
-    <v>12</v>
-    <v>Change (extended hours)</v>
-    <v>0</v>
-  </rv>
-  <rv s="3">
-    <v>12</v>
-    <v>Change % (extended hours)</v>
-    <v>0</v>
-  </rv>
   <rv s="0">
     <v>https://www.bing.com/financeapi/forcetrigger?t=a33knm&amp;q=10+Y+TSY+YLD+NDX&amp;form=skydnc</v>
     <v>Learn more on Bing</v>
   </rv>
-  <rv s="4">
+  <rv s="3">
     <v>5</v>
     <v>10 Y TSY YLD NDX</v>
     <v>6</v>
@@ -15667,28 +15625,28 @@
     <v>Powered by Refinitiv</v>
     <v>53.64</v>
     <v>39.47</v>
-    <v>0.38</v>
-    <v>7.4539999999999997E-3</v>
+    <v>-1.93</v>
+    <v>-3.7505000000000004E-2</v>
     <v>US</v>
-    <v>51.5</v>
+    <v>50.54</v>
     <v>Index</v>
-    <v>6</v>
-    <v>50.9</v>
+    <v>3</v>
+    <v>49.39</v>
     <v>10 Y TSY YLD NDX</v>
-    <v>50.9</v>
-    <v>50.98</v>
-    <v>51.36</v>
+    <v>50.4</v>
+    <v>51.46</v>
+    <v>49.53</v>
     <v>TNX</v>
     <v>10 Y TSY YLD NDX</v>
   </rv>
   <rv s="2">
-    <v>7</v>
+    <v>4</v>
   </rv>
 </rvData>
 </file>
 
 <file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
-<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="5">
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="4">
   <s t="_hyperlink">
     <k n="Address" t="s"/>
     <k n="Text" t="s"/>
@@ -15710,6 +15668,8 @@
     <k n="Beta"/>
     <k n="Change"/>
     <k n="Change (%)"/>
+    <k n="Change (Extended hours)"/>
+    <k n="Change % (Extended hours)"/>
     <k n="Currency" t="s"/>
     <k n="Description" t="s"/>
     <k n="Employees"/>
@@ -15730,6 +15690,7 @@
     <k n="P/E"/>
     <k n="Previous close"/>
     <k n="Price"/>
+    <k n="Price (Extended hours)"/>
     <k n="Shares outstanding"/>
     <k n="Ticker symbol" t="s"/>
     <k n="UniqueName" t="s"/>
@@ -15739,11 +15700,6 @@
   </s>
   <s t="_linkedentity">
     <k n="%cvi" t="r"/>
-  </s>
-  <s t="_error">
-    <k n="errorType" t="i"/>
-    <k n="field" t="s"/>
-    <k n="subType" t="i"/>
   </s>
   <s t="_linkedentitycore">
     <k n="_Display" t="spb"/>
@@ -15779,7 +15735,7 @@
 <file path=xl/richData/rdsupportingpropertybag.xml><?xml version="1.0" encoding="utf-8"?>
 <supportingPropertyBags xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2">
   <spbArrays count="2">
-    <a count="42">
+    <a count="45">
       <v t="s">%EntityServiceId</v>
       <v t="s">_Format</v>
       <v t="s">%IsRefreshable</v>
@@ -15790,13 +15746,16 @@
       <v t="s">Name</v>
       <v t="s">_SubLabel</v>
       <v t="s">Price</v>
+      <v t="s">Price (Extended hours)</v>
       <v t="s">Exchange</v>
       <v t="s">Official name</v>
       <v t="s">Last trade time</v>
       <v t="s">Ticker symbol</v>
       <v t="s">Exchange abbreviation</v>
       <v t="s">Change</v>
+      <v t="s">Change (Extended hours)</v>
       <v t="s">Change (%)</v>
+      <v t="s">Change % (Extended hours)</v>
       <v t="s">Currency</v>
       <v t="s">Previous close</v>
       <v t="s">Open</v>
@@ -15890,13 +15849,19 @@
       <v>8</v>
       <v>9</v>
       <v>4</v>
+      <v>1</v>
+      <v>1</v>
+      <v>5</v>
     </spb>
     <spb s="4">
-      <v>Real-Time Nasdaq Last Sale</v>
+      <v>at close</v>
       <v>from previous close</v>
       <v>from previous close</v>
       <v>Source: Nasdaq Last Sale</v>
       <v>GMT</v>
+      <v>Real-Time Nasdaq Last Sale</v>
+      <v>from close</v>
+      <v>from close</v>
     </spb>
     <spb s="0">
       <v>1</v>
@@ -15968,6 +15933,9 @@
     <k n="Year incorporated" t="i"/>
     <k n="`%EntityServiceId" t="i"/>
     <k n="Shares outstanding" t="i"/>
+    <k n="Price (Extended hours)" t="i"/>
+    <k n="Change (Extended hours)" t="i"/>
+    <k n="Change % (Extended hours)" t="i"/>
   </s>
   <s>
     <k n="Price" t="s"/>
@@ -15975,6 +15943,9 @@
     <k n="Change (%)" t="s"/>
     <k n="ExchangeID" t="s"/>
     <k n="Last trade time" t="s"/>
+    <k n="Price (Extended hours)" t="s"/>
+    <k n="Change (Extended hours)" t="s"/>
+    <k n="Change % (Extended hours)" t="s"/>
   </s>
   <s>
     <k n="UniqueName" t="spb"/>
@@ -16490,7 +16461,7 @@
       </c>
       <c r="F3" s="181">
         <f ca="1">Statement!AC143</f>
-        <v>4988394.0549999997</v>
+        <v>5095214.4250000007</v>
       </c>
       <c r="H3" s="179" t="str">
         <f>'AVG target price'!B5</f>
@@ -16498,7 +16469,7 @@
       </c>
       <c r="I3" s="205">
         <f ca="1">'AVG target price'!C5</f>
-        <v>114.4961108417382</v>
+        <v>117.23172915838408</v>
       </c>
       <c r="K3" s="238" t="s">
         <v>422</v>
@@ -16517,7 +16488,7 @@
       </c>
       <c r="F4" s="182">
         <f ca="1">Statement!AC144</f>
-        <v>4926221.0549999997</v>
+        <v>5033041.4250000007</v>
       </c>
       <c r="H4" s="179" t="str">
         <f>'AVG target price'!B6</f>
@@ -16525,7 +16496,7 @@
       </c>
       <c r="I4" s="205">
         <f ca="1">'AVG target price'!C6</f>
-        <v>229.63275447305054</v>
+        <v>231.44050669254096</v>
       </c>
       <c r="K4" s="238" t="s">
         <v>423</v>
@@ -16537,7 +16508,7 @@
       </c>
       <c r="C5" s="202" cm="1">
         <f t="array" aca="1" ref="C5" ca="1">_FV(C3,"Price",TRUE)</f>
-        <v>340.435</v>
+        <v>347.72500000000002</v>
       </c>
       <c r="E5" s="179" t="s">
         <v>237</v>
@@ -16552,7 +16523,7 @@
       </c>
       <c r="I5" s="205">
         <f ca="1">'AVG target price'!C7</f>
-        <v>201.200208242569</v>
+        <v>202.96135486625744</v>
       </c>
       <c r="K5" s="238" t="s">
         <v>424</v>
@@ -16562,16 +16533,16 @@
       <c r="B6" s="179" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="202" t="e" cm="1" vm="2">
-        <f t="array" ref="C6">_FV(C3,"Price (Extended hours)",TRUE)</f>
-        <v>#VALUE!</v>
+      <c r="C6" s="202" cm="1">
+        <f t="array" aca="1" ref="C6" ca="1">_FV(C3,"Price (Extended hours)",TRUE)</f>
+        <v>347.54</v>
       </c>
       <c r="E6" s="179" t="s">
         <v>231</v>
       </c>
       <c r="F6" s="184">
         <f ca="1">Statement!AC140</f>
-        <v>39.040711009174316</v>
+        <v>39.876720183486249</v>
       </c>
       <c r="H6" s="179" t="str">
         <f>'AVG target price'!B8</f>
@@ -16579,7 +16550,7 @@
       </c>
       <c r="I6" s="205">
         <f ca="1">'AVG target price'!C8</f>
-        <v>199.66010736869646</v>
+        <v>201.21244835591099</v>
       </c>
       <c r="K6" s="239" t="s">
         <v>425</v>
@@ -16591,14 +16562,14 @@
       </c>
       <c r="C7" s="6" cm="1">
         <f t="array" aca="1" ref="C7" ca="1">_FV(C3,"Change")</f>
-        <v>-2.5049999999999999</v>
+        <v>-0.495</v>
       </c>
       <c r="E7" s="180" t="s">
         <v>198</v>
       </c>
       <c r="F7" s="185">
         <f ca="1">Statement!AC141</f>
-        <v>10.77754043020588</v>
+        <v>11.008328303768238</v>
       </c>
       <c r="H7" s="179" t="str">
         <f>'AVG target price'!B9</f>
@@ -16606,23 +16577,23 @@
       </c>
       <c r="I7" s="205">
         <f ca="1">'AVG target price'!C9</f>
-        <v>213.69431720014197</v>
+        <v>215.36625038802489</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B8" s="179" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="6" t="e" cm="1" vm="3">
-        <f t="array" ref="C8">_FV(C3,"Change (extended hours)",TRUE)</f>
-        <v>#VALUE!</v>
+      <c r="C8" s="6" cm="1">
+        <f t="array" aca="1" ref="C8" ca="1">_FV(C3,"Change (extended hours)",TRUE)</f>
+        <v>-0.185</v>
       </c>
       <c r="E8" s="179" t="s">
         <v>259</v>
       </c>
       <c r="F8" s="186">
         <f ca="1">Statement!AC151</f>
-        <v>2.4652623398253169E-2</v>
+        <v>2.4135785021451767E-2</v>
       </c>
       <c r="H8" s="178" t="str">
         <f>'AVG target price'!B10</f>
@@ -16630,7 +16601,7 @@
       </c>
       <c r="I8" s="206">
         <f ca="1">'AVG target price'!C10</f>
-        <v>191.73669962523925</v>
+        <v>193.64245789222369</v>
       </c>
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.2">
@@ -16639,14 +16610,14 @@
       </c>
       <c r="C9" s="73" cm="1">
         <f t="array" aca="1" ref="C9" ca="1">_FV(C3,"Change (%)",TRUE)</f>
-        <v>-7.3040000000000006E-3</v>
+        <v>-1.4219999999999999E-3</v>
       </c>
       <c r="E9" s="179" t="s">
         <v>282</v>
       </c>
       <c r="F9" s="186">
         <f ca="1">Statement!AC152</f>
-        <v>2.5614287602626049E-2</v>
+        <v>2.5077288086850235E-2</v>
       </c>
       <c r="H9" s="178" t="str">
         <f>'AVG target price'!B12</f>
@@ -16654,23 +16625,23 @@
       </c>
       <c r="I9" s="207">
         <f ca="1">'AVG target price'!C12</f>
-        <v>-0.43678910915376135</v>
+        <v>-0.44311608917327289</v>
       </c>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B10" s="179" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="73" t="e" cm="1" vm="4">
-        <f t="array" ref="C10">_FV(C3,"Change % (extended hours)",TRUE)</f>
-        <v>#VALUE!</v>
+      <c r="C10" s="73" cm="1">
+        <f t="array" aca="1" ref="C10" ca="1">_FV(C3,"Change % (extended hours)",TRUE)</f>
+        <v>-5.3199999999999992E-4</v>
       </c>
       <c r="E10" s="179" t="s">
         <v>287</v>
       </c>
       <c r="F10" s="186">
         <f ca="1">Statement!AC154</f>
-        <v>1.6483461228886418E-2</v>
+        <v>1.613788805365144E-2</v>
       </c>
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.2">
@@ -16679,21 +16650,21 @@
       </c>
       <c r="C11" s="203" cm="1">
         <f t="array" aca="1" ref="C11" ca="1">_FV(C3,"52 week high",TRUE)</f>
-        <v>348.1499</v>
+        <v>351.73</v>
       </c>
       <c r="E11" s="180" t="s">
         <v>283</v>
       </c>
       <c r="F11" s="187">
         <f ca="1">Statement!AC153</f>
-        <v>3.0842892182061186E-3</v>
+        <v>3.0196275792652239E-3</v>
       </c>
       <c r="H11" s="178" t="s">
         <v>394</v>
       </c>
       <c r="I11" s="206">
         <f ca="1">DDM!C26</f>
-        <v>13.274851239824555</v>
+        <v>13.600871850759665</v>
       </c>
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.2">
@@ -16718,7 +16689,7 @@
       </c>
       <c r="C13" s="203" cm="1">
         <f t="array" aca="1" ref="C13" ca="1">_FV(C3,"Beta")</f>
-        <v>1.0789</v>
+        <v>1.077</v>
       </c>
       <c r="E13" s="179" t="s">
         <v>101</v>
@@ -16741,7 +16712,7 @@
       </c>
       <c r="C14" s="204" cm="1">
         <f t="array" aca="1" ref="C14" ca="1">_FV(C3,"Volume average",TRUE)</f>
-        <v>38617562</v>
+        <v>39174961</v>
       </c>
       <c r="E14" s="180" t="s">
         <v>102</v>
@@ -16755,7 +16726,7 @@
       </c>
       <c r="I14" s="241">
         <f ca="1">'Reverse DCF'!C16</f>
-        <v>342.00119694383932</v>
+        <v>351.30611132400372</v>
       </c>
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.2">
@@ -16764,7 +16735,7 @@
       </c>
       <c r="F15" s="186">
         <f ca="1">Statement!AC166</f>
-        <v>1.2463530209222817E-2</v>
+        <v>1.220223425631395E-2</v>
       </c>
     </row>
     <row r="16" spans="2:11" x14ac:dyDescent="0.2">
@@ -16797,7 +16768,7 @@
       </c>
       <c r="I17" s="236">
         <f ca="1">DCF!C15</f>
-        <v>9.8892924301031637E-2</v>
+        <v>9.7029602251831923E-2</v>
       </c>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.2">
@@ -16819,7 +16790,7 @@
       </c>
       <c r="I18" s="237">
         <f ca="1">Multiples!C54</f>
-        <v>9.9910499999999999E-2</v>
+        <v>9.7994999999999999E-2</v>
       </c>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
@@ -16887,12 +16858,12 @@
       <c r="C26" s="164">
         <v>0.21</v>
       </c>
-      <c r="E26" s="179" t="e" vm="5">
+      <c r="E26" s="179" t="e" vm="2">
         <v>#VALUE!</v>
       </c>
       <c r="F26" s="213" cm="1">
         <f t="array" aca="1" ref="F26" ca="1">_FV(E26,"Price")</f>
-        <v>51.36</v>
+        <v>49.53</v>
       </c>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.2">
@@ -16907,7 +16878,7 @@
       </c>
       <c r="F27" s="214">
         <f ca="1">F26/1000</f>
-        <v>5.1360000000000003E-2</v>
+        <v>4.9530000000000005E-2</v>
       </c>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.2">
@@ -21214,12 +21185,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="C3:G3"/>
-    <mergeCell ref="H3:L3"/>
-    <mergeCell ref="P3:W3"/>
-    <mergeCell ref="X3:Z3"/>
-    <mergeCell ref="C5:L5"/>
-    <mergeCell ref="P5:Z5"/>
     <mergeCell ref="C40:L40"/>
     <mergeCell ref="C11:L11"/>
     <mergeCell ref="P11:Z11"/>
@@ -21227,6 +21192,12 @@
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="C26:L26"/>
     <mergeCell ref="C33:L33"/>
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="H3:L3"/>
+    <mergeCell ref="P3:W3"/>
+    <mergeCell ref="X3:Z3"/>
+    <mergeCell ref="C5:L5"/>
+    <mergeCell ref="P5:Z5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -22286,16 +22257,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="C31:L31"/>
+    <mergeCell ref="C25:L25"/>
+    <mergeCell ref="C2:G2"/>
+    <mergeCell ref="H2:L2"/>
+    <mergeCell ref="S2:Z2"/>
     <mergeCell ref="AA2:AC2"/>
     <mergeCell ref="C4:L4"/>
     <mergeCell ref="S4:AC4"/>
     <mergeCell ref="C13:L13"/>
     <mergeCell ref="C18:L18"/>
-    <mergeCell ref="C31:L31"/>
-    <mergeCell ref="C25:L25"/>
-    <mergeCell ref="C2:G2"/>
-    <mergeCell ref="H2:L2"/>
-    <mergeCell ref="S2:Z2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -22417,7 +22388,7 @@
       </c>
       <c r="C6" s="133">
         <f ca="1">Overview!C5</f>
-        <v>340.435</v>
+        <v>347.72500000000002</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22426,7 +22397,7 @@
       </c>
       <c r="C7" s="134">
         <f ca="1">C5*C6</f>
-        <v>4988394.0549999997</v>
+        <v>5095214.4250000007</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22444,7 +22415,7 @@
       </c>
       <c r="C9" s="135">
         <f ca="1">Overview!F27</f>
-        <v>5.1360000000000003E-2</v>
+        <v>4.9530000000000005E-2</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22453,7 +22424,7 @@
       </c>
       <c r="C10" s="133">
         <f ca="1">Overview!C13</f>
-        <v>1.0789</v>
+        <v>1.077</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22496,7 +22467,7 @@
       </c>
       <c r="C16" s="46">
         <f ca="1">C8/(C8+C7)</f>
-        <v>1.6626918063877835E-2</v>
+        <v>1.6284013631914961E-2</v>
       </c>
     </row>
     <row r="17" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22505,7 +22476,7 @@
       </c>
       <c r="C17" s="46">
         <f ca="1">C7/(C8+C7)</f>
-        <v>0.98337308193612216</v>
+        <v>0.98371598636808499</v>
       </c>
     </row>
     <row r="18" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22523,7 +22494,7 @@
       </c>
       <c r="C19" s="46">
         <f ca="1">C9+C10*C11</f>
-        <v>9.9910499999999999E-2</v>
+        <v>9.7994999999999999E-2</v>
       </c>
     </row>
     <row r="20" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22532,7 +22503,7 @@
       </c>
       <c r="C20" s="46">
         <f ca="1">(C17*C19)+(C16*C18)</f>
-        <v>9.8892924301031637E-2</v>
+        <v>9.7029602251831923E-2</v>
       </c>
     </row>
   </sheetData>
@@ -22783,7 +22754,7 @@
       </c>
       <c r="L8" s="126">
         <f ca="1">L7*(1+C14)/(C15-C14)</f>
-        <v>1837359.0526591584</v>
+        <v>1881804.1949815061</v>
       </c>
       <c r="N8" s="91"/>
       <c r="O8" s="16"/>
@@ -22837,23 +22808,23 @@
       <c r="G10" s="138"/>
       <c r="H10" s="126">
         <f ca="1">H7/(1+$C$15)^H9</f>
-        <v>100427.45148504277</v>
+        <v>100598.02909234971</v>
       </c>
       <c r="I10" s="126">
         <f t="shared" ref="I10:L10" ca="1" si="0">I7/(1+$C$15)^I9</f>
-        <v>97097.551361446123</v>
+        <v>97427.674922636434</v>
       </c>
       <c r="J10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>93359.889040441572</v>
+        <v>93836.417239063201</v>
       </c>
       <c r="K10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>89353.869758090004</v>
+        <v>89962.494019650287</v>
       </c>
       <c r="L10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>88685.992558160317</v>
+        <v>89441.728231623725</v>
       </c>
       <c r="N10" s="91"/>
     </row>
@@ -22872,7 +22843,7 @@
       <c r="K11" s="137"/>
       <c r="L11" s="126">
         <f ca="1">L8/(1+C15)^L9</f>
-        <v>1146613.7579608092</v>
+        <v>1184357.1838524786</v>
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.2">
@@ -22895,7 +22866,7 @@
       </c>
       <c r="C15" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.8892924301031637E-2</v>
+        <v>9.7029602251831923E-2</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.2">
@@ -22910,7 +22881,7 @@
       </c>
       <c r="C19" s="64">
         <f ca="1">SUM(H10:L10)</f>
-        <v>468924.75420318078</v>
+        <v>471266.34350532334</v>
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.2">
@@ -22919,7 +22890,7 @@
       </c>
       <c r="C20" s="64">
         <f ca="1">L11</f>
-        <v>1146613.7579608092</v>
+        <v>1184357.1838524786</v>
       </c>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.2">
@@ -22928,7 +22899,7 @@
       </c>
       <c r="C21" s="94">
         <f ca="1">C19+C20</f>
-        <v>1615538.5121639899</v>
+        <v>1655623.527357802</v>
       </c>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.2">
@@ -22955,7 +22926,7 @@
       </c>
       <c r="C24" s="94">
         <f ca="1">C21+C22-C23</f>
-        <v>1677711.5121639899</v>
+        <v>1717796.527357802</v>
       </c>
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.2">
@@ -22973,7 +22944,7 @@
       </c>
       <c r="C26" s="235">
         <f ca="1">C24/C25</f>
-        <v>114.4961108417382</v>
+        <v>117.23172915838408</v>
       </c>
     </row>
   </sheetData>
@@ -23242,23 +23213,23 @@
       <c r="G9" s="138"/>
       <c r="H9" s="92">
         <f ca="1">DCF!H10</f>
-        <v>100427.45148504277</v>
+        <v>100598.02909234971</v>
       </c>
       <c r="I9" s="92">
         <f ca="1">DCF!I10</f>
-        <v>97097.551361446123</v>
+        <v>97427.674922636434</v>
       </c>
       <c r="J9" s="92">
         <f ca="1">DCF!J10</f>
-        <v>93359.889040441572</v>
+        <v>93836.417239063201</v>
       </c>
       <c r="K9" s="92">
         <f ca="1">DCF!K10</f>
-        <v>89353.869758090004</v>
+        <v>89962.494019650287</v>
       </c>
       <c r="L9" s="92">
         <f ca="1">DCF!L10</f>
-        <v>88685.992558160317</v>
+        <v>89441.728231623725</v>
       </c>
       <c r="N9" s="91"/>
     </row>
@@ -24044,7 +24015,7 @@
       </c>
       <c r="C41" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.8892924301031637E-2</v>
+        <v>9.7029602251831923E-2</v>
       </c>
     </row>
     <row r="42" spans="2:14" x14ac:dyDescent="0.2">
@@ -24070,7 +24041,7 @@
       </c>
       <c r="C44" s="24">
         <f ca="1">C43/(1+C41)^5</f>
-        <v>2922396.9896485889</v>
+        <v>2947300.129292103</v>
       </c>
     </row>
     <row r="45" spans="2:14" x14ac:dyDescent="0.2">
@@ -24079,7 +24050,7 @@
       </c>
       <c r="C45" s="108">
         <f ca="1">SUM(H9:K9)+C44</f>
-        <v>3302635.7512936094</v>
+        <v>3329124.7445658026</v>
       </c>
     </row>
     <row r="46" spans="2:14" x14ac:dyDescent="0.2">
@@ -24106,7 +24077,7 @@
       </c>
       <c r="C48" s="94">
         <f ca="1">C45+C46-C47</f>
-        <v>3364808.7512936094</v>
+        <v>3391297.7445658026</v>
       </c>
     </row>
     <row r="49" spans="2:3" x14ac:dyDescent="0.2">
@@ -24124,7 +24095,7 @@
       </c>
       <c r="C50" s="235">
         <f ca="1">C48/C49</f>
-        <v>229.63275447305054</v>
+        <v>231.44050669254096</v>
       </c>
     </row>
     <row r="52" spans="2:3" x14ac:dyDescent="0.2">
@@ -24148,7 +24119,7 @@
       </c>
       <c r="C54" s="135">
         <f ca="1">IF(Overview!C29&gt;0,Overview!C29,WACC!C19)</f>
-        <v>9.9910499999999999E-2</v>
+        <v>9.7994999999999999E-2</v>
       </c>
     </row>
     <row r="55" spans="2:3" x14ac:dyDescent="0.2">
@@ -24183,7 +24154,7 @@
       </c>
       <c r="C58" s="235">
         <f ca="1">C57/(1+C54)^5</f>
-        <v>201.200208242569</v>
+        <v>202.96135486625744</v>
       </c>
     </row>
     <row r="60" spans="2:3" x14ac:dyDescent="0.2">
@@ -24207,7 +24178,7 @@
       </c>
       <c r="C62" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.8892924301031637E-2</v>
+        <v>9.7029602251831923E-2</v>
       </c>
     </row>
     <row r="63" spans="2:3" x14ac:dyDescent="0.2">
@@ -24233,7 +24204,7 @@
       </c>
       <c r="C65" s="24">
         <f ca="1">C64/(1+C62)^5</f>
-        <v>2483207.7916284888</v>
+        <v>2504368.3904854641</v>
       </c>
     </row>
     <row r="66" spans="2:3" x14ac:dyDescent="0.2">
@@ -24242,7 +24213,7 @@
       </c>
       <c r="C66" s="108">
         <f ca="1">SUM(H9:K9)+C65</f>
-        <v>2863446.5532735093</v>
+        <v>2886193.0057591638</v>
       </c>
     </row>
     <row r="67" spans="2:3" x14ac:dyDescent="0.2">
@@ -24269,7 +24240,7 @@
       </c>
       <c r="C69" s="94">
         <f ca="1">C66+C67-C68</f>
-        <v>2925619.5532735093</v>
+        <v>2948366.0057591638</v>
       </c>
     </row>
     <row r="70" spans="2:3" x14ac:dyDescent="0.2">
@@ -24287,7 +24258,7 @@
       </c>
       <c r="C71" s="235">
         <f ca="1">C69/C70</f>
-        <v>199.66010736869646</v>
+        <v>201.21244835591099</v>
       </c>
     </row>
     <row r="73" spans="2:3" x14ac:dyDescent="0.2">
@@ -24311,7 +24282,7 @@
       </c>
       <c r="C75" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.8892924301031637E-2</v>
+        <v>9.7029602251831923E-2</v>
       </c>
     </row>
     <row r="76" spans="2:3" x14ac:dyDescent="0.2">
@@ -24337,7 +24308,7 @@
       </c>
       <c r="C78" s="24">
         <f ca="1">C77/(1+C75)^5</f>
-        <v>2688851.0682886597</v>
+        <v>2711764.0516620292</v>
       </c>
     </row>
     <row r="79" spans="2:3" x14ac:dyDescent="0.2">
@@ -24346,7 +24317,7 @@
       </c>
       <c r="C79" s="108">
         <f ca="1">SUM(H9:K9)+C78</f>
-        <v>3069089.8299336801</v>
+        <v>3093588.6669357289</v>
       </c>
     </row>
     <row r="80" spans="2:3" x14ac:dyDescent="0.2">
@@ -24373,7 +24344,7 @@
       </c>
       <c r="C82" s="94">
         <f ca="1">C79+C80-C81</f>
-        <v>3131262.8299336801</v>
+        <v>3155761.6669357289</v>
       </c>
     </row>
     <row r="83" spans="2:3" x14ac:dyDescent="0.2">
@@ -24391,22 +24362,22 @@
       </c>
       <c r="C84" s="235">
         <f ca="1">C82/C83</f>
-        <v>213.69431720014197</v>
+        <v>215.36625038802489</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="B73:C73"/>
-    <mergeCell ref="C27:L27"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="B60:C60"/>
     <mergeCell ref="C22:L22"/>
     <mergeCell ref="C2:G2"/>
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="C4:L4"/>
     <mergeCell ref="C11:L11"/>
     <mergeCell ref="C17:L17"/>
+    <mergeCell ref="B73:C73"/>
+    <mergeCell ref="C27:L27"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="B60:C60"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -24456,7 +24427,7 @@
       </c>
       <c r="C5" s="133">
         <f ca="1">DCF!C26</f>
-        <v>114.4961108417382</v>
+        <v>117.23172915838408</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -24465,7 +24436,7 @@
       </c>
       <c r="C6" s="133">
         <f ca="1">Multiples!C50</f>
-        <v>229.63275447305054</v>
+        <v>231.44050669254096</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
@@ -24474,7 +24445,7 @@
       </c>
       <c r="C7" s="133">
         <f ca="1">Multiples!C58</f>
-        <v>201.200208242569</v>
+        <v>202.96135486625744</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
@@ -24483,7 +24454,7 @@
       </c>
       <c r="C8" s="133">
         <f ca="1">Multiples!C71</f>
-        <v>199.66010736869646</v>
+        <v>201.21244835591099</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
@@ -24492,7 +24463,7 @@
       </c>
       <c r="C9" s="133">
         <f ca="1">Multiples!C84</f>
-        <v>213.69431720014197</v>
+        <v>215.36625038802489</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
@@ -24501,7 +24472,7 @@
       </c>
       <c r="C10" s="235">
         <f ca="1">AVERAGE(C5:C9)</f>
-        <v>191.73669962523925</v>
+        <v>193.64245789222369</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
@@ -24510,7 +24481,7 @@
       </c>
       <c r="C11" s="133">
         <f ca="1">Overview!C5</f>
-        <v>340.435</v>
+        <v>347.72500000000002</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.2">
@@ -24519,7 +24490,7 @@
       </c>
       <c r="C12" s="149">
         <f ca="1">(C10-C11)/C11</f>
-        <v>-0.43678910915376135</v>
+        <v>-0.44311608917327289</v>
       </c>
     </row>
   </sheetData>
@@ -25028,7 +24999,7 @@
       </c>
       <c r="C24" s="135">
         <f ca="1">IF(Overview!C29&gt;0,Overview!C29,WACC!C19)</f>
-        <v>9.9910499999999999E-2</v>
+        <v>9.7994999999999999E-2</v>
       </c>
     </row>
     <row r="25" spans="2:14" x14ac:dyDescent="0.2">
@@ -25045,7 +25016,7 @@
       </c>
       <c r="C26" s="235">
         <f ca="1">C23/(C24-C25)</f>
-        <v>13.274851239824555</v>
+        <v>13.600871850759665</v>
       </c>
     </row>
   </sheetData>
@@ -25282,7 +25253,7 @@
       <c r="K8" s="137"/>
       <c r="L8" s="126">
         <f ca="1">L7*(1+C20)/(C21-C20)</f>
-        <v>6326643.5245096758</v>
+        <v>6479683.0577803422</v>
       </c>
       <c r="N8" s="91"/>
       <c r="O8" s="16"/>
@@ -25336,23 +25307,23 @@
       <c r="G10" s="138"/>
       <c r="H10" s="126">
         <f ca="1">H7/(1+$C$21)^H9</f>
-        <v>111078.52669588511</v>
+        <v>111267.19532211016</v>
       </c>
       <c r="I10" s="126">
         <f t="shared" ref="I10:L10" ca="1" si="1">I7/(1+$C$21)^I9</f>
-        <v>143031.32889371528</v>
+        <v>143517.62346030437</v>
       </c>
       <c r="J10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>184175.66071174777</v>
+        <v>185115.73140732135</v>
       </c>
       <c r="K10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>237155.55368862467</v>
+        <v>238770.91320388051</v>
       </c>
       <c r="L10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>305375.62036160333</v>
+        <v>307977.87178210734</v>
       </c>
       <c r="N10" s="91"/>
     </row>
@@ -25371,15 +25342,15 @@
       <c r="K11" s="137"/>
       <c r="L11" s="126">
         <f ca="1">L8/(1+C21)^L9</f>
-        <v>3948175.7778468141</v>
+        <v>4078139.0534867868</v>
       </c>
     </row>
     <row r="13" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="14" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="B14" s="259" t="s">
+      <c r="B14" s="258" t="s">
         <v>219</v>
       </c>
-      <c r="C14" s="260"/>
+      <c r="C14" s="259"/>
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B15" s="150" t="s">
@@ -25387,7 +25358,7 @@
       </c>
       <c r="C15" s="151">
         <f ca="1">Overview!C5</f>
-        <v>340.435</v>
+        <v>347.72500000000002</v>
       </c>
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.2">
@@ -25396,7 +25367,7 @@
       </c>
       <c r="C16" s="151">
         <f ca="1">C36</f>
-        <v>342.00119694383932</v>
+        <v>351.30611132400372</v>
       </c>
     </row>
     <row r="17" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -25406,20 +25377,20 @@
       <c r="C17" s="153">
         <v>0.41499999999999998</v>
       </c>
-      <c r="E17" s="258" t="s">
+      <c r="E17" s="260" t="s">
         <v>222</v>
       </c>
-      <c r="F17" s="258"/>
-      <c r="G17" s="258"/>
-      <c r="H17" s="258"/>
-      <c r="I17" s="258"/>
+      <c r="F17" s="260"/>
+      <c r="G17" s="260"/>
+      <c r="H17" s="260"/>
+      <c r="I17" s="260"/>
     </row>
     <row r="18" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B19" s="259" t="s">
+      <c r="B19" s="258" t="s">
         <v>181</v>
       </c>
-      <c r="C19" s="260"/>
+      <c r="C19" s="259"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B20" s="154" t="s">
@@ -25435,7 +25406,7 @@
       </c>
       <c r="C21" s="216">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.8892924301031637E-2</v>
+        <v>9.7029602251831923E-2</v>
       </c>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.2">
@@ -25453,7 +25424,7 @@
       </c>
       <c r="C23" s="156">
         <f ca="1">C15*C22</f>
-        <v>4968308.3899999997</v>
+        <v>5074698.6500000004</v>
       </c>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.2">
@@ -25480,15 +25451,15 @@
       </c>
       <c r="C26" s="157">
         <f ca="1">C23+C25-C24</f>
-        <v>4906135.3899999997</v>
+        <v>5012525.6500000004</v>
       </c>
     </row>
     <row r="27" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="28" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B28" s="259" t="s">
+      <c r="B28" s="258" t="s">
         <v>183</v>
       </c>
-      <c r="C28" s="260"/>
+      <c r="C28" s="259"/>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B29" s="154" t="s">
@@ -25496,7 +25467,7 @@
       </c>
       <c r="C29" s="156">
         <f ca="1">SUM(H10:L10)</f>
-        <v>980816.6903515762</v>
+        <v>986649.33517572377</v>
       </c>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
@@ -25505,7 +25476,7 @@
       </c>
       <c r="C30" s="156">
         <f ca="1">L11</f>
-        <v>3948175.7778468141</v>
+        <v>4078139.0534867868</v>
       </c>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.2">
@@ -25514,7 +25485,7 @@
       </c>
       <c r="C31" s="159">
         <f ca="1">C29+C30</f>
-        <v>4928992.4681983907</v>
+        <v>5064788.3886625106</v>
       </c>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.2">
@@ -25541,7 +25512,7 @@
       </c>
       <c r="C34" s="159">
         <f ca="1">C31+C32-C33</f>
-        <v>4991165.4681983907</v>
+        <v>5126961.3886625106</v>
       </c>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.2">
@@ -25559,21 +25530,21 @@
       </c>
       <c r="C36" s="162">
         <f ca="1">C34/C35</f>
-        <v>342.00119694383932</v>
+        <v>351.30611132400372</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="E17:I17"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="H3:L3"/>
     <mergeCell ref="P3:W3"/>
     <mergeCell ref="X3:Z3"/>
     <mergeCell ref="C5:L5"/>
     <mergeCell ref="P5:Z5"/>
     <mergeCell ref="B14:C14"/>
-    <mergeCell ref="E17:I17"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="C3:G3"/>
-    <mergeCell ref="H3:L3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -32078,7 +32049,7 @@
       </c>
       <c r="AC114" s="63">
         <f ca="1">Overview!C5</f>
-        <v>340.435</v>
+        <v>347.72500000000002</v>
       </c>
     </row>
     <row r="115" spans="1:31" x14ac:dyDescent="0.2">
@@ -32149,7 +32120,7 @@
       </c>
       <c r="AC115" s="65">
         <f ca="1">AC114/AC84</f>
-        <v>340.435</v>
+        <v>347.72500000000002</v>
       </c>
     </row>
     <row r="117" spans="1:31" x14ac:dyDescent="0.2">
@@ -33063,7 +33034,7 @@
       <c r="AA140" s="49"/>
       <c r="AC140" s="72">
         <f ca="1">AC115/Statement!AC25</f>
-        <v>39.040711009174316</v>
+        <v>39.876720183486249</v>
       </c>
     </row>
     <row r="141" spans="2:29" x14ac:dyDescent="0.2">
@@ -33100,7 +33071,7 @@
       <c r="AA141" s="49"/>
       <c r="AC141" s="72">
         <f ca="1">AC115/(Statement!AC5/Statement!AC21)</f>
-        <v>10.77754043020588</v>
+        <v>11.008328303768238</v>
       </c>
     </row>
     <row r="142" spans="2:29" x14ac:dyDescent="0.2">
@@ -33161,7 +33132,7 @@
       </c>
       <c r="AC142" s="72">
         <f ca="1">AC115/(Statement!AC48/Statement!AC74)</f>
-        <v>46.20822535342262</v>
+        <v>47.197718098958333</v>
       </c>
     </row>
     <row r="143" spans="2:29" x14ac:dyDescent="0.2">
@@ -33222,7 +33193,7 @@
       </c>
       <c r="AC143" s="141">
         <f ca="1">Statement!AC115*Statement!AC77</f>
-        <v>4988394.0549999997</v>
+        <v>5095214.4250000007</v>
       </c>
     </row>
     <row r="144" spans="2:29" x14ac:dyDescent="0.2">
@@ -33283,7 +33254,7 @@
       </c>
       <c r="AC144" s="141">
         <f ca="1">AC143+AC106-AC105+AC47+AC44</f>
-        <v>4926221.0549999997</v>
+        <v>5033041.4250000007</v>
       </c>
     </row>
     <row r="145" spans="2:29" x14ac:dyDescent="0.2">
@@ -33320,7 +33291,7 @@
       <c r="AA145" s="49"/>
       <c r="AC145" s="177">
         <f ca="1">AC144/AC5</f>
-        <v>10.552652836299838</v>
+        <v>10.781476973071166</v>
       </c>
     </row>
     <row r="146" spans="2:29" x14ac:dyDescent="0.2">
@@ -33357,7 +33328,7 @@
       <c r="AA146" s="49"/>
       <c r="AC146" s="177">
         <f ca="1">AC144/AC11</f>
-        <v>31.811009079226906</v>
+        <v>32.500800244093021</v>
       </c>
     </row>
     <row r="147" spans="2:29" x14ac:dyDescent="0.2">
@@ -33492,7 +33463,7 @@
       <c r="AA149" s="49"/>
       <c r="AC149" s="72">
         <f t="shared" ref="AC149:AC150" ca="1" si="137">AC143/AC147</f>
-        <v>40.563634297470259</v>
+        <v>41.432255015165445</v>
       </c>
     </row>
     <row r="150" spans="2:29" x14ac:dyDescent="0.2">
@@ -33529,7 +33500,7 @@
       <c r="AA150" s="49"/>
       <c r="AC150" s="72">
         <f t="shared" ca="1" si="137"/>
-        <v>40.217608400689151</v>
+        <v>41.089688593987901</v>
       </c>
     </row>
     <row r="151" spans="2:29" x14ac:dyDescent="0.2">
@@ -33566,7 +33537,7 @@
       <c r="AA151" s="49"/>
       <c r="AC151" s="74">
         <f t="shared" ref="AC151" ca="1" si="140">AC147/AC143</f>
-        <v>2.4652623398253169E-2</v>
+        <v>2.4135785021451767E-2</v>
       </c>
     </row>
     <row r="152" spans="2:29" x14ac:dyDescent="0.2">
@@ -33603,7 +33574,7 @@
       <c r="AA152" s="49"/>
       <c r="AC152" s="74">
         <f ca="1">AC25/AC115</f>
-        <v>2.5614287602626049E-2</v>
+        <v>2.5077288086850235E-2</v>
       </c>
     </row>
     <row r="153" spans="2:29" x14ac:dyDescent="0.2">
@@ -33640,7 +33611,7 @@
       <c r="AA153" s="49"/>
       <c r="AC153" s="149">
         <f ca="1">AC81/AC115</f>
-        <v>3.0842892182061186E-3</v>
+        <v>3.0196275792652239E-3</v>
       </c>
     </row>
     <row r="154" spans="2:29" x14ac:dyDescent="0.2">
@@ -33677,7 +33648,7 @@
       <c r="AA154" s="49"/>
       <c r="AC154" s="149">
         <f ca="1">-AC62/AC143</f>
-        <v>1.6483461228886418E-2</v>
+        <v>1.613788805365144E-2</v>
       </c>
     </row>
     <row r="155" spans="2:29" x14ac:dyDescent="0.2">
@@ -33714,7 +33685,7 @@
       <c r="AA155" s="49"/>
       <c r="AC155" s="149">
         <f ca="1">-(AC62+AC63)/AC143</f>
-        <v>1.9618738800698053E-2</v>
+        <v>1.9207435023698729E-2</v>
       </c>
     </row>
     <row r="156" spans="2:29" x14ac:dyDescent="0.2">
@@ -34217,7 +34188,7 @@
       <c r="AA166" s="49"/>
       <c r="AC166" s="149">
         <f ca="1">(AC105-AC106)/AC143</f>
-        <v>1.2463530209222817E-2</v>
+        <v>1.220223425631395E-2</v>
       </c>
     </row>
     <row r="167" spans="1:31" x14ac:dyDescent="0.2">
@@ -36269,7 +36240,7 @@
       </c>
       <c r="C5" s="166">
         <f ca="1">Overview!C5</f>
-        <v>340.435</v>
+        <v>347.72500000000002</v>
       </c>
       <c r="E5" s="12"/>
       <c r="F5" s="132" t="s">
@@ -36285,7 +36256,7 @@
       </c>
       <c r="C6" s="167">
         <f ca="1">Statement!AC143</f>
-        <v>4988394.0549999997</v>
+        <v>5095214.4250000007</v>
       </c>
       <c r="E6" s="20" t="s">
         <v>19</v>
@@ -36305,7 +36276,7 @@
       </c>
       <c r="C7" s="167">
         <f ca="1">Statement!AC144</f>
-        <v>4926221.0549999997</v>
+        <v>5033041.4250000007</v>
       </c>
       <c r="E7" s="20" t="s">
         <v>29</v>
@@ -36325,7 +36296,7 @@
       </c>
       <c r="C8" s="168">
         <f ca="1">Statement!AC140</f>
-        <v>39.040711009174316</v>
+        <v>39.876720183486249</v>
       </c>
       <c r="E8" s="20" t="s">
         <v>237</v>
@@ -36345,7 +36316,7 @@
       </c>
       <c r="C9" s="168">
         <f ca="1">Statement!AC141</f>
-        <v>10.77754043020588</v>
+        <v>11.008328303768238</v>
       </c>
       <c r="E9" s="20" t="s">
         <v>238</v>
@@ -36365,7 +36336,7 @@
       </c>
       <c r="C10" s="168">
         <f ca="1">Statement!AC142</f>
-        <v>46.20822535342262</v>
+        <v>47.197718098958333</v>
       </c>
       <c r="E10" s="20" t="s">
         <v>1</v>
@@ -36385,7 +36356,7 @@
       </c>
       <c r="C11" s="168">
         <f ca="1">Statement!AC145</f>
-        <v>10.552652836299838</v>
+        <v>10.781476973071166</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.2">
@@ -36394,7 +36365,7 @@
       </c>
       <c r="C12" s="168">
         <f ca="1">Statement!AC146</f>
-        <v>31.811009079226906</v>
+        <v>32.500800244093021</v>
       </c>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.2">
@@ -36630,7 +36601,7 @@
       </c>
       <c r="C38" s="169">
         <f ca="1">Statement!AC152</f>
-        <v>2.5614287602626049E-2</v>
+        <v>2.5077288086850235E-2</v>
       </c>
       <c r="E38" s="20" t="s">
         <v>264</v>
@@ -36646,7 +36617,7 @@
       </c>
       <c r="C39" s="209">
         <f ca="1">Statement!AC151</f>
-        <v>2.4652623398253169E-2</v>
+        <v>2.4135785021451767E-2</v>
       </c>
       <c r="E39" s="20" t="s">
         <v>266</v>
@@ -36662,7 +36633,7 @@
       </c>
       <c r="C40" s="169">
         <f ca="1">Statement!AC153</f>
-        <v>3.0842892182061186E-3</v>
+        <v>3.0196275792652239E-3</v>
       </c>
       <c r="E40" s="20" t="s">
         <v>267</v>
@@ -36678,7 +36649,7 @@
       </c>
       <c r="C41" s="169">
         <f ca="1">Statement!AC154</f>
-        <v>1.6483461228886418E-2</v>
+        <v>1.613788805365144E-2</v>
       </c>
     </row>
     <row r="42" spans="2:6" x14ac:dyDescent="0.2">
@@ -36687,7 +36658,7 @@
       </c>
       <c r="C42" s="169">
         <f ca="1">Statement!AC155</f>
-        <v>1.9618738800698053E-2</v>
+        <v>1.9207435023698729E-2</v>
       </c>
     </row>
     <row r="45" spans="2:6" x14ac:dyDescent="0.2">
@@ -36731,7 +36702,7 @@
       </c>
       <c r="F48" s="169">
         <f ca="1">Statement!AC166</f>
-        <v>1.2463530209222817E-2</v>
+        <v>1.220223425631395E-2</v>
       </c>
     </row>
     <row r="51" spans="2:6" x14ac:dyDescent="0.2">
@@ -36910,7 +36881,7 @@
       </c>
       <c r="I6" s="166">
         <f ca="1">Statement!AC114</f>
-        <v>340.435</v>
+        <v>347.72500000000002</v>
       </c>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.2">
@@ -36939,7 +36910,7 @@
       </c>
       <c r="I7" s="167">
         <f ca="1">Statement!AC143</f>
-        <v>4988394.0549999997</v>
+        <v>5095214.4250000007</v>
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
@@ -36968,7 +36939,7 @@
       </c>
       <c r="I8" s="167">
         <f ca="1">Statement!AC144</f>
-        <v>4926221.0549999997</v>
+        <v>5033041.4250000007</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
@@ -36997,7 +36968,7 @@
       </c>
       <c r="I9" s="168">
         <f ca="1">Statement!AC140</f>
-        <v>39.040711009174316</v>
+        <v>39.876720183486249</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.2">
@@ -37026,7 +36997,7 @@
       </c>
       <c r="I10" s="168">
         <f ca="1">Statement!AC141</f>
-        <v>10.77754043020588</v>
+        <v>11.008328303768238</v>
       </c>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.2">
@@ -37055,7 +37026,7 @@
       </c>
       <c r="I11" s="168">
         <f ca="1">Statement!AC142</f>
-        <v>46.20822535342262</v>
+        <v>47.197718098958333</v>
       </c>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.2">
@@ -37084,7 +37055,7 @@
       </c>
       <c r="I12" s="168">
         <f ca="1">Statement!AC145</f>
-        <v>10.552652836299838</v>
+        <v>10.781476973071166</v>
       </c>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
@@ -37113,7 +37084,7 @@
       </c>
       <c r="I13" s="168">
         <f ca="1">Statement!AC146</f>
-        <v>31.811009079226906</v>
+        <v>32.500800244093021</v>
       </c>
     </row>
     <row r="15" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -37886,7 +37857,7 @@
       </c>
       <c r="I51" s="169">
         <f ca="1">Statement!AC152</f>
-        <v>2.5614287602626049E-2</v>
+        <v>2.5077288086850235E-2</v>
       </c>
     </row>
     <row r="52" spans="2:9" x14ac:dyDescent="0.2">
@@ -37915,7 +37886,7 @@
       </c>
       <c r="I52" s="169">
         <f ca="1">Statement!AC151</f>
-        <v>2.4652623398253169E-2</v>
+        <v>2.4135785021451767E-2</v>
       </c>
     </row>
     <row r="53" spans="2:9" x14ac:dyDescent="0.2">
@@ -37944,7 +37915,7 @@
       </c>
       <c r="I53" s="169">
         <f ca="1">Statement!AC153</f>
-        <v>3.0842892182061186E-3</v>
+        <v>3.0196275792652239E-3</v>
       </c>
     </row>
     <row r="54" spans="2:9" x14ac:dyDescent="0.2">
@@ -37973,7 +37944,7 @@
       </c>
       <c r="I54" s="169">
         <f ca="1">Statement!AC154</f>
-        <v>1.6483461228886418E-2</v>
+        <v>1.613788805365144E-2</v>
       </c>
     </row>
     <row r="55" spans="2:9" x14ac:dyDescent="0.2">
@@ -38002,7 +37973,7 @@
       </c>
       <c r="I55" s="169">
         <f ca="1">Statement!AC155</f>
-        <v>1.9618738800698053E-2</v>
+        <v>1.9207435023698729E-2</v>
       </c>
     </row>
     <row r="57" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -38238,7 +38209,7 @@
       </c>
       <c r="I68" s="190">
         <f ca="1">Statement!AC166</f>
-        <v>1.2463530209222817E-2</v>
+        <v>1.220223425631395E-2</v>
       </c>
     </row>
     <row r="70" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -38930,14 +38901,14 @@
     <row r="1" spans="2:7" ht="12" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="3" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B3" s="8"/>
-      <c r="C3" s="249" t="s">
+      <c r="C3" s="247" t="s">
         <v>307</v>
       </c>
-      <c r="D3" s="250"/>
-      <c r="F3" s="251" t="s">
+      <c r="D3" s="248"/>
+      <c r="F3" s="249" t="s">
         <v>308</v>
       </c>
-      <c r="G3" s="250"/>
+      <c r="G3" s="248"/>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B4" s="8"/>
@@ -39004,19 +38975,19 @@
       <c r="B7" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C7" s="247">
+      <c r="C7" s="250">
         <f>Statement!AA88</f>
         <v>-1.5892574471146927E-2</v>
       </c>
-      <c r="D7" s="248"/>
-      <c r="F7" s="247">
+      <c r="D7" s="251"/>
+      <c r="F7" s="250">
         <f>IF(F6=0,
 IF(G6=0,0,IF(G6&gt;0,1,-1)),
 (G6-F6)/ABS(F6)
 )</f>
         <v>0.16356501765281381</v>
       </c>
-      <c r="G7" s="248"/>
+      <c r="G7" s="251"/>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B8" s="201" t="s">
@@ -39043,19 +39014,19 @@
       <c r="B9" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C9" s="247">
+      <c r="C9" s="250">
         <f>Statement!AA89</f>
         <v>-3.1133095757317875E-2</v>
       </c>
-      <c r="D9" s="248"/>
-      <c r="F9" s="247">
+      <c r="D9" s="251"/>
+      <c r="F9" s="250">
         <f>IF(F8=0,
 IF(G8=0,0,IF(G8&gt;0,1,-1)),
 (G8-F8)/ABS(F8)
 )</f>
         <v>8.6032831193608647E-2</v>
       </c>
-      <c r="G9" s="248"/>
+      <c r="G9" s="251"/>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B10" s="201" t="s">
@@ -39082,19 +39053,19 @@
       <c r="B11" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C11" s="247">
+      <c r="C11" s="250">
         <f>Statement!AA90</f>
         <v>-2.0079954728829339E-4</v>
       </c>
-      <c r="D11" s="248"/>
-      <c r="F11" s="247">
+      <c r="D11" s="251"/>
+      <c r="F11" s="250">
         <f>IF(F10=0,
 IF(G10=0,0,IF(G10&gt;0,1,-1)),
 (G10-F10)/ABS(F10)
 )</f>
         <v>0.25280204949906215</v>
       </c>
-      <c r="G11" s="248"/>
+      <c r="G11" s="251"/>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B12" s="201" t="s">
@@ -39121,19 +39092,19 @@
       <c r="B13" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C13" s="247">
+      <c r="C13" s="250">
         <f>Statement!AA93</f>
         <v>9.4729043183742583E-3</v>
       </c>
-      <c r="D13" s="248"/>
-      <c r="F13" s="247">
+      <c r="D13" s="251"/>
+      <c r="F13" s="250">
         <f>IF(F12=0,
 IF(G12=0,0,IF(G12&gt;0,1,-1)),
 (G12-F12)/ABS(F12)
 )</f>
         <v>0.22937612786800721</v>
       </c>
-      <c r="G13" s="248"/>
+      <c r="G13" s="251"/>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B14" s="201" t="s">
@@ -39160,19 +39131,19 @@
       <c r="B15" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C15" s="247">
+      <c r="C15" s="250">
         <f>Statement!AA94</f>
         <v>-5.2946913752264175E-3</v>
       </c>
-      <c r="D15" s="248"/>
-      <c r="F15" s="247">
+      <c r="D15" s="251"/>
+      <c r="F15" s="250">
         <f>IF(F14=0,
 IF(G14=0,0,IF(G14&gt;0,1,-1)),
 (G14-F14)/ABS(F14)
 )</f>
         <v>0.26569037656903766</v>
       </c>
-      <c r="G15" s="248"/>
+      <c r="G15" s="251"/>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B16" s="201" t="s">
@@ -39199,19 +39170,19 @@
       <c r="B17" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C17" s="247">
+      <c r="C17" s="250">
         <f>Statement!AA96</f>
         <v>7.1336804381635002E-3</v>
       </c>
-      <c r="D17" s="248"/>
-      <c r="F17" s="247">
+      <c r="D17" s="251"/>
+      <c r="F17" s="250">
         <f>IF(F16=0,
 IF(G16=0,0,IF(G16&gt;0,1,-1)),
 (G16-F16)/ABS(F16)
 )</f>
         <v>0.27118716394981651</v>
       </c>
-      <c r="G17" s="248"/>
+      <c r="G17" s="251"/>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B18" s="201" t="s">
@@ -39238,22 +39209,22 @@
       <c r="B19" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C19" s="247">
+      <c r="C19" s="250">
         <f>IF(C18=0,
 IF(D18=0,0,IF(D18&gt;0,1,-1)),
 (D18-C18)/ABS(C18)
 )</f>
         <v>-7.4697813391280731E-4</v>
       </c>
-      <c r="D19" s="248"/>
-      <c r="F19" s="247">
+      <c r="D19" s="251"/>
+      <c r="F19" s="250">
         <f>IF(F18=0,
 IF(G18=0,0,IF(G18&gt;0,1,-1)),
 (G18-F18)/ABS(F18)
 )</f>
         <v>-1.5587369547765587E-2</v>
       </c>
-      <c r="G19" s="248"/>
+      <c r="G19" s="251"/>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B20" s="201" t="s">
@@ -39280,22 +39251,22 @@
       <c r="B21" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C21" s="247">
+      <c r="C21" s="250">
         <f>IF(C20=0,
 IF(D20=0,0,IF(D20&gt;0,1,-1)),
 (D20-C20)/ABS(C20)
 )</f>
         <v>4.975124378109568E-3</v>
       </c>
-      <c r="D21" s="248"/>
-      <c r="F21" s="247">
+      <c r="D21" s="251"/>
+      <c r="F21" s="250">
         <f>IF(F20=0,
 IF(G20=0,0,IF(G20&gt;0,1,-1)),
 (G20-F20)/ABS(F20)
 )</f>
         <v>0.28662420382165599</v>
       </c>
-      <c r="G21" s="248"/>
+      <c r="G21" s="251"/>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23" s="8" t="s">
@@ -39343,22 +39314,22 @@
       <c r="B25" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C25" s="247">
+      <c r="C25" s="250">
         <f>IF(C24=0,
 IF(D24=0,0,IF(D24&gt;0,1,-1)),
 (D24-C24)/ABS(C24)
 )</f>
         <v>1.5257357017718937E-2</v>
       </c>
-      <c r="D25" s="248"/>
-      <c r="F25" s="247">
+      <c r="D25" s="251"/>
+      <c r="F25" s="250">
         <f>IF(F24=0,
 IF(G24=0,0,IF(G24&gt;0,1,-1)),
 (G24-F24)/ABS(F24)
 )</f>
         <v>0.11124326423612797</v>
       </c>
-      <c r="G25" s="248"/>
+      <c r="G25" s="251"/>
     </row>
     <row r="26" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B26" s="20" t="s">
@@ -39385,22 +39356,22 @@
       <c r="B27" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C27" s="247">
+      <c r="C27" s="250">
         <f>IF(C26=0,
 IF(D26=0,0,IF(D26&gt;0,1,-1)),
 (D26-C26)/ABS(C26)
 )</f>
         <v>4.7692033505613969E-2</v>
       </c>
-      <c r="D27" s="248"/>
-      <c r="F27" s="247">
+      <c r="D27" s="251"/>
+      <c r="F27" s="250">
         <f>IF(F26=0,
 IF(G26=0,0,IF(G26&gt;0,1,-1)),
 (G26-F26)/ABS(F26)
 )</f>
         <v>0.22399433663696178</v>
       </c>
-      <c r="G27" s="248"/>
+      <c r="G27" s="251"/>
     </row>
     <row r="28" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B28" s="20" t="s">
@@ -39427,22 +39398,22 @@
       <c r="B29" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C29" s="247">
+      <c r="C29" s="250">
         <f>IF(C28=0,
 IF(D28=0,0,IF(D28&gt;0,1,-1)),
 (D28-C28)/ABS(C28)
 )</f>
         <v>-8.2012001756354591E-2</v>
       </c>
-      <c r="D29" s="248"/>
-      <c r="F29" s="247">
+      <c r="D29" s="251"/>
+      <c r="F29" s="250">
         <f>IF(F28=0,
 IF(G28=0,0,IF(G28&gt;0,1,-1)),
 (G28-F28)/ABS(F28)
 )</f>
         <v>0.22428264688658989</v>
       </c>
-      <c r="G29" s="248"/>
+      <c r="G29" s="251"/>
     </row>
     <row r="30" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B30" s="20" t="s">
@@ -39469,22 +39440,22 @@
       <c r="B31" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C31" s="247">
+      <c r="C31" s="250">
         <f>IF(C30=0,
 IF(D30=0,0,IF(D30&gt;0,1,-1)),
 (D30-C30)/ABS(C30)
 )</f>
         <v>-0.21985477919295321</v>
       </c>
-      <c r="D31" s="248"/>
-      <c r="F31" s="247">
+      <c r="D31" s="251"/>
+      <c r="F31" s="250">
         <f>IF(F30=0,
 IF(G30=0,0,IF(G30&gt;0,1,-1)),
 (G30-F30)/ABS(F30)
 )</f>
         <v>0.1335178139052231</v>
       </c>
-      <c r="G31" s="248"/>
+      <c r="G31" s="251"/>
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B32" s="20" t="s">
@@ -39511,22 +39482,22 @@
       <c r="B33" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C33" s="247">
+      <c r="C33" s="250">
         <f>IF(C32=0,
 IF(D32=0,0,IF(D32&gt;0,1,-1)),
 (D32-C32)/ABS(C32)
 )</f>
         <v>-2.9218647406434668E-2</v>
       </c>
-      <c r="D33" s="248"/>
-      <c r="F33" s="247">
+      <c r="D33" s="251"/>
+      <c r="F33" s="250">
         <f>IF(F32=0,
 IF(G32=0,0,IF(G32&gt;0,1,-1)),
 (G32-F32)/ABS(F32)
 )</f>
         <v>0.15613189104652678</v>
       </c>
-      <c r="G33" s="248"/>
+      <c r="G33" s="251"/>
     </row>
     <row r="35" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B35" s="224" t="s">
@@ -39553,22 +39524,22 @@
       <c r="B36" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C36" s="247">
+      <c r="C36" s="250">
         <f>IF(C35=0,
 IF(D35=0,0,IF(D35&gt;0,1,-1)),
 (D35-C35)/ABS(C35)
 )</f>
         <v>-4.8110327402884512E-2</v>
       </c>
-      <c r="D36" s="248"/>
-      <c r="F36" s="247">
+      <c r="D36" s="251"/>
+      <c r="F36" s="250">
         <f>IF(F35=0,
 IF(G35=0,0,IF(G35&gt;0,1,-1)),
 (G35-F35)/ABS(F35)
 )</f>
         <v>0.21690368310080302</v>
       </c>
-      <c r="G36" s="248"/>
+      <c r="G36" s="251"/>
     </row>
     <row r="37" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B37" s="224" t="s">
@@ -39595,22 +39566,22 @@
       <c r="B38" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C38" s="247">
+      <c r="C38" s="250">
         <f>IF(C37=0,
 IF(D37=0,0,IF(D37&gt;0,1,-1)),
 (D37-C37)/ABS(C37)
 )</f>
         <v>0.23252768186688891</v>
       </c>
-      <c r="D38" s="248"/>
-      <c r="F38" s="247">
+      <c r="D38" s="251"/>
+      <c r="F38" s="250">
         <f>IF(F37=0,
 IF(G37=0,0,IF(G37&gt;0,1,-1)),
 (G37-F37)/ABS(F37)
 )</f>
         <v>0.28660203827989061</v>
       </c>
-      <c r="G38" s="248"/>
+      <c r="G38" s="251"/>
     </row>
     <row r="39" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B39" s="224" t="s">
@@ -39637,22 +39608,22 @@
       <c r="B40" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C40" s="247">
+      <c r="C40" s="250">
         <f>IF(C39=0,
 IF(D39=0,0,IF(D39&gt;0,1,-1)),
 (D39-C39)/ABS(C39)
 )</f>
         <v>-0.10457043679490888</v>
       </c>
-      <c r="D40" s="248"/>
-      <c r="F40" s="247">
+      <c r="D40" s="251"/>
+      <c r="F40" s="250">
         <f>IF(F39=0,
 IF(G39=0,0,IF(G39&gt;0,1,-1)),
 (G39-F39)/ABS(F39)
 )</f>
         <v>-5.9261510408752466E-2</v>
       </c>
-      <c r="G40" s="248"/>
+      <c r="G40" s="251"/>
     </row>
     <row r="41" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B41" s="224" t="s">
@@ -39679,22 +39650,22 @@
       <c r="B42" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C42" s="247">
+      <c r="C42" s="250">
         <f>IF(C41=0,
 IF(D41=0,0,IF(D41&gt;0,1,-1)),
 (D41-C41)/ABS(C41)
 )</f>
         <v>-2.2781926338438173E-3</v>
       </c>
-      <c r="D42" s="248"/>
-      <c r="F42" s="247">
+      <c r="D42" s="251"/>
+      <c r="F42" s="250">
         <f>IF(F41=0,
 IF(G41=0,0,IF(G41&gt;0,1,-1)),
 (G41-F41)/ABS(F41)
 )</f>
         <v>6.4694759589411135E-2</v>
       </c>
-      <c r="G42" s="248"/>
+      <c r="G42" s="251"/>
     </row>
     <row r="43" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B43" s="224" t="s">
@@ -39721,55 +39692,25 @@
       <c r="B44" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C44" s="247">
+      <c r="C44" s="250">
         <f>IF(C43=0,
 IF(D43=0,0,IF(D43&gt;0,1,-1)),
 (D43-C43)/ABS(C43)
 )</f>
         <v>-7.6510847107438013E-3</v>
       </c>
-      <c r="D44" s="248"/>
-      <c r="F44" s="247">
+      <c r="D44" s="251"/>
+      <c r="F44" s="250">
         <f>IF(F43=0,
 IF(G43=0,0,IF(G43&gt;0,1,-1)),
 (G43-F43)/ABS(F43)
 )</f>
         <v>0.12092039528862633</v>
       </c>
-      <c r="G44" s="248"/>
+      <c r="G44" s="251"/>
     </row>
   </sheetData>
   <mergeCells count="38">
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="F36:G36"/>
     <mergeCell ref="C44:D44"/>
     <mergeCell ref="F44:G44"/>
     <mergeCell ref="C38:D38"/>
@@ -39778,6 +39719,36 @@
     <mergeCell ref="F40:G40"/>
     <mergeCell ref="C42:D42"/>
     <mergeCell ref="F42:G42"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="F36:G36"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="F9:G9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>

</xml_diff>

<commit_message>
Updated the list file and added metrics to some of the stocks
</commit_message>
<xml_diff>
--- a/AAPL.xlsx
+++ b/AAPL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/KINGSTON/MyStockData/Finance-StockLists/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28F5C13A-E116-8A49-A165-25B31C0AEF2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5E1A667-BA76-D142-909E-6D5DAE5E4113}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="14400" xr2:uid="{AEC0C047-6E16-294C-82BD-58123BA913A1}"/>
   </bookViews>
@@ -2391,6 +2391,12 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="168" fontId="18" fillId="17" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="18" fillId="17" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2398,12 +2404,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="18" fillId="17" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="18" fillId="17" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="5" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2424,14 +2424,14 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -15571,11 +15571,11 @@
     <v>Powered by Refinitiv</v>
     <v>351.73</v>
     <v>243.42</v>
-    <v>1.077</v>
-    <v>-0.495</v>
-    <v>-1.4219999999999999E-3</v>
-    <v>-0.185</v>
-    <v>-5.3199999999999992E-4</v>
+    <v>1.0749</v>
+    <v>-3.8149999999999999</v>
+    <v>-1.0971E-2</v>
+    <v>0.33</v>
+    <v>9.5960000000000001E-4</v>
     <v>USD</v>
     <v>Apple Inc. designs, manufactures and markets smartphones, personal computers, tablets, wearables and accessories, and sells a variety of related services. Its product categories include iPhone, Mac, iPad, Wearables, Home and Accessories. Its services include advertising, AppleCare, cloud services, digital content, and payment services. The Company operates various platforms, including the App Store, that allow customers to discover and download applications and digital content, such as books, music, video, games and podcasts. It also offers digital content through subscription-based services, including Apple Arcade, Apple Fitness+, Apple Music, Apple News+, and Apple TV+. Its wearables include smartwatches, wireless headphones, and spatial computers. Its products include iPhone 16 Pro, iPhone 16, iPhone 15, iPhone 14, iPhone SE, MacBook Air, MacBook Pro, iMac, Mac mini, Mac Studio, Mac Pro, iPad Pro, iPad Air, AirPods, AirPods Pro, AirPods Max, Apple TV, Apple Vision Pro and others.</v>
     <v>166000</v>
@@ -15583,25 +15583,25 @@
     <v>XNAS</v>
     <v>XNAS</v>
     <v>One Apple Park Way, CUPERTINO, CA, 95014 US</v>
-    <v>351.73</v>
+    <v>347.09</v>
     <v>Computers, Phones &amp; Household Electronics</v>
     <v>Stock</v>
-    <v>46318.958116758593</v>
+    <v>46321.85777778906</v>
     <v>0</v>
-    <v>345.75</v>
-    <v>5074761240500</v>
+    <v>341.03</v>
+    <v>5019084443800</v>
     <v>APPLE INC.</v>
     <v>APPLE INC.</v>
-    <v>349.11500000000001</v>
-    <v>40.0687</v>
-    <v>348.22</v>
+    <v>343.92</v>
+    <v>39.572600000000001</v>
     <v>347.72500000000002</v>
-    <v>347.54</v>
+    <v>343.91</v>
+    <v>344.24</v>
     <v>14594180000</v>
     <v>AAPL</v>
     <v>APPLE INC. (XNAS:AAPL)</v>
-    <v>39502829</v>
-    <v>39174961</v>
+    <v>42220287</v>
+    <v>37293021</v>
     <v>1977</v>
   </rv>
   <rv s="2">
@@ -15625,17 +15625,17 @@
     <v>Powered by Refinitiv</v>
     <v>53.64</v>
     <v>39.47</v>
-    <v>-1.93</v>
-    <v>-3.7505000000000004E-2</v>
+    <v>0.35</v>
+    <v>7.0660000000000002E-3</v>
     <v>US</v>
-    <v>50.54</v>
+    <v>50.03</v>
     <v>Index</v>
     <v>3</v>
-    <v>49.39</v>
+    <v>49.55</v>
     <v>10 Y TSY YLD NDX</v>
-    <v>50.4</v>
-    <v>51.46</v>
+    <v>49.92</v>
     <v>49.53</v>
+    <v>49.88</v>
     <v>TNX</v>
     <v>10 Y TSY YLD NDX</v>
   </rv>
@@ -16461,7 +16461,7 @@
       </c>
       <c r="F3" s="181">
         <f ca="1">Statement!AC143</f>
-        <v>5095214.4250000007</v>
+        <v>5039313.2300000004</v>
       </c>
       <c r="H3" s="179" t="str">
         <f>'AVG target price'!B5</f>
@@ -16469,7 +16469,7 @@
       </c>
       <c r="I3" s="205">
         <f ca="1">'AVG target price'!C5</f>
-        <v>117.23172915838408</v>
+        <v>116.87080807776867</v>
       </c>
       <c r="K3" s="238" t="s">
         <v>422</v>
@@ -16488,7 +16488,7 @@
       </c>
       <c r="F4" s="182">
         <f ca="1">Statement!AC144</f>
-        <v>5033041.4250000007</v>
+        <v>4977140.2300000004</v>
       </c>
       <c r="H4" s="179" t="str">
         <f>'AVG target price'!B6</f>
@@ -16496,7 +16496,7 @@
       </c>
       <c r="I4" s="205">
         <f ca="1">'AVG target price'!C6</f>
-        <v>231.44050669254096</v>
+        <v>231.20590979823791</v>
       </c>
       <c r="K4" s="238" t="s">
         <v>423</v>
@@ -16508,7 +16508,7 @@
       </c>
       <c r="C5" s="202" cm="1">
         <f t="array" aca="1" ref="C5" ca="1">_FV(C3,"Price",TRUE)</f>
-        <v>347.72500000000002</v>
+        <v>343.91</v>
       </c>
       <c r="E5" s="179" t="s">
         <v>237</v>
@@ -16523,7 +16523,7 @@
       </c>
       <c r="I5" s="205">
         <f ca="1">'AVG target price'!C7</f>
-        <v>202.96135486625744</v>
+        <v>202.72537726530837</v>
       </c>
       <c r="K5" s="238" t="s">
         <v>424</v>
@@ -16535,14 +16535,14 @@
       </c>
       <c r="C6" s="202" cm="1">
         <f t="array" aca="1" ref="C6" ca="1">_FV(C3,"Price (Extended hours)",TRUE)</f>
-        <v>347.54</v>
+        <v>344.24</v>
       </c>
       <c r="E6" s="179" t="s">
         <v>231</v>
       </c>
       <c r="F6" s="184">
         <f ca="1">Statement!AC140</f>
-        <v>39.876720183486249</v>
+        <v>39.439220183486249</v>
       </c>
       <c r="H6" s="179" t="str">
         <f>'AVG target price'!B8</f>
@@ -16550,7 +16550,7 @@
       </c>
       <c r="I6" s="205">
         <f ca="1">'AVG target price'!C8</f>
-        <v>201.21244835591099</v>
+        <v>201.01099985192954</v>
       </c>
       <c r="K6" s="239" t="s">
         <v>425</v>
@@ -16562,14 +16562,14 @@
       </c>
       <c r="C7" s="6" cm="1">
         <f t="array" aca="1" ref="C7" ca="1">_FV(C3,"Change")</f>
-        <v>-0.495</v>
+        <v>-3.8149999999999999</v>
       </c>
       <c r="E7" s="180" t="s">
         <v>198</v>
       </c>
       <c r="F7" s="185">
         <f ca="1">Statement!AC141</f>
-        <v>11.008328303768238</v>
+        <v>10.887552482418391</v>
       </c>
       <c r="H7" s="179" t="str">
         <f>'AVG target price'!B9</f>
@@ -16577,7 +16577,7 @@
       </c>
       <c r="I7" s="205">
         <f ca="1">'AVG target price'!C9</f>
-        <v>215.36625038802489</v>
+        <v>215.14928068353927</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.2">
@@ -16586,14 +16586,14 @@
       </c>
       <c r="C8" s="6" cm="1">
         <f t="array" aca="1" ref="C8" ca="1">_FV(C3,"Change (extended hours)",TRUE)</f>
-        <v>-0.185</v>
+        <v>0.33</v>
       </c>
       <c r="E8" s="179" t="s">
         <v>259</v>
       </c>
       <c r="F8" s="186">
         <f ca="1">Statement!AC151</f>
-        <v>2.4135785021451767E-2</v>
+        <v>2.4403523731744689E-2</v>
       </c>
       <c r="H8" s="178" t="str">
         <f>'AVG target price'!B10</f>
@@ -16601,7 +16601,7 @@
       </c>
       <c r="I8" s="206">
         <f ca="1">'AVG target price'!C10</f>
-        <v>193.64245789222369</v>
+        <v>193.39247513535673</v>
       </c>
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.2">
@@ -16610,14 +16610,14 @@
       </c>
       <c r="C9" s="73" cm="1">
         <f t="array" aca="1" ref="C9" ca="1">_FV(C3,"Change (%)",TRUE)</f>
-        <v>-1.4219999999999999E-3</v>
+        <v>-1.0971E-2</v>
       </c>
       <c r="E9" s="179" t="s">
         <v>282</v>
       </c>
       <c r="F9" s="186">
         <f ca="1">Statement!AC152</f>
-        <v>2.5077288086850235E-2</v>
+        <v>2.5355470908086413E-2</v>
       </c>
       <c r="H9" s="178" t="str">
         <f>'AVG target price'!B12</f>
@@ -16625,7 +16625,7 @@
       </c>
       <c r="I9" s="207">
         <f ca="1">'AVG target price'!C12</f>
-        <v>-0.44311608917327289</v>
+        <v>-0.43766544986956846</v>
       </c>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.2">
@@ -16634,14 +16634,14 @@
       </c>
       <c r="C10" s="73" cm="1">
         <f t="array" aca="1" ref="C10" ca="1">_FV(C3,"Change % (extended hours)",TRUE)</f>
-        <v>-5.3199999999999992E-4</v>
+        <v>9.5960000000000001E-4</v>
       </c>
       <c r="E10" s="179" t="s">
         <v>287</v>
       </c>
       <c r="F10" s="186">
         <f ca="1">Statement!AC154</f>
-        <v>1.613788805365144E-2</v>
+        <v>1.6316905944741202E-2</v>
       </c>
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.2">
@@ -16657,14 +16657,14 @@
       </c>
       <c r="F11" s="187">
         <f ca="1">Statement!AC153</f>
-        <v>3.0196275792652239E-3</v>
+        <v>3.0531243639324241E-3</v>
       </c>
       <c r="H11" s="178" t="s">
         <v>394</v>
       </c>
       <c r="I11" s="206">
         <f ca="1">DDM!C26</f>
-        <v>13.600871850759665</v>
+        <v>13.556462898000653</v>
       </c>
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.2">
@@ -16689,7 +16689,7 @@
       </c>
       <c r="C13" s="203" cm="1">
         <f t="array" aca="1" ref="C13" ca="1">_FV(C3,"Beta")</f>
-        <v>1.077</v>
+        <v>1.0749</v>
       </c>
       <c r="E13" s="179" t="s">
         <v>101</v>
@@ -16712,7 +16712,7 @@
       </c>
       <c r="C14" s="204" cm="1">
         <f t="array" aca="1" ref="C14" ca="1">_FV(C3,"Volume average",TRUE)</f>
-        <v>39174961</v>
+        <v>37293021</v>
       </c>
       <c r="E14" s="180" t="s">
         <v>102</v>
@@ -16726,7 +16726,7 @@
       </c>
       <c r="I14" s="241">
         <f ca="1">'Reverse DCF'!C16</f>
-        <v>351.30611132400372</v>
+        <v>350.07811261770382</v>
       </c>
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.2">
@@ -16735,7 +16735,7 @@
       </c>
       <c r="F15" s="186">
         <f ca="1">Statement!AC166</f>
-        <v>1.220223425631395E-2</v>
+        <v>1.2337593866932537E-2</v>
       </c>
     </row>
     <row r="16" spans="2:11" x14ac:dyDescent="0.2">
@@ -16768,7 +16768,7 @@
       </c>
       <c r="I17" s="236">
         <f ca="1">DCF!C15</f>
-        <v>9.7029602251831923E-2</v>
+        <v>9.7270363408778412E-2</v>
       </c>
     </row>
     <row r="18" spans="2:9" x14ac:dyDescent="0.2">
@@ -16790,7 +16790,7 @@
       </c>
       <c r="I18" s="237">
         <f ca="1">Multiples!C54</f>
-        <v>9.7994999999999999E-2</v>
+        <v>9.8250499999999991E-2</v>
       </c>
     </row>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
@@ -16863,7 +16863,7 @@
       </c>
       <c r="F26" s="213" cm="1">
         <f t="array" aca="1" ref="F26" ca="1">_FV(E26,"Price")</f>
-        <v>49.53</v>
+        <v>49.88</v>
       </c>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.2">
@@ -16878,7 +16878,7 @@
       </c>
       <c r="F27" s="214">
         <f ca="1">F26/1000</f>
-        <v>4.9530000000000005E-2</v>
+        <v>4.9880000000000001E-2</v>
       </c>
     </row>
     <row r="28" spans="2:9" x14ac:dyDescent="0.2">
@@ -21185,6 +21185,12 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="C3:G3"/>
+    <mergeCell ref="H3:L3"/>
+    <mergeCell ref="P3:W3"/>
+    <mergeCell ref="X3:Z3"/>
+    <mergeCell ref="C5:L5"/>
+    <mergeCell ref="P5:Z5"/>
     <mergeCell ref="C40:L40"/>
     <mergeCell ref="C11:L11"/>
     <mergeCell ref="P11:Z11"/>
@@ -21192,12 +21198,6 @@
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="C26:L26"/>
     <mergeCell ref="C33:L33"/>
-    <mergeCell ref="C3:G3"/>
-    <mergeCell ref="H3:L3"/>
-    <mergeCell ref="P3:W3"/>
-    <mergeCell ref="X3:Z3"/>
-    <mergeCell ref="C5:L5"/>
-    <mergeCell ref="P5:Z5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -22257,16 +22257,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="AA2:AC2"/>
+    <mergeCell ref="C4:L4"/>
+    <mergeCell ref="S4:AC4"/>
+    <mergeCell ref="C13:L13"/>
+    <mergeCell ref="C18:L18"/>
     <mergeCell ref="C31:L31"/>
     <mergeCell ref="C25:L25"/>
     <mergeCell ref="C2:G2"/>
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="S2:Z2"/>
-    <mergeCell ref="AA2:AC2"/>
-    <mergeCell ref="C4:L4"/>
-    <mergeCell ref="S4:AC4"/>
-    <mergeCell ref="C13:L13"/>
-    <mergeCell ref="C18:L18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -22388,7 +22388,7 @@
       </c>
       <c r="C6" s="133">
         <f ca="1">Overview!C5</f>
-        <v>347.72500000000002</v>
+        <v>343.91</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22397,7 +22397,7 @@
       </c>
       <c r="C7" s="134">
         <f ca="1">C5*C6</f>
-        <v>5095214.4250000007</v>
+        <v>5039313.2300000004</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22415,7 +22415,7 @@
       </c>
       <c r="C9" s="135">
         <f ca="1">Overview!F27</f>
-        <v>4.9530000000000005E-2</v>
+        <v>4.9880000000000001E-2</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22424,7 +22424,7 @@
       </c>
       <c r="C10" s="133">
         <f ca="1">Overview!C13</f>
-        <v>1.077</v>
+        <v>1.0749</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22467,7 +22467,7 @@
       </c>
       <c r="C16" s="46">
         <f ca="1">C8/(C8+C7)</f>
-        <v>1.6284013631914961E-2</v>
+        <v>1.6461678877765208E-2</v>
       </c>
     </row>
     <row r="17" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22476,7 +22476,7 @@
       </c>
       <c r="C17" s="46">
         <f ca="1">C7/(C8+C7)</f>
-        <v>0.98371598636808499</v>
+        <v>0.98353832112223483</v>
       </c>
     </row>
     <row r="18" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22494,7 +22494,7 @@
       </c>
       <c r="C19" s="46">
         <f ca="1">C9+C10*C11</f>
-        <v>9.7994999999999999E-2</v>
+        <v>9.8250499999999991E-2</v>
       </c>
     </row>
     <row r="20" spans="2:3" ht="17" customHeight="1" x14ac:dyDescent="0.2">
@@ -22503,7 +22503,7 @@
       </c>
       <c r="C20" s="46">
         <f ca="1">(C17*C19)+(C16*C18)</f>
-        <v>9.7029602251831923E-2</v>
+        <v>9.7270363408778412E-2</v>
       </c>
     </row>
   </sheetData>
@@ -22754,7 +22754,7 @@
       </c>
       <c r="L8" s="126">
         <f ca="1">L7*(1+C14)/(C15-C14)</f>
-        <v>1881804.1949815061</v>
+        <v>1875940.8169003951</v>
       </c>
       <c r="N8" s="91"/>
       <c r="O8" s="16"/>
@@ -22808,23 +22808,23 @@
       <c r="G10" s="138"/>
       <c r="H10" s="126">
         <f ca="1">H7/(1+$C$15)^H9</f>
-        <v>100598.02909234971</v>
+        <v>100575.95604756652</v>
       </c>
       <c r="I10" s="126">
         <f t="shared" ref="I10:L10" ca="1" si="0">I7/(1+$C$15)^I9</f>
-        <v>97427.674922636434</v>
+        <v>97384.924790873134</v>
       </c>
       <c r="J10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>93836.417239063201</v>
+        <v>93774.662520188504</v>
       </c>
       <c r="K10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>89962.494019650287</v>
+        <v>89883.562346361927</v>
       </c>
       <c r="L10" s="126">
         <f t="shared" ca="1" si="0"/>
-        <v>89441.728231623725</v>
+        <v>89343.645540190482</v>
       </c>
       <c r="N10" s="91"/>
     </row>
@@ -22843,7 +22843,7 @@
       <c r="K11" s="137"/>
       <c r="L11" s="126">
         <f ca="1">L8/(1+C15)^L9</f>
-        <v>1184357.1838524786</v>
+        <v>1179372.1995183637</v>
       </c>
     </row>
     <row r="13" spans="1:28" x14ac:dyDescent="0.2">
@@ -22866,7 +22866,7 @@
       </c>
       <c r="C15" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.7029602251831923E-2</v>
+        <v>9.7270363408778412E-2</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.2">
@@ -22881,7 +22881,7 @@
       </c>
       <c r="C19" s="64">
         <f ca="1">SUM(H10:L10)</f>
-        <v>471266.34350532334</v>
+        <v>470962.75124518061</v>
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.2">
@@ -22890,7 +22890,7 @@
       </c>
       <c r="C20" s="64">
         <f ca="1">L11</f>
-        <v>1184357.1838524786</v>
+        <v>1179372.1995183637</v>
       </c>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.2">
@@ -22899,7 +22899,7 @@
       </c>
       <c r="C21" s="94">
         <f ca="1">C19+C20</f>
-        <v>1655623.527357802</v>
+        <v>1650334.9507635443</v>
       </c>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.2">
@@ -22926,7 +22926,7 @@
       </c>
       <c r="C24" s="94">
         <f ca="1">C21+C22-C23</f>
-        <v>1717796.527357802</v>
+        <v>1712507.9507635443</v>
       </c>
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.2">
@@ -22944,7 +22944,7 @@
       </c>
       <c r="C26" s="235">
         <f ca="1">C24/C25</f>
-        <v>117.23172915838408</v>
+        <v>116.87080807776867</v>
       </c>
     </row>
   </sheetData>
@@ -23213,23 +23213,23 @@
       <c r="G9" s="138"/>
       <c r="H9" s="92">
         <f ca="1">DCF!H10</f>
-        <v>100598.02909234971</v>
+        <v>100575.95604756652</v>
       </c>
       <c r="I9" s="92">
         <f ca="1">DCF!I10</f>
-        <v>97427.674922636434</v>
+        <v>97384.924790873134</v>
       </c>
       <c r="J9" s="92">
         <f ca="1">DCF!J10</f>
-        <v>93836.417239063201</v>
+        <v>93774.662520188504</v>
       </c>
       <c r="K9" s="92">
         <f ca="1">DCF!K10</f>
-        <v>89962.494019650287</v>
+        <v>89883.562346361927</v>
       </c>
       <c r="L9" s="92">
         <f ca="1">DCF!L10</f>
-        <v>89441.728231623725</v>
+        <v>89343.645540190482</v>
       </c>
       <c r="N9" s="91"/>
     </row>
@@ -24015,7 +24015,7 @@
       </c>
       <c r="C41" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.7029602251831923E-2</v>
+        <v>9.7270363408778412E-2</v>
       </c>
     </row>
     <row r="42" spans="2:14" x14ac:dyDescent="0.2">
@@ -24041,7 +24041,7 @@
       </c>
       <c r="C44" s="24">
         <f ca="1">C43/(1+C41)^5</f>
-        <v>2947300.129292103</v>
+        <v>2944068.09056859</v>
       </c>
     </row>
     <row r="45" spans="2:14" x14ac:dyDescent="0.2">
@@ -24050,7 +24050,7 @@
       </c>
       <c r="C45" s="108">
         <f ca="1">SUM(H9:K9)+C44</f>
-        <v>3329124.7445658026</v>
+        <v>3325687.1962735802</v>
       </c>
     </row>
     <row r="46" spans="2:14" x14ac:dyDescent="0.2">
@@ -24077,7 +24077,7 @@
       </c>
       <c r="C48" s="94">
         <f ca="1">C45+C46-C47</f>
-        <v>3391297.7445658026</v>
+        <v>3387860.1962735802</v>
       </c>
     </row>
     <row r="49" spans="2:3" x14ac:dyDescent="0.2">
@@ -24095,7 +24095,7 @@
       </c>
       <c r="C50" s="235">
         <f ca="1">C48/C49</f>
-        <v>231.44050669254096</v>
+        <v>231.20590979823791</v>
       </c>
     </row>
     <row r="52" spans="2:3" x14ac:dyDescent="0.2">
@@ -24119,7 +24119,7 @@
       </c>
       <c r="C54" s="135">
         <f ca="1">IF(Overview!C29&gt;0,Overview!C29,WACC!C19)</f>
-        <v>9.7994999999999999E-2</v>
+        <v>9.8250499999999991E-2</v>
       </c>
     </row>
     <row r="55" spans="2:3" x14ac:dyDescent="0.2">
@@ -24154,7 +24154,7 @@
       </c>
       <c r="C58" s="235">
         <f ca="1">C57/(1+C54)^5</f>
-        <v>202.96135486625744</v>
+        <v>202.72537726530837</v>
       </c>
     </row>
     <row r="60" spans="2:3" x14ac:dyDescent="0.2">
@@ -24178,7 +24178,7 @@
       </c>
       <c r="C62" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.7029602251831923E-2</v>
+        <v>9.7270363408778412E-2</v>
       </c>
     </row>
     <row r="63" spans="2:3" x14ac:dyDescent="0.2">
@@ -24204,7 +24204,7 @@
       </c>
       <c r="C65" s="24">
         <f ca="1">C64/(1+C62)^5</f>
-        <v>2504368.3904854641</v>
+        <v>2501622.0751253334</v>
       </c>
     </row>
     <row r="66" spans="2:3" x14ac:dyDescent="0.2">
@@ -24213,7 +24213,7 @@
       </c>
       <c r="C66" s="108">
         <f ca="1">SUM(H9:K9)+C65</f>
-        <v>2886193.0057591638</v>
+        <v>2883241.1808303236</v>
       </c>
     </row>
     <row r="67" spans="2:3" x14ac:dyDescent="0.2">
@@ -24240,7 +24240,7 @@
       </c>
       <c r="C69" s="94">
         <f ca="1">C66+C67-C68</f>
-        <v>2948366.0057591638</v>
+        <v>2945414.1808303236</v>
       </c>
     </row>
     <row r="70" spans="2:3" x14ac:dyDescent="0.2">
@@ -24258,7 +24258,7 @@
       </c>
       <c r="C71" s="235">
         <f ca="1">C69/C70</f>
-        <v>201.21244835591099</v>
+        <v>201.01099985192954</v>
       </c>
     </row>
     <row r="73" spans="2:3" x14ac:dyDescent="0.2">
@@ -24282,7 +24282,7 @@
       </c>
       <c r="C75" s="135">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.7029602251831923E-2</v>
+        <v>9.7270363408778412E-2</v>
       </c>
     </row>
     <row r="76" spans="2:3" x14ac:dyDescent="0.2">
@@ -24308,7 +24308,7 @@
       </c>
       <c r="C78" s="24">
         <f ca="1">C77/(1+C75)^5</f>
-        <v>2711764.0516620292</v>
+        <v>2708790.3041509106</v>
       </c>
     </row>
     <row r="79" spans="2:3" x14ac:dyDescent="0.2">
@@ -24317,7 +24317,7 @@
       </c>
       <c r="C79" s="108">
         <f ca="1">SUM(H9:K9)+C78</f>
-        <v>3093588.6669357289</v>
+        <v>3090409.4098559008</v>
       </c>
     </row>
     <row r="80" spans="2:3" x14ac:dyDescent="0.2">
@@ -24344,7 +24344,7 @@
       </c>
       <c r="C82" s="94">
         <f ca="1">C79+C80-C81</f>
-        <v>3155761.6669357289</v>
+        <v>3152582.4098559008</v>
       </c>
     </row>
     <row r="83" spans="2:3" x14ac:dyDescent="0.2">
@@ -24362,22 +24362,22 @@
       </c>
       <c r="C84" s="235">
         <f ca="1">C82/C83</f>
-        <v>215.36625038802489</v>
+        <v>215.14928068353927</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="B73:C73"/>
+    <mergeCell ref="C27:L27"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="B60:C60"/>
     <mergeCell ref="C22:L22"/>
     <mergeCell ref="C2:G2"/>
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="C4:L4"/>
     <mergeCell ref="C11:L11"/>
     <mergeCell ref="C17:L17"/>
-    <mergeCell ref="B73:C73"/>
-    <mergeCell ref="C27:L27"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="B60:C60"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
@@ -24427,7 +24427,7 @@
       </c>
       <c r="C5" s="133">
         <f ca="1">DCF!C26</f>
-        <v>117.23172915838408</v>
+        <v>116.87080807776867</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -24436,7 +24436,7 @@
       </c>
       <c r="C6" s="133">
         <f ca="1">Multiples!C50</f>
-        <v>231.44050669254096</v>
+        <v>231.20590979823791</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
@@ -24445,7 +24445,7 @@
       </c>
       <c r="C7" s="133">
         <f ca="1">Multiples!C58</f>
-        <v>202.96135486625744</v>
+        <v>202.72537726530837</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
@@ -24454,7 +24454,7 @@
       </c>
       <c r="C8" s="133">
         <f ca="1">Multiples!C71</f>
-        <v>201.21244835591099</v>
+        <v>201.01099985192954</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
@@ -24463,7 +24463,7 @@
       </c>
       <c r="C9" s="133">
         <f ca="1">Multiples!C84</f>
-        <v>215.36625038802489</v>
+        <v>215.14928068353927</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
@@ -24472,7 +24472,7 @@
       </c>
       <c r="C10" s="235">
         <f ca="1">AVERAGE(C5:C9)</f>
-        <v>193.64245789222369</v>
+        <v>193.39247513535673</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
@@ -24481,7 +24481,7 @@
       </c>
       <c r="C11" s="133">
         <f ca="1">Overview!C5</f>
-        <v>347.72500000000002</v>
+        <v>343.91</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.2">
@@ -24490,7 +24490,7 @@
       </c>
       <c r="C12" s="149">
         <f ca="1">(C10-C11)/C11</f>
-        <v>-0.44311608917327289</v>
+        <v>-0.43766544986956846</v>
       </c>
     </row>
   </sheetData>
@@ -24999,7 +24999,7 @@
       </c>
       <c r="C24" s="135">
         <f ca="1">IF(Overview!C29&gt;0,Overview!C29,WACC!C19)</f>
-        <v>9.7994999999999999E-2</v>
+        <v>9.8250499999999991E-2</v>
       </c>
     </row>
     <row r="25" spans="2:14" x14ac:dyDescent="0.2">
@@ -25016,7 +25016,7 @@
       </c>
       <c r="C26" s="235">
         <f ca="1">C23/(C24-C25)</f>
-        <v>13.600871850759665</v>
+        <v>13.556462898000653</v>
       </c>
     </row>
   </sheetData>
@@ -25253,7 +25253,7 @@
       <c r="K8" s="137"/>
       <c r="L8" s="126">
         <f ca="1">L7*(1+C20)/(C21-C20)</f>
-        <v>6479683.0577803422</v>
+        <v>6459493.4802914327</v>
       </c>
       <c r="N8" s="91"/>
       <c r="O8" s="16"/>
@@ -25307,23 +25307,23 @@
       <c r="G10" s="138"/>
       <c r="H10" s="126">
         <f ca="1">H7/(1+$C$21)^H9</f>
-        <v>111267.19532211016</v>
+        <v>111242.78126740745</v>
       </c>
       <c r="I10" s="126">
         <f t="shared" ref="I10:L10" ca="1" si="1">I7/(1+$C$21)^I9</f>
-        <v>143517.62346030437</v>
+        <v>143454.64959463268</v>
       </c>
       <c r="J10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>185115.73140732135</v>
+        <v>184993.90482560924</v>
       </c>
       <c r="K10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>238770.91320388051</v>
+        <v>238561.41937073204</v>
       </c>
       <c r="L10" s="126">
         <f t="shared" ca="1" si="1"/>
-        <v>307977.87178210734</v>
+        <v>307640.1401755797</v>
       </c>
       <c r="N10" s="91"/>
     </row>
@@ -25342,15 +25342,15 @@
       <c r="K11" s="137"/>
       <c r="L11" s="126">
         <f ca="1">L8/(1+C21)^L9</f>
-        <v>4078139.0534867868</v>
+        <v>4060974.0803088089</v>
       </c>
     </row>
     <row r="13" spans="1:28" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="14" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="B14" s="258" t="s">
+      <c r="B14" s="259" t="s">
         <v>219</v>
       </c>
-      <c r="C14" s="259"/>
+      <c r="C14" s="260"/>
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.2">
       <c r="B15" s="150" t="s">
@@ -25358,7 +25358,7 @@
       </c>
       <c r="C15" s="151">
         <f ca="1">Overview!C5</f>
-        <v>347.72500000000002</v>
+        <v>343.91</v>
       </c>
     </row>
     <row r="16" spans="1:28" x14ac:dyDescent="0.2">
@@ -25367,7 +25367,7 @@
       </c>
       <c r="C16" s="151">
         <f ca="1">C36</f>
-        <v>351.30611132400372</v>
+        <v>350.07811261770382</v>
       </c>
     </row>
     <row r="17" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -25377,20 +25377,20 @@
       <c r="C17" s="153">
         <v>0.41499999999999998</v>
       </c>
-      <c r="E17" s="260" t="s">
+      <c r="E17" s="258" t="s">
         <v>222</v>
       </c>
-      <c r="F17" s="260"/>
-      <c r="G17" s="260"/>
-      <c r="H17" s="260"/>
-      <c r="I17" s="260"/>
+      <c r="F17" s="258"/>
+      <c r="G17" s="258"/>
+      <c r="H17" s="258"/>
+      <c r="I17" s="258"/>
     </row>
     <row r="18" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="19" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B19" s="258" t="s">
+      <c r="B19" s="259" t="s">
         <v>181</v>
       </c>
-      <c r="C19" s="259"/>
+      <c r="C19" s="260"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B20" s="154" t="s">
@@ -25406,7 +25406,7 @@
       </c>
       <c r="C21" s="216">
         <f ca="1">IF(Overview!C28&gt;0,Overview!C28,WACC!C20)</f>
-        <v>9.7029602251831923E-2</v>
+        <v>9.7270363408778412E-2</v>
       </c>
     </row>
     <row r="22" spans="2:9" x14ac:dyDescent="0.2">
@@ -25424,7 +25424,7 @@
       </c>
       <c r="C23" s="156">
         <f ca="1">C15*C22</f>
-        <v>5074698.6500000004</v>
+        <v>5019022.54</v>
       </c>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.2">
@@ -25451,15 +25451,15 @@
       </c>
       <c r="C26" s="157">
         <f ca="1">C23+C25-C24</f>
-        <v>5012525.6500000004</v>
+        <v>4956849.54</v>
       </c>
     </row>
     <row r="27" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="28" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B28" s="258" t="s">
+      <c r="B28" s="259" t="s">
         <v>183</v>
       </c>
-      <c r="C28" s="259"/>
+      <c r="C28" s="260"/>
     </row>
     <row r="29" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B29" s="154" t="s">
@@ -25467,7 +25467,7 @@
       </c>
       <c r="C29" s="156">
         <f ca="1">SUM(H10:L10)</f>
-        <v>986649.33517572377</v>
+        <v>985892.89523396117</v>
       </c>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.2">
@@ -25476,7 +25476,7 @@
       </c>
       <c r="C30" s="156">
         <f ca="1">L11</f>
-        <v>4078139.0534867868</v>
+        <v>4060974.0803088089</v>
       </c>
     </row>
     <row r="31" spans="2:9" x14ac:dyDescent="0.2">
@@ -25485,7 +25485,7 @@
       </c>
       <c r="C31" s="159">
         <f ca="1">C29+C30</f>
-        <v>5064788.3886625106</v>
+        <v>5046866.9755427698</v>
       </c>
     </row>
     <row r="32" spans="2:9" x14ac:dyDescent="0.2">
@@ -25512,7 +25512,7 @@
       </c>
       <c r="C34" s="159">
         <f ca="1">C31+C32-C33</f>
-        <v>5126961.3886625106</v>
+        <v>5109039.9755427698</v>
       </c>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.2">
@@ -25530,21 +25530,21 @@
       </c>
       <c r="C36" s="162">
         <f ca="1">C34/C35</f>
-        <v>351.30611132400372</v>
+        <v>350.07811261770382</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="P3:W3"/>
+    <mergeCell ref="X3:Z3"/>
+    <mergeCell ref="C5:L5"/>
+    <mergeCell ref="P5:Z5"/>
+    <mergeCell ref="B14:C14"/>
     <mergeCell ref="E17:I17"/>
     <mergeCell ref="B19:C19"/>
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="C3:G3"/>
     <mergeCell ref="H3:L3"/>
-    <mergeCell ref="P3:W3"/>
-    <mergeCell ref="X3:Z3"/>
-    <mergeCell ref="C5:L5"/>
-    <mergeCell ref="P5:Z5"/>
-    <mergeCell ref="B14:C14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -32049,7 +32049,7 @@
       </c>
       <c r="AC114" s="63">
         <f ca="1">Overview!C5</f>
-        <v>347.72500000000002</v>
+        <v>343.91</v>
       </c>
     </row>
     <row r="115" spans="1:31" x14ac:dyDescent="0.2">
@@ -32120,7 +32120,7 @@
       </c>
       <c r="AC115" s="65">
         <f ca="1">AC114/AC84</f>
-        <v>347.72500000000002</v>
+        <v>343.91</v>
       </c>
     </row>
     <row r="117" spans="1:31" x14ac:dyDescent="0.2">
@@ -33034,7 +33034,7 @@
       <c r="AA140" s="49"/>
       <c r="AC140" s="72">
         <f ca="1">AC115/Statement!AC25</f>
-        <v>39.876720183486249</v>
+        <v>39.439220183486249</v>
       </c>
     </row>
     <row r="141" spans="2:29" x14ac:dyDescent="0.2">
@@ -33071,7 +33071,7 @@
       <c r="AA141" s="49"/>
       <c r="AC141" s="72">
         <f ca="1">AC115/(Statement!AC5/Statement!AC21)</f>
-        <v>11.008328303768238</v>
+        <v>10.887552482418391</v>
       </c>
     </row>
     <row r="142" spans="2:29" x14ac:dyDescent="0.2">
@@ -33132,7 +33132,7 @@
       </c>
       <c r="AC142" s="72">
         <f ca="1">AC115/(Statement!AC48/Statement!AC74)</f>
-        <v>47.197718098958333</v>
+        <v>46.679897135416667</v>
       </c>
     </row>
     <row r="143" spans="2:29" x14ac:dyDescent="0.2">
@@ -33193,7 +33193,7 @@
       </c>
       <c r="AC143" s="141">
         <f ca="1">Statement!AC115*Statement!AC77</f>
-        <v>5095214.4250000007</v>
+        <v>5039313.2300000004</v>
       </c>
     </row>
     <row r="144" spans="2:29" x14ac:dyDescent="0.2">
@@ -33254,7 +33254,7 @@
       </c>
       <c r="AC144" s="141">
         <f ca="1">AC143+AC106-AC105+AC47+AC44</f>
-        <v>5033041.4250000007</v>
+        <v>4977140.2300000004</v>
       </c>
     </row>
     <row r="145" spans="2:29" x14ac:dyDescent="0.2">
@@ -33291,7 +33291,7 @@
       <c r="AA145" s="49"/>
       <c r="AC145" s="177">
         <f ca="1">AC144/AC5</f>
-        <v>10.781476973071166</v>
+        <v>10.661728813704553</v>
       </c>
     </row>
     <row r="146" spans="2:29" x14ac:dyDescent="0.2">
@@ -33328,7 +33328,7 @@
       <c r="AA146" s="49"/>
       <c r="AC146" s="177">
         <f ca="1">AC144/AC11</f>
-        <v>32.500800244093021</v>
+        <v>32.139818996635654</v>
       </c>
     </row>
     <row r="147" spans="2:29" x14ac:dyDescent="0.2">
@@ -33463,7 +33463,7 @@
       <c r="AA149" s="49"/>
       <c r="AC149" s="72">
         <f t="shared" ref="AC149:AC150" ca="1" si="137">AC143/AC147</f>
-        <v>41.432255015165445</v>
+        <v>40.977688754807815</v>
       </c>
     </row>
     <row r="150" spans="2:29" x14ac:dyDescent="0.2">
@@ -33500,7 +33500,7 @@
       <c r="AA150" s="49"/>
       <c r="AC150" s="72">
         <f t="shared" ca="1" si="137"/>
-        <v>41.089688593987901</v>
+        <v>40.633311922186159</v>
       </c>
     </row>
     <row r="151" spans="2:29" x14ac:dyDescent="0.2">
@@ -33537,7 +33537,7 @@
       <c r="AA151" s="49"/>
       <c r="AC151" s="74">
         <f t="shared" ref="AC151" ca="1" si="140">AC147/AC143</f>
-        <v>2.4135785021451767E-2</v>
+        <v>2.4403523731744689E-2</v>
       </c>
     </row>
     <row r="152" spans="2:29" x14ac:dyDescent="0.2">
@@ -33574,7 +33574,7 @@
       <c r="AA152" s="49"/>
       <c r="AC152" s="74">
         <f ca="1">AC25/AC115</f>
-        <v>2.5077288086850235E-2</v>
+        <v>2.5355470908086413E-2</v>
       </c>
     </row>
     <row r="153" spans="2:29" x14ac:dyDescent="0.2">
@@ -33611,7 +33611,7 @@
       <c r="AA153" s="49"/>
       <c r="AC153" s="149">
         <f ca="1">AC81/AC115</f>
-        <v>3.0196275792652239E-3</v>
+        <v>3.0531243639324241E-3</v>
       </c>
     </row>
     <row r="154" spans="2:29" x14ac:dyDescent="0.2">
@@ -33648,7 +33648,7 @@
       <c r="AA154" s="49"/>
       <c r="AC154" s="149">
         <f ca="1">-AC62/AC143</f>
-        <v>1.613788805365144E-2</v>
+        <v>1.6316905944741202E-2</v>
       </c>
     </row>
     <row r="155" spans="2:29" x14ac:dyDescent="0.2">
@@ -33685,7 +33685,7 @@
       <c r="AA155" s="49"/>
       <c r="AC155" s="149">
         <f ca="1">-(AC62+AC63)/AC143</f>
-        <v>1.9207435023698729E-2</v>
+        <v>1.9420503456182261E-2</v>
       </c>
     </row>
     <row r="156" spans="2:29" x14ac:dyDescent="0.2">
@@ -34188,7 +34188,7 @@
       <c r="AA166" s="49"/>
       <c r="AC166" s="149">
         <f ca="1">(AC105-AC106)/AC143</f>
-        <v>1.220223425631395E-2</v>
+        <v>1.2337593866932537E-2</v>
       </c>
     </row>
     <row r="167" spans="1:31" x14ac:dyDescent="0.2">
@@ -36240,7 +36240,7 @@
       </c>
       <c r="C5" s="166">
         <f ca="1">Overview!C5</f>
-        <v>347.72500000000002</v>
+        <v>343.91</v>
       </c>
       <c r="E5" s="12"/>
       <c r="F5" s="132" t="s">
@@ -36256,7 +36256,7 @@
       </c>
       <c r="C6" s="167">
         <f ca="1">Statement!AC143</f>
-        <v>5095214.4250000007</v>
+        <v>5039313.2300000004</v>
       </c>
       <c r="E6" s="20" t="s">
         <v>19</v>
@@ -36276,7 +36276,7 @@
       </c>
       <c r="C7" s="167">
         <f ca="1">Statement!AC144</f>
-        <v>5033041.4250000007</v>
+        <v>4977140.2300000004</v>
       </c>
       <c r="E7" s="20" t="s">
         <v>29</v>
@@ -36296,7 +36296,7 @@
       </c>
       <c r="C8" s="168">
         <f ca="1">Statement!AC140</f>
-        <v>39.876720183486249</v>
+        <v>39.439220183486249</v>
       </c>
       <c r="E8" s="20" t="s">
         <v>237</v>
@@ -36316,7 +36316,7 @@
       </c>
       <c r="C9" s="168">
         <f ca="1">Statement!AC141</f>
-        <v>11.008328303768238</v>
+        <v>10.887552482418391</v>
       </c>
       <c r="E9" s="20" t="s">
         <v>238</v>
@@ -36336,7 +36336,7 @@
       </c>
       <c r="C10" s="168">
         <f ca="1">Statement!AC142</f>
-        <v>47.197718098958333</v>
+        <v>46.679897135416667</v>
       </c>
       <c r="E10" s="20" t="s">
         <v>1</v>
@@ -36356,7 +36356,7 @@
       </c>
       <c r="C11" s="168">
         <f ca="1">Statement!AC145</f>
-        <v>10.781476973071166</v>
+        <v>10.661728813704553</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.2">
@@ -36365,7 +36365,7 @@
       </c>
       <c r="C12" s="168">
         <f ca="1">Statement!AC146</f>
-        <v>32.500800244093021</v>
+        <v>32.139818996635654</v>
       </c>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.2">
@@ -36601,7 +36601,7 @@
       </c>
       <c r="C38" s="169">
         <f ca="1">Statement!AC152</f>
-        <v>2.5077288086850235E-2</v>
+        <v>2.5355470908086413E-2</v>
       </c>
       <c r="E38" s="20" t="s">
         <v>264</v>
@@ -36617,7 +36617,7 @@
       </c>
       <c r="C39" s="209">
         <f ca="1">Statement!AC151</f>
-        <v>2.4135785021451767E-2</v>
+        <v>2.4403523731744689E-2</v>
       </c>
       <c r="E39" s="20" t="s">
         <v>266</v>
@@ -36633,7 +36633,7 @@
       </c>
       <c r="C40" s="169">
         <f ca="1">Statement!AC153</f>
-        <v>3.0196275792652239E-3</v>
+        <v>3.0531243639324241E-3</v>
       </c>
       <c r="E40" s="20" t="s">
         <v>267</v>
@@ -36649,7 +36649,7 @@
       </c>
       <c r="C41" s="169">
         <f ca="1">Statement!AC154</f>
-        <v>1.613788805365144E-2</v>
+        <v>1.6316905944741202E-2</v>
       </c>
     </row>
     <row r="42" spans="2:6" x14ac:dyDescent="0.2">
@@ -36658,7 +36658,7 @@
       </c>
       <c r="C42" s="169">
         <f ca="1">Statement!AC155</f>
-        <v>1.9207435023698729E-2</v>
+        <v>1.9420503456182261E-2</v>
       </c>
     </row>
     <row r="45" spans="2:6" x14ac:dyDescent="0.2">
@@ -36702,7 +36702,7 @@
       </c>
       <c r="F48" s="169">
         <f ca="1">Statement!AC166</f>
-        <v>1.220223425631395E-2</v>
+        <v>1.2337593866932537E-2</v>
       </c>
     </row>
     <row r="51" spans="2:6" x14ac:dyDescent="0.2">
@@ -36881,7 +36881,7 @@
       </c>
       <c r="I6" s="166">
         <f ca="1">Statement!AC114</f>
-        <v>347.72500000000002</v>
+        <v>343.91</v>
       </c>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.2">
@@ -36910,7 +36910,7 @@
       </c>
       <c r="I7" s="167">
         <f ca="1">Statement!AC143</f>
-        <v>5095214.4250000007</v>
+        <v>5039313.2300000004</v>
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
@@ -36939,7 +36939,7 @@
       </c>
       <c r="I8" s="167">
         <f ca="1">Statement!AC144</f>
-        <v>5033041.4250000007</v>
+        <v>4977140.2300000004</v>
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.2">
@@ -36968,7 +36968,7 @@
       </c>
       <c r="I9" s="168">
         <f ca="1">Statement!AC140</f>
-        <v>39.876720183486249</v>
+        <v>39.439220183486249</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.2">
@@ -36997,7 +36997,7 @@
       </c>
       <c r="I10" s="168">
         <f ca="1">Statement!AC141</f>
-        <v>11.008328303768238</v>
+        <v>10.887552482418391</v>
       </c>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.2">
@@ -37026,7 +37026,7 @@
       </c>
       <c r="I11" s="168">
         <f ca="1">Statement!AC142</f>
-        <v>47.197718098958333</v>
+        <v>46.679897135416667</v>
       </c>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.2">
@@ -37055,7 +37055,7 @@
       </c>
       <c r="I12" s="168">
         <f ca="1">Statement!AC145</f>
-        <v>10.781476973071166</v>
+        <v>10.661728813704553</v>
       </c>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.2">
@@ -37084,7 +37084,7 @@
       </c>
       <c r="I13" s="168">
         <f ca="1">Statement!AC146</f>
-        <v>32.500800244093021</v>
+        <v>32.139818996635654</v>
       </c>
     </row>
     <row r="15" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -37857,7 +37857,7 @@
       </c>
       <c r="I51" s="169">
         <f ca="1">Statement!AC152</f>
-        <v>2.5077288086850235E-2</v>
+        <v>2.5355470908086413E-2</v>
       </c>
     </row>
     <row r="52" spans="2:9" x14ac:dyDescent="0.2">
@@ -37886,7 +37886,7 @@
       </c>
       <c r="I52" s="169">
         <f ca="1">Statement!AC151</f>
-        <v>2.4135785021451767E-2</v>
+        <v>2.4403523731744689E-2</v>
       </c>
     </row>
     <row r="53" spans="2:9" x14ac:dyDescent="0.2">
@@ -37915,7 +37915,7 @@
       </c>
       <c r="I53" s="169">
         <f ca="1">Statement!AC153</f>
-        <v>3.0196275792652239E-3</v>
+        <v>3.0531243639324241E-3</v>
       </c>
     </row>
     <row r="54" spans="2:9" x14ac:dyDescent="0.2">
@@ -37944,7 +37944,7 @@
       </c>
       <c r="I54" s="169">
         <f ca="1">Statement!AC154</f>
-        <v>1.613788805365144E-2</v>
+        <v>1.6316905944741202E-2</v>
       </c>
     </row>
     <row r="55" spans="2:9" x14ac:dyDescent="0.2">
@@ -37973,7 +37973,7 @@
       </c>
       <c r="I55" s="169">
         <f ca="1">Statement!AC155</f>
-        <v>1.9207435023698729E-2</v>
+        <v>1.9420503456182261E-2</v>
       </c>
     </row>
     <row r="57" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -38209,7 +38209,7 @@
       </c>
       <c r="I68" s="190">
         <f ca="1">Statement!AC166</f>
-        <v>1.220223425631395E-2</v>
+        <v>1.2337593866932537E-2</v>
       </c>
     </row>
     <row r="70" spans="2:9" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -38901,14 +38901,14 @@
     <row r="1" spans="2:7" ht="12" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="3" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B3" s="8"/>
-      <c r="C3" s="247" t="s">
+      <c r="C3" s="249" t="s">
         <v>307</v>
       </c>
-      <c r="D3" s="248"/>
-      <c r="F3" s="249" t="s">
+      <c r="D3" s="250"/>
+      <c r="F3" s="251" t="s">
         <v>308</v>
       </c>
-      <c r="G3" s="248"/>
+      <c r="G3" s="250"/>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B4" s="8"/>
@@ -38975,19 +38975,19 @@
       <c r="B7" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C7" s="250">
+      <c r="C7" s="247">
         <f>Statement!AA88</f>
         <v>-1.5892574471146927E-2</v>
       </c>
-      <c r="D7" s="251"/>
-      <c r="F7" s="250">
+      <c r="D7" s="248"/>
+      <c r="F7" s="247">
         <f>IF(F6=0,
 IF(G6=0,0,IF(G6&gt;0,1,-1)),
 (G6-F6)/ABS(F6)
 )</f>
         <v>0.16356501765281381</v>
       </c>
-      <c r="G7" s="251"/>
+      <c r="G7" s="248"/>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B8" s="201" t="s">
@@ -39014,19 +39014,19 @@
       <c r="B9" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C9" s="250">
+      <c r="C9" s="247">
         <f>Statement!AA89</f>
         <v>-3.1133095757317875E-2</v>
       </c>
-      <c r="D9" s="251"/>
-      <c r="F9" s="250">
+      <c r="D9" s="248"/>
+      <c r="F9" s="247">
         <f>IF(F8=0,
 IF(G8=0,0,IF(G8&gt;0,1,-1)),
 (G8-F8)/ABS(F8)
 )</f>
         <v>8.6032831193608647E-2</v>
       </c>
-      <c r="G9" s="251"/>
+      <c r="G9" s="248"/>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B10" s="201" t="s">
@@ -39053,19 +39053,19 @@
       <c r="B11" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C11" s="250">
+      <c r="C11" s="247">
         <f>Statement!AA90</f>
         <v>-2.0079954728829339E-4</v>
       </c>
-      <c r="D11" s="251"/>
-      <c r="F11" s="250">
+      <c r="D11" s="248"/>
+      <c r="F11" s="247">
         <f>IF(F10=0,
 IF(G10=0,0,IF(G10&gt;0,1,-1)),
 (G10-F10)/ABS(F10)
 )</f>
         <v>0.25280204949906215</v>
       </c>
-      <c r="G11" s="251"/>
+      <c r="G11" s="248"/>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B12" s="201" t="s">
@@ -39092,19 +39092,19 @@
       <c r="B13" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C13" s="250">
+      <c r="C13" s="247">
         <f>Statement!AA93</f>
         <v>9.4729043183742583E-3</v>
       </c>
-      <c r="D13" s="251"/>
-      <c r="F13" s="250">
+      <c r="D13" s="248"/>
+      <c r="F13" s="247">
         <f>IF(F12=0,
 IF(G12=0,0,IF(G12&gt;0,1,-1)),
 (G12-F12)/ABS(F12)
 )</f>
         <v>0.22937612786800721</v>
       </c>
-      <c r="G13" s="251"/>
+      <c r="G13" s="248"/>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B14" s="201" t="s">
@@ -39131,19 +39131,19 @@
       <c r="B15" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C15" s="250">
+      <c r="C15" s="247">
         <f>Statement!AA94</f>
         <v>-5.2946913752264175E-3</v>
       </c>
-      <c r="D15" s="251"/>
-      <c r="F15" s="250">
+      <c r="D15" s="248"/>
+      <c r="F15" s="247">
         <f>IF(F14=0,
 IF(G14=0,0,IF(G14&gt;0,1,-1)),
 (G14-F14)/ABS(F14)
 )</f>
         <v>0.26569037656903766</v>
       </c>
-      <c r="G15" s="251"/>
+      <c r="G15" s="248"/>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B16" s="201" t="s">
@@ -39170,19 +39170,19 @@
       <c r="B17" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C17" s="250">
+      <c r="C17" s="247">
         <f>Statement!AA96</f>
         <v>7.1336804381635002E-3</v>
       </c>
-      <c r="D17" s="251"/>
-      <c r="F17" s="250">
+      <c r="D17" s="248"/>
+      <c r="F17" s="247">
         <f>IF(F16=0,
 IF(G16=0,0,IF(G16&gt;0,1,-1)),
 (G16-F16)/ABS(F16)
 )</f>
         <v>0.27118716394981651</v>
       </c>
-      <c r="G17" s="251"/>
+      <c r="G17" s="248"/>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B18" s="201" t="s">
@@ -39209,22 +39209,22 @@
       <c r="B19" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C19" s="250">
+      <c r="C19" s="247">
         <f>IF(C18=0,
 IF(D18=0,0,IF(D18&gt;0,1,-1)),
 (D18-C18)/ABS(C18)
 )</f>
         <v>-7.4697813391280731E-4</v>
       </c>
-      <c r="D19" s="251"/>
-      <c r="F19" s="250">
+      <c r="D19" s="248"/>
+      <c r="F19" s="247">
         <f>IF(F18=0,
 IF(G18=0,0,IF(G18&gt;0,1,-1)),
 (G18-F18)/ABS(F18)
 )</f>
         <v>-1.5587369547765587E-2</v>
       </c>
-      <c r="G19" s="251"/>
+      <c r="G19" s="248"/>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B20" s="201" t="s">
@@ -39251,22 +39251,22 @@
       <c r="B21" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C21" s="250">
+      <c r="C21" s="247">
         <f>IF(C20=0,
 IF(D20=0,0,IF(D20&gt;0,1,-1)),
 (D20-C20)/ABS(C20)
 )</f>
         <v>4.975124378109568E-3</v>
       </c>
-      <c r="D21" s="251"/>
-      <c r="F21" s="250">
+      <c r="D21" s="248"/>
+      <c r="F21" s="247">
         <f>IF(F20=0,
 IF(G20=0,0,IF(G20&gt;0,1,-1)),
 (G20-F20)/ABS(F20)
 )</f>
         <v>0.28662420382165599</v>
       </c>
-      <c r="G21" s="251"/>
+      <c r="G21" s="248"/>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23" s="8" t="s">
@@ -39314,22 +39314,22 @@
       <c r="B25" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C25" s="250">
+      <c r="C25" s="247">
         <f>IF(C24=0,
 IF(D24=0,0,IF(D24&gt;0,1,-1)),
 (D24-C24)/ABS(C24)
 )</f>
         <v>1.5257357017718937E-2</v>
       </c>
-      <c r="D25" s="251"/>
-      <c r="F25" s="250">
+      <c r="D25" s="248"/>
+      <c r="F25" s="247">
         <f>IF(F24=0,
 IF(G24=0,0,IF(G24&gt;0,1,-1)),
 (G24-F24)/ABS(F24)
 )</f>
         <v>0.11124326423612797</v>
       </c>
-      <c r="G25" s="251"/>
+      <c r="G25" s="248"/>
     </row>
     <row r="26" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B26" s="20" t="s">
@@ -39356,22 +39356,22 @@
       <c r="B27" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C27" s="250">
+      <c r="C27" s="247">
         <f>IF(C26=0,
 IF(D26=0,0,IF(D26&gt;0,1,-1)),
 (D26-C26)/ABS(C26)
 )</f>
         <v>4.7692033505613969E-2</v>
       </c>
-      <c r="D27" s="251"/>
-      <c r="F27" s="250">
+      <c r="D27" s="248"/>
+      <c r="F27" s="247">
         <f>IF(F26=0,
 IF(G26=0,0,IF(G26&gt;0,1,-1)),
 (G26-F26)/ABS(F26)
 )</f>
         <v>0.22399433663696178</v>
       </c>
-      <c r="G27" s="251"/>
+      <c r="G27" s="248"/>
     </row>
     <row r="28" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B28" s="20" t="s">
@@ -39398,22 +39398,22 @@
       <c r="B29" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C29" s="250">
+      <c r="C29" s="247">
         <f>IF(C28=0,
 IF(D28=0,0,IF(D28&gt;0,1,-1)),
 (D28-C28)/ABS(C28)
 )</f>
         <v>-8.2012001756354591E-2</v>
       </c>
-      <c r="D29" s="251"/>
-      <c r="F29" s="250">
+      <c r="D29" s="248"/>
+      <c r="F29" s="247">
         <f>IF(F28=0,
 IF(G28=0,0,IF(G28&gt;0,1,-1)),
 (G28-F28)/ABS(F28)
 )</f>
         <v>0.22428264688658989</v>
       </c>
-      <c r="G29" s="251"/>
+      <c r="G29" s="248"/>
     </row>
     <row r="30" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B30" s="20" t="s">
@@ -39440,22 +39440,22 @@
       <c r="B31" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C31" s="250">
+      <c r="C31" s="247">
         <f>IF(C30=0,
 IF(D30=0,0,IF(D30&gt;0,1,-1)),
 (D30-C30)/ABS(C30)
 )</f>
         <v>-0.21985477919295321</v>
       </c>
-      <c r="D31" s="251"/>
-      <c r="F31" s="250">
+      <c r="D31" s="248"/>
+      <c r="F31" s="247">
         <f>IF(F30=0,
 IF(G30=0,0,IF(G30&gt;0,1,-1)),
 (G30-F30)/ABS(F30)
 )</f>
         <v>0.1335178139052231</v>
       </c>
-      <c r="G31" s="251"/>
+      <c r="G31" s="248"/>
     </row>
     <row r="32" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B32" s="20" t="s">
@@ -39482,22 +39482,22 @@
       <c r="B33" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C33" s="250">
+      <c r="C33" s="247">
         <f>IF(C32=0,
 IF(D32=0,0,IF(D32&gt;0,1,-1)),
 (D32-C32)/ABS(C32)
 )</f>
         <v>-2.9218647406434668E-2</v>
       </c>
-      <c r="D33" s="251"/>
-      <c r="F33" s="250">
+      <c r="D33" s="248"/>
+      <c r="F33" s="247">
         <f>IF(F32=0,
 IF(G32=0,0,IF(G32&gt;0,1,-1)),
 (G32-F32)/ABS(F32)
 )</f>
         <v>0.15613189104652678</v>
       </c>
-      <c r="G33" s="251"/>
+      <c r="G33" s="248"/>
     </row>
     <row r="35" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B35" s="224" t="s">
@@ -39524,22 +39524,22 @@
       <c r="B36" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C36" s="250">
+      <c r="C36" s="247">
         <f>IF(C35=0,
 IF(D35=0,0,IF(D35&gt;0,1,-1)),
 (D35-C35)/ABS(C35)
 )</f>
         <v>-4.8110327402884512E-2</v>
       </c>
-      <c r="D36" s="251"/>
-      <c r="F36" s="250">
+      <c r="D36" s="248"/>
+      <c r="F36" s="247">
         <f>IF(F35=0,
 IF(G35=0,0,IF(G35&gt;0,1,-1)),
 (G35-F35)/ABS(F35)
 )</f>
         <v>0.21690368310080302</v>
       </c>
-      <c r="G36" s="251"/>
+      <c r="G36" s="248"/>
     </row>
     <row r="37" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B37" s="224" t="s">
@@ -39566,22 +39566,22 @@
       <c r="B38" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C38" s="250">
+      <c r="C38" s="247">
         <f>IF(C37=0,
 IF(D37=0,0,IF(D37&gt;0,1,-1)),
 (D37-C37)/ABS(C37)
 )</f>
         <v>0.23252768186688891</v>
       </c>
-      <c r="D38" s="251"/>
-      <c r="F38" s="250">
+      <c r="D38" s="248"/>
+      <c r="F38" s="247">
         <f>IF(F37=0,
 IF(G37=0,0,IF(G37&gt;0,1,-1)),
 (G37-F37)/ABS(F37)
 )</f>
         <v>0.28660203827989061</v>
       </c>
-      <c r="G38" s="251"/>
+      <c r="G38" s="248"/>
     </row>
     <row r="39" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B39" s="224" t="s">
@@ -39608,22 +39608,22 @@
       <c r="B40" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C40" s="250">
+      <c r="C40" s="247">
         <f>IF(C39=0,
 IF(D39=0,0,IF(D39&gt;0,1,-1)),
 (D39-C39)/ABS(C39)
 )</f>
         <v>-0.10457043679490888</v>
       </c>
-      <c r="D40" s="251"/>
-      <c r="F40" s="250">
+      <c r="D40" s="248"/>
+      <c r="F40" s="247">
         <f>IF(F39=0,
 IF(G39=0,0,IF(G39&gt;0,1,-1)),
 (G39-F39)/ABS(F39)
 )</f>
         <v>-5.9261510408752466E-2</v>
       </c>
-      <c r="G40" s="251"/>
+      <c r="G40" s="248"/>
     </row>
     <row r="41" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B41" s="224" t="s">
@@ -39650,22 +39650,22 @@
       <c r="B42" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C42" s="250">
+      <c r="C42" s="247">
         <f>IF(C41=0,
 IF(D41=0,0,IF(D41&gt;0,1,-1)),
 (D41-C41)/ABS(C41)
 )</f>
         <v>-2.2781926338438173E-3</v>
       </c>
-      <c r="D42" s="251"/>
-      <c r="F42" s="250">
+      <c r="D42" s="248"/>
+      <c r="F42" s="247">
         <f>IF(F41=0,
 IF(G41=0,0,IF(G41&gt;0,1,-1)),
 (G41-F41)/ABS(F41)
 )</f>
         <v>6.4694759589411135E-2</v>
       </c>
-      <c r="G42" s="251"/>
+      <c r="G42" s="248"/>
     </row>
     <row r="43" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B43" s="224" t="s">
@@ -39692,25 +39692,55 @@
       <c r="B44" s="200" t="s">
         <v>309</v>
       </c>
-      <c r="C44" s="250">
+      <c r="C44" s="247">
         <f>IF(C43=0,
 IF(D43=0,0,IF(D43&gt;0,1,-1)),
 (D43-C43)/ABS(C43)
 )</f>
         <v>-7.6510847107438013E-3</v>
       </c>
-      <c r="D44" s="251"/>
-      <c r="F44" s="250">
+      <c r="D44" s="248"/>
+      <c r="F44" s="247">
         <f>IF(F43=0,
 IF(G43=0,0,IF(G43&gt;0,1,-1)),
 (G43-F43)/ABS(F43)
 )</f>
         <v>0.12092039528862633</v>
       </c>
-      <c r="G44" s="251"/>
+      <c r="G44" s="248"/>
     </row>
   </sheetData>
   <mergeCells count="38">
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="C25:D25"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="C27:D27"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="C29:D29"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="C31:D31"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="C36:D36"/>
+    <mergeCell ref="F36:G36"/>
     <mergeCell ref="C44:D44"/>
     <mergeCell ref="F44:G44"/>
     <mergeCell ref="C38:D38"/>
@@ -39719,36 +39749,6 @@
     <mergeCell ref="F40:G40"/>
     <mergeCell ref="C42:D42"/>
     <mergeCell ref="F42:G42"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="C36:D36"/>
-    <mergeCell ref="F36:G36"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="C27:D27"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="C9:D9"/>
-    <mergeCell ref="F9:G9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>

</xml_diff>